<commit_message>
fix: prevent insurer row duplication in Pass 3 secondary root matching
  Secondary root matching used allow_sharing=True, which let the same
  insurer row be claimed by multiple partial groups. This caused insurer
  rows to appear duplicated across groups in the Partial Matches sheet
  (e.g., FAIRSTONE rows appearing in both the FAIRSTONE primary group
  and TAMARIN SAVANNAH secondary group via the shared fragment
  "CONTRACTORS"). Changed to allow_sharing=False so that once an insurer
  row is claimed by a primary group, secondary groups cannot reclaim it.
</commit_message>
<xml_diff>
--- a/data/history.xlsx
+++ b/data/history.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_43C55FAC0A5A7B599DFF561A1C56D84A4F6ECDDF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EE7B733-E70F-48FE-A32A-9F634321852D}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_1D42FFDF252A7E4E413E56FC0C13C9644F653085" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA32C618-A899-4F91-BE1C-506345A51F8B}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="127">
   <si>
     <t>ActionType</t>
   </si>
@@ -72,118 +72,346 @@
     <t>move</t>
   </si>
   <si>
+    <t>["-546|-546|66.67|15|CAFE MAME LTD|-0.33|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|Mise en demeure|03/12/2025|479.35|67|01-07-2025 to 01-09-2025|POL-F&amp;A-Jun-21-16\\R3|POL-F&amp;A-Jun-21-16\\R3\\E1|101.56|33594/25|444.46|-479.33244203509025|","-99|-99|14.79|15|CAFE MAME LTD|-0.21|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|Mise en demeure|03/12/2025|84.16|15|01-07-2025 to 01-09-2025|POL-EL-Jun-21-22\\R3|POL-EL-Jun-21-22\\R3\\E1|0.35|33594/25|98.6|-84.20252652854977|","-112|-112|16.71|15|CAFE MAME LTD|-0.29|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)|Mise en demeure|03/12/2025|95.11|17|01-07-2025 to 01-09-2025|POL-LOP(F&amp;A)-Jun-21-8\\R3|POL-LOP(F&amp;A)-Jun-21-8\\R3\\E1|0.39|33594/25|111.43|-95.26310141298515|","-94|-94|14.05|15|CAFE MAME LTD|0.05|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT|Mise en demeure|03/12/2025|79.92|14|01-07-2025 to 01-09-2025|POL-EE-Jun-21-8\\R3|POL-EE-Jun-21-8\\R3\\E1|0.33|33594/25|93.64|-79.94551452591253|","-320|-320|47.76|15|CAFE MAME LTD|-0.24|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY|Mise en demeure|03/12/2025|271.75|48|01-07-2025 to 01-09-2025|POL-PPL-Jun-21-1009\\R3|POL-PPL-Jun-21-1009\\R3\\E1|1.11|33594/25|318.4|-272.1667553441207|","-29885|-29885|5172.56|8|DALAIS MARIE ANNE JACQUELINE MRS|3984.98|0||MUR|01/08/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH|Mise en demeure|14/08/2025|59884.44|1187.58|01-08-2025 to 01-08-2026|POL-HEALTH-Jul-19-2912\\R6|POL-HEALTH-Jul-19-2912\\R6|400|MD17M00728/4/R6|64657|-27508.899724856663|","-19880|-19880|10365.12|12|DOOKHONY HEENA MRS|7990.64|0||MUR|01/01/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH|Mise en demeure|25/04/2025|76410.88|2374.48|01-01-2025 to 01-01-2026|POL-HEALTH-Feb-25-20|POL-HEALTH-Feb-25-20|400|MED/2025/00428|86376|-17505.396588918593|","38332|38332|-3066.58|8|MASSOOD BIBI THARAA SARAH MISS|0.42|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH|Mise en demeure|15/10/2025|-35265.61|-3067|01-09-2025 to 01-06-2026|POL-HEALTH-May-23-37\\R2|POL-HEALTH-May-23-37\\R2\\E1|0|MED/2023/01143/R2|-38332.19|35265.43520002379|","-51650|-51650|4100|8|MASSOOD BIBI THARAA SARAH MISS|0|0||MUR|01/06/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH|Mise en demeure|12/06/2025|47550|4100|01-06-2025 to 01-06-2026|POL-HEALTH-May-23-37\\R2|POL-HEALTH-May-23-37\\R2|400|MED/2023/01143/R2|51250|-47550|","-5487|-5487|805.2|15|MR WENDIP APPAYA|0.2|100||MUR|01/11/2024|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE|Mise en demeure|20/11/2024|4681.6|805|01-11-2024 to 01-11-2025|POL-MV-Jun-19-6016\\R5|POL-MV-Jun-19-6016\\R5|18.8|18607/19|5368|-4681.770649558941|"]</t>
+  </si>
+  <si>
     <t>[]</t>
   </si>
   <si>
-    <t>["||WEST BY MJ LTD (SITE A)||14/01/2026||153696|01/05/2023 - 30/06/2026|DN52706012026000004|153696|||0","||WEST BY MJ LTD (SITE B)||14/01/2026||759983|01/05/2024 - 31/12/2026|DN52706012026000005|759983|||0"]</t>
-  </si>
-  <si>
-    <t>["Payment done after 30.06.2026","Payment done after 30.06.2026"]</t>
+    <t>["Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure"]</t>
   </si>
   <si>
     <t>no-match</t>
   </si>
   <si>
+    <t>mise_en_demeure</t>
+  </si>
+  <si>
+    <t>2026-07-28T06:36:25.730Z</t>
+  </si>
+  <si>
+    <t>["-62.85|422|CANDY PALACE LTD|01/09/2026||Payment done after 30.06.2026|01/07/25 to 30/06/26|POL-MVF-Dec-22-1017\\R3\\E11|31142/22/R3/E6|POL-MVF-Dec-22-1017\\R3\\E11|359.15|24/06/2026|JRNI.260624.210|Motor","-35128.35|235109|DANIELLE DE FLEURIOT ENTERPRISE LTD|01/09/2026||Payment done after 30.06.2026|01/07/26 to 30/06/27|POL-MV-Jul-25-301\\R1|19158/25/R1|POL-MV-Jul-25-301\\R1|199980.65|16/06/2026|JRNI.260616.52|Motor","-2696.85|18142|FAYDHERBE DE MAUDAVE Marie Anne Sylvie|01/09/2026||Payment done after 30.06.2026|01/07/26 to 30/06/27|POL-MV-Jul-20-1275\\R6|13575/20/R6|POL-MV-Jul-20-1275\\R6|15445.15|16/06/2026|JRNI.260616.245|Motor","-2502.45|16841|Kian Fat Valerie|01/07/2026|9559.58|Payment done after 30.06.2026|01/05/26 to 30/04/27|POL-MV-Jun-19-6033\\R7|17498/19/R7|POL-MV-Jun-19-6033\\R7|9559.58|27/04/2026|JRNI.260427.85|Motor","-3636|24525|LINCOLN Joseph Yves|01/07/2026|20889|Payment done after 30.06.2026|01/05/26 to 30/04/27|POL-MIS-May-23-71\\R3|11986/23/R3|POL-MIS-May-23-71\\R3|20889|15/04/2026|JRNI.260415.92|Motor","-3045.9|20577|MILLE FEUX LTEE|01/07/2026|17531.1|Payment done after 30.06.2026|01/04/26 to 31/03/27|POL-GIT-Apr-20-1020\\R6|19292/14/R12|POL-GIT-Apr-20-1020\\R6|17531.1|22/04/2026|JRNI.260422.338|Inland Transit","-4781.7|32090|MOOTOOSAMY Aelander Ishwaree|01/11/2025|27308.3|Payment done after 30.06.2026|01/09/25 to 31/08/26|POL-MV-May-19-2370\\R7|29682/18/R7|POL-MV-May-19-2370\\R7|27308.3|26/08/2025|JRNI.250826.79|Motor","-18312|2670|The Brandhouse Ltd|01/10/2025||Payment done after 30.06.2026|28/03/25 to 27/03/26||22482/25/N/E1||-15642|19/09/2025|JRNI.250919.324|Non-Motor Corporate","-49|6.9|The Brandhouse Ltd|22/09/2025||Payment done after 30.06.2026|26/03/25 to 30/09/25||23712/25/N/E1||-42.1|22/09/2025|JRNI.250922.289|Non-Motor Corporate"]</t>
+  </si>
+  <si>
+    <t>["CBL Payment done after 30.06.2026","CBL Payment done after 30.06.2026","CBL Payment done after 30.06.2026","CBL Payment done after 30.06.2026","CBL Payment done after 30.06.2026","CBL Payment done after 30.06.2026","CBL Payment done after 30.06.2026","CBL Payment done after 30.06.2026","CBL Payment done after 30.06.2026"]</t>
+  </si>
+  <si>
     <t>timing_differences</t>
   </si>
   <si>
-    <t>2026-07-29T11:09:15.516Z</t>
-  </si>
-  <si>
-    <t>["-464472|-464472|86336.25|15|KI SIGNATURE VILLAS LTD &amp;/OR SUBSEQUENT OWNERS|17267.51|0|MUR|31/01/2024|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|31/03/2023|494253.26|69068.74|31-01-2024 to 31-01-2034|POL-DEF-Feb-23-1001|POL-DEF-Feb-23-1001|5014.51||575575|-395402.94170785137|","-407563|-407563|75703.13|15|KI SIGNATURE VILLAS LTD &amp;/OR SUBSEQUENT OWNERS|15140.79|0|MUR|04/12/2024|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|16/11/2023|433750.78|60562.34|04-12-2024 to 04-12-2034|POL-DEF-Oct-23-1027|POL-DEF-Oct-23-1027|4766.41||504687.5|-347000.5150203676|","-2976332|-2976332|493876.77|15|TAMARIN SAVANNAH LTD &amp;/OR SUBSEQUENT OWNERS|49387.51|0|MUR|01/04/2025|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|31/08/2023|2813158.83|444489.26|01-04-2025 to 01-04-2035|POL-DEF-Jul-23-1022|POL-DEF-Jul-23-1022|14523.79||3292511.81|-2531842.9129736493|","-2748986|-2748986|456117.89|15|TAMARIN SAVANNAH LTD &amp;/OR SUBSEQUENT OWNERS|45611.7|0|MUR|01/04/2025|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|31/08/2023|2598310.82|410506.19|01-04-2025 to 01-04-2035|POL-DEF-Jul-23-1023|POL-DEF-Jul-23-1023|13642.75||3040785.96|-2338479.8749578674|","-3230|-3230|759810.42|15|TAMARIN SAVANNAH LTD &amp;/OR SUBSEQUENT OWNERS|759328.25|0|MUR|01/09/2025|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|31/08/2023|4326321.29|482.169999999925|01-09-2025 to 01-09-2035|POL-DEF-Jul-23-1024|POL-DEF-Jul-23-1024|20728.91||5065402.8|-2747.4746159689994|","-4417745|-4417745|733125|15|WESTBYMJ LTD &amp;/OR SUBSEQUENT OWNERS,|73312.5600000001|0|MUR|01/07/2024|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|13/12/2023|4175481.25|659812.44|01-07-2024 to 01-07-2034|POL-DEF-Oct-23-1025|POL-DEF-Oct-23-1025|21106.25|.|4887500|-3757932.5933468896|","-6040593|-6040593|1002656.25|15|WESTBYMJ LTD &amp;/OR SUBSEQUENT OWNERS,|100265.87|0|MUR|01/01/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|15/05/2024|5709114.06|902390.38|01-01-2026 to 01-01-2036|POL-DEF-Oct-23-1026|POL-DEF-Oct-23-1026|27395.31|.|6684375|-5138202.416679181|","-639491|-639491|95589.15|15|FRENCH TOUCH LTD &amp;/OR SUBSEQUENT OWNERS|0.15|0|MUR|06/02/2024|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|18/06/2024|543902.26|95589|06-02-2024 to 06-02-2034|POL-DEF-Jun-24-1007|POL-DEF-Jun-24-1007|2230.41||637261|-543901.9112855011|","-2623057|-2623057|488986.76|15|AZURI SMART CITY COMPANY LTD &amp;/OR SUBSEQUENT OWNERS|97797.07|0|MUR|01/05/2027|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|22/09/2025|2789834.69|391189.69|01-05-2027 to 30-04-2037|POL-DEF-Aug-25-1023|POL-DEF-Aug-25-1023|18909.69|DN52706092025000018|3259911.76|-2231867.6158615863|Timing Difference","-8540560|-8540560|1594275|15|AZURI SMART CITY COMPANY LTD &amp;/OR SUBSEQUENT OWNERS|318855.01|0|MUR|19/06/2027|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|23/06/2025|9081424.75|1275419.99|19-06-2027 to 18-06-2037|POL-DEF-Jun-25-1019|POL-DEF-Jun-25-1019|47199.75|DN52706092025000010|10628500|-7265139.970132637|Timing Difference","-2843778|-2843778|530227.62|15|AZURI SMART CITY COMPANY LTD &amp;/OR SUBSEQUENT OWNERS|106045.21|0|MUR|01/10/2025|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|15/05/2024|3024495.13|424182.41|01-10-2025 to 01-10-2035|POL-DEF-May-24-1006|POL-DEF-May-24-1006|19871.98||3534850.77|-2419595.933832291|","-1006700|-1006700|187500|15|AMARE17.1  LTD &amp;/OR MNJ PROPERTIES LTD &amp;/OR SUBSEQUENT OWNERS|37500|0|MUR|27/10/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|16/07/2025|1070875|150000|27-10-2026 to 26-10-2036|POL-DEF-Dec-24-1017|POL-DEF-Dec-24-1017\\E2|8375||1250000|-856700|Timing Difference","-2261875|-2261875|421875|15|SEKOYA17 LTD &amp;/OR MNJ PROPERTIES LTD &amp;/OR SUBSEQUENT OWNERS|84375.04|0|MUR|01/01/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|28/06/2024|2405468.75|337499.96|01-01-2026 to 01-01-2036|POL-DEF-Jun-24-1009|POL-DEF-Jun-24-1009|14843.75||2812500|-1924375|","-3371779|-3371779|628882.45|15|DIL PROPERTY DEVELOPMENT LTD &amp;/OR SUBSEQUENT OWNERS|125776.98|0|MUR|01/03/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|17/12/2024|3585841.16|503105.47|01-03-2026 to 01-03-2036|POL-DEF-Nov-24-1016|POL-DEF-Nov-24-1016|22173.92|DN52706092024000012|4192549.69|-2868673.023288386|","-603117|-603117|89703.54|15|CREATIVE PROPERTIES LTD &amp;/OR SUBSEQUENT OWNERS|-0.46|0|MUR|20/03/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|08/05/2025|513413.13|89704|20-03-2026 to 19-03-2036|POL-DEF-Feb-25-1008|POL-DEF-Feb-25-1008\\E2|5093.08||598023.59|-513413.41091800696|","-440325|-440325|65519.51|15|CREATIVE PROPERTIES LTD &amp;/OR SUBSEQUENT OWNERS|-0.49|0|MUR|21/03/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|08/05/2025|374805.98|65520|21-03-2026 to 20-03-2036|POL-DEF-Feb-25-1007|POL-DEF-Feb-25-1007\\E2|3528.79||436796.7|-374805.562910973|","-763225|-763225|113635.98|15|CREATIVE PROPERTIES LTD &amp;/OR SUBSEQUENT OWNERS|-0.02|0|MUR|02/06/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|08/05/2025|649588.73|113636|02-06-2026 to 01-06-2036|POL-DEF-Feb-25-1009|POL-DEF-Feb-25-1009\\E2|5651.51||757573.2|-649588.9768221078|","-510696|-510696|75888.79|15|CREATIVE PROPERTIES LTD &amp;/OR SUBSEQUENT OWNERS|-0.210000000009313|0|MUR|21/01/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|08/05/2025|434807.24|75889|21-01-2026 to 20-01-2036|POL-DEF-Feb-25-1010|POL-DEF-Feb-25-1010\\E2|4770.74||505925.29|-434807.21445796243|","-1272734|-1272734|273316.91|15|CREATIVE PROPERTIES LTD &amp;/OR SUBSEQUENT OWNERS|83487.77|0|MUR|15/01/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|24/04/2025|1559173.18|189829.14|15-01-2026 to 14-01-2036|POL-DEF-Mar-25-1011|POL-DEF-Mar-25-1011|10377.39||1822112.7|-1082905.020279875|","-444491|-444491|82603.06|15|SOCIETE EXSARTUM &amp;/OR SUBSEQUENT OWNERS|16520.69|0|MUR|04/03/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|12/05/2025|473011.39|66082.37|04-03-2026 to 04-03-2036|POL-DEF-Apr-25-1014|POL-DEF-Apr-25-1014|4927.4|DN52706092025000004|550687.05|-378408.63525505865|","-438652|-438652|81512|15|SOCIETE EXSARTUM &amp;/OR SUBSEQUENT OWNERS|16302.39|0|MUR|04/03/2026|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|12/05/2025|466803.3|65209.61|04-03-2026 to 04-03-2036|POL-DEF-Apr-25-1013|POL-DEF-Apr-25-1013|4901.95|DN52706092025000005|543413.35|-373442.4356781582|"]</t>
-  </si>
-  <si>
-    <t>["DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE"]</t>
+    <t>2026-07-28T06:37:30.917Z</t>
+  </si>
+  <si>
+    <t>["-9497|-440755.76999999996|1417.5|15|ACCUVISE ADMINISTRATORS LIMITED||0|Correction to be done by CBL amount not same as in aging|USD|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PI-D&amp;O|||8079.75||01-07-2026 to 30-06-2027|POL-D&amp;O+PI-Jul-20-1004\\R7|POL-D&amp;O+PI-Jul-20-1004\\R7|47.25||9450|-374971.32671641785|Timing Difference","-43000|-43000|6412.5|15|ARTEMIS CASCAVELLE HOSPITAL LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY|||36587.12||01-07-2026 to 01-07-2027|POL-MON-Jun-26-13|POL-MON-Jun-26-13|249.62||42750|-36587.44333089455|Timing Difference","-66231|-66231|9900|15|ARTEMIS CUREPIPE HOSPITAL LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY|||56331||01-07-2026 to 01-07-2027|POL-MON-Jul-25-6\\R1|POL-MON-Jul-25-6\\R1|231||66000|-56331|Timing Difference","-100329|-100329|14996.88|15|ARTEMIS CUREPIPE HOSPITAL LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|||85332.25||01-07-2026 to 01-07-2027|POL-PA-Jul-25-1005\\R1|POL-PA-Jul-25-1005\\R1|349.93||99979.2|-85332.1394319875|Timing Difference","-924866|-924866|138171.25|15|ARTEMIS CUREPIPE HOSPITAL LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|ASSETS ALL RISKS &amp; BUSINESS INTERRUPTION|||786694.4||01-07-2026 to 01-07-2027|POL-AAR+BI-Jul-25-3\\R1|POL-AAR+BI-Jul-25-3\\R1|3724||921141.65|-786694.6977113918|Timing Difference","-66231|-66231|9899.98|15|ARTEMIS CUREPIPE HOSPITAL LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|||56330.86||01-07-2026 to 01-07-2027|POL-EL-Jul-25-23\\R1|POL-EL-Jul-25-23\\R1|231||65999.84|-56330.996083697566|Timing Difference","-58402|-58402|8662.5|15|ARTEMIS CUREPIPE HOSPITAL LTD &amp;/OR ST HELENE CLINIC CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY|||49739.63||01-07-2026 to 01-07-2027|POL-PL-Jul-25-50\\R1|POL-PL-Jul-25-50\\R1|652.13||57750|-49739.519282259054|Timing Difference","-110560|-110560|8812.8|8|BLANDIN DE CHALAIN MARIE ANNE ODILE MRS|858.399999999999|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||14/07/2026|101747.2|7954.4|01-07-2026 to 01-07-2027|POL-HEALTH-Jul-22-69\\R4|POL-HEALTH-Jul-22-69\\R4|400|MED/2022/00715/R4|110160|-101747.2|Timing Difference","-20210|-20210|3021|15|CRANS &amp; COMPANY LIMITED|6041.93|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY|||17189.49|-3020.93|01-07-2026 to 01-07-2027|POL-PPL-Sep-19-1135\\R7|POL-PPL-Sep-19-1135\\R7|70.49||20140|-17189.073243647235|Timing Difference","-9152|-9152|1368|15|CRANS &amp; COMPANY LIMITED|2736.01|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|||7783.92|-1368.01|01-07-2026 to 01-07-2027|POL-EL-Sep-19-1400\\R7|POL-EL-Sep-19-1400\\R7|31.92||9120|-7783.988041853512|Timing Difference","-8580|-8580|1282.5|15|CRANS &amp; COMPANY LIMITED|2565.01|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR TRADE|||7297.42|-1282.51|01-07-2026 to 01-07-2027|POL-MT-Sep-19-1015\\R7|POL-MT-Sep-19-1015\\R7|29.92||8550|-7297.488041846544|Timing Difference","-14300|-14300|2137.5|15|CRANS &amp; COMPANY LIMITED|4275.02|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)|||12162.37|-2137.52|01-07-2026 to 01-07-2027|POL-ARMISC-Jul-24-13\\R2|POL-ARMISC-Jul-24-13\\R2|49.87||14250|-12162.480568005163|Timing Difference","-31746|-31746|4745.25|15|CRANS &amp; COMPANY LIMITED|9490.54|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|||27000.47|-4745.29|01-07-2026 to 01-07-2027|POL-PA-Jul-24-24\\R2|POL-PA-Jul-24-24\\R2|110.72||31635|-27000.708146483998|Timing Difference","-176374|-176374|26289.15|15|CRANS &amp; COMPANY LIMITED|52578.24|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|||150085.28|-26289.09|01-07-2026 to 01-07-2027|POL-F&amp;A-Sep-19-1482\\R7|POL-F&amp;A-Sep-19-1482\\R7|1113.43||175261|-150084.91409281947|Timing Difference","-100767|-100767|8029.36|8|D'UNIENVILLE JOSEPH CHARLES HENRI MR|0|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||10/07/2026|92737.64|8029.36|01-07-2026 to 01-07-2027|POL-HEALTH-Aug-24-55\\R2|POL-HEALTH-Aug-24-55\\R2|400|MED/2024/00723/R2|100367|-92737.64|Timing Difference","-29901|-29901|4455|15|DR RAYMOND JEAN-LOUP D'HOTMAN DE VILLIERS||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|MEDICAL MALPRACTICE|||25445.5||01-07-2026 to 30-06-2027|POL-PI-Nov-19-1442\\R7|POL-PI-Nov-19-1442\\R7|200.5||29700|-25445.925502918013|Timing Difference","-37700|-37700|5625|15|ENASANS INTERIORS LTD||0||MUR|01/08/2026|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY|||32075.25||01-08-2026 to 31-07-2027|POL-F-PI-Aug-25-1019\\R1|POL-F-PI-Aug-25-1019\\R1|200.25||37500|-32075.037300813656|Timing Difference","-2196|-2196|253.49|15|GMF LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|||1942.32||01-07-2026 to 01-07-2027|POL-F&amp;A-Jun-19-1328\\R7|POL-F&amp;A-Jun-19-1328\\R7|505.91||1689.9|-1942.4880659073417|Timing Difference","-10455|-10455|1562.85|15|GMF LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY|||8892.62||01-07-2026 to 01-07-2027|POL-PL-Jun-19-1230\\R7|POL-PL-Jun-19-1230\\R7|36.47||10419|-8892.220254087095|Timing Difference","-12837|-12837|1918.8|15|GMF LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|||10917.97||01-07-2026 to 01-07-2027|POL-EL-Jun-19-1240\\R7|POL-EL-Jun-19-1240\\R7|44.77||12792|-10918.165620323492|Timing Difference","-69091|-69091|10327.5|15|GMF LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|||58763.48||01-07-2026 to 01-07-2027|POL-PA-Jun-19-1308\\R7|POL-PA-Jun-19-1308\\R7|240.98||68850|-58763.497010463594|Timing Difference","-14535|-14535|2172.63|15|GMF LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT|||12362.26||01-07-2026 to 01-07-2027|POL-EE-Jun-19-1140\\R7|POL-EE-Jun-19-1140\\R7|50.69||14484.2|-12362.353557543263|Timing Difference","-2077|-2077|310.5|15|GMF LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)|||1766.75||01-07-2026 to 01-07-2027|POL-ARMISC-Jun-26-13|POL-ARMISC-Jun-26-13|7.25||2070|-1766.537369117824|Timing Difference","-49839|-49839|4317.6|8|HARTER CATHERINE DIANE MARIE MRS|359.81|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||14/07/2026|50052.4|3957.79|01-07-2026 to 01-07-2027|POL-HEALTH-Jul-25-85\\R1|POL-HEALTH-Jul-25-85\\R1|400|MED/2025/01120/R1|53970|-45881.21323524002|Timing Difference","-84783|-84783|7366.96|8|HARTER JEAN LUC MR|613.65|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||10/07/2026|85120.04|6753.31|01-07-2026 to 01-07-2027|POL-HEALTH-Jul-25-86\\R1|POL-HEALTH-Jul-25-86\\R1|400|MED/2025/01001/R1|92087|-78029.6944578157|Timing Difference","-34307|-34307|2962|8|HARTER JULIEN LEO MR|246.77|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/07/2026|34463|2715.23|01-07-2026 to 01-07-2027|POL-HEALTH-Jul-25-87\\R1|POL-HEALTH-Jul-25-87\\R1|400|MED/2025/00960/R1|37025|-31591.7739746159|Timing Difference","-60112|-60112|8985.3|15|JBA INVESTMENT HOLDINGS LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|||51126.36||01-07-2026 to 01-07-2027|POL-PA-Jun-19-1347\\R7|POL-PA-Jun-19-1347\\R7|209.66||59902|-51126.64917787997|Timing Difference","-3596|-3596|537.47|15|JBA INVESTMENT HOLDINGS LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT|||3058.2||01-07-2026 to 01-07-2027|POL-EE-Jun-19-1160\\R7|POL-EE-Jun-19-1160\\R7|12.54||3583.13|-3058.48067258675|Timing Difference","-664|-664|99.23|15|JBA INVESTMENT HOLDINGS LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)|||564.59||01-07-2026 to 01-07-2027|POL-ARMISC-Jul-23-19\\R3|POL-ARMISC-Jul-23-19\\R3|2.32||661.5|-564.7430930071405|Timing Difference","-1798|-1798|268.74|15|JBA INVESTMENT HOLDINGS LTD &amp;/OR JBA &amp; PARTNERS LTD &amp;/OR MR &amp; MRS JUGMOHUN BHURTUN||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|||1529.11||01-07-2026 to 01-07-2027|POL-EL-Jun-19-1284\\R7|POL-EL-Jun-19-1284\\R7|6.27||1791.58|-1529.2375782184276|Timing Difference","-18966|-18966|2835|15|JBA INVESTMENT HOLDINGS LTD &amp;/OR JBA &amp; PARTNERS LTD &amp;/OR MR &amp; MRS JUGMOHUN BHURTUN||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY|||16131.15||01-07-2026 to 01-07-2027|POL-PL-Jun-19-1269\\R7|POL-PL-Jun-19-1269\\R7|66.15||18900|-16131.022421524664|Timing Difference","-9957|-9957|1488.38|15|JBA INVESTMENT HOLDINGS LTD &amp;/OR JBA &amp; PARTNERS LTD &amp;/OR MR &amp; MRS JUGMOHUN BHURTUN||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|||8468.85||01-07-2026 to 01-07-2027|POL-PA-Jun-20-1179\\R6|POL-PA-Jun-20-1179\\R6|34.73||9922.5|-8468.654379782329|Timing Difference","-175608|-175608|26174.53|15|JBA INVESTMENT HOLDINGS LTD &amp;/OR MR J. &amp; MRS S. K. BHURTUN &amp;/OR MR B. BHURTUN &amp;/OR MRS PRISHAN BHURTUN JUGROO||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|||149433.09||01-07-2026 to 01-07-2027|POL-F&amp;A-Jun-19-1372\\R7|POL-F&amp;A-Jun-19-1372\\R7|1110.74||174496.88|-149433.4133605364|Timing Difference","-50412|-50412|4000.96|8|JEETOO MAHEROO NESSA SAMSOODEEN|400.08|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||10/07/2026|46411.04|3600.88|01-07-2026 to 01-07-2027|POL-HEALTH-Oct-20-327\\R6|POL-HEALTH-Oct-20-327\\R6|400|MD20M01109/1/R5|50012|-46411.04|Timing Difference","-92710|-92710|7384.8|8|JEETOO YUSUF MAHOMED MR|738.48|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||10/07/2026|85325.2|6646.32|01-07-2026 to 01-07-2027|POL-HEALTH-Oct-20-326\\R6|POL-HEALTH-Oct-20-326\\R6|400|MD20M01108/1/R5|92310|-85325.2|Timing Difference","-385486|-385486|82193.15|15|KI SIGNATURE VILLAS LTD &amp;/OR SUBSEQUENT OWNERS|24658.05|0||MUR|01/09/2026|MAURITIUS UNION ASSURANCE CO LTD|DEFECTS INSURANCE||13/06/2025|468501.15|57535.1|01-09-2026 to 01-09-2036|POL-DEF-Apr-25-1012|POL-DEF-Apr-25-1012|2740||547954.3|-327950.7964925368|Timing Difference","-225864|-225864|27055.68|12|LAGESSE MARIE MICHEL JEAN OCTAVE|-0.32|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/07/2026|198808.32|27056|01-07-2026 to 01-07-2027|POL-HEALTH-Jun-25-56\\R1|POL-HEALTH-Jun-25-56\\R1|400|MED/2025/00830/R1|225464|-198808.32|Timing Difference","-184141|-184141|27450|15|MONDO PROPERTIES LTD &amp;/OR NASARA RESIDENCE LTD &amp;/OR CONTRACTORS &amp;/OR SUB-CONTRACTORS|0|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||30/06/2026|156690.5|27450|01-07-2026 to 01-07-2028|POL-CAR-TPL-Jun-26-36|POL-CAR-TPL-Jun-26-36|1140.5||183000|-156690.92546452302|Timing Difference","-15200|-15200|2250|15|MRS LIM KIN BEATRICE||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY|||12950||01-07-2026 to 30-06-2027|POL-F-PI-Jun-26-24|POL-F-PI-Jun-26-24|200|4013/09|15000|-12950|Timing Difference","-2103165|-2103165|313905.15|15|NASARA RESIDENCE LTD &amp;/OR SUBSEQUENT OWNERS|0.150000000037253|0||MUR|01/07/2028|MAURITIUS UNION ASSURANCE CO LTD|DEFECTS INSURANCE||30/06/2026|1789259.85|313905|01-07-2028 to 01-07-2038|POL-DEF-Jun-26-1007|POL-DEF-Jun-26-1007|10464||2092701|-1789259.85|Timing Difference","-86476|-86476|6886.08|8|PUDDOO DAYARAM MR.|0|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||10/07/2026|79589.92|6886.08|01-07-2026 to 01-07-2027|POL-HEALTH-Jul-19-2908\\R7|POL-HEALTH-Jul-19-2908\\R7|400|MD17M00548/4/R5|86076|-79589.92|Timing Difference","-8053|-8053|1181.25|15|SOCIETE C&amp;R||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY|||6871.31||01-07-2026 to 01-07-2027|POL-PL-Jun-19-1244\\R7|POL-PL-Jun-19-1244\\R7|177.56||7875|-6871.685455308622|Timing Difference","-95763|-95763|14269.5|15|SOCIETE C&amp;R||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|||81493.46||01-07-2026 to 01-07-2027|POL-F&amp;A-Jun-19-1344\\R7|POL-F&amp;A-Jun-19-1344\\R7|632.96||95130|-81493.49403965792|Timing Difference"]</t>
+  </si>
+  <si>
+    <t>["After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026","After 30.06.2026"]</t>
+  </si>
+  <si>
+    <t>2026-07-28T06:39:26.666Z</t>
+  </si>
+  <si>
+    <t>["1|1|4692.75|15|AKINI TRAVEL &amp; CO LTD|4692.71|200|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||31/12/2019|26901.76|0.0399999999999636|01-07-2019 to 01-07-2020|POL-MV-May-19-1179\\R1|POL-MV-May-19-1179\\R1|109.51|32245/18/R1|31285|0.8514694483313715|","-20.68|-20.68|413.4|15|BEAUTES DE CHINE &amp;/OR AH TONG CHAO &amp; CIE|413.4|0|Correction to be done by CBL amount not in aging|MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||26/09/2025|2490.73|0|01-07-2025 to 01-07-2026|POL-PL-Jun-19-1202\\R6|POL-PL-Jun-19-1202\\R6|10.13|11411/07|2894|-17.736222689755625|","-120520|-120520|18000|15|BLUE MOUNTAIN CONTRACTING SERVICES LTD|0|0|Correction to be done by CBL amount not in aging|MUR|01/04/2019|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||14/07/2020|102520|18000|01-04-2019 to 01-04-2020|POL-CAR-TPL-May-19-1003|POL-CAR-TPL-May-19-1003|520|to close with POL-CAR-TPL-Oct-19-1144\\E1 as per mail from PP on 13.07 - MUA NOT PROCESSED PLACING SLIP|120000|-102520|","120520|120520|-18000|15|BLUE MOUNTAIN CONTRACTING SERVICES LTD &amp;/OR MIMUSOPS CO LTD &amp;/OR SUB CONTRACTORS|0|0|Correction to be done by CBL amount not in aging|MUR|01/04/2019|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||14/07/2020|-102520|-18000|01-04-2019 to 30-10-2019|POL-CAR-TPL-Oct-19-1144|POL-CAR-TPL-Oct-19-1144\\E1|-520|to close with1819/04/0723 as per mail from PP on 13.07 - MUA NOT PROCESSED PLACING SLIP|-120000|102520|","-12694|-12694|1875|15|CAPE POINT LTD|0|0|Correction to be done by CBL amount not in aging|MUR|01/03/2021|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||31/03/2021|10818.75|1875|01-03-2021 to 01-03-2022|POL-PL-Feb-20-1095\\R1|POL-PL-Feb-20-1095\\R1|193.75|21139/17|12500|-10818.96307237814|","12694|12694|4270.13|15|CAPE POINT LTD|6147.96|0|Correction to be done by CBL amount not in aging|MUR|01/03/2021|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||31/03/2021|24597.01|-1877.83|01-03-2021 to 01-03-2022|POL-F&amp;A-Feb-20-1097\\R1|POL-F&amp;A-Feb-20-1097\\R1|399.64|21139/17|28467.5|10816.258380289839|","0.01|0.5278|2867.15|15|CEMENTIS SERVICES LTD &amp;/OR MAUCIMENT INVESTMENT LTD &amp;/OR CEMENTIS INDIAN OCEAN LTD &amp;/OR CEMENTIS MADAGASCAR SA &amp;/OR CEMENTIS MADAGASCAR IMMOBILIER SAS &amp;/OR BINASTORE &amp;/OR CHAUMAD FINANCES SARL &amp;/OR CHAUX DE MADAGASCAR SARL|2867.27|0|Correction to be done by CBL amount not in aging|EUR|26/08/2022|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||30/04/2023|16324.09|-0.119999999999891|26-08-2022 to 01-01-2023|POL-F&amp;A-Sep-22-1045|POL-F&amp;A-Sep-22-1045|76.9|NO DOCS TO FOLLOW|19114.34|0.44894726458530043|","0.64|0.64|1275|15|CONSULTANCY COMPANY LTD (CCL)|1275.09|0|Correction to be done by CBL amount not in aging|MUR|03/07/2019|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||30/09/2019|7255|-0.0899999999999181|03-07-2019 to 03-07-2020|POL-PA-Jul-19-1372|POL-PA-Jul-19-1372|30|MD08K01172/R11|8500|0.544337631887456|","376|376|15375|15|CROWN COURT BUILDING|15429.96|0|Correction to be done by CBL amount not in aging|MUR|01/04/2020|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||29/05/2020|87983.75|-54.9599999999973|01-04-2020 to 01-04-2021|POL-FO-Mar-20-1001|POL-FO-Mar-20-1001|858.75|13635/12/R8|102500|320.068596030815|","-376|-376|56.25|15|CROWN COURT BUILDING|0.25|0|Correction to be done by CBL amount not in aging|MUR|01/04/2020|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||28/05/2020|320.06|56|01-04-2020 to 01-04-2021|POL-EE-Mar-20-1058|POL-EE-Mar-20-1058|1.31|13635/12/R8|375|-319.79633812548167|","-2302|-2302|344.06|15|DB VISION LIMITED &amp;/OR DB DESIGN AND CONCEPT LTD|0.06|0|Correction to be done by CBL amount not in aging|MUR|01/09/2020|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||18/03/2021|1957.68|344|01-09-2020 to 01-09-2021|POL-EL-Aug-19-1395\\R1|POL-EL-Aug-19-1395\\R1|8.03|18762/08/R12|2293.71|-1957.9011356625856|","-17513|-17513|2617.83|15|DB VISION LIMITED &amp;/OR DB DESIGN AND CONCEPT LTD|-0.17|0|Correction to be done by CBL amount not in aging|MUR|01/09/2020|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||18/03/2021|14895.44|2618|01-09-2020 to 01-09-2021|POL-ARMISC-Aug-19-1122\\R1|POL-ARMISC-Aug-19-1122\\R1|61.08|18762/08/R12|17452.19|-14895.210358773662|","-6523|-6523|975|15|DB VISION LIMITED &amp;/OR DB DESIGN AND CONCEPT LTD|0|0|Correction to be done by CBL amount not in aging|MUR|01/09/2020|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||18/03/2021|5547.75|975|01-09-2020 to 01-09-2021|POL-PL-Aug-19-1374\\R1|POL-PL-Aug-19-1374\\R1|22.75|18762/08/R12|6500|-5547.962630792227|","37387|37387|9480.15|15|DB VISION LIMITED &amp;/OR DB DESIGN AND CONCEPT LTD|14961.89|0|Correction to be done by CBL amount not in aging|MUR|01/09/2020|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||26/03/2021|54442.06|-5481.74|01-09-2020 to 01-09-2021|POL-F&amp;A-Aug-19-1478\\R1|POL-F&amp;A-Aug-19-1478\\R1|721.21|18762/08/R12|63201|31842.223496653198|","-9985|-9985|1492.5|15|DB VISION LIMITED &amp;/OR DB DESIGN AND CONCEPT LTD|-0.5|0|Correction to be done by CBL amount not in aging|MUR|01/09/2020|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||18/03/2021|8492.33|1493|01-09-2020 to 01-09-2021|POL-PA-Aug-19-1475\\R1|POL-PA-Aug-19-1475\\R1|34.83|18762/08/R12|9950|-8492.47458895144|","-1064|-1064|159|15|DB VISION LIMITED &amp;/OR DB DESIGN AND CONCEPT LTD|0|0|Correction to be done by CBL amount not in aging|MUR|01/09/2020|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||18/03/2021|904.71|159|01-09-2020 to 01-09-2021|POL-LOP(F&amp;A)-Aug-19-1130\\R1|POL-LOP(F&amp;A)-Aug-19-1130\\R1|3.71|18762/08/R12|1060|-904.9566517189835|","-500.12|-500.12|1582.1696|8|EDL CONSULTING LIMITED|1542.16|0|Correction to be done by CBL amount not in aging|MUR|01/05/2018|MAURITIUS UNION ASSURANCE CO LTD|HEALTH|||18194.9504|40.0095999999999|01-05-2018 to 01-05-2019|POL-HEALTH-May-19-1734|POL-HEALTH-May-19-1734|0|MD16M00344/MED/R02 MD16M00348/MCSGP/R02|19777.12|-460.1104|","-4651|-4651|695.25|15|FRIENDS IN HOPE|0.25|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||18/02/2021|3955.99|695|01-01-2021 to 01-01-2022|POL-PA-Jun-20-1173\\R1|POL-PA-Jun-20-1173\\R1|16.22|MD09K00164/R12|4635.02|-3955.7858743044867|","-1691|-1691|252.82|15|FRIENDS IN HOPE|-0.18|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||18/02/2021|1438.54|253|01-01-2021 to 01-01-2022|POL-EL-Jun-20-1182\\R1|POL-EL-Jun-20-1182\\R1|5.9||1685.46|-1438.2338118437233|","-9032|-9032|1350|15|FRIENDS IN HOPE|0|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||18/02/2021|7681.5|1350|01-01-2021 to 01-01-2022|POL-PL-Jun-20-1198\\R1|POL-PL-Jun-20-1198\\R1|31.5|MD09K00164/R12|9000|-7681.925261584454|","-1292|-1292|148.26|15|FRIENDS IN HOPE|0.26|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||19/02/2021|843.56|148|01-01-2021 to 01-01-2022|POL-EE-Jun-20-1095\\R1|POL-EE-Jun-20-1095\\R1|3.45|MD09K00164/R12|988.37|-1098.86826238632|","16666|16666|172.5|15|FRIENDS IN HOPE|1910.1|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||30/04/2021|1481.53|-1737.6|01-01-2021 to 01-01-2022|POL-F&amp;A-Jun-20-1202\\R1|POL-F&amp;A-Jun-20-1202\\R1|504.03|MD09K00164/R12|1150|14927.890654945799|","1|1|3750|15|GREGORY GEBERT OSTEOPATHE D.O (BRN: 118006529) &amp;/OR GEBERT JEAN FRANCOIS GREGORY MR|3750.15|0|Correction to be done by CBL amount not in aging|MUR|01/08/2019|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY||31/07/2019|21450|-0.150000000000091|01-08-2019 to 01-08-2020|POL-PI-Jul-19-1073|POL-PI-Jul-19-1073|200|29754/18/R1|25000|0.8511904761904762|","1000|1000|0|15|LAVASTONE PROPERTIES LTD &amp;/OR PRINCIPALS &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS||0|Correction to be done by CBL amount not in aging|MUR|01/10/2020|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||17/02/2021|-1000||01-10-2020 to 01-10-2021|POL-CAR-TPL(BC)-Oct-19-1050\\R1|POL-CAR-TPL(BC)-Oct-19-1050\\R1\\E1|-1000|33502/19|0|1000|","-500|-500|5722.5|15|LAVASTONE PROPERTIES LTD &amp;/OR PRINCIPALS &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|5796.81|0|Correction to be done by CBL amount not in aging|MUR|01/10/2020|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||30/11/2020|32561.03|-74.3100000000004|01-10-2020 to 01-10-2021|POL-CAR-TPL(BC)-Oct-19-1050\\R1|POL-CAR-TPL(BC)-Oct-19-1050\\R1|133.53|33502/19|38150|-425.26159421558043|","1258|1258|-188.01|15|MAUCIMENT INVESTMENT LTD &amp;/OR CEMENTIS (MAURITIUS) LTD &amp;/OR CEMENTIS INVESTMENT LTD &amp;/OR SUBSIDIARIES|-0.01|0|Correction to be done by CBL amount not in aging|MUR|01/11/2022|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||18/05/2023|-1069.8|-188|01-11-2022 to 01-01-2023|POL-ARM(P&amp;M)-Nov-22-1011|POL-ARM(P&amp;M)-Nov-22-1011\\E1|-4.39|INTERNAL PURPOSE|-1253.42|1069.9615999236769|","1|1|-225|15|MAURIPLAGE INVESTMENT LTD T/A SANDS SUITES RESORT &amp; SPA &amp;/OR MAURIPLAGE BEACH RESORT LTD T/A MARADIVA VILLAS RESORT &amp; SPA|-225|0|Correction to be done by CBL amount not in aging|MUR|01/10/2020|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||19/01/2021|-1280.26|0|01-10-2020 to 01-10-2021|POL-FID-Oct-19-1066\\R1|POL-FID-Oct-19-1066\\R1\\E1|-5.26|40547/17/R3|-1500|0.8505241619388013|","-6543|-6543|-978.08|15|MR DULLOO BEN TARIK|-1956.08|0|Correction to be done by CBL amount not in aging|MUR|23/10/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||13/01/2020|-5565.24|978|23-10-2019 to 01-04-2020|POL-MV-May-19-1670|POL-MV-May-19-1670\\E1|-22.82|13384/19/N|-6520.5|-5564.967832843266|","-5469|-5469|810|15|MR EVAN MERCIER|0|50|Correction to be done by CBL amount not in aging|MUR|01/10/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||21/01/2020|4658.9|810|01-10-2019 to 01-10-2020|POL-MV-May-19-2318\\R1|POL-MV-May-19-2318\\R1|18.9|49358/17/R2|5400|-4658.985188977674|","1124|1124|1734|15|MR LOICK LACOSTE|1898.93|100|Correction to be done by CBL amount not in aging|MUR|01/04/2021|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||21/04/2021|9966.47|-164.93|01-04-2021 to 01-04-2022|POL-MV-Mar-21-74|POL-MV-Mar-21-74|40.47|5525/21/N|11560|957.4241274068478|","5469|5469|||MR. EVAN MERCIER||0|Correction to be done by CBL amount not in aging|MUR|20/08/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR INDIVIDUAL SCHEMES||31/03/2021||-810|20-08-2019 to 01-04-2020|POL-MIS-May-19-1632|POL-MIS-May-19-1632\\E1||09/2019 8362 - CANNOT CLOSE VOUCHER 0\nCLOSED WITHOUT DOCS\nINS LAPSED||5469|","21|974.6099999999999|0|0|ONE &amp; ONLY LE SAINT GERAN LTD||0|Correction to be done by CBL amount not same as in aging|USD|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||08/05/2026|-20.53||01-10-2025 to 30-09-2026|POL-PL-Nov-21-43\\R4|POL-PL-Nov-21-43\\R4\\E1|-20.53|33871/25/N|0|974.6099999999999|","0.01|0.5278|1118.7|15|ORANGE BUSINESS SERVICES MAURITIUS LIMITED &amp;/OR EQUANT MAURITIUS HOLDINGS LTD|1118.39|0|Correction to be done by CBL amount not in aging|EUR|01/11/2024|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||09/01/2025|6368.4|0.309999999999945|01-11-2024 to 31-10-2025|POL-CP-Mar-20-1014\\R6|POL-CP-Mar-20-1014\\R6|29.1|10945/21|7458|0.44893770885923795|","-10666|-10666|1594.25|15|POOL SOLUTIONS LTD|0.25|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||03/08/2020|9071.26|1594|01-07-2020 to 01-07-2021|POL-EE-Aug-19-1195\\R1|POL-EE-Aug-19-1195\\R1|37.21|31416/12/R8|10628.3|-9071.67675619825|","-1505|-1505|225|15|POOL SOLUTIONS LTD|0|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||03/08/2020|1280.25|225|01-07-2020 to 01-07-2021|POL-ARMISC-Jul-20-1039|POL-ARMISC-Jul-20-1039|5.25|31416/12/R8|1500|-1280.0373692077728|","80637|80637|951.56|15|POOL SOLUTIONS LTD|12126.69|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||03/08/2020|5914.4|-11175.13|01-07-2020 to 01-07-2021|POL-F&amp;A-Aug-19-1446\\R1|POL-F&amp;A-Aug-19-1446\\R1|522.21|31416/12/R8|6343.75|69461.44061427681|","-7526|-7526|1125|15|POOL SOLUTIONS LTD &amp;/OR NCF CO LTD|0|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||03/08/2020|6401.25|1125|01-07-2020 to 01-07-2021|POL-PL-Jun-19-1200\\R1|POL-PL-Jun-19-1200\\R1|26.25|31416/12/R8|7500|-6401.037369207773|","-25618|-25618|3829.35|15|POOL SOLUTIONS LTD &amp;/OR NCF CO LTD|0.35|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||03/08/2020|21789|3829|01-07-2020 to 01-07-2021|POL-PA-Jun-19-1282\\R1|POL-PA-Jun-19-1282\\R1|89.35|31416/12/R8|25529|-21788.702316893945|","-27596|-27596|4125|15|POOL SOLUTIONS LTD &amp;/OR NCF CO LTD &amp;/OR PRINCIPALS &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB-CONTRACTORS|0|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||03/08/2020|23471.25|4125|01-07-2020 to 01-07-2021|POL-CAR-TPL(BC)-Jun-19-1021\\R1|POL-CAR-TPL(BC)-Jun-19-1021\\R1|96.25|31416/12/R8|27500|-23471.037369207774|","-7726|-7726|1154.85|15|POOL SOLUTIONS LTD &amp;/or NCF CO LTD|-0.150000000000146|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||03/08/2020|6571.1|1155|01-07-2020 to 01-07-2021|POL-EL-Jun-19-1207\\R1|POL-EL-Jun-19-1207\\R1|26.95|31416/12/R8|7699|-6571.1425261618315|","-1170|-71725.68000000001|174.45|15|PORT LOUIS MANAGEMENT SERVICES LTD &amp;/OR ORCHIDEE INTERNATIONAL LIMITED &amp;/OR JASMINA HOLDINGSLTD &amp;/OR HORIZONWORLD LTD &amp;/OR PMSL TRUSTEES LTD||0|Correction to be done by CBL amount not same as in aging|GBP|31/05/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PI-D&amp;O|||995.63||31-05-2026 to 30-06-2026|POL-D&amp;O+PI-Jun-19-1006\\R6|POL-D&amp;O+PI-Jun-19-1006\\R6\\E1|7.07||1163.01|-61031.928396690826|","79990|79990|2351.25|15|RESMAU LTD T/A KAS POZ|13939.74|0|Correction to be done by CBL amount not in aging|MUR|01/11/2020|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||02/04/2021|13878.62|-11588.49|01-11-2020 to 01-11-2021|POL-F&amp;A-Oct-19-1563\\R1|POL-F&amp;A-Oct-19-1563\\R1|554.87|27726/13/R7|15675|68401.70708699453|","-5942|-5942|888.15|15|RESMAU LTD T/A KAS POZ|0.15|0|Correction to be done by CBL amount not in aging|MUR|01/11/2020|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||04/03/2021|5053.58|888|01-11-2020 to 01-11-2021|POL-LOP(F&amp;A)-Oct-19-1159\\R1|POL-LOP(F&amp;A)-Oct-19-1159\\R1|20.73|27726/13/R7|5921|-5053.809641299756|"]</t>
+  </si>
+  <si>
+    <t>["NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING","NOT IN AGING/AMOUNT NOT SAME IN AGING"]</t>
+  </si>
+  <si>
+    <t>correction_to_be_done_by_cbl</t>
+  </si>
+  <si>
+    <t>2026-07-28T06:45:42.915Z</t>
+  </si>
+  <si>
+    <t>continuation</t>
+  </si>
+  <si>
+    <t>["-60210|-60210|9000|15|RESMAU LTD T/A KAS POZ|0|0|Correction to be done by CBL amount not in aging|MUR|01/11/2020|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||04/03/2021|51210|9000|01-11-2020 to 01-11-2021|POL-PPL-Oct-19-1158\\R1|POL-PPL-Oct-19-1158\\R1|210|27726/13/R7|60000|-51210|","-5018|-5018|750|15|RESMAU LTD T/A KAS POZ|0|0|Correction to be done by CBL amount not in aging|MUR|01/11/2020|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||04/03/2021|4267.5|750|01-11-2020 to 01-11-2021|POL-EE-Oct-19-1244\\R1|POL-EE-Oct-19-1244\\R1|17.5|27726/13/R7|5000|-4267.925261584454|","-3512|-3512|525|15|RESMAU LTD T/A KAS POZ|0|0|Correction to be done by CBL amount not in aging|MUR|01/11/2020|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||04/03/2021|2987.25|525|01-11-2020 to 01-11-2021|POL-FID-Oct-19-1071\\R1|POL-FID-Oct-19-1071\\R1|12.25|27726/13/R7|3500|-2987.037369207773|","-1996|-1996|298.35|15|RESMAU LTD T/A KAS POZ|0.350000000000036|0|Correction to be done by CBL amount not in aging|MUR|01/11/2020|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||04/03/2021|1697.61|298|01-11-2020 to 01-11-2021|POL-EL-Oct-19-1478\\R1|POL-EL-Oct-19-1478\\R1|6.96|27726/13/R7|1989|-1697.6440209222628|","-3312|-3312|495|15|RESMAU LTD T/A KAS POZ|0|0|Correction to be done by CBL amount not in aging|MUR|01/11/2020|MAURITIUS UNION ASSURANCE CO LTD|MONEY||04/03/2021|2816.55|495|01-11-2020 to 01-11-2021|POL-MON-Oct-19-1170\\R1|POL-MON-Oct-19-1170\\R1|11.55|27726/13/R7|3300|-2816.932735426009|","-4526|-4526|3344.56|8|SEEGOBIN RINA|2985.47|0|Correction to be done by CBL amount not in aging|MUR|01/10/2019|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/04/2020|38862.44|359.09|01-10-2019 to 01-10-2020|POL-HEALTH-Sep-19-3112|POL-HEALTH-Sep-19-3112|400|MD18M01189/MESIP/R01|41807|-4167.35146871372|","13774|13774|2339.7|15|SKYFLEET LTD|4399.82|67|Correction to be done by CBL amount not in aging|MUR|29/10/2018|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET|||13380.3|-2060.12|29-10-2018 to 29-10-2019|POL-MVF-May-19-1505|POL-MVF-May-19-1505|55|27042/17/R1|15598|11723.93461832061|","-730|-730|-109.2|15|SKYFLEET LTD|-218.4|0|Correction to be done by CBL amount not in aging|MUR|29/03/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET|||-620.8|109.2|29-03-2019 to 29-03-2020|POL-MVF-May-19-1520|POL-MVF-May-19-1520|-2|27042/17/R1|-728|-620.8|","-2874|-2874|-437.25|15|SKYFLEET LTD|-866.85|51|Correction to be done by CBL amount not in aging|MUR|28/12/2018|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET|||-2436.75|429.6|28-12-2018 to 28-12-2019|POL-MVF-May-19-1528|POL-MVF-May-19-1528|-10|27042/17/R1|-2915|-2436.75|","-4198|-4198|-627.45|15|SKYFLEET LTD|-1254.9|0|Correction to be done by CBL amount not in aging|MUR|12/11/2018|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET|||-3570.55|627.45|12-11-2018 to 12-11-2019|POL-MVF-May-19-1529|POL-MVF-May-19-1529|-15|27042/17/R1|-4183|-3570.55|","943|943|139.67|15|SKYFLEET LTD|557.97|8.74|Correction to be done by CBL amount not in aging|MUR|30/05/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||28/08/2020|803.48|-418.3|30-05-2019 to 01-07-2019|POL-MV-Oct-19-6278|POL-MV-Oct-19-6278|3.27|27042/17/R1/E35|931.14|803.3522133276786|","-398|-398|-59.51|15|SKYFLEET LTD|-118.49|0|Correction to be done by CBL amount not in aging|MUR|29/05/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||31/10/2019|-338.6|58.98|29-05-2019 to 01-07-2019|POL-MVF-Jul-19-1925|POL-MVF-Jul-19-1925\\E2|-1.39||-396.72|-338.5064429429052|","-528|-528|-78.9|15|SKYFLEET LTD|-157.8|0|Correction to be done by CBL amount not in aging|MUR|24/04/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/05/2019|-449.1|78.9|24-04-2019 to 24-04-2020|POL-MVF-May-19-1206|POL-MVF-May-19-1206|-2|27042/17/R1|-526|-449.1|","897|897|133.95|15|SKYFLEET LTD|267.9|0|Correction to be done by CBL amount not in aging|MUR|11/04/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET|||763.05|-133.95|11-04-2019 to 11-04-2020|POL-MVF-May-19-1550|POL-MVF-May-19-1550|4|27042/17/R1|893|763.05|","-310|-310|-46.32|15|SKYFLEET LTD|-93|0|Correction to be done by CBL amount not in aging|MUR|29/05/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||31/10/2019|-263.57|46.68|29-05-2019 to 01-07-2019|POL-MVF-Jul-19-1925|POL-MVF-Jul-19-1925\\E1|-1.08||-308.81|-263.6635580367227|","-994|-994|-148.5|15|SKYFLEET LTD|-297|0|Correction to be done by CBL amount not in aging|MUR|24/04/2019|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/05/2019|-845.5|148.5|24-04-2019 to 24-04-2020|POL-MVF-May-19-1207|POL-MVF-May-19-1207|-4|27042/17/R1|-990|-845.5|","-8580|-8580|-1282.5|15|SKYFLEET LTD|-2565|0|Correction to be done by CBL amount not in aging|MUR|12/11/2018|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET|||-7297.5|1282.5|12-11-2018 to 12-11-2019|POL-MVF-May-19-1530|POL-MVF-May-19-1530|-30|27042/17/R1|-8550|-7297.5|","900|900|5811|15|SKYFLEET LTD|5945.4|129|Correction to be done by CBL amount not in aging|MUR|08/11/2018|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET|||33195|-134.400000000001|08-11-2018 to 08-11-2019|POL-MVF-May-19-1501|POL-MVF-May-19-1501|137|27042/17/R1|38740|765.9206275957545|","-4014|-4014|1275|15|SOCIETE A.E. PATEL &amp; CIE|675.04|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||05/08/2020|7254.75|599.96|01-07-2020 to 01-07-2021|POL-FID-Jun-19-1032\\R1|POL-FID-Jun-19-1032\\R1|29.75|28513/17|8500|-3414|","-1535|-1535|229.5|15|SOCIETE A.E. PATEL &amp; CIE|-0.5|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|MONEY||28/07/2020|1305.86|230|01-07-2020 to 01-07-2021|POL-MON-Jun-19-1072\\R1|POL-MON-Jun-19-1072\\R1|5.36|28513/17|1530|-1305.5538114839517|","126053|126053|8092.5|15|SOCIETE A.E. PATEL &amp; CIE|26761.59|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||28/07/2020|46546.33|-18669.09|01-07-2020 to 01-07-2021|POL-F&amp;A-Jun-19-1315\\R1|POL-F&amp;A-Jun-19-1315\\R1|688.83|28513/17|53950|107383.42192704347|","-7546|-7546|1128|15|SOCIETE A.E. PATEL &amp; CIE|0|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/07/2020|6418.32|1128|01-07-2020 to 01-07-2021|POL-PA-Jun-19-1298\\R1|POL-PA-Jun-19-1298\\R1|26.32|28513/17|7520|-6418.047832585949|","-18262|-18262|2625|15|SOCIETE A.E. PATEL &amp; CIE|-83.35|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY||25/03/2021|15074.25|2708.35|01-07-2020 to 01-07-2021|POL-PI-Jun-19-1049\\R1|POL-PI-Jun-19-1049\\R1|199.25|41856/17|17500|-15553.53777702445|","-35123|-35123|5250|15|SOCIETE A.E. PATEL &amp; CIE|0|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||28/07/2020|29872.5|5250|01-07-2020 to 01-07-2021|POL-PPL-Jun-19-1086\\R1|POL-PPL-Jun-19-1086\\R1|122.5|28513/17|35000|-29872.925261584453|","-15053|-15053|2250|15|SOCIETE A.E. PATEL &amp; CIE|0|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||28/02/2021|13002.5|2250|01-07-2020 to 01-07-2021|POL-GIT-Jun-19-1062\\R1|POL-GIT-Jun-19-1062\\R1|252.5|23241/18/R2|15000|-12832.429601704638|","-22724|-22724|3396.75|15|SOCIETE A.E. PATEL &amp; CIE|-0.25|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||28/07/2020|19327.51|3397|01-07-2020 to 01-07-2021|POL-LOP(F&amp;A)-Jun-19-1076\\R1|POL-LOP(F&amp;A)-Jun-19-1076\\R1|79.26|28513/17|22645|-19327.288863971808|","-5268|-5268|787.5|15|SOCIETE A.E. PATEL &amp; CIE|-0.5|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||28/07/2020|4480.88|788|01-07-2020 to 01-07-2021|POL-EE-Jun-19-1135\\R1|POL-EE-Jun-19-1135\\R1|18.38|28513/17|5250|-4480.556801141907|","-11059|-11059|1653|15|SOCIETE A.E. PATEL &amp; CIE|0|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN||28/07/2020|9405.57|1653|01-07-2020 to 01-07-2021|POL-M B-D-Jun-19-1027\\R1|POL-M B-D-Jun-19-1027\\R1|38.57|28513/17|11020|-9405.93572496263|","-5469|-5469|817.5|15|SOCIETE A.E. PATEL &amp; CIE|-0.5|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||28/07/2020|4651.58|818|01-07-2020 to 01-07-2021|POL-EL-Jun-19-1227\\R1|POL-EL-Jun-19-1227\\R1|19.08|28513/17|5450|-4651.511958135555|","-25984|-25984|3884.02|15|SOCIETE HARBOUR VIEW|0.02|0|Correction to be done by CBL amount not in aging|MUR|16/07/2023|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||26/10/2023|22100.05|3884|16-07-2023 to 01-07-2024|POL-PL-Jun-19-1216\\R4|POL-PL-Jun-19-1216\\R4|90.63|22560/23/N|25893.44|-22099.99046338776|","-1809|-1809|270.37|15|SOCIETE HARBOUR VIEW|0.37|0|Correction to be done by CBL amount not in aging|MUR|16/07/2023|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||26/10/2023|1538.4|270|16-07-2023 to 01-07-2024|POL-EE-Jun-19-1133\\R4|POL-EE-Jun-19-1133\\R4|6.3|22560/23/N|1802.47|-1538.5956202281109|","-2531|-2531|378.27|15|SOCIETE HARBOUR VIEW|0.27|0|Correction to be done by CBL amount not in aging|MUR|16/07/2023|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||26/10/2023|2152.34|378|16-07-2023 to 01-07-2024|POL-EL-Jun-19-1222\\R4|POL-EL-Jun-19-1222\\R4|8.82|22560/23/N|2521.79|-2152.6717036603823|","-8170|-8170|1221.26|15|SOCIETE HARBOUR VIEW|0.26|0|Correction to be done by CBL amount not in aging|MUR|16/07/2023|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||26/10/2023|6948.99|1221|16-07-2023 to 01-07-2024|POL-PA-Jun-19-1294\\R4|POL-PA-Jun-19-1294\\R4|28.5|22560/23/N|8141.75|-6948.777369113552|","38494|38494|53811.97|15|SOCIETE HARBOUR VIEW|59557.93|0|Correction to be done by CBL amount not in aging|MUR|16/07/2023|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||26/10/2023|306690.1|-5745.96000000003|16-07-2023 to 01-07-2024|POL-F&amp;A-Jun-19-1309\\R4|POL-F&amp;A-Jun-19-1309\\R4|1755.61|22560/23/N|358746.46|32748.019198336366|","2|2|16382.06|8|SOLUTION INTEGRAL LIMITED|16382.34|0|Correction to be done by CBL amount not in aging|MUR|01/02/2024|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/04/2024|189826.69|-0.279999999997017|01-02-2024 to 01-02-2025|POL-HEALTH-Mar-20-133\\R4|POL-HEALTH-Mar-20-133\\R4|1433|MED/2023/00744/R1|204775.75|1.8411118829826572|","-8530|-8530|1275|15|SYNDICAT DES CO PROP. DES \"RESIDENCES DU NORD\"|0|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||25/01/2021|7254.75|1275|01-01-2021 to 01-01-2022|POL-PL-Nov-19-1500\\R1|POL-PL-Nov-19-1500\\R1|29.75|12616/13/R8|8500|-7254.962630792227|","-72885|-72885|10819.95|15|SYNDICAT DES CO PROP. DES \"RESIDENCES DU NORD\"|-0.05|0|Correction to be done by CBL amount not in aging|MUR|01/01/2023|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||13/07/2023|62065.53|10820|01-01-2023 to 01-01-2024|POL-F&amp;A-Nov-19-1601\\R3|POL-F&amp;A-Nov-19-1601\\R3|752.48|12616/13|72133|-62065.12125666182|","-1109|-1109|165.75|15|SYNDICAT DES CO PROP. DES \"RESIDENCES DU NORD\"|-0.25|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||25/01/2021|943.12|166|01-01-2021 to 01-01-2022|POL-EL-Nov-19-1510\\R1|POL-EL-Nov-19-1510\\R1|3.87|12616/13/R8|1105|-943.2305680557685|","81415|81415|165.75|15|SYNDICAT DES CO PROP. DES \"RESIDENCES DU NORD\"|12335.15|0|Correction to be done by CBL amount not in aging|MUR|01/01/2023|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||14/07/2023|943.12|-12169.4|01-01-2023 to 01-01-2024|POL-EL-Nov-19-1510\\R3|POL-EL-Nov-19-1510\\R3|3.87|12616/13|1105|69245.37123377853|","9639|9639|10819.95|15|SYNDICAT DES CO PROP. DES \"RESIDENCES DU NORD\"|12250.75|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||25/01/2021|62065.53|-1430.8|01-01-2021 to 01-01-2022|POL-F&amp;A-Nov-19-1601\\R1|POL-F&amp;A-Nov-19-1601\\R1|752.48|12616/13/R8|72133|8208.077159812901|","-8530|-8530|1275|15|SYNDICAT DES CO PROP. DES \"RESIDENCES DU NORD\"|0|0|Correction to be done by CBL amount not in aging|MUR|01/01/2023|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||30/06/2023|7254.75|1275|01-01-2023 to 01-01-2024|POL-PL-Nov-19-1500\\R3|POL-PL-Nov-19-1500\\R3|29.75|12616/13|8500|-7254.962630792227|","-160800|-160800|24000|15|SYSTEMS BUILDING CONTRACTING LTD|0|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY||31/12/2019|136800|24000|01-07-2019 to 01-07-2020|POL-PI-Jun-19-1061|POL-PI-Jun-19-1061|800|17885/09|160000|-136800|","2294|121077.32|-288|12.5|THE MAURITIUS COMMERCIAL BANK LTD &amp;/OR THE MAURITIUS COMMERCIAL BANK (MADAGASCAR) S.A - (FOR ACCOUNT OF VISA PLATINUM DEBIT CARDHOLDERS)|0|0|Correction to be done by CBL amount not same as in aging|EUR|01/12/2024|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL &amp; PERSONAL ACCIDENT||30/09/2025|-2006.03|-288|01-12-2024 to 30-06-2025|POL-TRPA-Nov-24-1|POL-TRPA-Nov-24-1\\E1|10|31924/24/N|-2304.03|105876.87878519463|","0.01|0.5278|1166.57|12.5|THE MAURITIUS COMMERCIAL BANK LTD &amp;/OR THE MAURITIUS COMMERCIAL BANK (MADAGASCAR) S.A - (FOR ACCOUNT OF VISA PLATINUM DEBIT CARDHOLDERS)|1166.2|0|Correction to be done by CBL amount not in aging|EUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL &amp; PERSONAL ACCIDENT||31/07/2025|8175.98|0.369999999999891|01-07-2025 to 30-06-2026|POL-TRPA-Nov-24-1\\R1|POL-TRPA-Nov-24-1\\R1|10|31924/24/N/R1|9332.55|0.46189554714719216|","0.01|0.5278|1945.83|12.5|THE MAURITIUS COMMERCIAL BANK LTD (FOR ACCOUNT OF FCY CARDHOLDERS)|1945.71|0|Correction to be done by CBL amount not in aging|EUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL &amp; PERSONAL ACCIDENT||31/10/2024|13630.84|0.119999999999891|01-10-2024 to 30-06-2025|POL-TRPA-Oct-23-1\\R1|POL-TRPA-Oct-23-1\\R1|10|FOREIGN CURRENCY CREDIT CARD|15566.67|0.46186748207415323|","0.01|0.5278|8142.88|12.5|THE MAURITIUS COMMERCIAL BANK LTD (FOR ACCOUNT OF INDIVIDUAL GOLD &amp; CORPORATE CARDHOLDERS)|8142.76|0|Correction to be done by CBL amount not in aging|EUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL &amp; PERSONAL ACCIDENT||31/07/2025|57010.16|0.119999999999891|01-10-2024 to 30-06-2025|POL-TRPA-Jul-19-1005\\R5|POL-TRPA-Jul-19-1005\\R5\\E1|10|28685/24/N|65143.04|0.46183512615834965|","-0.01|-0.5278|-1535.37|12.5|THE MAURITIUS COMMERCIAL BANK LTD (FOR ACCOUNT OF THE AMEX GOLD &amp; GREEN CARDHOLDERS)|-1535.75|0|Correction to be done by CBL amount not in aging|EUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL &amp; PERSONAL ACCIDENT||31/07/2025|-10737.59|0.380000000000109|01-10-2024 to 30-06-2025|POL-TRPA-Jul-19-1004\\R5|POL-TRPA-Jul-19-1004\\R5\\E1|10|28612/24/N|-12282.96|-0.461771243611973|"]</t>
+  </si>
+  <si>
+    <t>["0.01|0.5278|4983.63|12.5|THE MAURITIUS COMMERCIAL BANK LTD (FOR ACCOUNT OF THE AMEX GOLD &amp; GREEN CARDHOLDERS)|4983.26|0|Correction to be done by CBL amount not in aging|EUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL &amp; PERSONAL ACCIDENT||31/07/2025|34895.43|0.369999999999891|01-07-2025 to 30-06-2026|POL-TRPA-Jul-19-1004\\R6|POL-TRPA-Jul-19-1004\\R6|10|28612/24/N/R1|39869.06|0.46184157685762905|","0.01|0.5278|530.37|12.5|THE MAURITIUS COMMERCIAL BANK LTD (FOR ACCOUNT OF THE PLATINUM CARDHOLDERS)|530.75|0|Correction to be done by CBL amount not in aging|EUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL &amp; PERSONAL ACCIDENT||31/07/2025|3722.56|-0.379999999999995|01-10-2024 to 30-06-2025|POL-TRPA-Nov-19-1011\\R5|POL-TRPA-Nov-19-1011\\R5\\E1|10|28687/24/N|4242.93|0.46197966296176995|","0.01|0.5278|751.88|12.5|THE MAURITIUS COMMERCIAL BANK LTD - SEYCHELLES (FOR ACCOUNT OF INDIVIDUAL GOLD CARDHOLDERS)|751.76|0|Correction to be done by CBL amount not in aging|EUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL &amp; PERSONAL ACCIDENT||31/10/2024|5273.13|0.120000000000005|01-10-2024 to 30-06-2025|POL-TRPA-Aug-20-1003\\R4|POL-TRPA-Aug-20-1003\\R4|10|VISA GOLD - SEYCHELLES|6015.01|0.4619341733872641|","901.82|901.82|567|15|THOMAS MORE (INTERNATIONAL) LTD|701.81|0|Correction to be done by CBL amount not in aging|MUR|24/05/2019|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||11/07/2019|3228|-134.81|24-05-2019 to 01-04-2020|POL-EE-Jun-19-1123|POL-EE-Jun-19-1123|13|17410/19/N|3782|767.0816758893282|","-2418|-2418|||THOMAS MORE (INTERNATIONAL) LTD||0|Correction to be done by CBL amount not in aging|MUR|24/05/2019|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||31/05/2021||888.01|24-05-2019 to 01-04-2020|POL-EE-Jun-19-1125|POL-EE-Jun-19-1125\\E1||P/10/6D99/18/1975/000/01 VOUCHER NOT OK||-2418|","1515.96|1515.96|394|15|THOMAS MORE (INTERNATIONAL) LTD|620.61|0|Correction to be done by CBL amount not in aging|MUR|24/05/2019|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||11/07/2019|2239|-226.61|24-05-2019 to 01-04-2020|POL-EL-Jun-19-1194|POL-EL-Jun-19-1194|9|17410/19/N|2624|1289.112966198253|"]</t>
+  </si>
+  <si>
+    <t>["-84794|-84794|42185.95|15|AMALA VILLAS LTD AND THE SUCCESSIVE OWNERS OF THE BUILDINGS|29530.12|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|DEFECTS INSURANCE||03/03/2025|240459.71|12655.83|01-01-2026 to 01-01-2036|POL-DEF-Feb-25-1004|POL-DEF-Feb-25-1004|1406|-|281239.66|-72138.16992534044|","-570854|-570854|142003.65|15|ONE T-APARTMENT LTD &amp;/OR SUBSEQUQNT OWNERS|56801.17|0||MUR|12/09/2025|MAURITIUS UNION ASSURANCE CO LTD|DEFECTS INSURANCE||07/08/2025|809420.38|85202.48|12-09-2025 to 12-09-2035|POL-DEF-Jul-25-1022|POL-DEF-Jul-25-1022|4733||946691.03|-485651.87238808756|"]</t>
+  </si>
+  <si>
+    <t>["Defects Insurance","Defects Insurance"]</t>
+  </si>
+  <si>
+    <t>miscellaneous</t>
+  </si>
+  <si>
+    <t>2026-07-28T06:47:46.081Z</t>
+  </si>
+  <si>
+    <t>["-6298|-6298|16165.44|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|15224.66|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||31/08/2024|91981.33|940.780000000002|01-07-2024 to 30-06-2025|POL-EE-Jul-19-1186\\R5|POL-EE-Jul-19-1186\\R5|377.19|23694/19/R5|107769.58|-5356.594712352482|","-73|-73|5663.74|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|5652.77|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||31/08/2024|32726.68|10.9700000000003|01-07-2024 to 30-06-2025|POL-F&amp;A-Jul-19-1421\\R5|POL-F&amp;A-Jul-19-1421\\R5|632.15|23694/19/R4|37758.27|-62.23030745691243|","-14017|-14017|11960.19|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|11871.34|0||MUR|01/07/2023|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||28/09/2023|68053.5|88.8499999999985|01-07-2023 to 30-06-2024|POL-EL-Jul-19-1343\\R4|POL-EL-Jul-19-1343\\R4|279.06|23694/19/R4|79734.63|-11921.783753505182|","-6722.37|-6722.37|34277.43|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|33966.35|0||MUR|01/07/2023|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/09/2023|195038.57|311.080000000002|01-07-2023 to 30-06-2024|POL-PA-Jul-19-1407\\R4|POL-PA-Jul-19-1407\\R4|799.81|23694/19/R4|228516.19|-5717.5314056188845|","-35164|-35164|5767.11|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|900.54|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||31/07/2025|33314.87|4866.57|01-07-2025 to 30-06-2026|POL-F&amp;A-Jul-19-1421\\R6|POL-F&amp;A-Jul-19-1421\\R6|634.58|23694/19/R6 23694/19/R6/E3|38447.4|-29975.044475228737|","-18064|-18064|4725|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR VIVO ENERYGY MAURITIUS LTD &amp;/OR SUBSIDIARIES|2700.16|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||31/07/2025|26885.25|2024.84|01-07-2025 to 30-06-2026|POL-PPL-Jul-19-1117\\R6|POL-PPL-Jul-19-1117\\R6|110.25|23694/19/R6|31500|-15363.850523168909|","-257115|-257115|46578.65|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|15790.82|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||31/07/2025|265032.5|30787.83|01-07-2025 to 30-06-2026|POL-PA-Jul-19-1407\\R6|POL-PA-Jul-19-1407\\R6|1086.83|23694/19/R6|310524.32|-218682.2622922832|","-76431.99|-76431.99|18373.44|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|10764.87|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||31/07/2025|104544.89|7608.57|01-07-2025 to 30-06-2026|POL-EE-Jul-19-1186\\R6|POL-EE-Jul-19-1186\\R6|428.7|23694/19/R6|122489.63|-65007.17986512753|","-3056|-3056|10833.88|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|10377.01|0||MUR|01/07/2023|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||28/09/2023|61644.76|456.869999999999|01-07-2023 to 30-06-2024|POL-EE-Jul-19-1186\\R4|POL-EE-Jul-19-1186\\R4|252.79|23694/19/R4|72225.85|-2599.1986957812674|","-4516|-4516|4725|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR VIVO ENERYGY MAURITIUS LTD &amp;/OR SUBSIDIARIES|4050.23|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||31/08/2024|26885.25|674.77|01-07-2024 to 30-06-2025|POL-PPL-Jul-19-1117\\R5|POL-PPL-Jul-19-1117\\R5|110.25|23694/19/R5|31500|-3840.9626307922276|","-192|-192|5168.14|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|5139.63|0||MUR|01/07/2023|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||28/09/2023|29906.69|28.5099999999993|01-07-2023 to 30-06-2024|POL-F&amp;A-Jul-19-1421\\R4|POL-F&amp;A-Jul-19-1421\\R4|620.58|23694/19/R4|34454.25|-163.70954556301484|","-2881|-133707.21|430.05|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|0|0|Correction to be done by CBL amount not same as in aging|USD|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|DIRECTORS &amp; OFFICERS LIABILITY||16/07/2026|2451.02|430.05|01-07-2026 to 30-06-2027|POL-D&amp;O-Jul-19-1054\\R7|POL-D&amp;O-Jul-19-1054\\R7|14.07||2867|-113749.07442519619|Timing Difference","-72683|-72683|10864.43|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|0.43|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||31/07/2025|61818.57|10864|01-07-2025 to 30-06-2026|POL-LOP(F&amp;A)-Jul-19-1113\\R6|POL-LOP(F&amp;A)-Jul-19-1113\\R6|253.5|23694/19/R6|72429.5|-61818.57|","-41394|-41394|6187.5|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|-0.5|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||31/07/2025|35206.88|6188|01-07-2025 to 30-06-2026|POL-PA-Jul-19-1408\\R6|POL-PA-Jul-19-1408\\R6|144.38|23694/19/R6|41250|-35206.556801188955|","-33822|-33822|5055.6|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|484.650000000001|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|MONEY||31/07/2025|28766.37|4570.95|01-07-2025 to 30-06-2026|POL-MON-Jul-19-1117\\R6|POL-MON-Jul-19-1117\\R6|117.97|23694/19/R6|33704|-28766.395515695862|","-65875|-65875|18482.44|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|11523.45|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||31/07/2025|105165.08|6958.99|01-07-2025 to 30-06-2026|POL-ARM(P&amp;M)-Jul-19-1099\\R6|POL-ARM(P&amp;M)-Jul-19-1099\\R6|431.26|23694/19/R6|123216.26|-56028.213465179084|","-92161|-92161|16646.43|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|5309.4|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||31/07/2025|94718.24|11337.03|01-07-2025 to 30-06-2026|POL-EL-Jul-19-1343\\R6|POL-EL-Jul-19-1343\\R6|388.42|23694/19/R6|110976.25|-78385.07236307529|","-2865|-2865|6375|15|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR VIVO ENERYGY MAURITIUS LTD &amp;/OR SUBSIDIARIES|5946.62|0||MUR|01/07/2023|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||28/09/2023|36273.75|428.379999999999|01-07-2023 to 30-06-2024|POL-PPL-Jul-19-1117\\R4|POL-PPL-Jul-19-1117\\R4|148.75|23694/19/R4|42500|-2436.748878923767|","-213|-213|16.88|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|-0.12|0||MUR|14/08/2024|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||04/11/2024|196.07|17|14-08-2024 to 01-07-2025|POL-CP-Jul-23-8\\R1|POL-CP-Jul-23-8\\R1\\E2|100.39|19358/23|112.56|-196.1160366283165|","-48350|-48350|7212.33|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|0.33|0||MUR|06/03/2025|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||04/06/2025|41138.15|7212|06-03-2025 to 01-07-2025|POL-CP-Jul-23-8\\R1|POL-CP-Jul-23-8\\R1\\E4|268.29|19358/23|48082.19|-41137.74160049704|","-380|-380|656.95|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD|600.25|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||26/08/2024|3738.02|56.7|01-07-2024 to 01-07-2025|POL-ARMISC-Jul-23-23\\R1|POL-ARMISC-Jul-23-23\\R1|15.32|17111/23/N/E6|4379.65|-323.1984746198495|","-6643.98|-6643.98|21304.23|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|20311.45|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||26/08/2024|121221.13|992.779999999999|01-07-2024 to 01-07-2025|POL-EL-Jul-23-1039\\R1|POL-EL-Jul-23-1039\\R1|497.11|17111/23/R1|142028.25|-5650.859350907094|","-4424|-4424|1653|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|991.78|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||05/08/2025|9405.57|661.22|01-07-2025 to 01-07-2026|POL-FID-Jul-23-10\\R2|POL-FID-Jul-23-10\\R2|38.57|17111/23/R1|11020|-3762.714499252616|","-6556|-6556|1966.76|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR MR VINCENT LAGARDE &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD &amp;/OR THE HOUSE CANTEEN LTD|986.9|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|MONEY||05/08/2025|11190.87|979.86|01-07-2025 to 01-07-2026|POL-MON-Jul-23-6\\R2|POL-MON-Jul-23-6\\R2|45.93|17111/23/R1|13111.7|-5576.030312449887|","-1952|-1952|276.8|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|-0.2|0||MUR|13/08/2024|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||28/01/2025|1675|277|13-08-2024 to 01-07-2025|POL-CP-Jul-23-8\\R1|POL-CP-Jul-23-8\\R1\\E1|106.46|19358/23|1845.34|-1675.1716364381596|","-948865|-948865|251449.49|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|109616.49|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||05/08/2025|1431247.57|141833|01-07-2025 to 01-07-2026|POL-CP-Jul-23-8\\R2|POL-CP-Jul-23-8\\R2|6367.13|19358/23|1676329.93|-807073.8089410163|","-1054|-1054|1496.25|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|1338.96|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||26/08/2024|8513.67|157.29|01-07-2024 to 01-07-2025|POL-FID-Jul-23-10\\R1|POL-FID-Jul-23-10\\R1|34.92|17111/23/R1|9975|-896.4515380742304|","-39859|-39859|127825.41|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|121867.84|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||26/08/2024|727326.58|5957.56999999998|01-07-2024 to 01-07-2025|POL-PA-Jul-23-1051\\R1|POL-PA-Jul-23-1051\\R1|2982.59|17111/23/R1|852169.4|-33901.00296933181|","-813|-813|106.6|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD|-0.4|0||MUR|01/09/2023|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||20/03/2024|706.57|107|01-09-2023 to 01-07-2024|POL-CP-Jul-23-8|POL-CP-Jul-23-8\\E2|102.49|19358/23/N/E3|710.68|-706.4222856229325|","-400|-400|83.61|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD|38.33|0||MUR|01/09/2023|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||20/03/2024|575.75|45.28|01-09-2023 to 01-07-2024|POL-ARMISC-Jul-23-23|POL-ARMISC-Jul-23-23\\E1|101.95|17111/23/E4|557.41|-349.27808784275663|","-4178|-4178|2285.71|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR MR VINCENT LAGARDE &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|1661.15|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|MONEY||26/08/2024|13005.66|624.559999999999|01-07-2024 to 01-07-2025|POL-MON-Jul-23-6\\R1|POL-MON-Jul-23-6\\R1|53.29|17111/23/R1|15238.08|-3553.4845785564016|","-4272|-4272|638.47|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD|0.47|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||05/08/2025|3632.89|638|01-07-2025 to 01-07-2026|POL-ARMISC-Jul-23-23\\R2|POL-ARMISC-Jul-23-23\\R2|14.9|17111/23/N/E6|4256.46|-3633.434334731795|","-861|-861|113.81|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|-0.19|0||MUR|30/01/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||29/05/2025|747.6|114|30-01-2025 to 01-07-2025|POL-EL-Jul-23-1039\\R1|POL-EL-Jul-23-1039\\R1\\E1|102.66|17111/23/R1/E1|758.75|-747.2441694431224|","-14622|-14622|5827.5|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|3642.5|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||26/08/2024|33158.51|2185|01-07-2024 to 01-07-2025|POL-PL-Jul-23-1040\\R1|POL-PL-Jul-23-1040\\R1|136.01|17111/23/R1|38850|-12436.351737969595|","-12923|-12923|1916.71|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|-0.29|0||MUR|17/03/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||26/05/2026|11006.09|1917|17-03-2026 to 01-07-2026|POL-CP-Jul-23-8\\R2|POL-CP-Jul-23-8\\R2\\E4|144.72||12778.08|-11006.260335995295|"]</t>
+  </si>
+  <si>
+    <t>["-140405.66|939813.95|RHT HOLDING LTD &amp;/OR RHT BUS SERVICES LTD &amp;/OR SUBSIDIARIES|01/10/2025|544657.1||01/07/25 to 30/06/26||23694/19/R6||544657.1|23/07/2025|JRNI.250723.428|Non-Motor Corporate","-251449.5|1682697|NATEC MEDICAL LTD|01/10/2025|792773.85||01/07/25 to 30/06/26||19358/23/R2||792773.85|22/07/2025|JRNI.250722.446|Non-Motor Corporate","-130910.83|876293.97|NATEC MEDICAL LTD|01/10/2025|186105.45||01/07/25 to 30/06/26||17111/23/R2||186105.45|19/07/2025|JRNI.250719.27|Non-Motor Corporate","-7684.95|51512|NATEC MEDICAL LTD|01/08/2026|||01/07/25 to 30/06/26||19358/23/R2/E5||43827.05|28/05/2026|JRNI.260528.560|Non-Motor Corporate","-1916.7|12923|NATEC MEDICAL LTD|01/07/2026|11006.3||01/07/25 to 30/06/26||19358/23/R2/E4||11006.3|15/04/2026|JRNI.260415.301|Non-Motor Corporate","-9152|1368|Bank of Mauritius|29/09/2025|||01/07/25 to 30/06/26||19120/25/N/E1||-7784|29/09/2025|JRNI.250929.287|Travel","-12763.8|85840|Syndicat des Coproprietaires de L`Immeuble Residence St Clement Court|01/04/2026|31079.96||02/01/26 to 31/12/26||13617/08/R17||31079.96|22/01/2026|JRNI.260122.442|Non-Motor Corporate","-9204|1475.8|DUCHENNE Loic Damien|27/01/2026|||09/01/25 to 31/01/26||996/25/N/E1||-7828.2|27/01/2026|JRNI.260127.81|Yacht Hull/Tpl","-48123.31|3849.86|CAY MANAGEMENT CPY LTD|30/11/2025|||01/10/25 to 30/09/26|MD16M00777|MD16M00777/R9/E2|MD16M00777|-44273.45|25/05/2026|JRNNHZ.260525.14|Medical","-868.43|10855.49|CAY MANAGEMENT CPY LTD|30/11/2025|9987.06||01/10/25 to 30/09/26|MD16M00777|MD16M00777/R9/E3|MD16M00777|9987.06|24/06/2026|JRNNHZ.260624.34|Medical","-23068.5|155078|Kasa Textile &amp; Co Ltd|01/04/2026|73338.2|Payment done after 30.06.2026|01/01/26 to 31/12/26||26063/21/R4||73338.2|06/01/2026|JRNI.260106.450|Motor","-3143.28|39291|Kasa Textile &amp; Co Ltd|01/07/2026|20749.66||01/03/26 to 28/02/27|MD08M01085|MD08M01085/R18|MD08M01085|20749.66|31/05/2026|JRNNHZ.260531.65|Medical","-3260|40750|Kasa Textile &amp; Co Ltd|01/08/2026|||01/03/26 to 28/02/27|MD08M01085|MD08M01085/R18|MD08M01085|37490|30/06/2026|JRNNHZ.260630.468|Medical","-6919.33|46789.96|Tartuffe Ltee|01/10/2025|19409.18||01/07/25 to 30/06/26||25773/16/R9||19409.18|28/07/2025|JRNI.250728.434|Non-Motor Corporate","-11540.96|1825.13|Tartuffe Ltee|28/04/2026|100||01/07/25 to 30/06/26||25773/16/R9/E2||-9715.83|17/04/2026|JRNI.260417.279|Non-Motor Corporate","-6750|45358|ERC Levage Ltee|12/06/2026|38608|Payment done after 30.06.2026|11/05/26 to 11/05/26|POL-GIT-May-26-18|11642/26/N|POL-GIT-May-26-18|38608|12/05/2026|JRNI.260512.238|Inland Transit","-1024.8|7156|Royal Car Rental Ltd|01/02/2026|6131.2||17/10/25 to 31/10/26||32587/25/N||6131.2|20/11/2025|JRNI.251120.318|Non-Motor Corporate","-1292958.7|8666994|Royal Car Rental Ltd|15/10/2026|2938487.62||01/01/26 to 31/12/26||31162/23/R2||5167497.43|06/01/2026|JRNI.260106.423|Motor","-5260.05|35290|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/09/2026|||01/05/25 to 30/04/26||9314/08/R17/E2||30029.95|29/06/2026|JRNI.260629.452|Non-Motor Corporate","-2730.9|18570|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/08/2026|||01/05/26 to 30/04/27||22405/20/R6||15839.1|13/05/2026|JRNI.260513.103|Non-Motor Corporate","-374330.06|2504767.95|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/08/2026|||01/05/26 to 30/04/27||9314/08/R18||2130437.89|25/05/2026|JRNI.260525.474|Non-Motor Corporate","-22567.5|151477|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/06/2026|128909.5||11/07/25 to 11/09/26||7049/26/N||128909.5|26/03/2026|JRNI.260326.415|Non-Motor Corporate","-106601.08|1353604.63|A.E. Patel &amp; Co. Ltd|31/03/2026|291872.13||01/10/25 to 30/09/26|MD17M00713|MD17M00713/R9|MD17M00713|291872.13|24/11/2025|JRNNHZ.251124.36|Medical","-234.45|1572|A.E. Patel &amp; Co. Ltd|01/09/2026|||01/07/25 to 30/06/26||21522/17/R9/E10||1337.55|17/06/2026|JRNI.260617.192|Motor","-37642|5726.65|Lavastone Ltd &amp;/or Subsidiaries|09/01/2026|100||01/10/25 to 30/09/26||33502/19/R6/E1||-31915.35|08/01/2026|JRNI.260108.274|Non-Motor Corporate","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.38|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.37|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.36|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|3327.96||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|3327.96|10/03/2026|JRNNHZ.260310.35|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.252|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.251|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|57.63||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|57.63|25/06/2026|JRNNHZ.260625.250|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|10/03/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.248|Medical","-68.64|572.05|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/03/2026|75.26||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E78|MED/2025/01055|75.26|19/02/2026|JRNNHZ.260219.82|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/03/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.61|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.60|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.59|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|1624.17||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.17|19/02/2026|JRNNHZ.260219.58|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.57|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/10/2025|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.56|Medical","-367.1|3059.17|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|2692.07||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E74|MED/2025/01055|2692.07|19/02/2026|JRNNHZ.260219.37|Medical","-3396.48|28304|HARDY HENRY &amp; CIE LTEE|01/08/2026||Payment done after 30.06.2026|01/10/25 to 30/06/26|MED/2023/01269|MED/2023/01269/R2|MED/2023/01269|24907.52|30/06/2026|JRNNHZ.260630.789|Medical","-62149.68|517914|Hardy Henry Services Ltd|01/08/2026|||01/10/25 to 30/06/26|MD18M01064|MD18M01064/R7|MD18M01064|455764.32|30/06/2026|JRNNHZ.260630.599|Medical","-1014.36|8453|HARDY HENRY &amp; CIE LTEE|01/08/2026|||01/10/25 to 30/06/26|MD18M01063|MD18M01063/R7|MD18M01063|7438.64|30/06/2026|JRNNHZ.260630.598|Medical","-17714.88|147624|HARDY HENRY MANAGEMENT LTD|01/08/2026|||01/10/25 to 30/06/26|MD18M01062|MD18M01062/R7|MD18M01062|129909.12|30/06/2026|JRNNHZ.260630.597|Medical","-5604.96|46708|HARDY HENRY TEXTILES LTEE|01/08/2026|||01/10/25 to 30/06/26|MD18M01051|MD18M01051/R7|MD18M01051|41103.04|30/06/2026|JRNNHZ.260630.595|Medical","-195.99|1636|HARDY HENRY TEXTILES LTEE|01/08/2026|||01/10/25 to 30/06/26|MD04M00390|MD04M00390/R22|MD04M00390|1440.01|30/06/2026|JRNNHZ.260630.456|Medical","-3835.92|31966|Hardy Henry Services Ltd|01/08/2026|||01/10/25 to 30/06/26|MD02M00616|MD02M00616/R24|MD02M00616|28130.08|30/06/2026|JRNNHZ.260630.450|Medical","-3396.48|28304|HARDY HENRY &amp; CIE LTEE|01/07/2026|17476.02|Payment done after 30.06.2026|01/10/25 to 30/06/26|MED/2023/01269|MED/2023/01269/R2|MED/2023/01269|17476.02|31/05/2026|JRNNHZ.260531.397|Medical","-63366.36|528053|Hardy Henry Services Ltd|01/07/2026|418832.06||01/10/25 to 30/06/26|MD18M01064|MD18M01064/R7|MD18M01064|418832.06|31/05/2026|JRNNHZ.260531.197|Medical","-17714.88|147624|HARDY HENRY MANAGEMENT LTD|01/07/2026|76436.11||01/10/25 to 30/06/26|MD18M01062|MD18M01062/R7|MD18M01062|76436.11|31/05/2026|JRNNHZ.260531.195|Medical","-5604.96|46708|HARDY HENRY TEXTILES LTEE|01/07/2026|41103.04||01/10/25 to 30/06/26|MD18M01051|MD18M01051/R7|MD18M01051|41103.04|31/05/2026|JRNNHZ.260531.193|Medical","-3835.92|31966|Hardy Henry Services Ltd|01/07/2026|28130.08||01/10/25 to 30/06/26|MD02M00616|MD02M00616/R24|MD02M00616|28130.08|31/05/2026|JRNNHZ.260531.47|Medical","-86931.38|582070.94|H.VAULBERT DE CHANTILLY LTD (HVC LTD)|01/04/2026|495139.56||01/01/26 to 31/12/26||2321/20/R6||495139.56|30/01/2026|JRNI.260130.518|Non-Motor Corporate","-22324.99|1785.99|ORANGE EIGHT LTD ORANGE EIGHT LTD|31/03/2026|||01/10/25 to 30/09/26|MED/2022/01410|MED/2022/01410/R3/E7|MED/2022/01410|-20539|02/06/2026|JRNNHZ.260602.5|Medical","-45701.76|575270.9|ORANGE EIGHT LTD ORANGE EIGHT LTD|31/03/2026|217638.96||01/10/25 to 30/09/26|MED/2022/01410|MED/2022/01410/R3|MED/2022/01410|217638.96|28/11/2025|JRNNHZ.251128.28|Medical","-3865.35|26359|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/04/2026|22493.65||01/02/26 to 31/01/27||6162/25/R2||22493.65|28/01/2026|JRNI.260128.450|Non-Motor Corporate","-750|5118|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/08/2026|||16/11/25 to 15/06/26||36726/25/N/E2||4368|13/05/2026|JRNI.260513.284|Car/Ear (One Off)","-74398.8|498228|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/03/2026|278436.63||01/12/25 to 30/11/26||46037/12/R13||278436.63|30/12/2025|JRNI.251230.598|Non-Motor Corporate","-900|6121|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/09/2026|||16/11/25 to 15/08/26||36731/25/N/E3||5221|29/06/2026|JRNI.260629.604|Non-Motor Corporate","-450|3111|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/07/2026|2661||16/11/25 to 15/05/26||36731/25/N/E1||2661|23/04/2026|JRNI.260423.350|Non-Motor Corporate","-2756.85|18543|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/02/2026|9278.51||16/10/23 to 15/10/26||27489/23/N/E2||9278.51|28/11/2025|JRNI.251128.356|Car/Ear (One Off)","-18900|126630|Golden Fund Management Services Ltd &amp;/or The Mauritius Development Investment Trust Co Ltd|01/08/2026||Payment done after 30.06.2026|01/05/26 to 30/04/27|POL-C+PI-Jun-19-1003\\R7|15398/18/R8|POL-C+PI-Jun-19-1003\\R7|107730|28/05/2026|JRNI.260528.571|Financial","-7735.12|97089|Paris Onezime Marie Stephanie|02/03/2026|43569.57||01/01/26 to 31/12/26|MED/2023/00006|MED/2023/00006/R3|MED/2023/00006|43569.57|29/12/2025|JRNNHZ.251229.18|Medical","-2299.8|28747.56|Paris Onezime Marie Stephanie|02/03/2026|4969.88||01/01/26 to 31/12/26|MED/2023/00006|MED/2023/00006/R3/E1|MED/2023/00006|4969.88|22/05/2026|JRNNHZ.260522.141|Medical","-20182.35|135220|Hefty Ltd|01/06/2026|115037.65||01/04/26 to 31/03/27||6400/26/N||115037.65|20/03/2026|JRNI.260320.119|Motor","-8891.25|59582|Hefty Ltd|01/06/2026|50690.75||01/04/26 to 31/03/27||6368/26/N||50690.75|20/03/2026|JRNI.260320.18|Motor","-27536.85|184322|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/05/26||12718/24/N/E5||156785.15|30/06/2026|JRNI.260630.570|Car/Ear (One Off)","-18000|120520|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/05/26||12718/24/N/E4||102520|30/06/2026|JRNI.260630.548|Car/Ear (One Off)","-108000|722620|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/08/26||12718/24/N/E7||614620|30/06/2026|JRNI.260630.605|Car/Ear (One Off)","-20045.25|134266|Rehm Grinaker Construction Co. Ltd|01/06/2026|114220.75||01/01/26 to 31/12/26||10936/21/R4/E2||114220.75|09/03/2026|JRNI.260309.20|Motor","-44294.4|557555.76|CREDIT GUARANTEE INSURANCE CO LTD|02/03/2026|238039.16||01/01/26 to 31/12/26|MD11M00167|MD11M00167/R15|MD11M00167|238039.16|14/01/2026|JRNNHZ.260114.222|Medical","-589.95|3947|Impact Production Ltd &amp;/or Event Strategy Ltd &amp;/or Mille Feux Ltd &amp;/or Marquee Design Ltd|01/09/2026|||01/04/26 to 31/03/27||8040/21/R5/E1||3357.05|04/06/2026|JRNI.260604.342|Non-Motor Corporate","-68411.52|458172.96|Impact Production Ltd &amp;/or Event Strategy Ltd &amp;/or Mille Feux Ltd &amp;/or Marquee Design Ltd|01/07/2026|389761.44||01/04/26 to 31/03/27||8040/21/R5||389761.44|30/04/2026|JRNI.260430.631|Non-Motor Corporate","-7372.5|49772|IMPACT PRODUCTION LTD|01/04/2026|42399.5||01/01/26 to 31/12/26||54552/15/R10||42399.5|06/01/2026|JRNI.260106.400|Motor","-6255.68|78196|KASA CORPORATE SERVICES LTD|01/07/2026|71940.32||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|71940.32|31/05/2026|JRNNHZ.260531.63|Medical","-13161.28|171425.68|KASA CORPORATE SERVICES LTD|01/06/2026|158264.4||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|158264.4|30/04/2026|JRNNHZ.260430.476|Medical","-76806|514632|KASA CORPORATE SERVICES LTD|01/04/2026|243234.45|Payment done after 30.06.2026|01/01/26 to 31/12/26||32859/23/R2||243234.45|06/01/2026|JRNI.260106.408|Motor","-3986.32|49829|KASA CORPORATE SERVICES LTD|01/08/2026|||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|45842.68|30/06/2026|JRNNHZ.260630.466|Medical","-121776.21|815182.95|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|01/07/2026|462223.22||01/03/26 to 28/02/27||8187/26/N||462223.22|07/04/2026|JRNI.260407.284|Non-Motor Corporate","-57631|8614.5|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|18/05/2026|||01/12/25 to 30/11/26||29742/23/R2/E1||-49016.5|18/05/2026|JRNI.260518.268|Motor","-38187|255971|CURRIMJEE JEEWANJEE AND COMPANY LIMITED|01/04/2026|27828.27|Payment done after 30.06.2026|01/01/26 to 31/12/26||1915/26/N||27828.27|28/01/2026|JRNI.260128.526|Non-Motor Corporate","-429672.4|2875008.96|Currimjee Jeewanjee &amp; Co Ltd|01/04/2026|729243.58|Payment done after 30.06.2026|01/01/26 to 31/12/26||1918/26/N||729243.58|28/01/2026|JRNI.260128.522|Non-Motor Corporate"]</t>
+  </si>
+  <si>
+    <t>["Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference"]</t>
+  </si>
+  <si>
+    <t>["Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference","Timing Difference"]</t>
   </si>
   <si>
     <t>partial</t>
   </si>
   <si>
-    <t>2026-07-29T11:13:19.856Z</t>
-  </si>
-  <si>
-    <t>["-2706390|-2706390|505697.43|15|BLUE GREEN SIGNATURE CO LTD AND THE SUBSEQUENT OWNERS|102050.13|0|MUR|01/12/2024|SANLAM GENERAL INSURANCE LTD|DEFECTS INSURANCE|08/06/2023|2884918.4|403647.3|01-12-2024 to 01-12-2034|POL-DEF-May-23-1012|POL-DEF-May-23-1012|19299.61|PY52706092023000011|3371316.22|-2302742.245079414|"]</t>
-  </si>
-  <si>
-    <t>["DEFECTS INSURANCE"]</t>
-  </si>
-  <si>
-    <t>2026-07-29T11:13:53.434Z</t>
-  </si>
-  <si>
-    <t>["||||||21976651.46|||14237413.36|||7739238.1"]</t>
-  </si>
-  <si>
-    <t>["Total"]</t>
-  </si>
-  <si>
-    <t>miscellaneous</t>
-  </si>
-  <si>
-    <t>2026-07-29T11:33:21.330Z</t>
-  </si>
-  <si>
-    <t>["570911.38||WEST BY MJ LTD (SITE B)||15/05/2024||674778|01/01/2026 - 31/12/2035|DN52706092024000007|103866.62|09/09/2024|RC0012024004120|570911.38","214175||AMARE 17.1 LTD &amp;/OR SUBSEQUENT OWNERS||21/02/2025||254875|27/10/2026 - 26/10/2036|DN52706092025000002|40700|24/11/2025|RC5272025000016|214175","524906||AZURI SMART CITY COMPANY LTD &amp;/OR SUBSEQUENT OWNERS||14/05/2025||3502314|01/01/2025 - 31/12/2034|DN52706092025000007|2977408|14/05/2025|RC0012025002049|524906","557966.09||AZURI SMART CITY COMPANY LTD &amp;/OR SUBSEQUENT OWNERS||15/09/2025||661764|01/05/2027 - 30/04/2037|DN52706092025000018|103797.91|28/02/2026|RC5272026000014|557966.09","159795.44||AZURI SMART CITY COMPANY LTD &amp;/OR SUBSEQUENT OWNERS||05/11/2025||2835991|01/09/2025 - 31/08/2035|DN52706092025000019|2142572.56|28/02/2026|RC5272026000015|693418.44","442554||MNJ PROPERTIES LTD||17/11/2025||2217718|01/06/2024 - 31/05/2034|DN52706092025000020|1775164|19/11/2025|RC5272025000012|442554"]</t>
-  </si>
-  <si>
-    <t>["DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE"]</t>
-  </si>
-  <si>
-    <t>2026-07-29T11:55:34.875Z</t>
-  </si>
-  <si>
-    <t>["||JEAN YAN MAYER||11/06/2026||43762|01/08/2026 - 31/07/2027|DN52708032026000005|43762|||0"]</t>
-  </si>
-  <si>
-    <t>["Transaction after 30.06.2026"]</t>
-  </si>
-  <si>
-    <t>2026-07-29T11:55:53.467Z</t>
-  </si>
-  <si>
-    <t>["259851.19||TAMARIN SAVANNAH LTD (PHASE 1B)||11/03/2024||309512|16/06/2025 - 15/06/2035|DN52706092024000005|49660.81|03/05/2024|RC0012024001764|259851.19","28721.32||AZURI SMART CITY COMPANY LTD||26/08/2024||292704|16/07/2024 - 15/07/2034|DN52706092024000010|80946.94|04/02/2025|RC0012025000412|211757.06","524906||AZURI SMART CITY COMPANY LTD &amp;/OR SUBSEQUENT OWNERS||14/05/2025||3502314|01/01/2025 - 31/12/2034|DN52706092025000007|2977408|14/05/2025|RC0012025002049|524906","557966.09||AZURI SMART CITY COMPANY LTD &amp;/OR SUBSEQUENT OWNERS||15/09/2025||661764|01/05/2027 - 30/04/2037|DN52706092025000018|103797.91|28/02/2026|RC5272026000014|557966.09","159795.44||AZURI SMART CITY COMPANY LTD &amp;/OR SUBSEQUENT OWNERS||05/11/2025||2835991|01/09/2025 - 31/08/2035|DN52706092025000019|2142572.56|28/02/2026|RC5272026000015|693418.44","604899.41||AZURI SMART CITY COMPANY LTD &amp;/OR CONTRACTORS &amp;/OR SUB CONTRACTORS||13/05/2024||716944|01/10/2025 - 30/09/2035|DN52706092024000006|112044.59|23/07/2024|RC0012024003219|604899.41","717168.47|| DIL PROPERTY DEVELOPMENT LTD||03/12/2024||848945|01/03/2026 - 29/02/2036|DN52706092024000012|131776.53|20/02/2025|RC0012025000649|717168.47","||CREATIVE PROPERTIES LTD||20/08/2025||104539.15|21/01/2026 - 20/01/2036|DN52706092025000012|104539.15|||0","||CREATIVE PROPERTIES LTD||20/08/2025||123023.42|20/03/2026 - 19/03/2036|DN52706092025000013|123023.42|||0","||CREATIVE PROPERTIES LTD||20/08/2025||89665|21/03/2026 - 20/03/2036|DN52706092025000014|89665|||0","||CREATIVE PROPERTIES LTD||20/08/2025||155045|02/06/2026 - 01/06/2036|DN52706092025000015|155045|||0","||CREATIVE PROPERTIES LTD||21/08/2025||72375|13/01/2026 - 12/01/2036|DN52706092025000016|72375|||0","||CREATIVE PROPERTIES LTD||21/08/2025||104539|28/11/2026 - 27/11/2036|DN52706092025000017|104539|||0","94602.37||SOCIETE EXSARTUM||02/05/2025||113523|03/03/2026 - 02/03/2036|DN52706092025000004|18920.63|04/06/2025|RC0012025002443|94602.37","93360.61||SOCIETE EXSARTUM||02/05/2025||112063|03/03/2026 - 02/03/2036|DN52706092025000005|18702.39|04/06/2025|RC0012025002442|93360.61","1816284.99||AZURI SMART CITY COMPANY LTD &amp;/OR CONTRACTORS &amp;/OR SUB CONTRACTORS||26/06/2025||2143140|19/07/2027 - 18/06/2037|DN52706092025000010|326855.01|14/10/2025|RC5272025000004|1816284.99","604899.41||AZURI SMART CITY COMPANY LTD &amp;/OR CONTRACTORS &amp;/OR SUB CONTRACTORS||13/05/2024||716944|01/10/2025 - 30/09/2035|DN52706092024000006|112044.59|23/07/2024|RC0012024003219|604899.41"]</t>
-  </si>
-  <si>
-    <t>["DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE","DEFECTS INSURANCE"]</t>
-  </si>
-  <si>
-    <t>2026-07-29T11:58:56.483Z</t>
-  </si>
-  <si>
-    <t>["||TAMARIN SAVANNAH LTD||29/06/2026||764882|01/01/2028 - 31/12/2037|DN52706092026000001|764882|||0","1816284.99||AZURI SMART CITY COMPANY LTD &amp;/OR CONTRACTORS &amp;/OR SUB CONTRACTORS||26/06/2025||2143140|19/07/2027 - 18/06/2037|DN52706092025000010|326855.01|14/10/2025|RC5272025000004|1816284.99"]</t>
-  </si>
-  <si>
-    <t>["After 30.06.2026","After 30.06.2026"]</t>
-  </si>
-  <si>
-    <t>2026-07-29T11:59:52.481Z</t>
-  </si>
-  <si>
-    <t>["||AZURI SMART CITY COMPANY LTD &amp;/OR CONTRACTORS &amp;/OR SUB CONTRACTORS||30/04/2026||251051|03/06/2024 - 31/08/2026|DN52706012026000016|251051|||0"]</t>
+    <t>2026-07-28T07:15:33.776Z</t>
+  </si>
+  <si>
+    <t>["-25014|-25014|6118.95|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD &amp;/OR THE HOUSE CANTEEN LTD &amp;/OR AVA DCB LTD|2380.07|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||05/08/2025|34816.81|3738.88|01-07-2025 to 01-07-2026|POL-PL-Jul-23-1040\\R2|POL-PL-Jul-23-1040\\R2|142.76|19358/23|40793|-21274.98513133749|","-696|-696|89.03|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|0.03|0||MUR|31/03/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||04/06/2025|606.55|89|31-03-2025 to 01-07-2025|POL-EL-Jul-23-1039\\R1|POL-EL-Jul-23-1039\\R1\\E2|102.08|17111/23/R1|593.5|-606.9162425601656|","-4581|-4581|684.75|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|-0.25|0||MUR|30/01/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||29/05/2025|3896.23|685|30-01-2025 to 01-07-2025|POL-PA-Jul-23-1051\\R1|POL-PA-Jul-23-1051\\R1\\E1|15.98|17111/23/R1|4565|-3896.2470104650097|","-135920.99|-135920.99|103307.13|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD &amp;/OR AVA ENERGY LTD &amp;/OR THE HOUSE CANTEEN LTD|82990.12|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||05/08/2025|587817.58|20317.01|01-07-2025 to 01-07-2026|POL-PA-Jul-23-1051\\R2|POL-PA-Jul-23-1051\\R2|2410.5|17111/23/R1|688714.21|-115603.95143881369|","-11|-11|1.72|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR MR VINCENT LAGARDE &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|-0.28|0||MUR|30/01/2025|MAURITIUS UNION ASSURANCE CO LTD|MONEY||29/05/2025|9.77|2|30-01-2025 to 01-07-2025|POL-MON-Jul-23-6\\R1|POL-MON-Jul-23-6\\R1\\E1|0.04|17111/23/R1|11.45|-9.353350739773717|","-26119|-26119|17226.53|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD &amp;/OR AVA ENERGY LTD &amp;/OR THE HOUSE CANTEEN LTD|13321.94|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||05/08/2025|98018.96|3904.59|01-07-2025 to 01-07-2026|POL-EL-Jul-23-1039\\R2|POL-EL-Jul-23-1039\\R2|401.96|17111/23/R1|114843.53|-22214.814794401063|","-656|-656|98.12|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|0.12|0||MUR|30/01/2025|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||29/05/2025|558.27|98|30-01-2025 to 01-07-2025|POL-FID-Jul-23-10\\R1|POL-FID-Jul-23-10\\R1\\E1|2.29|17111/23/R1|654.1|-557.9382988771919|","-262939|-262939|208834.57|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|169530.66|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||26/08/2024|1188768.79|39303.91|01-07-2024 to 01-07-2025|POL-CP-Jul-23-8\\R1|POL-CP-Jul-23-8\\R1|5372.83|19358/23|1392230.53|-223649.7749073886|","-3573|-3573|534.15|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|0.15|0||MUR|31/03/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||04/06/2025|3039.28|534|31-03-2025 to 01-07-2025|POL-PA-Jul-23-1051\\R1|POL-PA-Jul-23-1051\\R1\\E2|12.46|17111/23/R1|3560.97|-3038.9142756399315|","9048|9048|-1352.46|15|BANK OF MAURITIUS|-0.46|0||MUR|17/01/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||18/02/2025|-7695.49|-1352|17-01-2025 to 01-07-2025|POL-PA-Jun-22-34\\R2|POL-PA-Jun-22-34\\R2\\E1|-31.55|19698/24/N/E1|-9016.4|7695.532526152332|","-12744|-12744|1875|15|BANK OF MAURITIUS|0|0||MUR|07/10/2025|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||16/10/2025|10868.75|1875|07-10-2025 to 07-10-2025|POL-GIT-Oct-25-9|POL-GIT-Oct-25-9|243.75|27948/25/N|12500|-10868.963217263365|","8124|8124|-1229.36|15|BANK OF MAURITIUS|-0.359999999999854|0||MUR|29/09/2025|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL (ANNUAL COVER)||28/10/2025|-6895.08|-1229|29-09-2025 to 01-07-2026|POL-TR-ANN-Jun-25-5|POL-TR-ANN-Jun-25-5\\E3|71.31|19120/25/N/E3|-8195.75|6894.7065791611485|","-7338|-7338|1081.84|15|BANK OF MAURITIUS|-0.160000000000146|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL (ANNUAL COVER)||24/11/2025|6255.66|1082|01-11-2025 to 01-07-2026|POL-TR-ANN-Jun-25-5|POL-TR-ANN-Jun-25-5\\E4|125.24|19120/25/N|7212.26|-6256.0862800681425|","9120|9120|-1367.95|15|BANK OF MAURITIUS|0.05|0||MUR|29/08/2025|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL (ANNUAL COVER)||06/10/2025|-7751.69|-1368|29-08-2025 to 01-07-2026|POL-TR-ANN-Jun-25-5|POL-TR-ANN-Jun-25-5\\E1|0||-9119.64|7751.995999842099|","-46415|-46415|6923|15|BANK OF MAURITIUS|0|0||MUR|08/11/2024|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||15/01/2025|39491.9|6923|08-11-2024 to 01-07-2025|POL-CP-Jun-22-7\\R2|POL-CP-Jun-22-7\\R2\\E2|261.54|18672/24/N|46153.36|-39491.98508453104|","-3687|-3687|506.25|15|BANK OF MAURITIUS|0.25|0||MUR|02/10/2024|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||13/11/2024|3180.56|506|02-10-2024 to 01-01-2025|POL-F&amp;A-Oct-24-1030|POL-F&amp;A-Oct-24-1030|311.81|3601.902454|3375|-3180.7239103723814|","-12738|-12738|11340.67|15|SYNDICAT DES COPROPRIETAIRES DE L’IMMEUBLE RESIDENCE ST CLEMENT COURT|9440.05|0||MUR|01/01/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|Mise en demeure|20/02/2025|64678.41|1900.62|01-01-2025 to 01-01-2026|POL-F&amp;A-Jul-19-1426\\R6|POL-F&amp;A-Jul-19-1426\\R6|414.61|13617/08/R15|75604.47|-10837.721090284176|","-36765|-36765|11907.68|15|SYNDICAT DES COPROPRIETAIRES DE L’IMMEUBLE RESIDENCE ST CLEMENT COURT|10737.15|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|Mise en demeure|25/02/2026|67904.7|1170.53|01-01-2026 to 01-01-2027|POL-F&amp;A-Jul-19-1426\\R7|POL-F&amp;A-Jul-19-1426\\R7|427.85|13617/08/R17|79384.53|-31279.812674424695|","-14657|-14657|2161.05|15|DUCHENNE LOIC DAMIEN MR|0.050000000000291|0||MUR|09/01/2025|MAURITIUS UNION ASSURANCE CO LTD|MARINE HULL &amp; TPL|Mise en demeure|30/01/2025|12496.41|2161|09-01-2025 to 01-02-2026|POL-MH+TPL-Jan-25-1002|POL-MH+TPL-Jan-25-1002|250.43|996/25/N|14407.03|-12496.01782095943|","9104|9104|-1375.72|15|DUCHENNE LOIC DAMIEN MR|0.28|0||MUR|30/05/2025|MAURITIUS UNION ASSURANCE CO LTD|MARINE HULL &amp; TPL|Mise en demeure|19/02/2026|-7727.88|-1376|30-05-2025 to 01-02-2026|POL-MH+TPL-Jan-25-1002|POL-MH+TPL-Jan-25-1002\\E1|67.89|996/25/N/E1 \nA/C No : 3601.902454|-9171.49|7728.219552704425|","25661|25661|-2052.84|8|CAY MANAGEMENT CPY LTD|0.16|0||MUR|01/01/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/01/2025|-23607.66|-2053|01-01-2025 to 01-10-2025|POL-HEALTH-Oct-19-3183\\R5|POL-HEALTH-Oct-19-3183\\R5\\E4|0|MD16M00777/5/R3/EQ/5|-25660.5|23608.12|","-3757|-3757|300.58|8|CAY MANAGEMENT CPY LTD|-0.42|0||MUR|01/05/2024|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/03/2025|3456.7|301|01-05-2024 to 01-10-2024|POL-HEALTH-Oct-19-3183\\R4|POL-HEALTH-Oct-19-3183\\R4\\E5|0|NO DOCS WILL FOLLOW - POL-HEALTH-Oct-19-3183\\R4\\E3|3757.28|-3456.4423998211473|","-10856|-10856|868.44|8|CAY MANAGEMENT CPY LTD|0.44|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/06/2026|9987.06|868|01-07-2026 to 01-10-2026|POL-HEALTH-Oct-19-3183\\R6|POL-HEALTH-Oct-19-3183\\R6\\E2|0|MD16M00777/5/R4/EQ/3|10855.5|-9987.52|Timing Difference","48123|48123|-3849.87|8|CAY MANAGEMENT CPY LTD|0.13|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|-44273.45|-3850|01-05-2026 to 01-10-2026|POL-HEALTH-Oct-19-3183\\R6|POL-HEALTH-Oct-19-3183\\R6\\E1|0|MD16M00777/5/R4/EQ/2|-48123.32|44273.155600029255|","-2926|-2926|33870.72|8|KASA TEXTILE &amp; CO LTD|33638.02|0||MUR|01/03/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/05/2025|392476.97|232.700000000004|01-03-2025 to 01-03-2026|POL-HEALTH-Jun-19-2719\\R48|POL-HEALTH-Jun-19-2719\\R48|2963.69|MED/2024/00392/R1\nMD08M01085/13/R4|423384|-2693.547170901759|","-68923|-68923|23068.5|15|KASA TEXTILE &amp; CO LTD|12815.38|750||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||20/02/2026|132009.77|10253.12|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1067\\R4|POL-MVF-Dec-21-1067\\R4|538.27|26063/21/R4|153790|-58670.43382486792|","-314174|-314174|37719.36|8|KASA TEXTILE &amp; CO LTD|12760.49|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/05/2026|437072.64|24958.87|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2719\\R49|POL-HEALTH-Jun-19-2719\\R49|3300|MD08M01085/13/R5|471492|-289214.7710984178|","-13131|-13131|1050.48|8|KASA TEXTILE &amp; CO LTD|0.48|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/06/2026|12080.52|1050|01-06-2026 to 01-03-2027|POL-HEALTH-Jun-19-2719\\R49|POL-HEALTH-Jun-19-2719\\R49\\E1|0|MD08M01085/13/R5/EQ/2|13131|-12080.52|","-385|-385|3565.85|15|TARTUFFE LTEE|3509.4|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|Mise en demeure|09/09/2025|20789.69|56.4499999999998|01-07-2025 to 01-07-2026|POL-F&amp;A-Jun-19-1359\\R6|POL-F&amp;A-Jun-19-1359\\R6|583.21|25773/16|23772.33|-328.6328551943418|","1131|1131|-169.04|15|TARTUFFE LTEE|-0.04|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY|Mise en demeure|15/05/2026|-961.85|-169|01-04-2026 to 01-07-2026|POL-PPL-Jun-19-1092\\R6|POL-PPL-Jun-19-1092\\R6\\E2|-3.94|25773/16/R9/E2|-1126.95|961.9435577288684|","1673|1673|-250.01|15|TARTUFFE LTEE|-0.01|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)|Mise en demeure|15/05/2026|-1422.57|-250|01-04-2026 to 01-07-2026|POL-LOP(F&amp;A)-Jun-19-1088\\R6|POL-LOP(F&amp;A)-Jun-19-1088\\R6\\E2|-5.83|25773/16/R9/E2|-1666.75|1422.92722022265|","5448|5448|-889.02|15|TARTUFFE LTEE|-0.02|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|Mise en demeure|15/05/2026|-4558.53|-889|01-04-2026 to 01-07-2026|POL-F&amp;A-Jun-19-1359\\R6|POL-F&amp;A-Jun-19-1359\\R6\\E2|479.26|25773/16/R9/E2|-5926.81|4558.906561665336|","-4917|-4917|735|15|TARTUFFE LTEE|0|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|Mise en demeure|09/09/2025|4182.15|735|01-07-2025 to 01-07-2026|POL-PA-Jun-19-1329\\R6|POL-PA-Jun-19-1329\\R6|17.15|25773/16|4900|-4182.0224215246635|","-6709|-6709|1002.8|15|TARTUFFE LTEE|-0.2|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)|Mise en demeure|09/09/2025|5705.9|1003|01-07-2025 to 01-07-2026|POL-LOP(F&amp;A)-Jun-19-1088\\R6|POL-LOP(F&amp;A)-Jun-19-1088\\R6|23.4|25773/16|6685.3|-5706.155156736775|","1564|1564|-233.78|15|TARTUFFE LTEE|0.22|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|Mise en demeure|15/05/2026|-1330.18|-234|01-04-2026 to 01-07-2026|POL-EL-Jun-19-1268\\R6|POL-EL-Jun-19-1268\\R6\\E2|-5.45|25773/16/R9/E2|-1558.51|1330.2140208189467|","-6273|-6273|937.67|15|TARTUFFE LTEE|-0.33|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|Mise en demeure|09/09/2025|5335.37|938|01-07-2025 to 01-07-2026|POL-EL-Jun-19-1268\\R6|POL-EL-Jun-19-1268\\R6|21.88|25773/16|6251.16|-5335.335979046842|","-4536|-4536|678.03|15|TARTUFFE LTEE|0.03|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY|Mise en demeure|09/09/2025|3857.99|678|01-07-2025 to 01-07-2026|POL-PPL-Jun-19-1092\\R6|POL-PPL-Jun-19-1092\\R6|15.82|25773/16|4520.2|-3857.972989537083|","1226|1226|-183.25|15|TARTUFFE LTEE|-0.25|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|Mise en demeure|15/05/2026|-1042.67|-183|01-04-2026 to 01-07-2026|POL-PA-Jun-19-1329\\R6|POL-PA-Jun-19-1329\\R6\\E2|-4.28|25773/16/R9/E2|-1221.64|1042.7380416340382|","-85498|-85498|12750|15|ERC LEVAGE LTEE|0|0||MUR|30/01/2026|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||17/06/2026|72747.5|12750|30-01-2026 to 30-01-2026|POL-GIT-Jan-26-1|POL-GIT-Jan-26-1|497.5|2217/26/N|85000|-72747.92543641626|","-20270|-20270|3000|15|ERC LEVAGE LTEE|0|0||MUR|17/06/2025|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||31/07/2025|17270|3000|17-06-2025 to 17-06-2025|POL-GIT-Jun-25-5|POL-GIT-Jun-25-5|270|20990/25/N|20000|-17270|","-9881440|-9881440|2222028.75|15|ROYAL CAR RENTAL LTD|891753.83|31400||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||30/01/2026|12674744.08|1330274.92|01-01-2026 to 01-01-2027|POL-MVF-Jul-19-6113\\R7|POL-MVF-Jul-19-6113\\R7|51847.8299999998|31069/23 / 31162/23 / 31191/23|14813525|-8407507.087014845|","40842|40842|-6064.8|15|ROYAL CAR RENTAL LTD|0.2|-268||MUR|25/06/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/01/2026|-34776.72|-6065|25-06-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E43|-141.52|31162/23/R1/E35|-40432|34777.128721947665|","7452|7452|-1113.86|15|ROYAL CAR RENTAL LTD|0.140000000000146|0||MUR|26/08/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/01/2026|-6337.88|-1114|26-08-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E34|-25.99|31162/23/R1/E25|-7425.75|6338.101136110492|","-10111|-10111|1502.72|15|ROYAL CAR RENTAL LTD|-0.28|57.53||MUR|27/11/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||27/11/2025|8608.01|1503|27-11-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E47|35.06|31069/23/R1/E10|10018.14|-8608.23987090942|","-779717|-779717|116549.62|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.38|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||28/05/2026|663167.34|116550|01-05-2026 to 01-05-2027|POL-ARMISC-May-19-1048\\R7|POL-ARMISC-May-19-1048\\R7|2719.49||776997.47|-663167.3740209268|"]</t>
+  </si>
+  <si>
+    <t>["-150000|1005000|Currimjee Jeewanjee &amp; Co Ltd|01/04/2026|249278.65||01/01/26 to 31/12/26|POL-TER&amp;SAB-Mar-21-1002\\R5|6361/26/N|POL-TER&amp;SAB-Mar-21-1002\\R5|249278.65|18/03/2026|JRNI.260318.354|Special","-30754|4697.05|Currimjee Jeewanjee &amp; Co Ltd|03/03/2026|100||01/01/26 to 31/12/26||1918/26/N/E1||-26056.95|27/02/2026|JRNI.260227.565|Non-Motor Corporate","-29145.6|366870.24|RENTACOLOR (MAURITIUS) LTD|31/01/2026|266766.27||01/01/26 to 31/12/26|MD21M00252|MD21M00252/R5|MD21M00252|266766.27|23/02/2026|JRNNHZ.260223.99|Medical","-20809.54|1664.76|SAMENA CAPITAL MAURITIUS MANAGEMENT|31/07/2025|||01/07/25 to 30/06/26|MED/2023/01023|MED/2023/01023/R2/E1|MED/2023/01023|-19144.78|23/01/2026|JRNNHZ.260123.6|Medical","-20809.54|1664.76|SAMENA CAPITAL MAURITIUS MANAGEMENT|31/07/2025|||01/07/25 to 30/06/26|MED/2023/01023|MED/2023/01023/R2/E1|MED/2023/01023|-19144.78|23/01/2026|JRNNHZ.260123.6|Medical","-6290.76|52423|MAURITOURS LTD MAURITOURS LTD|01/08/2026|||01/01/26 to 31/12/26|MED/2023/00018|MED/2023/00018/R3|MED/2023/00018|46132.24|30/06/2026|JRNNHZ.260630.738|Medical","-27489.12|233886.6|MAURITOURS LTD MAURITOURS LTD|01/06/2026|206397.48||01/01/26 to 31/12/26|MED/2023/00018|MED/2023/00018/R3|MED/2023/00018|206397.48|30/04/2026|JRNNHZ.260430.757|Medical","-6872.28|57269|MAURITOURS LTD MAURITOURS LTD|01/07/2026|50396.72||01/01/26 to 31/12/26|MED/2023/00018|MED/2023/00018/R3|MED/2023/00018|50396.72|31/05/2026|JRNNHZ.260531.343|Medical","-6663.2|83290|Nassau Services Ltd|01/08/2026|||01/01/26 to 31/12/26|MD10M00493|MD10M00493/R16|MD10M00493|76626.8|30/06/2026|JRNNHZ.260630.483|Medical","-6901.04|86263|Nassau Services Ltd|01/07/2026|16093.06||01/01/26 to 31/12/26|MD10M00493|MD10M00493/R16|MD10M00493|16093.06|31/05/2026|JRNNHZ.260531.81|Medical","-31162.48|208789|Nassau Services Ltd|30/08/2026|44406.63||01/06/26 to 31/05/27||12779/21/R5||177626.52|11/06/2026|JRNI.260611.328|Financial","-27050.95|2164.07|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2026|||01/01/26 to 31/12/26|MD11M00166|MD11M00166/R15/E6|MD11M00166|-24886.88|20/03/2026|JRNNHZ.260320.336|Medical","-12682.38|1014.59|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E14|MD11M00166|-8562.88|03/10/2025|JRNNHZ.251003.354|Medical","-22907.97|1832.63|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E6|MD11M00166|-7943.33|12/06/2025|JRNNHZ.250612.280|Medical","-37909.31|3032.74|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2026|||01/01/26 to 31/12/26|MD11M00166|MD11M00166/R15/E8|MD11M00166|-34876.57|05/06/2026|JRNNHZ.260605.487|Medical","-12682.38|1014.59|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E14|MD11M00166|-8562.88|03/10/2025|JRNNHZ.251003.354|Medical","-22907.97|1832.63|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E6|MD11M00166|-7943.33|12/06/2025|JRNNHZ.250612.280|Medical","-19196.43|1535.71|NEWREST (MAURITIUS) LTD NEWREST (MAURITIUS) LTD|31/03/2026|||01/10/25 to 30/09/26|MED/2024/01202|MED/2024/01202/R1/E7|MED/2024/01202|-17660.72|08/06/2026|JRNNHZ.260608.239|Medical","-895792.5|6006552|JAG SERVICES LTD|15/10/2026|2008438.85||01/01/26 to 31/12/26||31069/23/R2||3155697.21|06/01/2026|JRNI.260106.421|Motor","-52010|6861.3|JAG SERVICES LTD|13/02/2026|||01/01/26 to 31/12/26||31069/23/R2/E4||-45148.7|13/02/2026|JRNI.260213.86|Motor","-1.05|110|Panache &amp; Co.Ltd|01/09/2026|||01/07/25 to 30/06/26||17835/22/R3/E1||108.95|18/06/2026|JRNI.260618.308|Non-Motor Corporate","-48.6|325|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|26/03/26 to 26/03/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14790/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|276.4|09/06/2026|JRNI.260609.338|Marine","-37.5|251|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|08/05/26 to 08/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14789/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|213.5|09/06/2026|JRNI.260609.337|Marine","-60.9|407|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|04/05/26 to 04/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14786/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|346.1|09/06/2026|JRNI.260609.336|Marine","-37.5|251|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|01/05/26 to 01/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14778/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|213.5|09/06/2026|JRNI.260609.335|Marine","-37.5|351|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|05/05/26 to 05/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14777/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|313.5|09/06/2026|JRNI.260609.334|Marine","-180.9|1210|Panache &amp; Co.Ltd|01/09/2026|||01/07/25 to 30/06/26||9084/09/R16/E7||1029.1|03/06/2026|JRNI.260603.144|Motor","-661.05|4438|Panache &amp; Co.Ltd|01/08/2026|||01/07/25 to 30/06/26||9084/09/R16/E6||3776.95|28/05/2026|JRNI.260528.372|Motor","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|18/04/26 to 18/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12372/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.300|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|14/04/26 to 14/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12371/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.299|Marine","-304.8|2039|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|18/04/26 to 18/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12370/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|1734.2|18/05/2026|JRNI.260518.298|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|17/04/26 to 17/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12369/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.297|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|16/04/26 to 16/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12367/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.296|Marine","-57.75|386|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|09/04/26 to 09/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12366/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|328.25|18/05/2026|JRNI.260518.295|Marine","-48.6|325|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|15/04/26 to 15/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12365/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|276.4|18/05/2026|JRNI.260518.294|Marine","-104.7|700|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|02/03/26 to 02/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12364/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|595.3|18/05/2026|JRNI.260518.293|Marine","-123.15|824|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|02/02/26 to 02/02/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12363/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|700.85|18/05/2026|JRNI.260518.292|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|16/04/26 to 16/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12361/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.291|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|08/03/26 to 08/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12360/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.290|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|09/04/26 to 09/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12358/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.289|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|06/04/26 to 06/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12357/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.288|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|25/03/26 to 25/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12356/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.287|Marine","-54|461|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|28/03/26 to 28/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12355/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|407|18/05/2026|JRNI.260518.286|Marine","-5407|808.2|Panache &amp; Co.Ltd|24/04/2026|||01/07/25 to 30/06/26||9084/09/R16/E5||-4598.8|24/04/2026|JRNI.260424.167|Motor","-44.4|397|Scott &amp; Co Ltd|01/07/2026|352.6||01/10/25 to 30/09/26||33954/19/R6/E2||352.6|09/01/2026|JRNI.260109.314|Non-Motor Corporate","-457.5|3161|Scott &amp; Co Ltd|01/07/2026|2703.5||01/10/25 to 30/09/26||33954/19/R6/E1||2703.5|07/01/2026|JRNI.260107.260|Non-Motor Corporate","-195955.8|1311444|HIGHWAY PROPERTIES LTD|01/08/2026|||01/05/26 to 30/04/27||13781/26/N||1115488.2|28/05/2026|JRNI.260528.581|Non-Motor Corporate","-24269.23|162860.98|HIGHWAY PROPERTIES LTD|01/09/2026|||01/05/26 to 30/04/27||14246/26/R1||138591.75|09/06/2026|JRNI.260609.339|Non-Motor Corporate","-2059.76|14279.97|HIGHWAY PROPERTIES LTD|05/06/2026|12220.21||01/04/26 to 30/04/26||14246/26/N||12220.21|03/06/2026|JRNI.260603.381|Non-Motor Corporate","-19264.65|129381|HIGHWAY PROPERTIES LTD|06/05/2026|110116.35||01/04/26 to 30/04/26||10767/26/N||110116.35|23/04/2026|JRNI.260423.353|Non-Motor Corporate","-38641.95|258710|HIGHWAY PROPERTIES LTD|01/07/2026|176087.63|Payment done after 30.06.2026|10/04/26 to 31/03/27|POL-MV-Apr-26-95|8591/26/N|POL-MV-Apr-26-95|176087.63|10/04/2026|JRNI.260410.163|Motor","-11997.59|80763.97|ACBMS LTD|01/08/2026|||01/05/26 to 30/04/27||12079/22/R4||45845.27|07/05/2026|JRNI.260507.165|Non-Motor Corporate","-16786.56|211300.82|GAYA COLLECTIONS LIMITEE GAYA COLLECTIONS LIMITEE|30/06/2026|160619.77|Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2023/00969|MED/2023/00969/R3|MED/2023/00969|160619.77|13/05/2026|JRNNHZ.260513.423|Medical","-2119.73|26496.72|GAYA COLLECTIONS LIMITEE GAYA COLLECTIONS LIMITEE|30/06/2026|1913.1||01/05/26 to 30/04/27|MED/2023/00969|MED/2023/00969/R3/E1|MED/2023/00969|1913.1|11/06/2026|JRNNHZ.260611.54|Medical","-12676.72|158459|BELLE RIVIERE HOTEL LTD|01/08/2026|||01/05/26 to 30/04/27|MED/2025/00947|MED/2025/00947/R1|MED/2025/00947|145782.28|30/06/2026|JRNNHZ.260630.904|Medical","-11476.08|155614.12|BELLE RIVIERE HOTEL LTD|01/07/2026|131974.92||01/05/26 to 30/04/27|MED/2025/00947|MED/2025/00947/R1|MED/2025/00947|131974.92|31/05/2026|JRNNHZ.260531.511|Medical","-6485.7|43689|Osman Rezah|01/09/2026|||01/06/26 to 31/05/27||13626/10/R16||37203.3|01/06/2026|JRNI.260601.332|Non-Motor Corporate","-38910|5816.1|Partsionate Ltd|24/06/2026|||06/05/26 to 30/04/27||11100/26/N/E1||-33093.9|24/06/2026|JRNI.260624.288|Motor","-123515|18462.6|Partsionate Ltd|05/06/2026|||06/05/26 to 30/04/27||11084/26/N/E2||-105052.4|05/06/2026|JRNI.260605.166|Motor","-83312.02|557857.94|ALL TO THE MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTIPLANTES LTEE &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED|01/09/2026|||01/06/26 to 30/06/27||22063/19/R7||474545.92|16/06/2026|JRNI.260616.372|Non-Motor Corporate","-3078|21042|ASSOCIATION SYNDICALE DU LOTISSEMENT LES VILLAS DE CASCAVELLE|01/03/2026|17964||01/11/25 to 31/10/26||9507/20/R6||17964|03/12/2025|JRNI.251203.405|Non-Motor Corporate","-1383.3|9754|ASSOCIATION SYNDICALE MORCELLEMENT VILLAZE|01/08/2026|||01/05/26 to 30/04/27||17184/24/R2||8370.7|11/05/2026|JRNI.260511.317|Non-Motor Corporate","-1524.6|10400|Pajeli Co Ltd|01/07/2026|8875.4||01/05/26 to 30/04/27|POL-MV-Apr-24-1124\\R2|11196/24/R2|POL-MV-Apr-24-1124\\R2|8875.4|15/04/2026|JRNI.260415.32|Motor","-35741.69|239611.97|Pajeli Co Ltd|01/09/2026|||01/07/26 to 30/06/27||19583/24/R2||203870.28|01/06/2026|JRNI.260601.418|Non-Motor Corporate","-263.98|1915.99|LES CAMPECHES LTEE|01/09/2026|||12/06/26 to 11/12/26||16082/26/N||1652.01|24/06/2026|JRNI.260624.397|Non-Motor Corporate","-11504.7|77466|SYNDICAT DES COPROPRIÉTAIRES DE L`ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|01/03/2026|65961.3||01/10/25 to 30/09/26||2595/17/R9||65961.3|03/12/2025|JRNI.251203.296|Non-Motor Corporate","-408.45|2783|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|01/01/2026|2374.55||01/11/25 to 31/10/26||31161/22/R3||2374.55|13/10/2025|JRNI.251013.122|Motor","-13346.85|89390|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|01/08/2026|||01/06/26 to 31/05/27||31169/22/R3||76043.15|29/05/2026|JRNI.260529.51|Motor","-457|68.25|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|08/10/2025|||01/01/25 to 31/10/25||31161/22/R2/E2||-388.75|08/10/2025|JRNI.251008.78|Motor","-408.75|2785|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|01/04/2026|2376.25||01/02/26 to 31/01/27||31164/22/R3||2376.25|12/01/2026|JRNI.260112.141|Motor","-7549.5|50606|The General Construction Company Limited|01/01/2026|43056.5||01/04/25 to 31/03/26||10359/24/R1/E1||43056.5|01/10/2025|JRNI.251001.326|Non-Motor Corporate","-242123.1|1619804|The General Construction Company Limited|17/06/2026|1377680.9||16/12/24 to 15/12/34||17764/25/N/E1||1377680.9|15/06/2026|JRNI.260615.361|Special","-768028.95|5138114|The General Construction Company Limited|01/07/2026|1456887.07||01/04/26 to 31/03/27||10359/24/R2||1456887.07|16/04/2026|JRNI.260416.322|Non-Motor Corporate","-322312.92|2156773.96|The General Construction Company Limited|01/07/2026|589013.49||01/04/26 to 31/03/27||7186/22/R4||589013.49|16/04/2026|JRNI.260416.317|Non-Motor Corporate","-12916.35|86534|The General Construction Company Limited|01/11/2025|73617.65||01/04/25 to 31/03/26||MT9900043297/R25/E15||73617.65|18/08/2025|JRNI.250818.221|Motor","-11576.25|77945|The General Construction Company Limited|01/07/2026|44248.1||01/04/26 to 31/03/27||8694/22/R4||44248.1|15/04/2026|JRNI.260415.201|Non-Motor Corporate","-9325|1393.8|The General Construction Company Limited|27/10/2025|||01/04/25 to 31/03/26||MT9900043297/R25/E27||-7931.2|27/10/2025|JRNI.251027.157|Motor","-1308|195.45|The General Construction Company Limited|05/02/2026|||01/04/25 to 31/03/26||MT9900043297/R25/E38||-1112.55|05/02/2026|JRNI.260205.45|Motor","-4762.35|32003|The General Construction Company Limited|01/10/2025|27240.65||01/04/25 to 31/03/26|POL-MVF-May-19-1121\\R6\\E14|MT9900043297/R25/E11|POL-MVF-May-19-1121\\R6\\E14|27240.65|14/07/2025|JRNI.250714.129|Motor","-3359|502.05|The General Construction Company Limited|06/11/2025|||01/04/25 to 31/03/26||MT9900043297/R25/E30||-2856.95|06/11/2025|JRNI.251106.243|Motor","-75873.75|513095|The General Construction Company Limited|01/07/2026|437221.25||01/04/26 to 31/03/27||9151/18/R8||437221.25|01/04/2026|JRNI.260401.326|Motor","-10350|69442|The General Construction Company Limited|01/07/2026|59092||01/04/26 to 31/03/27||13092/25/R1||59092|01/04/2026|JRNI.260401.324|Motor","-924635.68|6216812.99|The General Construction Company Limited|01/07/2026|3362379.92||01/04/26 to 31/03/27||MT9900043297/R26||3362379.92|01/04/2026|JRNI.260401.322|Motor"]</t>
+  </si>
+  <si>
+    <t>["-3485|-3485|520.93|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.0700000000000728|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||28/05/2026|2964.09|521|01-05-2026 to 01-05-2027|POL-MON-Apr-20-1058\\R6|POL-MON-Apr-20-1058\\R6|12.15||3472.87|-2964.07298953808|","-429|-429|825|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|762.01|0|Correction to be done by CBL amount not in aging|MUR|01/11/2018|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||4794|62.99|01-11-2018 to 01-11-2019|POL-CAR-TPL-May-19-1036|POL-CAR-TPL-May-19-1036|119|17636/16/N|5500|-366.01281366791244|","-95011|-95011|14202|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR PRINCIPALS &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||28/05/2026|80809.38|14202|01-05-2026 to 01-05-2027|POL-CAR-TPL(BC)-May-25-4\\R1|POL-CAR-TPL(BC)-May-25-4\\R1|331.38||94680|-80809.05680119581|","-7350|-7350|1098.64|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.359999999999854|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||28/05/2026|6251.25|1099|01-05-2026 to 01-05-2027|POL-EE-Apr-20-1086\\R6|POL-EE-Apr-20-1086\\R6|25.64||7324.25|-6251.343557522629|","-906872|-906872|135556.38|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR FASTMIX  CO LTD|0.38|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||28/05/2026|771315.81|135556|01-05-2026 to 01-05-2027|POL-ARM(P&amp;M)-Feb-20-1010\\R7|POL-ARM(P&amp;M)-Feb-20-1010\\R7|3163.01||903709.18|-771315.6484005976|","-107514|-107514|16070.81|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR FASTMIX CO LTD|-0.19|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||28/05/2026|91442.88|16071|01-05-2026 to 01-05-2027|POL-EL-Apr-20-1161\\R6|POL-EL-Apr-20-1161\\R6|374.98|9314/08/R18|107138.71|-91443.14366216991|","-92643|-92643|13848|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR FAST MIX CO LTD|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/05/2026|78795.12|13848|01-05-2026 to 01-05-2027|POL-PA-Apr-20-1154\\R6|POL-PA-Apr-20-1154\\R6|323.12||92320|-78795.01793721973|","-112057|-112057|16675.17|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR SOCIETE FOUR TWELVE &amp;/ORDISTRI-T TRADING LTD|0.169999999997672|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||28/05/2026|95381.69|16675|01-05-2026 to 01-05-2027|POL-F&amp;A-Apr-20-1182\\R6|POL-F&amp;A-Apr-20-1182\\R6|889.09|9314/08/R18|111167.77|-95381.80916661417|","-276484|-276484|41328|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/05/2026|235156.32|41328|01-05-2026 to 01-05-2027|POL-PA-Apr-20-1155\\R6|POL-PA-Apr-20-1155\\R6|964.32||275520|-235156.04783258596|","-117828|-117828|17612.55|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.45|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/05/2026|100215.41|17613|01-05-2026 to 01-05-2027|POL-PA-Apr-20-1153\\R6|POL-PA-Apr-20-1153\\R6|410.96||117417|-100215.44402092678|","-5808|-5808|868.2|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR SOCIETE FOUR TWELVE &amp;/ORDISTRI-T TRADING LTD &amp;/OR FASTMIX CO LTD|0.2|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||28/05/2026|4940.06|868|01-05-2026 to 01-05-2027|POL-PL-Apr-20-1178\\R6|POL-PL-Apr-20-1178\\R6|20.26|9314/08/R18|5788|-4939.838863962701|","-85584|-85584|12718.13|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|||72866.13||01-07-2026 to 01-07-2027|POL-F&amp;A-Jun-19-1315\\R7|POL-F&amp;A-Jun-19-1315\\R7|796.76||84787.5|-72865.90863693862|Timing Difference","-16859|-16859|2520|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)|||14338.81||01-07-2026 to 01-07-2027|POL-LOP(F&amp;A)-Jun-19-1076\\R7|POL-LOP(F&amp;A)-Jun-19-1076\\R7|58.81||16800|-14338.97159941894|Timing Difference","-41394|-41394|6187.5|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY|||35206.88||01-07-2026 to 01-07-2027|POL-PPL-Jun-19-1086\\R7|POL-PPL-Jun-19-1086\\R7|144.38||41250|-35206.556801188955|Timing Difference","-134198|-134198|106612.8|8|A.E. PATEL &amp; CO.LTD|95951.41|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/11/2025|1235376.2|10661.39|01-10-2025 to 01-10-2026|POL-HEALTH-Aug-19-3002\\R8|POL-HEALTH-Aug-19-3002\\R8|9329|MD17M00713/4/R5|1332660|-123536.79149948322|","-58895|-58895|8803.46|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|||50091.71||01-07-2026 to 01-07-2027|POL-PA-Jun-19-1298\\R7|POL-PA-Jun-19-1298\\R7|205.42||58689.75|-50091.56541105153|Timing Difference","-33276|-33276|4961.25|15|A.E. PATEL &amp; CO. LTD|0|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY||16/07/2026|28314.51|4961.25|01-07-2026 to 30-06-2027|POL-PI-Jun-19-1049\\R7|POL-PI-Jun-19-1049\\R7|200.76|41856/17/R9|33075|-28314.714217195942|Timing Difference","-10044|-10044|1501.38|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY|||8542.85||01-07-2026 to 01-07-2027|POL-MON-Jun-19-1072\\R7|POL-MON-Jun-19-1072\\R7|35.03||10009.2|-8542.654379678681|Timing Difference","-14200|-14200|2122.58|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|DETERIORATION OF STOCK|||12077.45||01-07-2026 to 01-07-2027|POL-DOS-Sep-22-1\\R4|POL-DOS-Sep-22-1\\R4|49.53||14150.5|-12077.42448431447|Timing Difference","-9502|-9502|1420.35|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE|||8081.79||01-07-2026 to 01-07-2027|POL-FID-Jun-19-1032\\R7|POL-FID-Jun-19-1032\\R7|33.14||9469|-8081.670926759656|Timing Difference","-15003|-15003|2242.63|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT|||12760.55||01-07-2026 to 01-07-2027|POL-EE-Jun-19-1135\\R7|POL-EE-Jun-19-1135\\R7|52.33||14950.85|-12760.396905855958|Timing Difference","-11064|-11064|1653.75|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (MACHINERY BREAKDOWN)|||9409.84||01-07-2026 to 01-07-2027|POL-LOP(M B-D)-Oct-22-1\\R4|POL-LOP(M B-D)-Oct-22-1\\R4|38.59||11025|-9410.1887145131|Timing Difference","-6322|-6322|945|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN|||5377.05||01-07-2026 to 01-07-2027|POL-M B-D-Jun-19-1027\\R7|POL-M B-D-Jun-19-1027\\R7|22.05||6300|-5377.007473841555|Timing Difference","-7931|-7931|1185.48|15|A.E. PATEL &amp; CO. LTD &amp;/OR PHARMACY A. E. PATEL &amp; CO LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|||6745.35||01-07-2026 to 01-07-2027|POL-EL-Jun-19-1227\\R7|POL-EL-Jun-19-1227\\R7|27.66||7903.17|-6745.4945888387465|Timing Difference","1028|1028|-168.63|15|LAVASTONE LTD &amp;/OR SUBSIDIARIES &amp;/OR AFFILIATED COMPANIES|0.37|0||MUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||10/10/2025|-859.48|-169|01-10-2024 to 30-09-2025|POL-EL-Oct-19-1469\\R5|POL-EL-Oct-19-1469\\R5\\E1|96.07|33502/19/R5/E1|-1124.18|859.3880421355692|","5077|5077|-758.83|15|LAVASTONE LTD &amp;/OR SUBSIDIARIES &amp;/OR AFFILIATED COMPANIES|0.17|0||MUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||13/10/2025|-4317.73|-759|01-10-2024 to 30-09-2025|POL-PA-Oct-19-1546\\R5|POL-PA-Oct-19-1546\\R5\\E1|-17.71|33502/19/R5/E1|-5058.85|4318.104230029784|","-16533|-16533|1983.95|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.05|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|14548.96|1984|01-11-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E25|0|MED/2025/01055/EQ/55|16532.91|-14549.039199995645|","-25782|-25782|3093.89|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.11|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|22688.55|3094|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E41|0|MED/2025/01055/EQ/96|25782.44|-22688.162799952217|","7844|7844|-941.33|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.33|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|-6903.12|-941|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E40|0|MED/2025/01055/EQ/94|-7844.45|6902.723999770538|","-6277|-6277|753.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|5523.89|753|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E51|0|MED/2025/01055/EQ/112|6277.15|-5523.758000047792|","-1836|-1836|220.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||05/06/2026|1615.25|220|01-06-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E54|0|MED/2025/01055/EQ/118|1835.51|-1615.681200320347|","-6277|-6277|753.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||05/06/2026|5523.89|753|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E53|0|MED/2025/01055/EQ/114|6277.15|-5523.758000047792|","-13731|-13731|1647.68|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.32|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|12082.95|1648|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E28|0|MED/2025/01055/EQ/64|13730.63|-12083.275599881434|","3119|3119|-374.24|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.24|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/05/2026|-2744.44|-374|01-06-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E52|0|MED/2025/01055/EQ/113|-3118.68|2744.721600164172|","-11074|-11074|1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|9745.31|1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E29|0|MED/2025/01055/EQ/56|11074.22|-9745.116400071518|","-18355|-18355|2202.61|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.39|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|16152.45|2203|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E36|0|MED/2025/01055/EQ/74|18355.06|-16152.397200009153|","-7464|-7464|895.73|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.27|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|6568.66|896|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E43|0|MED/2025/01055/EQ/95|7464.39|-6568.316800167194|","-139140|-139140|16696.8|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.2|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||27/02/2026|122443.2|16697|01-07-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E19|0|MED/2025/01055/EQ/84|139140|-122443.2|","-7274|-7274|872.88|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.12|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|6401.09|873|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E35|0|MED/2025/01055/EQ/81|7273.97|-6401.116399985152|","-11074|-11074|1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/02/2026|9745.31|1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E34|0|MED/2025/01055/EQ/75|11074.22|-9745.116400071518|","11074|11074|-1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/02/2026|-9745.31|-1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E33|0|MED/2025/01055/EQ/76|-11074.22|9745.116400071518|","-42083|-42083|5049.99|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.01|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|37033.25|5050|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E37|0|MED/2025/01055/EQ/80|42083.24|-37033.03880000684|","-31700|-31700|3803.97|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.03|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|27895.75|3804|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E38|0|MED/2025/01055/EQ/72|31699.72|-27895.9963999682|","-2374|-2374|284.94|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.06|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|2089.55|285|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E45|0|MED/2025/01055/EQ/107|2374.49|-2089.118800247632|","24936|24936|-2992.32|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.32|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/10/2025|-21943.68|-2992|01-07-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E14|0|MED/2025/01055|-24936|21943.68|","-2082|-2082|249.87|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.13|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|1832.41|250|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E46|0|MED/2025/01055/EQ/116|2082.28|-1832.1635995159154|","-9763|-9763|1171.52|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.48|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|8591.15|1172|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E47|0|MED/2025/01055/EQ/102|9762.67|-8591.440400013522|","-6616|-6616|793.93|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.07|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|5822.15|794|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E48|0|MED/2025/01055/EQ/101|6616.08|-5822.079600004837|","-111444|-111444|13373.34|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.34|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|98071.15|13373|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E42|0|MED/2025/01055/EQ/97|111444.49|-98070.71880000527|","38769|38769|-4636.02|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.0200000000005821|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|-34132.74|-4636|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E39|-135.22|MED/2025/01055|-38633.54|34132.951300480076|","53793|53793|-6455.21|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.21|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|-47338.2|-6455|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E22|0|MED/2025/01055/EQ/51|-53793.41|47337.8392000061|"]</t>
+  </si>
+  <si>
+    <t>["-581|86.85|The General Construction Company Limited|27/10/2025|||01/04/25 to 31/03/26||9151/18/R7/E5||-494.15|27/10/2025|JRNI.251027.149|Motor","-9693.45|64949|DESVAUX DE MARIGNY Alain Laurent|01/09/2026|||01/07/26 to 30/06/27||21359/25/R1||55255.55|16/06/2026|JRNI.260616.212|Motor","-8462.43|106180.44|Desvaux De Marigny-Montocchio Marie Pascale Anne|31/10/2026|||01/05/26 to 30/04/27|MD21M00643|MD21M00643/R5|MD21M00643|87946.25|11/05/2026|JRNNHZ.260511.367|Medical","-11246.4|94120|CHEUNG Willy|30/04/2026|66298.88|Payment done after 30.06.2026|01/03/26 to 28/02/27|MED/2026/00365|MED/2026/00365/N|MED/2026/00365|66298.88|24/04/2026|JRNNHZ.260424.75|Medical","-4703.04|39592|RAMPUTH NEELESH|30/04/2026|27911.52|Payment done after 30.06.2026|01/03/26 to 28/02/27|MED/2026/00315|MED/2026/00315/N|MED/2026/00315|27911.52|16/04/2026|JRNNHZ.260416.32|Medical","-7197.12|60376|Boodiah Maureen Vivianna|31/05/2026|53178.88|Payment done after 30.06.2026|01/04/26 to 31/03/27|MED/2026/00362|MED/2026/00362/N|MED/2026/00362|53178.88|24/04/2026|JRNNHZ.260424.21|Medical","-8138.25|54545|Comptoir Ouest OI Ltee|01/07/2026|38670.45||01/05/26 to 30/04/27|POL-MV-Apr-25-150|11301/25/R1|POL-MV-Apr-25-150|38670.45|16/04/2026|JRNI.260416.191|Motor","-5517.02|69362.87|NOMBRO MARY LYSIE IVY|30/11/2026|||01/06/26 to 31/05/27|MED/2023/00781|MED/2023/00781/R3|MED/2023/00781|56493.34|03/06/2026|JRNNHZ.260603.72|Medical","-4165.05|52563.19|Pro Wire Electrical &amp; Mechanical Ltd Pro Wire Electrical &amp; Mechanical Ltd|30/11/2026||Payment done after 30.06.2026|01/06/26 to 31/05/27|MED/2022/00714|MED/2022/00714/R4|MED/2022/00714|48398.14|15/06/2026|JRNNHZ.260615.19|Medical","-2803.5|18855|MEDLOG (MAURITIUS) LTD|01/09/2026|||01/08/25 to 31/07/26||26048/24/R1/E2||16051.5|01/06/2026|JRNI.260601.416|Non-Motor Corporate","-14031.3|93969|G. DE VILLIERS PAINT CONTRACTORS LTD|01/08/2026|||01/06/26 to 31/05/27||18210/25/R1||79937.7|27/05/2026|JRNI.260527.92|Motor","-5408.25|36381|G. DE VILLIERS PAINT CONTRACTORS LTD|01/09/2025|22655.11||01/07/25 to 30/06/26||18205/25/N||22655.11|26/06/2025|JRNI.250626.416|Motor","-8518.95|57192|G. DE VILLIERS PAINT CONTRACTORS LTD|01/09/2025|27592.64||01/07/25 to 30/06/26||18193/25/N||27592.64|26/06/2025|JRNI.250626.408|Motor","-8902.65|59759|G. DE VILLIERS PAINT CONTRACTORS LTD|01/07/2026|50856.35||01/05/26 to 30/04/27||18193/25/R1||50856.35|30/04/2026|JRNI.260430.161|Motor","-5711.1|38407|G. DE VILLIERS PAINT CONTRACTORS LTD|01/08/2026|||01/06/26 to 31/05/27||18205/25/R1||32695.9|27/05/2026|JRNI.260527.85|Motor","-13435.2|112360|SAWMYNADEN Kisnasamy Poulay|31/05/2026|78739.85||01/04/26 to 31/03/27|MED/2026/00453|MED/2026/00453/N|MED/2026/00453|78739.85|21/05/2026|JRNNHZ.260521.163|Medical","-5286.24|44452|HUET Louise Lilette Nicole|30/06/2026|32240.48|Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2026/00429|MED/2026/00429/N|MED/2026/00429|32240.48|19/05/2026|JRNNHZ.260519.161|Medical","-10680.48|89404|SOORJUN SOTEEHALL MANISHA|30/06/2026|70314.39|Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2026/00515|MED/2026/00515/N|MED/2026/00515|70314.39|02/06/2026|JRNNHZ.260602.2|Medical","-150406.35|1006718|IKO (MAURITIUS) HOTEL LIMITED T/A CONSTANCE LE CHALAND IKO - MAURITIUS|01/04/2026|856311.65||01/01/26 to 31/12/26||1595/26/N||856311.65|23/01/2026|JRNI.260123.385|Non-Motor Corporate","-52.2|449|IKO (MAURITIUS) HOTEL LIMITED T/A CONSTANCE LE CHALAND IKO - MAURITIUS|01/09/2026|||01/01/26 to 31/12/26||1595/26/N/E3||396.8|17/06/2026|JRNI.260617.355|Non-Motor Corporate","-3529.35|23729|MERIDIS FINANCIAL SOLUTIONS LTD|01/09/2026|||04/05/26 to 30/04/27|POL-F-PI-Jun-26-23|16950/26/N|POL-F-PI-Jun-26-23|20199.65|30/06/2026|JRNI.260630.583|Financial","-30644.25|205312|The Peak Panorama Ltd and The Successive Owners of the Buildings|30/07/2026|||01/09/27 to 01/09/37|POL-DEF-Jun-26-1005|16305/26/N|POL-DEF-Jun-26-1005|174667.75|26/06/2026|JRNI.260626.112|Special","-8112.45|54472|COUVE Remy Andre Edgar|01/10/2025|||01/07/25 to 30/06/26|POL-MH+TPL-Jun-24-26/R1|18654/24/R1|POL-MH+TPL-Jun-24-26/R1|0.01|04/07/2025|JRNI.250704.7|Yacht Hull/Tpl","-5666.25|38007|LALLJEE Chandunnee|01/09/2026|||01/07/26 to 30/06/27||19149/25/R1||32340.75|15/06/2026|JRNI.260615.28|Motor","-8579.52|71896.01|LABELLE VICTOIRE Marie Cindy Anabelle|31/07/2026|||01/06/26 to 31/05/27|MED/2026/00624|MED/2026/00624/N|MED/2026/00624|63316.49|30/06/2026|JRNNHZ.260630.280|Medical","-3969.76|49622|VISIONWAY LTD|01/08/2026|||01/09/25 to 31/08/26|MD16M00704|MD16M00704/R9|MD16M00704|45652.24|30/06/2026|JRNNHZ.260630.553|Medical","-11250|75507|RIVALLAND CHRISTIAN ROBERT XAVIER|01/05/2026|64257||09/02/26 to 30/04/27|POL-MV-Feb-26-32|3064/26/N|POL-MV-Feb-26-32|64257|09/02/2026|JRNI.260209.147|Motor","-2808|336.96|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E7|MED/2025/00586|-2471.04|03/04/2026|JRNNHZ.260403.10|Medical","-5709.6|685.15|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E6|MED/2025/00586|-5024.45|09/03/2026|JRNNHZ.260309.114|Medical","-2808|336.96|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E7|MED/2025/00586|-2471.04|03/04/2026|JRNNHZ.260403.10|Medical","-22270.08|280324.64|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|31/10/2026||Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2025/00586|MED/2025/00586/R1|MED/2025/00586|248010.54|19/05/2026|JRNNHZ.260519.212|Medical","-5709.6|685.15|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E6|MED/2025/00586|-5024.45|09/03/2026|JRNNHZ.260309.114|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.35|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.34|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.33|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.32|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.31|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.30|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.158|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.157|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.156|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.155|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.154|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.153|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.152|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.151|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.150|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.149|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.148|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.147|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.93|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.92|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.91|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.90|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.89|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.88|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.87|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.86|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.85|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.84|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.83|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.82|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.311|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.310|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.309|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.308|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.307|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.306|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.305|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.304|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.303|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.302|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.301|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.300|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.17|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.16|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.15|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.14|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.13|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.12|Medical"]</t>
+  </si>
+  <si>
+    <t>["31285|31285|-3754.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.26|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/02/2026|-27531.21|-3754|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E30|0|MED/2025/01055/EQ/73|-31285.47|27530.79640005408|","-16585|-16585|1990.24|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.24|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|14595.08|1990|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E50|0|MED/2025/01055/EQ/110|16585.32|-14594.798400030872|","6550|6550|-785.99|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.01|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||22/04/2026|-5763.91|-786|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E44|0|MED/2025/01055/EQ/99|-6549.9|5763.997999969465|","-41854|-41854|5022.48|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.479999999999418|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/01/2026|36831.55|5022|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E24|0|MED/2025/01055/EQ/48|41854.03|-36831.52359999742|","18600|18600|-2231.98|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.02|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||07/01/2026|-16367.82|-2232|01-09-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E8|0|MED/2025/01055/EQ/7|-18599.8|16367.99599995699|","-50256|-50256|6030.71|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.29|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|44225.23|6031|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E49|0|MED/2025/01055/EQ/111|50255.94|-44225.28280000334|","27159|27159|-3259.13|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.13|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/01/2026|-23900.26|-3259|01-10-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E23|0|MED/2025/01055/EQ/47|-27159.39|23899.91680004595|","33030|33030|-3963.6|12|HARDY HENRY SERVICES LTEE|0.4|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-29066.4|-3964|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E7|0|MD18M01064/3/R4/EQ/15|-33030|29066.4|","47208|47208|-5664.96|12|HARDY HENRY SERVICES LTEE|0.04|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-41543.04|-5665|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E9|0|MD18M01064/3/R4/EQ/17|-47208|41543.04|","-1884|-1884|226.08|12|HARDY HENRY SERVICES LTEE|226.16|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||01/07/2026|1657.92|-0.0800000000000125|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E21|0|MD18M01064/3/R4/EQ/43|1884|-1657.92|","-5790|-5790|694.8|12|HARDY HENRY SERVICES LTEE|-0.2|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|5095.2|695|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E10|0|MD18M01064/3/R4/EQ/18|5790|-5095.2|","-9420|-9420|1130.4|12|HARDY HENRY SERVICES LTEE|0.400000000000146|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|8289.6|1130|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E12|0|MD18M01064/3/R4/EQ/19|9420|-8289.6|","9400|9400|-1128|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/06/2026|-8272|-1128|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E22|0|MD18M01064/3/R4/EQ/42|-9400|8272|","-18840|-18840|2260.8|12|HARDY HENRY SERVICES LTEE|-0.199999999999709|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|16579.2|2261|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E8|0|MD18M01064/3/R4/EQ/16|18840|-16579.2|","-4626|-4626|555.12|12|HARDY HENRY SERVICES LTEE|0.12|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/05/2026|4070.88|555|01-05-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E18|0|MD18M01064/3/R4/EQ/30|4626|-4070.88|","-3900|-3900|468|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||01/03/2026|3432|468|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E13|0|MD18M01064/3/R4/EQ/23|3900|-3432|","27591|27591|-3310.92|12|HARDY HENRY SERVICES LTEE|0.08|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|-24280.08|-3311|01-04-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E16|0|MD18M01064/3/R4/EQ/28|-27591|24280.08|","-2111|-2111|253.32|12|HARDY HENRY SERVICES LTEE|0.32|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||14/06/2026|1857.68|253|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E20|0|MD18M01064/3/R4/EQ/37|2111|-1857.68|","17780|17780|-2133.6|12|HARDY HENRY SERVICES LTEE|0.4|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||17/12/2025|-15646.4|-2134|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E3|0|MD18M01064/3/R4/EQ/3|-17780|15646.4|","24815|24815|-2977.8|12|HARDY HENRY SERVICES LTEE|0.2|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/12/2025|-21837.2|-2978|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E6|0|MD18M01064/3/R4/EQ/12|-24815|21837.2|","6167|6167|-740.04|12|HARDY HENRY SERVICES LTEE|-0.04|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-5426.96|-740|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E5|0|MD18M01064/3/R4/EQ/14|-6167|5426.96|","-29379|-29379|3525.48|12|HARDY HENRY SERVICES LTEE|0.48|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/12/2025|25853.52|3525|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E4|0|MD18M01064/3/R4/EQ/10|29379|-25853.52|","-1762|-1762|211.44|12|HARDY HENRY SERVICES LTEE|0.44|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/05/2026|1550.56|211|01-05-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E17|0|MD18M01064/3/R4/EQ/32|1762|-1550.56|","-24687|-24687|2962.44|12|HARDY HENRY SERVICES LTEE|0.44|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/12/2025|21724.56|2962|01-10-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E1|0|MD18M01064/3/R4/EQ/9\nMD18M01064/3/R4/EQ/8\nMD02M00616/19/R5/EQ/2|24687|-21724.56|","12700|12700|-1524|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/02/2026|-11176|-1524|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E11|0|MD18M01064/3/R4/EQ/21|-12700|11176|","-14180|-14180|1701.6|12|HARDY HENRY SERVICES LTEE|-0.4|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|12478.4|1702|01-03-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E14|0|MD18M01064/3/R4/EQ/25|14180|-12478.4|","13536|13536|-1624.32|12|HARDY HENRY SERVICES LTEE|-0.32|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|-11911.68|-1624|01-04-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E15|0|MD18M01064/3/R4/EQ/26|-13536|11911.68|","1884|1884|-226.08|12|HARDY HENRY SERVICES LTEE|-0.08|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/06/2026|-1657.92|-226|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E19|0|MD18M01064/3/R4/EQ/38|-1884|1657.92|","-17559|-17559|2624.7|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.3|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||12/02/2026|14934.55|2625|01-01-2026 to 01-01-2027|POL-FID-Dec-21-9\\R4|POL-FID-Dec-21-9\\R4|61.25|2321/20/R6|17498|-14934.337369192875|","-22618|-22618|3380.83|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.17|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||12/02/2026|19236.93|3381|01-01-2026 to 01-01-2027|POL-EE-Dec-21-20\\R4|POL-EE-Dec-21-20\\R4|78.88|2321/20/R6|22538.88|-19237.134125572116|","-12042|-12042|1800|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||12/02/2026|10242|1800|01-01-2026 to 01-01-2027|POL-MON-Jan-20-1008\\R6|POL-MON-Jan-20-1008\\R6|42|2321/20/R6|12000|-10242|","-105713|-105713|15801.59|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.41|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||12/02/2026|89911.08|15802|01-01-2026 to 01-01-2027|POL-PA-Mar-20-1110\\R6|POL-PA-Mar-20-1110\\R6|368.71|2321/20/R6|105343.96|-89911.36067266109|","-34386|-34386|5139.87|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.13|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||12/02/2026|29245.89|5140|01-01-2026 to 01-01-2027|POL-EL-Jan-20-1023\\R6|POL-EL-Jan-20-1023\\R6|119.93|2321/20/R6|34265.83|-29246.094125591524|","-120816|-120816|18059.27|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.27|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||12/02/2026|102757.21|18059|01-01-2026 to 01-01-2027|POL-PPL-Jan-20-1005\\R6|POL-PPL-Jan-20-1005\\R6|421.38|2321/20/R6|120395.1|-102756.80174890049|","-136980|-136980|20475.37|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.37|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||12/02/2026|116504.87|20475|01-01-2026 to 01-01-2027|POL-LOP(F&amp;A)-Jan-20-1009\\R6|POL-LOP(F&amp;A)-Jan-20-1009\\R6|477.76|2321/20/R6|136502.48|-116504.66587443562|","-131417|-131417|19569.12|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.12|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||12/02/2026|111848.29|19569|01-01-2026 to 01-01-2027|POL-F&amp;A-Jan-20-1022\\R6|POL-F&amp;A-Jan-20-1022\\R6|956.61|2321/20/R6|130460.8|-111847.94105233089|","-2277|-2277|317.95|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.05|0||MUR|20/11/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||09/02/2026|1959.16|318|20-11-2025 to 01-01-2026|POL-F&amp;A-Jan-20-1022\\R5|POL-F&amp;A-Jan-20-1022\\R5\\E1|157.42|2321/20/R5/E2|2119.69|-1959.0653591613932|","-272603|-272603|45701.76|8|ORANGE EIGHT LTD|31739.35|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/11/2025|529569.24|13962.41|01-10-2025 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4|3999|MED/2022/01410/R3|571272|-250946.36011848328|","-30551|-30551|2444.12|8|ORANGE EIGHT LTD|2444.2|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||22/04/2026|28107.35|-0.0799999999999272|01-04-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E1|0|MED/2022/01410/R3/EQ/5|30551.47|-28106.917600036923|","25543|25543|-2043.44|8|ORANGE EIGHT LTD|-2043.88|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|-23499.6|0.440000000000055|01-05-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E3|0|MED/2022/01410/R3/EQ/6|-25543.04|23499.563199994987|","56735|56735|-4538.8|8|ORANGE EIGHT LTD|-4538.6|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||16/04/2026|-52196.22|-0.199999999999818|01-04-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E2|0|MED/2022/01410/R3/EQ/4|-56735.02|52196.20159999943|","22325|22325|-1786|8|ORANGE EIGHT LTD|-1786|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||03/06/2026|-20539|0|01-06-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E4|0|MED/2022/01410/R3/EQ/7|-22325|20539|","-26357|-26357|3865.03|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND\nCLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|0.03|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||02/02/2026|22492.04|3865|01-02-2026 to 01-02-2027|POL-CAR-TPL-Jun-20-1033\\R5|POL-CAR-TPL-Jun-20-1033\\R5|590.18|6162/25|25766.89|-22491.980264877697|","-5118|-5118|750|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR CONTRACTORS &amp;/OR SUB CONTRACTORS||0||MUR|15/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||4367.5||15-05-2026 to 15-06-2026|POL-CAR-TPL-Nov-25-1054|POL-CAR-TPL-Nov-25-1054\\E2|117.5||5000|-4367.926722032243|","-6121|-6121|900|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION)||0||MUR|15/06/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY|||5221||15-06-2026 to 15-08-2026|POL-PL-Nov-25-1105|POL-PL-Nov-25-1105\\E3|121||6000|-5221|","-130114|-130114|19449|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR ECOFUEL LTEE|0|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||15/01/2026|110664.81|19449|01-12-2025 to 01-12-2026|POL-PA-Dec-19-1603\\R6|POL-PA-Dec-19-1603\\R6|453.81|46037/12/R13|129660|-110664.9715994021|","-197263|-197263|36216.93|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR ECOFUEL LTEE|6730.58|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||15/01/2026|206074.31|29486.35|01-12-2025 to 01-12-2026|POL-ARM(P&amp;M)-Dec-19-1132\\R6|POL-ARM(P&amp;M)-Dec-19-1132\\R6|845.07|46037/12/R13|241446.17|-167776.74922762375|","-15329|-15329|2216.63|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT ,SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR DIRECT CONTRACTORS &amp;/OR SUBCONTRACTORS||0||MUR|11/06/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||13112.59||11-06-2026 to 11-09-2026|POL-CAR-TPL-Jun-26-34|POL-CAR-TPL-Jun-26-34|551.72||14777.5|-13112.401812355749|","-3111|-3111|450|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION)|0|0||MUR|16/03/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||15/04/2026|2660.5|450|16-03-2026 to 15-05-2026|POL-PL-Nov-25-1105|POL-PL-Nov-25-1105\\E1|110.5||3000|-2660.9276643626426|","368|368|15750|15|GOLDEN FUND MANAGEMENT SERVICES LTD|15804.73|0|Correction to be done by CBL amount not in aging|MUR|01/05/2019|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PI-CRIME||13/05/2019|90142.5|-54.7299999999996|01-05-2019 to 01-05-2020|POL-C+PI-Jun-19-1002|POL-C+PI-Jun-19-1002|892.5|15398/18/R1|105000|313.2652454139812|","-736|-736|0|15|GOLDEN FUND MANAGEMENT SERVICES LTD|0|0|Correction to be done by CBL amount not in aging|MUR|01/05/2019|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PI-CRIME||13/05/2019|-368|0|01-05-2019 to 01-05-2020|POL-C+PI-Jun-19-1003|POL-C+PI-Jun-19-1003|-368|15398/18/R1|0|-736|"]</t>
+  </si>
+  <si>
+    <t>["-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.11|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.10|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.9|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.8|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.7|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.6|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.41|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.40|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.39|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.38|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.37|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.36|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.35|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.34|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.33|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.32|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.31|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.30|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.158|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.157|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.156|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.155|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.154|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.153|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.152|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.151|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.150|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.149|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.148|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.147|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.93|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.92|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.91|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.90|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.89|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.88|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.87|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.86|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.85|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.84|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.83|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.82|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.311|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.310|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.309|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.308|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.307|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.306|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.305|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.304|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.303|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.302|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.301|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.300|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.17|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.16|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.15|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.14|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.13|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.12|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.11|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.10|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.9|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.8|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.7|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.6|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.41|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.40|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.39|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.38|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.37|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.36|Medical","-7529.76|94522|FON SING MARIE SANDRA PIT TSOU|30/09/2025|23164.95||01/08/25 to 31/07/26|MED/2024/00815|MED/2024/00815/R1|MED/2024/00815|23164.95|07/08/2025|JRNNHZ.250807.18|Medical","-12492.78|154944.97|Gaya Shyamsundur|30/09/2025|16428.91||01/08/25 to 31/07/26|MD08M01060|MD08M01060/R17|MD08M01060|16428.91|26/08/2025|JRNNHZ.250826.22|Medical","-5061.6|42580|COLLET-SERRET MARINE CELIA|30/11/2025|30014.72|Payment done after 30.06.2026|01/10/25 to 30/09/26|MED/2025/01440|MED/2025/01440/N|MED/2025/01440|30014.72|23/01/2026|JRNNHZ.260123.2|Medical","-6314.24|79328|SALEMOHAMED FAWZIA|30/11/2025|13801.66||01/10/25 to 30/09/26|MD06M00609|MD06M00609/R19|MD06M00609|13801.66|03/10/2025|JRNNHZ.251003.167|Medical","-9316.8|78040|BUCARD JOSEPHE MARIE CLAUDE|31/10/2025|14170.45||01/09/25 to 31/08/26|MED/2025/01312|MED/2025/01312/N|MED/2025/01312|14170.45|25/11/2025|JRNNHZ.251125.142|Medical","-5685.78|71572.3|BENZOU LTEE|31/12/2025|19267.44||01/11/25 to 31/10/26|MD18M01126|MD18M01126/R7|MD18M01126|19267.44|18/11/2025|JRNNHZ.251118.72|Medical"]</t>
+  </si>
+  <si>
+    <t>["-18271|-18271|2299.8|8|PARIS-ONEZIME MARIE STEPHANIE MRS|837.96|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||09/06/2026|26447.76|1461.84|01-05-2026 to 01-01-2027|POL-HEALTH-Dec-22-157\\R3|POL-HEALTH-Dec-22-157\\R3\\E1|0|MED/2023/00006/R3|28747.56|-16809.323050721523|","-48544|-48544|7735.12|8|PARIS-ONEZIME MARIE STEPHANIE MRS|4641.24|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/12/2025|89353.88|3093.88|01-01-2026 to 01-01-2027|POL-HEALTH-Dec-22-157\\R3|POL-HEALTH-Dec-22-157\\R3|400|MED/2023/00006/R3|96689|-44676.47983520275|","-43082.59|-43082.59|14673.79|15|ROGERS CAPITAL FINANCE LTD ON LEASE TO HEFTY LTD|8240.27|99.18||MUR|04/12/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||09/12/2025|83593.07|6433.52|04-12-2025 to 01-12-2026|POL-MV-Dec-25-503|POL-MV-Dec-25-503|342.39|34294/25|97825.29|-36649.242294414405|","-135220|-135220|20182.35|15|SPICE FINANCE LTD ON FINANCE LEASE TO HEFTY LTD|0.349999999997672|200||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||06/04/2026|115037.58|20182|01-04-2026 to 01-04-2027|POL-MV-Apr-23-97\\R3|POL-MV-Apr-23-97\\R3|470.93|6400/26|134549|-115037.63955209857|","-59581|-59581|8891.1|15|INDUSTRIAL FINANCE CORPORATION OF MAURITIUS LTD (IFCM) ON FINANCE LEASE TO HEFTY LTD|0.1|100||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||06/04/2026|50690.36|8891|01-04-2026 to 01-04-2027|POL-MV-Apr-23-105\\R3|POL-MV-Apr-23-105\\R3|207.46|6368/26|59274|-50689.96864393722|","-120520|-120520|18000|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR SUB-CONTRACTORS|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|102520|18000|01-05-2026 to 31-05-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E3|520|12718/24/N|120000|-102520|","-184322|-184322|27536.85|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB-CONTRACTORS|-0.15|0||MUR|28/04/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|156784.68|27537|28-04-2026 to 31-05-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E4|742.53|12718/24/N|183579|-156785.0797840057|","-123859|-123859|92122.96|15|REHM GRINAKER CONSTRUCTION CO. LTD|92122.96|3000||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||21/01/2026|527179.71|0|01-01-2026 to 01-01-2027|POL-MVF-Jun-21-1026\\R4|POL-MVF-Jun-21-1026\\R4|2149.59|10936/21/R4|614153.08|-105434.63618668073|","-722620|-722620|108000|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB-CONTRACTORS|0|0||MUR|31/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|614620|108000|31-05-2026 to 31-08-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E5|2620|12718/24/N|720000|-614620|","-278797|-278797|44294.4|8|CREDIT GUARANTEE INSURANCE CO LTD|22146.08|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/01/2026|513261.36|22148.32|01-01-2026 to 01-01-2027|POL-HEALTH-Jan-20-22\\R6|POL-HEALTH-Jan-20-22\\R6|3875.76|MD11M00167/10/R5|553680|-256648.2810327706|","-109903|-109903|11704.53|8|CREDIT GUARANTEE INSURANCE CO LTD|2911.85|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/04/2026|134602.04|8792.68|01-03-2026 to 01-01-2027|POL-HEALTH-Jan-20-22\\R6|POL-HEALTH-Jan-20-22\\R6\\E1|0|MD11M00167/10/R5/EQ/4|146306.57|-101110.75669479504|","-4204|-4204|628.35|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|0.35|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||05/05/2026|3575.32|628|01-04-2026 to 01-04-2027|POL-MON-Apr-20-1052\\R6|POL-MON-Apr-20-1052\\R6|14.67|8040/21/R5|4189|-3575.600672745482|","-21300|-21300|3183.83|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.17|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||05/05/2026|18115.96|3184|01-04-2026 to 01-04-2027|POL-EE-Apr-20-1072\\R6|POL-EE-Apr-20-1072\\R6|74.29|8040/21/R5|21225.5|-18116.13860981728|","-3947|-3947|589.95|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.0499999999999272|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||05/05/2026|3356.82|590|01-04-2026 to 01-04-2027|POL-ARMISC-Apr-26-7|POL-ARMISC-Apr-26-7|13.77|8040/21/R5|3933|-3357.0156203680476|","-52448|-52448|7839.71|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.29|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||05/05/2026|44607.96|7840|01-04-2026 to 01-04-2027|POL-EL-Apr-20-1145\\R6|POL-EL-Apr-20-1145\\R6|182.92|8040/21/R5|52264.75|-44608.240672655236|","-197614|-197614|29538.75|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.25|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||05/05/2026|168075.49|29539|01-04-2026 to 01-04-2027|POL-PL-Apr-20-1159\\R6|POL-PL-Apr-20-1159\\R6|689.24|8040/21/R5|196925|-168075.285874439|","-115877|-115877|17320.89|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.11|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||05/05/2026|98555.9|17321|01-04-2026 to 01-04-2027|POL-PA-Apr-20-1141\\R6|POL-PA-Apr-20-1141\\R6|404.16|8040/21/R5|115472.63|-98556.0786098752|","-219576|-219576|48227.25|15|IMPACT PRODUCTION LTD|15592.78|2500||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||30/01/2026|276913.07|32634.47|01-01-2026 to 01-01-2027|POL-MVF-Sep-19-6170\\R7|POL-MVF-Sep-19-6170\\R7|1125.32|49936/17/R8\n54552/15/R10\n19969/21/R5\n30665/22/R4\n49919/17/R8|321515|-187006.84141025634|","-66231|-66231|9900|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|0|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||05/05/2026|56331|9900|01-04-2026 to 01-04-2027|POL-PA-Apr-20-1140\\R6|POL-PA-Apr-20-1140\\R6|231|8040/21/R5|66000|-56331|","-228722|-228722|76806|15|KASA CORPORATE SERVICES LTD|42670.55|800||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||20/02/2026|437826.14|34135.45|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1065\\R4|POL-MVF-Dec-21-1065\\R4|1792.14|32859/23/R2|512040|-194586.5067678828|","16632|16632|-1330.56|8|KASA CORPORATE SERVICES LTD.|0.44|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/03/2026|-15301.44|-1331|01-12-2025 to 01-03-2026|POL-HEALTH-Jun-19-2718\\R48|POL-HEALTH-Jun-19-2718\\R48\\E3|0|MD08M01076/14/R4/EQ/8|-16632|15301.44|","22341|22341|-1787.28|8|KASA CORPORATE SERVICES LTD.|-0.28|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-20553.72|-1787|01-04-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49\\E1|0|MD08M01076/14/R5/EQ/2|-22341|20553.72|","-24663|-24663|1959.36|8|KASA CORPORATE SERVICES LTD.|0.36|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|22703.64|1959|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49\\E2|171|Please refer to POL-HEALTH-Jun-19-2718\\R49 - NO Docs to follow|24492|-22703.64|","-969342|-969342|77008.32|8|KASA CORPORATE SERVICES LTD.|0.320000000009313|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|892333.68|77008|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49|6738|MD08M01076/14/R5 - please refer to POL-HEALTH-Jun-19-2718\\R49\\E2 for adjustment in  premium|962604|-892333.6799999999|","-265806|-265806|79479.3|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|39747.84|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||17/03/2026|452237.22|39731.46|01-03-2026 to 28-02-2027|POL-ARM(P&amp;M)-Mar-20-1019\\R6|POL-ARM(P&amp;M)-Mar-20-1019\\R6|1854.52|8187/26/N|529862|-226074.16165914875|","-40914|-40914|12234.05|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|6118.43|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||17/03/2026|69611.76|6115.62|01-03-2026 to 28-02-2027|POL-PA-Mar-20-1103\\R6|POL-PA-Mar-20-1103\\R6|285.46|8187/26/N|81560.35|-34798.30609092879|","-30023|-30023|8977.5|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|4489.18|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||17/03/2026|51081.97|4488.32|01-03-2026 to 28-02-2027|POL-PPL-Mar-20-1021\\R6|POL-PPL-Mar-20-1021\\R6|209.47|8187/26/N|59850|-25535.25672654121|","-30023|-30023|8977.5|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE &amp;/OR PRINCIPAL &amp;/OR CONTRACTORS &amp;/OR SUB-CONTRACTORS|4489.18|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|EAR &amp; TPL||17/03/2026|51081.98|4488.32|01-03-2026 to 28-02-2027|POL-EAR-TPL-Mar-20-1005\\R6|POL-EAR-TPL-Mar-20-1005\\R6|209.48|8187/26/N|59850|-25535.25747375768|","-8931|-8931|2596.16|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1298.65|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||17/03/2026|15272.17|1297.51|01-03-2026 to 28-02-2027|POL-F&amp;A-Mar-20-1117\\R6|POL-F&amp;A-Mar-20-1117\\R6|560.58|8187/26/N|17307.75|-7633.379855308247|","-11765|-11765|3518.25|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1759.9|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||17/03/2026|20018.87|1758.35|01-03-2026 to 28-02-2027|POL-EE-Mar-20-1049\\R6|POL-EE-Mar-20-1049\\R6|82.12|8187/26/N|23455|-10006.407136896953|","-8998|-8998|2690.78|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1345.52|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||17/03/2026|15310.51|1345.26|01-03-2026 to 28-02-2027|POL-ARMISC-Mar-20-1024\\R6|POL-ARMISC-Mar-20-1024\\R6|62.79|8187/26/N|17938.5|-7653.005366837599|","-893|-893|267.15|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|133.77|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||17/03/2026|1520.08|133.38|01-03-2026 to 28-02-2027|POL-LOP(F&amp;A)-Mar-20-1029\\R6|POL-LOP(F&amp;A)-Mar-20-1029\\R6|6.23|8187/26/N|1781|-759.5169284311477|","-10152|-10152|3035.48|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1518.42|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||08/05/2026|17271.86|1517.06|01-03-2026 to 28-02-2027|POL-EL-Mar-20-1108\\R6|POL-EL-Mar-20-1108\\R6|70.83|8187/26/N|20236.51|-8634.50962656852|","-12154.99|-12154.99|68082.09|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED  &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE  PROPERTIES LTD &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE  &amp;/OR QUALITY BEVERAGES LIMITED &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR TRAMPOLINE LIMITEE  NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|68082.14|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||06/02/2026|387387.1|-0.0500000000029104|01-01-2026 to 01-01-2027|POL-EE-Jan-26-3|POL-EE-Jan-26-3|1588.61|1918/26/N|453880.58|-10338.100644368502|","-27563|-27563|172922.85|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LTD &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALLI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|172922.99|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||06/02/2026|983931.06|-0.14000000001397|01-01-2026 to 01-01-2027|POL-PA-Mar-20-1106\\R6|POL-PA-Mar-20-1106\\R6|4034.9|1918/26/N|1152819.01|-23442.97025955507|","-12710|-12710|37735.58|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES &amp;/OR CURRIMJEE LIMITED &amp;/OR  CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR PRINCIPALS &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|37735.3|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||06/02/2026|214715.44|0.279999999998836|01-01-2026 to 01-01-2027|POL-CAR-TPL(BC)-Mar-20-1010\\R6|POL-CAR-TPL(BC)-Mar-20-1010\\R6|880.52|1918/26/N|251570.5|-10810.149400069764|","-19711.99|-19711.99|38186.93|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LIMITEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED  &amp;/OR LATE BAI REHMATBAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASSALI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LIMITED &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LIMITED &amp;/OR QUALITY BEVERAGES LIMITED &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR EMTEL MFS CO LTD &amp;/OR E-SKILLS LIMITED &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LIMITEE &amp;/OR ZAC (PROPERTIES) LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|38186.78|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||06/02/2026|217783.65|0.149999999994179|01-01-2026 to 01-01-2027|POL-PPL-Mar-20-1020\\R6|POL-PPL-Mar-20-1020\\R6|1391.08|1915/26/N|254579.5|-16771.259927463147|"]</t>
+  </si>
+  <si>
+    <t>["-14063.8|176197.6|VETOPHARMA LTD|31/12/2025|69323.69|Payment done after 30.06.2026|01/11/25 to 31/10/26|MED/2024/01200|MED/2024/01200/R1|MED/2024/01200|69323.69|13/01/2026|JRNNHZ.260113.134|Medical","-13858.46|171357.66|Rivaud Marie Josee|30/01/2026|62999.68|Payment done after 30.06.2026|01/12/25 to 30/11/26|MED/2023/01267|MED/2023/01267/R2|MED/2023/01267|62999.68|03/12/2025|JRNNHZ.251203.80|Medical","-21358.72|176800.64|CARR-BROWN ALAN|30/11/2025|46634.61||01/10/25 to 30/09/26|MED/2025/01409|MED/2025/01409/N|MED/2025/01409|46634.61|30/12/2025|JRNNHZ.251230.48|Medical","-20207.28|252591|COMPAGNIE MAURICIENNE DE TEXTILE LTEE|01/07/2026|232383.72||01/12/25 to 30/11/26|MD16M00967|MD16M00967/R9|MD16M00967|232383.72|31/05/2026|JRNNHZ.260531.156|Medical","-20207.28|252591|COMPAGNIE MAURICIENNE DE TEXTILE LTEE|01/08/2026|||01/12/25 to 30/11/26|MD16M00967|MD16M00967/R9|MD16M00967|232383.72|30/06/2026|JRNNHZ.260630.558|Medical","-4099.07|51638.43|BUSSIER Robert Emmanuel Marie Angelo|30/06/2026|20655.92||01/01/26 to 31/12/26|MD21M00507|MD21M00507/R5|MD21M00507|20655.92|15/01/2026|JRNNHZ.260115.177|Medical","-9015.21|113090.24|VALAYDON-JOSEPHINE RUBBY PA|02/03/2026|51931.06||01/01/26 to 31/12/26|MD18M00171|MD18M00171/R8|MD18M00171|51931.06|14/01/2026|JRNNHZ.260114.35|Medical","-471641.58|3166407.94|Compagnie D`Exploitation Agricole Limitee (CEAL)|28/06/2026|2210635.51|Payment done after 30.06.2026|01/01/26 to 31/12/26||MT200001000114/R26||2662306.14|06/01/2026|JRNI.260106.373|Motor","-25914|3873.6|Compagnie D`Exploitation Agricole Limitee (CEAL)|05/06/2026|||01/01/26 to 31/12/26||MT200001000114/R26/E10||-22040.4|03/06/2026|JRNI.260603.375|Motor","-4140.15|27762|Compagnie D`Exploitation Agricole Limitee (CEAL)|01/08/2026|||01/01/26 to 31/12/26||MT200001000114/R26/E7||23621.85|14/05/2026|JRNI.260514.24|Motor","-4140.15|27762|Compagnie D`Exploitation Agricole Limitee (CEAL)|01/08/2026|||01/01/26 to 31/12/26||MT200001000114/R26/E6||23621.85|13/05/2026|JRNI.260513.32|Motor","-552.15|3694|Compagnie D`Exploitation Agricole Limitee (CEAL)|01/08/2026|||01/01/26 to 31/12/26|POL-MVF-Jun-19-1892\\R7\\E7|MT200001000114/R26/E8|POL-MVF-Jun-19-1892\\R7\\E7|3141.85|25/05/2026|JRNI.260525.419|Motor","-320037.58|2158926.99|Rey &amp; Lenferna Limited|07/07/2026|1783590.77||01/01/26 to 31/12/26||25114/21/R4||1783590.77|06/01/2026|JRNI.260106.427|Motor","-28900.5|195094|Watertech Limited|01/04/2026|92889.71||01/01/26 to 31/12/26||26138/21/R4||92889.71|06/01/2026|JRNI.260106.451|Motor","-17739.45|118736|Mediterranean Shipping Company (Mauritius) Ltd|01/08/2026|||01/01/26 to 31/12/26||25811/10/R15/E1||100996.55|29/05/2026|JRNI.260529.414|Motor","-43344.15|290372|Mediterranean Shipping Company (Mauritius) Ltd|01/04/2026|79196.93||01/01/26 to 31/12/26||25811/10/R15||79196.93|06/01/2026|JRNI.260106.424|Motor","-10784.22|134411.6|Rajkomar Vimla|02/04/2026|74154.66||01/02/26 to 31/01/27|FD10M00005|FD10M00005/R16|FD10M00005|74154.66|04/02/2026|JRNNHZ.260204.222|Medical","-4776.09|60101.2|SOOPRAMANIEN POTHEGADOO KAVINA|02/04/2026|30095.59|Payment done after 30.06.2026|01/02/26 to 31/01/27|MED/2025/00230|MED/2025/00230/R1|MED/2025/00230|30095.59|09/02/2026|JRNNHZ.260209.67|Medical","-31162.95|208980|LES VUES D ANBALABA|01/04/2026|1455.27||29/12/25 to 31/12/26||712/26/N||1455.27|14/01/2026|JRNI.260114.326|Non-Motor Corporate","-62081.28|781448.12|PREVOIR SOLUTIONS INFORMATIQUES LTD PREVOIR SOLUTIONS INFORMATIQUES LTD|03/03/2026|417733.72|Payment done after 30.06.2026|01/02/26 to 31/01/27|MED/2023/00358|MED/2023/00358/R3|MED/2023/00358|417733.72|19/02/2026|JRNNHZ.260219.64|Medical","-850.2|5888|SKYDIVE AUSTRAL LIMITED|01/04/2026|5037.8||01/02/26 to 31/01/27||1249/26/N||5037.8|21/01/2026|JRNI.260121.25|Motor","-850.2|5888|SKYDIVE AUSTRAL LIMITED|01/08/2026|||01/06/26 to 31/05/27||12179/26/N||5037.8|15/05/2026|JRNI.260515.213|Motor","-142500|954750|Currimjee Group of Companies|14/02/2026|34329.35||01/01/26 to 31/12/26||38813/12/R13||34329.35|21/01/2026|JRNI.260121.345|Financial","-22871.7|153512|AIKO RESIDENCE LTD|01/04/2026|130640.3||21/01/26 to 21/01/28||1847/26/N||130640.3|27/01/2026|JRNI.260127.396|Car/Ear (One Off)"]</t>
+  </si>
+  <si>
+    <t>["-172|-172|34905.3|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LTD &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR SYNDICAT DES COPROPRIETAIRES DE PHOENIX CENTRAL &amp;/OR FACILICARE LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|34905.52|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||06/02/2026|198611.18|-0.219999999993888|01-01-2026 to 01-01-2027|POL-MON-Mar-20-1043\\R6|POL-MON-Mar-20-1043\\R6|814.48|1918/26/N|232702|-146.28998758460216|","-180668|-180668|29880.75|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LTD &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR SYNDICAT DES COPROPRIETAIRES DE PHOENIX CENTRAL &amp;/OR FACILICARE LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|2889.59|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||16/03/2026|170121.48|26991.16|01-01-2026 to 01-01-2027|POL-MON-Mar-20-1043\\R6|POL-MON-Mar-20-1043\\R6\\E2|797.23|1918/26/N/E1|199205|-153675.82425775955|","229698|229698|-34477.8|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LTD &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR SYNDICAT DES COPROPRIETAIRES DE PHOENIX CENTRAL &amp;/OR FACILICARE LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|-128.050000000005|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||16/03/2026|-196078.7|-34349.75|01-01-2026 to 01-01-2027|POL-MON-Mar-20-1043\\R6|POL-MON-Mar-20-1043\\R6\\E1|-704.5|1918/26/N/E1|-229852|195348.58150865405|","-14974.99|-14974.99|108863.66|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED  &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE  PROPERTIES LIMITED  &amp;/OR  LATE BAI REHMATBAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE  NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|108863.22|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||06/02/2026|619434.25|0.44000000001688|01-01-2026 to 01-01-2027|POL-EL-Mar-20-1106\\R6|POL-EL-Mar-20-1106\\R6|2540.16|1918/26/N|725757.75|-12736.576024785652|","-26952|-26952|4013.77|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED  &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE  PROPERTIES LTD &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|-0.23|0||MUR|05/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ASSETS ALL RISKS &amp; BUSINESS INTERRUPTION||26/05/2026|22938.32|4014|05-03-2026 to 01-01-2027|POL-AAR+BI-Mar-20-1003\\R6|POL-AAR+BI-Mar-20-1003\\R6\\E1|193.65||26758.44|-22938.24340301624|","34442|34442|-2755.38|8|RENTACOLOR (MAURITIUS) LIMITED|-0.38|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-31686.92|-2755|01-05-2026 to 01-01-2027|POL-HEALTH-Jan-21-3\\R5|POL-HEALTH-Jan-21-3\\R5\\E1|0|MD21M00252/0/R5/EQ/2|-34442.3|31686.64399996516|","-366870|-366870|29145.6|8|RENTACOLOR (MAURITIUS) LIMITED|2428.45|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/02/2026|337724.64|26717.15|01-01-2026 to 01-01-2027|POL-HEALTH-Jan-21-3\\R5|POL-HEALTH-Jan-21-3\\R5|2550.24|MD21M00252/0/R5|364320|-337724.41906653426|","20810|20810|-1664.76|8|SAMENA CAPITAL MAURITIUS MANAGEMENT|-1664.56|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||23/01/2026|-19144.79|-0.200000000000045|01-01-2026 to 01-07-2026|POL-HEALTH-Jul-19-2918\\R6|POL-HEALTH-Jul-19-2918\\R6\\E1|0|MED/2023/01023/R2|-20809.55|19145.204000086498|","-238864|-238864|18976.32|8|SAMENA CAPITAL MAURITIUS MANAGEMENT|3163.38|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||10/07/2026|219887.68|15812.94|01-07-2026 to 01-07-2027|POL-HEALTH-Jul-19-2918\\R7|POL-HEALTH-Jul-19-2918\\R7|1660|MED/2023/01023/R3|237204|-219887.68|Timing Difference","-13076|-13076|1569.12|12|MAURITOURS LTD|0.12|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/05/2026|11506.88|1569|01-06-2026 to 01-01-2027|POL-HEALTH-Jan-26-3|POL-HEALTH-Jan-26-3\\E1|0|MED/2023/00018/R3/EQ/1|13076|-11506.880000000001|","-692039|-692039|82467.36|12|MAURITOURS LTD|27441.8|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||07/04/2026|609571.24|55025.56|01-01-2026 to 01-01-2027|POL-HEALTH-Jan-26-3|POL-HEALTH-Jan-26-3|4810.6|MED/2023/00018/R3|687228|-609571.5923336647|","-437069|-437069|69442.56|8|NASSAU SERVICES LTD|34719.69|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|804665.44|34722.87|01-01-2026 to 01-01-2027|POL-HEALTH-Feb-21-10\\R27|POL-HEALTH-Feb-21-10\\R27|6076|MD10M00493/11/R5|868032|-402346.52834130335|","-156592|-156592|31162.5|15|NASSAU SERVICES LTD &amp;/OR UHY HEERALALL &amp;/OR UHY LOSS ADJUSTERS LTD &amp;/OR UHY &amp; CO &amp;/OR UHY ADVISORY LTD &amp;/OR MR. NIRMAL HEERALALL &amp;/OR MR. DOMINIQUE SAMOUILHAN &amp;/OR MR. PRAVESH JAISHINGH PURGASS &amp;/OR MR. BENY KOWLESSUR &amp;/OR MR AVINASHSINGH MOORUTH &amp;/OR MR JEAN THOMAS SAMOUILHAN &amp;/OR CAS SERVICES LTD &amp;/OR UHY CORPORATE FINANCE LTD &amp;/OR MR ANDRE DE COMARMOND &amp;/OR MR VINCENT DESIRE NICOLAS LECORDIER &amp;/OR MR VIVEGAH THOPLAN &amp;/OR MRS SABRINA RAGAVOODOO|7790.1|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY||03/06/2026|177626.25|23372.4|01-06-2026 to 31-05-2027|POL-PI-Jun-21-15\\R5|POL-PI-Jun-21-15\\R5|1038.75|12779/21/R5 3601.902454|207750|-133220.05970149254|","-13812|-13812|1104.96|8|LA PRUDENCE LEASING FINANCE CO. LTD|-0.04|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||02/03/2026|12707.04|1105|01-01-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E2|0|MD11M00166/10/R5/EQ/2|13812|-12707.04|","27051|27051|-2164.08|8|LA PRUDENCE LEASING FINANCE CO. LTD|-0.08|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||14/04/2026|-24886.88|-2164|01-04-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E3|0|MD11M00166/10/R5/EQ/6|-27050.96|24886.91679999527|","37909|37909|-3032.75|8|LA PRUDENCE LEASING FINANCE CO. LTD|0.25|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-34876.57|-3033|01-04-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E6|0|MD11M00166/10/R5/EQ/8|-37909.32|34876.275600037145|","-21675|-21675|1734.04|8|LA PRUDENCE LEASING FINANCE CO. LTD|0.04|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/05/2026|19941.41|1734|01-05-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E5|0|MD11M00166/10/R5/EQ/7|21675.45|-19940.996000083043|","19196|19196|-1535.72|8|NEWREST (MAURITIUS) LTD|0.28|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-17660.74|-1536|01-06-2026 to 01-10-2026|POL-HEALTH-Dec-24-132\\R1|POL-HEALTH-Dec-24-132\\R1\\E3|0|MED/2024/01202/R1/EQ/7|-19196.46|17660.316800076682|","-6048|-6048|483.84|8|NEWREST (MAURITIUS) LTD|-0.16|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||10/02/2026|5564.16|484|01-02-2026 to 01-10-2026|POL-HEALTH-Dec-24-132\\R1|POL-HEALTH-Dec-24-132\\R1\\E2|0|MED/2024/01202/R1/EQ/6|6048|-5564.16|","-6447|-6447|959.67|15|MCB LEASING LIMITED ON LEASE TO JAG SERVICES LTD|-0.33|26.3||MUR|08/12/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/12/2025|5486.84|960|08-12-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E49|22.4|31069/23/R1/E12|6397.81|-5487.257055367943|","52031|52031|-7777.5|15|MCB LEASING LIMITED ON LEASE TO JAG SERVICES LTD|0.5|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||23/02/2026|-44253.98|-7778|01-01-2026 to 01-01-2027|POL-MVF-Jul-19-6113\\R7|POL-MVF-Jul-19-6113\\R7\\E2|-181.48|31069/23/R2/E4|-51850|44253.57174887203|","2|2|12938|15|PANACHE CO LTD|12937.8|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||14/09/2019|74114|0.200000000000728|01-07-2019 to 01-07-2020|POL-CAR-TPL(BC)-Jun-19-1024|POL-CAR-TPL(BC)-Jun-19-1024|802|MD07E00472/R12|86250|1.7027523778890779|","-110|-110|1.52|15|PANACHE AND COMPANY LIMITED|-0.48|0||MUR|10/06/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||30/06/2026|108.62|2|10-06-2026 to 30-06-2026|POL-CP-Jun-19-1040\\R6|POL-CP-Jun-19-1040\\R6\\E1|100.04||10.1|-108.48193208643545|","1|1|315|15|PANACHE CO LTD|315.15|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|MONEY||30/09/2019|1792|-0.149999999999977|01-07-2019 to 01-07-2020|POL-MON-Jun-19-1077|POL-MON-Jun-19-1077|7|5180/15/R5|2100|0.8504983388704319|","-1|-1|4703|15|PANACHE CO LTD|4702.35|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||30/09/2019|26756|0.649999999999636|01-07-2019 to 01-07-2020|POL-EL-Jun-19-1236|POL-EL-Jun-19-1236|109|5180/15/R5|31350|-0.8505038303824025|","-2|-2|8100|15|PANACHE CO LTD|8099.7|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||30/09/2019|46089|0.299999999999272|01-07-2019 to 01-07-2020|POL-PA-Jun-19-1304|POL-PA-Jun-19-1304|189|5180/15/R5|54000|-1.7010463378176381|","119807.99|119807.99|-102187.5|15|SCOTT &amp; CO LTD &amp;/OR RIVERSIDE HEALH LTD &amp;/OR SCOTT HEALTH LTD &amp;/OR BAGATELLE HEALTH LTD &amp;/OR GRAND BAIE FORME HEALTH LTD &amp;/OR THE BRANDHOUSE LTD &amp;/OR STANDARD PHARMACY LTD &amp;/OR BEAU VALLON HEALTH LTD &amp;/OR MOBISIL LTD &amp;/OR SCOTT TRIBECA HEALTH LTD &amp;/OR SCOTT AGROW LTD|-84278.57|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|TERRORISM &amp; SABOTAGE||09/04/2026|-584563.89|-17908.93|01-10-2025 to 01-10-2026|POL-TER&amp;SAB-Oct-19-1021\\R6|POL-TER&amp;SAB-Oct-19-1021\\R6\\E1|-5501.39||-681250|101980.75418162765|","-122866|-122866|102187.5|15|SCOTT &amp; CO LTD &amp;/OR RIVERSIDE HEALH LTD &amp;/OR SCOTT HEALTH LTD &amp;/OR BAGATELLE HEALTH LTD &amp;/OR GRAND BAIE FORME HEALTH LTD &amp;/OR THE BRANDHOUSE LTD &amp;/OR STANDARD PHARMACY LTD &amp;/OR BEAU VALLON HEALTH LTD &amp;/OR MOBISIL LTD &amp;/OR SCOTT TRIBECA HEALTH LTD &amp;/OR SCOTT AGROW LTD|83757.06|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|TERRORISM &amp; SABOTAGE||09/04/2026|582468.75|18430.44|01-10-2025 to 01-10-2026|POL-TER&amp;SAB-Oct-19-1021\\R7|POL-TER&amp;SAB-Oct-19-1021\\R7|3406.25|43624/16/R8|681250|-104527.79104477612|","-1|-1|-28.04|15|SCOTT &amp; CO LTD &amp;/OR SCOTT HEALTH LTD &amp;/OR BAGATELLE HEALTH LTD &amp;/OR GRAND BAIE FORME HEALTH LTD &amp;/OR THE BRANDHOUSE LTD &amp;/OR STANDARD PHARMACY LTD &amp;/OR BEAU VALLON HEALTH LTD &amp;/OR MOBISIL LTD &amp;/OR TRIBECA HEALTH LTD|-28.14|0|Correction to be done by CBL amount not in aging|MUR|20/03/2024|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||13/06/2024|-159.55|0.100000000000001|20-03-2024 to 01-10-2024|POL-ARMISC-Jul-19-1112\\R5|POL-ARMISC-Jul-19-1112\\R5\\E2|-0.66|33954/19/R2/E8|-186.93|-0.850525081294312|","-17956|-17956|3578.65|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|894.27|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||18/05/2026|20362.5|2684.38|01-05-2026 to 30-04-2027|POL-EL-Mar-26-19\\R1|POL-EL-Mar-26-19\\R1|83.5|14246/26/R1|23857.65|-15271.991946919843|","-103484|-103484|38642|15|SBM BANK (MAURITIUS) LTD ON LEASE TO HIGHWAY PROPERTIES LTD|23185.21|195.07||MUR|10/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||08/05/2026|220068.02|15456.79|10-04-2026 to 01-04-2027|POL-MV-Apr-26-95|POL-MV-Apr-26-95|901.65|8591/26|257613.3|-88027.20119491313|","-118107|-118107|17579.51|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.490000000002328|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||11/05/2026|100527.45|17580|01-04-2026 to 30-04-2026|POL-F&amp;A-Mar-26-1018|POL-F&amp;A-Mar-26-1018|910.2|10767/26/N|117196.76|-100527.4840462408|","-983582|-983582|195955.58|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|48988.52|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||18/05/2026|1115487.22|146967.06|01-05-2026 to 30-04-2027|POL-CP-May-26-1008|POL-CP-May-26-1008|5072.3|13781/26/N|1306370.5|-836615.3299419845|","-11265|-11265|1683.84|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.16|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||11/05/2026|9581.04|1684|01-04-2026 to 30-04-2026|POL-LOP(F&amp;A)-Mar-26-3|POL-LOP(F&amp;A)-Mar-26-3|39.29|10767/26/N|11225.59|-9581.142062764982|","-2773|-2773|339.81|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.19|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||11/05/2026|2433.49|340|01-04-2026 to 30-04-2026|POL-PL-Mar-26-21|POL-PL-Mar-26-21|507.93|14246/26/N|2265.37|-2433.2267587350807|","-1528|-1528|228.35|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|0.35|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||11/05/2026|1299.34|228|01-04-2026 to 30-04-2026|POL-EL-Mar-26-19|POL-EL-Mar-26-19|5.33|14246/26/N|1522.36|-1299.6036630468222|"]</t>
+  </si>
+  <si>
+    <t>["-48874|-48874|9740.63|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|2434.76|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||18/05/2026|55424.18|7305.87|01-05-2026 to 30-04-2027|POL-PA-Mar-26-17\\R1|POL-PA-Mar-26-17\\R1|227.28|14246/26/R1|64937.53|-41568.46883033957|","-1158|-1158|173.1|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|0.1|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||11/05/2026|984.92|173|01-04-2026 to 30-04-2026|POL-EE-Mar-26-8|POL-EE-Mar-26-8|4.04|14246/26/N|1153.98|-984.9029895856721|","-5001|-5001|747.58|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.42|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN||11/05/2026|4253.75|748|01-04-2026 to 30-04-2026|POL-M B-D-Mar-26-1003|POL-M B-D-Mar-26-1003|17.44|14246/26/N|4983.89|-4253.469327158976|","-55317|-55317|10950|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|2737.52|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||18/05/2026|62805.5|8212.48|01-05-2026 to 30-04-2027|POL-PL-Mar-26-21\\R1|POL-PL-Mar-26-21\\R1|755.5|14246/26/R1|73000|-47104.44432618584|","-3819|-3819|570.88|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.12|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||11/05/2026|3248.33|571|01-04-2026 to 30-04-2026|POL-PA-Mar-26-17|POL-PA-Mar-26-17|13.32|14246/26/N|3805.89|-3248.1513899471356|","-440|-440|197.03|15|ACBMS LTD|131.27|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||12/05/2026|1121.07|65.76|01-05-2026 to 01-05-2027|POL-EE-May-22-1007\\R4|POL-EE-May-22-1007\\R4|4.6|12079/22|1313.5|-374.22866246870495|","-400|-400|106.08|15|ACBMS LTD|71.1|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||12/05/2026|1103.6|34.98|01-05-2026 to 01-05-2027|POL-EL-May-22-28\\R4|POL-EL-May-22-28\\R4|502.48|12079/22|707.2|-364.9229548310297|","-6412|-6412|2874.45|15|ACBMS LTD|1916.45|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||12/05/2026|16355.62|958|01-05-2026 to 01-05-2027|POL-PA-May-22-18\\R4|POL-PA-May-22-18\\R4|67.07|12079/22|19163|-5453.554534122861|","-19672|-19672|8819.96|15|ACBMS LTD|5879.48|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||12/05/2026|50185.55|2940.48|01-05-2026 to 01-05-2027|POL-ARMISC-May-22-11\\R4|POL-ARMISC-May-22-11\\R4|205.81|12079/22|58799.7|-16731.4906624822|","-26497|-26497|2119.74|8|GAYA COLLECTIONS LIMITEE|-0.260000000000291|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/06/2026|24376.98|2120|01-06-2026 to 01-05-2027|POL-HEALTH-Aug-23-74\\R4|POL-HEALTH-Aug-23-74\\R4\\E1|0|MED/2023/00969/R3/EQ/1|26496.72|-24377.23759997464|","-140853|-140853|16786.56|8|GAYA COLLECTIONS LIMITEE|5596.22|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/05/2026|194514.44|11190.34|01-05-2026 to 01-05-2027|POL-HEALTH-Aug-23-74\\R4|POL-HEALTH-Aug-23-74\\R4|1469|MED/2023/00969/R3|209832|-129663.09869484763|","3953|3953|-474.36|12|BELLE RIVIERE HOTEL LTD|-474.72|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/05/2026|-3478.64|0.360000000000014|01-04-2026 to 01-05-2026|POL-HEALTH-Sep-21-95\\R4|POL-HEALTH-Sep-21-95\\R4\\E16|0|MED/2025/00947/EQ/40|-3953|3478.64|","-90048|-90048|7203.84|8|BELLE RIVIERE HOTEL LTD|-0.16|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/06/2026|82844.16|7204|01-05-2026 to 01-05-2027|POL-HEALTH-Sep-21-95\\R6|POL-HEALTH-Sep-21-95\\R6\\E2|0|MED/2025/00947/R1/EQ/2|90048|-82844.16|","16176|16176|-1294.08|8|BELLE RIVIERE HOTEL LTD|-0.08|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/06/2026|-14881.92|-1294|01-05-2026 to 01-05-2027|POL-HEALTH-Sep-21-95\\R6|POL-HEALTH-Sep-21-95\\R6\\E1|0|MED/2025/00947/R1/EQ/1|-16176|14881.92|","7164|7164|-859.68|12|BELLE RIVIERE HOTEL LTD|-859.36|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/05/2026|-6304.32|-0.32000000000005|01-03-2026 to 01-05-2026|POL-HEALTH-Sep-21-95\\R4|POL-HEALTH-Sep-21-95\\R4\\E15|0|MED/2025/00947/EQ/39|-7164|6304.32|","1876|1876|-225.12|12|BELLE RIVIERE HOTEL LTD|-0.12|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/04/2026|-1650.88|-225|01-03-2026 to 01-05-2026|POL-HEALTH-Sep-21-95\\R4|POL-HEALTH-Sep-21-95\\R4\\E14|0|MED/2025/00947/EQ/38|-1876|1650.88|","-1749046|-1749046|139007.04|8|BELLE RIVIERE HOTEL LTD|11584|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/07/2026|1610743.96|127423.04|01-05-2026 to 01-05-2027|POL-HEALTH-Sep-21-95\\R6|POL-HEALTH-Sep-21-95\\R6|12163|MED/2025/00947/R1|1737588|-1610094.9679481024|","-32934|-32934|4922.8|15|OSMAN DR REZAH|-0.2|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||30/06/2026|28010.71|4923|01-06-2026 to 01-06-2027|POL-ARMISC-May-20-1035\\R6|POL-ARMISC-May-20-1035\\R6|114.86|3601.902454|32818.65|-28011.12675630384|","-10906|-10906|1562.87|15|OSMAN DR REZAH|-0.13|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||30/06/2026|9342.72|1563|01-06-2026 to 01-06-2027|POL-F&amp;A-May-20-1193\\R6|POL-F&amp;A-May-20-1193\\R6|486.47|3601.902454|10419.12|-9343.071243279823|","123515|123515|-18462.61|15|PARTSIONATE LTD|0.39|0||MUR|11/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||29/06/2026|-105052.25|-18463|11-05-2026 to 01-05-2027|POL-MV-May-26-130|POL-MV-May-26-130\\E1|-430.79|11084/26|-123084.07|105052.36907324349|","38910|38910|-5816.1|15|PARTSIONATE LTD|-0.1|0||MUR|02/06/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||26/06/2026|-33093.58|-5816|02-06-2026 to 01-05-2027|POL-MV-May-26-132|POL-MV-May-26-132\\E1|-135.71|11100/26/N|-38773.97|33093.8521673784|","-41423|-41423|6191.74|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTI PLANTS LTD &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED &amp;/OR WE FARM LTD|-0.26|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||18/06/2026|35231|6192|01-06-2026 to 01-07-2027|POL-EL-Jun-19-1239\\R7|POL-EL-Jun-19-1239\\R7|144.48||41278.26|-35231.221136023356|","-1|-1|450|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTIPLANTES LTEE &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED|450.08|0|Correction to be done by CBL amount not in aging|MUR|01/06/2020|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||22/07/2020|2560.5|-0.0800000000000409|01-06-2020 to 01-06-2021|POL-FID-Jun-19-1034\\R1|POL-FID-Jun-19-1034\\R1|10.5|22063/19|3000|-0.8505231689088191|","-1|-1|2235|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTIPLANTES LTEE &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED|2234.98|0|Correction to be done by CBL amount not in aging|MUR|01/06/2020|MAURITIUS UNION ASSURANCE CO LTD|MONEY||22/07/2020|12717.16|0.0199999999999818|01-06-2020 to 01-06-2021|POL-MON-Jun-19-1079\\R1|POL-MON-Jun-19-1079\\R1|52.16|22063/19|14900|-0.8505232688788777|","-86896|-86896|12914.23|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTI PLANTS LTD &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED &amp;/OR WE FARM LTD|0.23|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||18/06/2026|73981.95|12914|01-06-2026 to 01-07-2027|POL-F&amp;A-Jun-19-1327\\R7|POL-F&amp;A-Jun-19-1327\\R7|801.33||86094.85|-73981.79675101944|","-116166|-116166|17364.18|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTI PLANTS LTd &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED &amp;/OR WE FARM LTD|0.18|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||18/06/2026|98802.17|17364|01-06-2026 to 01-07-2027|POL-PA-Jun-19-1307\\R7|POL-PA-Jun-19-1307\\R7|405.16||115761.19|-98801.87231689728|","-65159|-65159|9739.73|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE|-0.27|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||18/06/2026|55419.07|9740|01-06-2026 to 01-07-2027|POL-PA-Jun-19-1306\\R7|POL-PA-Jun-19-1306\\R7|227.28||64931.52|-55419.24010463667|","-9231|-9231|1379.79|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTI PLANTS LTD &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED &amp;/OR WE FARM LTD|-0.21|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||18/06/2026|7851.04|1380|01-06-2026 to 01-07-2027|POL-FID-Jun-19-1034\\R7|POL-FID-Jun-19-1034\\R7|32.2||9198.63|-7851.184589034789|","-2788|-2788|416.7|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTI PLANTS LTd &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED &amp;/OR WE FARM LTD &amp;/OR CAPITAL AUTOMOBILE LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|||2371.02||01-07-2026 to 01-07-2027|POL-PA-Jun-19-1307\\R7|POL-PA-Jun-19-1307\\R7\\E1|9.72||2778|-2371.2581464422537|Timing Difference","-987|-987|147.6|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTI PLANTS LTD &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED &amp;/OR WE FARM LTD &amp;/OR CAPITAL AUTOMOBILE LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|||839.84||01-07-2026 to 01-07-2027|POL-EL-Jun-19-1239\\R7|POL-EL-Jun-19-1239\\R7\\E1|3.44||984|-839.4657700721057|Timing Difference","-11600|-11600|1719|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTI PLANTS LTD &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED &amp;/OR WE FARM LTD &amp;/OR CAPITAL AUTOMOBILE LTD||0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|||9881.11||01-07-2026 to 01-07-2027|POL-F&amp;A-Jun-19-1327\\R7|POL-F&amp;A-Jun-19-1327\\R7\\E1|140.11||11460|-9881.016300707493|Timing Difference","-81871|-81871|12237.97|15|ALL TO ALL MARKETING LTD  &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR CURPEN CO LTD &amp;/OR WE FARM LTD|-0.03|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||18/06/2026|69634.02|12238|01-06-2026 to 01-07-2027|POL-LOP(F&amp;A)-Jun-19-1080\\R7|POL-LOP(F&amp;A)-Jun-19-1080\\R7|285.55||81586.44|-69633.17798211574|","-97396|-97396|14558.58|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTI PLANTS LTD &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED &amp;/OR WE FARM LTD|-0.42|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||18/06/2026|82838.37|14559|01-06-2026 to 01-07-2027|POL-PPL-Jun-19-1088\\R7|POL-PPL-Jun-19-1088\\R7|339.7||97057.25|-82837.56200291694|","-31021|-31021|4636.95|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTI PLANTS LTD &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED &amp;/OR WE FARM LTD|-0.05|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||18/06/2026|26384.28|4637|01-06-2026 to 01-07-2027|POL-MON-Jun-19-1079\\R7|POL-MON-Jun-19-1079\\R7|108.19||30913.04|-26384.084379632914|","-28682|-28682|4287.15|15|ALL TO ALL MARKETING LTD &amp;/OR HORTIBEL MAURICE LTEE &amp;/OR HORTI PLANTS LTD &amp;/OR CURPEN CO LTD &amp;/OR ARABELLA LIMITED &amp;/OR WE FARM LTD|0.149999999999418|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||18/06/2026|24393.86|4287|01-06-2026 to 01-07-2027|POL-EE+CL-Jun-19-1135\\R7|POL-EE+CL-Jun-19-1135\\R7|100.02||28580.99|-24394.70201781597|","-590|-590|88.2|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|0.2|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||01/06/2026|501.86|88|01-05-2026 to 01-05-2027|POL-EE-May-23-1015\\R3|POL-EE-May-23-1015\\R3|2.06|3601.902454|588|-501.80896857946647|","-2768|-2768|339|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||01/06/2026|2428.91|339|01-05-2026 to 01-05-2027|POL-F&amp;A-May-20-1192\\R6|POL-F&amp;A-May-20-1192\\R6|507.91|3601.902454|2260|-2428.9889772427573|","-587|-587|87.75|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|-0.25|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN||01/06/2026|499.29|88|01-05-2026 to 01-05-2027|POL-M B-D-May-23-1003\\R3|POL-M B-D-May-23-1003\\R3|2.04|3601.902454|585|-499.255979149632|","1|1|399|15|ASSOCIATION SYNDICALE TROPICA BAIE|399.58|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||31/07/2019|2773|-0.580000000000041|01-07-2019 to 01-07-2020|POL-F&amp;A-Jun-19-1353|POL-F&amp;A-Jun-19-1353|509|19391/18/R1|2663|0.8742118537200505|","-5809|-5809|868.35|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|0.35|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||01/06/2026|4940.91|868|01-05-2026 to 01-05-2027|POL-PL-May-20-1184\\R6|POL-PL-May-20-1184\\R6|20.26|3601.902454|5789|-4940.688863986119|","-5727|-5727|781.35|15|PAJELI CO LTD|781.67|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||07/07/2026|4945.88|-0.32000000000005|01-07-2026 to 01-07-2027|POL-PL-Jun-24-24\\R2|POL-PL-Jun-24-24\\R2|518.23|3601 902454|5209|-4945.681378257901|Timing Difference","-208526|-208526|31169.86|15|PAJELI CO LTD|31169.67|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||07/07/2026|177356.51|0.18999999999869|01-07-2026 to 01-07-2027|POL-ARM(P&amp;M)-Jun-24-5\\R2|POL-ARM(P&amp;M)-Jun-24-5\\R2|727.3|3601 902454|207799.07|-177356.19530642574|Timing Difference","-2788|-2788|416.75|15|PAJELI CO LTD|416.49|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||07/07/2026|2371.27|0.259999999999991|01-07-2026 to 01-07-2027|POL-EL-Jun-24-14\\R2|POL-EL-Jun-24-14\\R2|9.72|3601 902454|2778.3|-2371.252989576832|Timing Difference","-22570|-22570|3373.65|15|PAJELI CO LTD|3373.34|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||07/07/2026|19196.07|0.309999999999945|01-07-2026 to 01-07-2027|POL-PA-Jun-24-14\\R2|POL-PA-Jun-24-14\\R2|78.72|3601 902454|22491|-19196.308146490075|Timing Difference","-67592|-67592|10103.38|15|PAJELI CO LTD|10103.82|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||07/07/2026|57488.23|-0.440000000000509|01-07-2026 to 01-07-2027|POL-ARM(P&amp;M)-May-24-2\\R2|POL-ARM(P&amp;M)-May-24-2\\R2|235.75|3601 902454|67355.86|-57488.56170403398|Timing Difference","-67587|-67587|14755.47|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD|4653.23|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||31/08/2020|83958.61|10102.24|01-07-2020 to 01-07-2021|POL-LOP(F&amp;A)-Jul-19-1109\\R1|POL-LOP(F&amp;A)-Jul-19-1109\\R1|344.28|29448/16|98369.8|-57484.30795353611|","-21299|-21299|3376.13|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|192.5|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||31/08/2020|19210.17|3183.63|01-07-2020 to 01-07-2021|POL-EE-Jul-19-1181\\R1|POL-EE-Jul-19-1181\\R1|78.8|29448/16|22507.5|-18115.29160730177|","-52322|-52322|11250|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|3429|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||31/08/2020|64012.5|7821|01-07-2020 to 01-07-2021|POL-PL-Jul-19-1299\\R1|POL-PL-Jul-19-1299\\R1|262.5|29448/16|75000|-44501.07324364723|"]</t>
+  </si>
+  <si>
+    <t>["-8852|-8852|2883.87|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|1560.7|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||31/08/2020|16409.22|1323.17|01-07-2020 to 01-07-2021|POL-EL-Jul-19-1326\\R1|POL-EL-Jul-19-1326\\R1|67.29|29448/16|19225.8|-7528.831070606108|","170383|170383|25569.86|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD|50914.98|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||31/08/2020|145992.53|-25345.12|01-07-2020 to 01-07-2021|POL-F&amp;A-Jul-19-1410\\R1|POL-F&amp;A-Jul-19-1410\\R1|1096.64|29448/16|170465.75|144988.91767006743|","-20323|-20323|6724.8|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|3686.8|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||31/08/2020|38264.12|3038|01-07-2020 to 01-07-2021|POL-PA-Jul-19-1389\\R1|POL-PA-Jul-19-1389\\R1|156.92|29448/16/R4|44832|-17285.182901923406|","-1452|-1452|217.05|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|217.09|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN||19/12/2025|1235.04|-0.039999999999992|01-10-2025 to 01-10-2026|POL-M B-D-Dec-19-1066\\R6|POL-M B-D-Dec-19-1066\\R6|5.06|2595/17|1447.03|-1234.963452678553|","-58|-58|7373.44|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|7314.34|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||03/05/2021|42454.85|59.1000000000004|01-01-2021 to 01-01-2022|POL-F&amp;A-Dec-19-1623\\R1|POL-F&amp;A-Dec-19-1623\\R1|672.04|2595/17/R4 voucher not ok|49156.25|-49.41733501189786|","-987|-987|147.52|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|147.05|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||19/12/2025|839.38|0.469999999999999|01-10-2025 to 01-10-2026|POL-EL-Dec-19-1533\\R6|POL-EL-Dec-19-1533\\R6|3.44|2595/17|983.46|-839.4650521836052|","-17425|-17425|2604.6|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|2604.23|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||19/12/2025|14820.17|0.369999999999891|01-10-2025 to 01-10-2026|POL-PL-Dec-19-1523\\R6|POL-PL-Dec-19-1523\\R6|60.77|2595/17|17364|-14820.365620320958|","-57604|-57604|8535.72|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|8535.44|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||19/12/2025|49068.24|0.280000000000655|01-10-2025 to 01-10-2026|POL-F&amp;A-Dec-19-1623\\R6|POL-F&amp;A-Dec-19-1623\\R6|699.17|2595/17|56904.79|-49068.27407282416|","-2785|-2785|408.75|15|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|-0.25|50||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||27/01/2026|2375.79|409|01-02-2026 to 01-02-2027|POL-MV-Dec-24-1525\\R1|POL-MV-Dec-24-1525\\R1|9.54|31164/22|2725|-2376.18247538193|","-947|-947|786393.6|8|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|786318.01|0||MUR|01/10/2022|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/01/2023|9112335.4|75.589999999851|01-10-2022 to 01-10-2023|POL-HEALTH-Nov-21-120\\R1|POL-HEALTH-Nov-21-120\\R1|68809|MED/2021/00123/R1\nMED/2021/00123/R1/EQ/3\nMED/2021/00123/R1/EQ/4|9829920|-871.7666302209102|","-89390|-89390|13346.85|15|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|-0.15|100||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||01/06/2026|76043.58|13347|01-06-2026 to 01-06-2027|POL-MV-Dec-24-1523\\R1|POL-MV-Dec-24-1523\\R1|311.43|31169/22|88979|-76043.21420313114|","-2266447|-2266447|1031407.49|15|THE GENERAL CONSTRUCTION COMPANY LIMITED|694454.94|36900||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||28/04/2026|5905608.78|336952.55|01-04-2026 to 01-04-2027|POL-MVF-May-19-1121\\R7|POL-MVF-May-19-1121\\R7|24066.37|MT9900043297/R26/9151/18/ 13764/23/ 13092/25|6876049.9|-1929467.76851147|","-84944|-84944|8462.4|8|DESVAUX DE MARIGNY-MONTOCCHIO MARIE PASCALE ANNE MRS|2539.12|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|97717.6|5923.28|01-05-2026 to 01-05-2027|POL-HEALTH-Jul-21-75\\R5|POL-HEALTH-Jul-21-75\\R5|400|MD21M00643/0/R5|105780|-78174.08|","-65884|-65884|11246.4|12|CHEUNG WILLY SOON MR|3374.32|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||27/04/2026|82873.6|7872.08|01-03-2026 to 01-03-2027|POL-HEALTH-Mar-26-26|POL-HEALTH-Mar-26-26|400|MED/2026/00365|93720|-58011.520000000004|","-27715|-27715|4703.04|12|RAMPUTH NEELESH MR|1410.88|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||16/04/2026|34888.96|3292.16|01-03-2026 to 01-03-2027|POL-HEALTH-Apr-26-28|POL-HEALTH-Apr-26-28|400|MED/2026/00315|39192|-24422.80072741968|","-54338|-54338|7197.12|12|BOODIAH MAUREEN VIVIANNA MRS|719.88|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/04/2026|53178.88|6477.24|01-04-2026 to 01-04-2027|POL-HEALTH-Apr-26-32|POL-HEALTH-Apr-26-32|400|MED/2026/00362|59976|-47860.63968199285|","-36325|-36325|8138.25|15|COMPTOIR OUEST OI LTEE|2718.72|100||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||13/05/2026|46406.64|5419.53|01-05-2026 to 01-05-2027|POL-MV-Apr-25-150\\R1|POL-MV-Apr-25-150\\R1|189.89|11301/25|54255|-30905.208498907963|","-62427|-62427|8275.56|12|NOMBRO MARY LYSIE IVY MRS|1654.6|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||04/06/2026|61087.44|6620.96|01-06-2026 to 01-06-2027|POL-HEALTH-Jul-23-49\\R3|POL-HEALTH-Jul-23-49\\R3|400|MED/2023/00781/R3|68963|-54978.96020760348|","-43008|-43008|4165.12|8|PRO WIRE ELECTRICAL &amp; MECHANICAL LTD|757.32|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/06/2026|48398.88|3407.8|01-06-2026 to 01-06-2027|POL-HEALTH-Jul-22-68\\R4|POL-HEALTH-Jul-22-68\\R4|500|MED/2022/00714/R4|52064|-39600.0881028841|","-18666|-18666|2775.13|15|MEDLOG (MAURITIUS) LTD|0.13|0||MUR|24/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||20/05/2026|15890.48|2775|24-04-2026 to 31-07-2026|POL-ARM(P&amp;M)-Jul-21-3\\R4|POL-ARM(P&amp;M)-Jul-21-3\\R4\\E2|164.75|P/10/6D99/21/3262/000/01|18500.86|-15890.812016323067|","-59758|-59758|8902.5|15|SPICE FINANCE LTD ON FINANCIAL LEASE TO G. DE VILLIERS PAINT CONTRACTORS LTD|-0.5|200||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||05/05/2026|50855.23|8903|01-05-2026 to 01-05-2027|POL-MV-Apr-26-119|POL-MV-Apr-26-119|207.73|18193/25|59350|-50855.45977633354|","-89888|-89888|13435.2|12|SAWMYNADEN KISNASAMY POULAY MR|2687.24|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|98924.8|10747.96|01-04-2026 to 01-04-2027|POL-HEALTH-Apr-26-41|POL-HEALTH-Apr-26-41|400|MED/2026/00453|111960|-79139.84|","-33338.5|-33338.5|5286.24|12|HUET LOUISE LILETTE NICOLE|1321.86|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|39165.76|3964.38|01-05-2026 to 01-05-2027|POL-HEALTH-May-26-45|POL-HEALTH-May-26-45|400|MED/2026/00429|44052|-29373.879460091783|","-71848|-71848|10680.48|12|SOORJUN SOTEEHALL MANISHA MRS|2097.77|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||04/06/2026|78723.52|8582.71|01-05-2026 to 01-05-2027|POL-HEALTH-May-26-46|POL-HEALTH-May-26-46|400|MED/2026/00515|89004|-63264.814381459444|","-449|-449|52.21|15|IKO (MAURITIUS) HOTEL LIMITED T/A ANANTARA MAURITIUS RESORTS &amp; VILLAS|0.21|0||MUR|15/05/2026|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||25/06/2026|397.09|52|15-05-2026 to 01-01-2027|POL-FID-Aug-19-1061\\R6|POL-FID-Aug-19-1061\\R6\\E2|101.22|1595/26/N|348.08|-396.82486089472513|","-23536|-23536|3500.34|15|MERIDIS FINANCIAL SOLUTIONS LTD|0.34|0||MUR|04/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY||18/06/2026|20035.27|3500|04-05-2026 to 30-04-2027|POL-F-PI-Jun-26-23|POL-F-PI-Jun-26-23|200|3601.902454 16950/26/N|23335.61|-20035.601997143902|","-513281|-513281|76609.07|15|THE PEAK PANORAMA LTD AND THE SUCCESSIVE OWNERS OF THE BUILDINGS|0.0700000000093132|0||MUR|01/09/2027|MAURITIUS UNION ASSURANCE CO LTD|DEFECTS INSURANCE||25/06/2026|436672.03|76609|01-09-2027 to 01-09-2037|POL-DEF-Jun-26-1005|POL-DEF-Jun-26-1005|2554||510727.1|-436671.9449253635|Timing Difference","-54472|-54472|8112.43|15|COUVE MR REMY ANDRE EDGAR|0.43|0||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|MARINE HULL &amp; TPL||07/07/2026|46359.74|8112|01-07-2026 to 01-07-2027|POL-MH+TPL-Jun-24-26\\R2|POL-MH+TPL-Jun-24-26\\R2|389.29|3601 902454|54082.88|-46359.59531775584|Timing Difference","-23084|-23084|5666.25|15|SBM BANK (MAURITIUS) ON FINANCE LEASE TO MRS LALLJEE CHANDUNNEE|2225.02|100||MUR|01/07/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||03/07/2026|32340.96|3441.23|01-07-2026 to 01-07-2027|POL-MV-Jul-25-300\\R1|POL-MV-Jul-25-300\\R1|132.21|19149/25|37775|-19642.555205709654|Timing Difference","-71896|-71896|5719.68|8|LABELLE-VICTOIRE MARIE CINDY ANABELLE MRS|0|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/07/2026|66176.32|5719.68|01-06-2026 to 01-06-2027|POL-HEALTH-Jun-26-60|POL-HEALTH-Jun-26-60|400|MED/2026/00624|71496|-66176.32|","-93564|-93564|44603.52|8|VISIONWAY LTD|37170.16|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/09/2025|516842.13|7433.36|01-09-2025 to 01-09-2026|POL-HEALTH-Sep-19-3082\\R6|POL-HEALTH-Sep-19-3082\\R6|3901.65|MD16M00704/5/R4|557544|-86130.89628768162|","-75385|-75385|11250.05|15|MR RIVALLAND CHRISTIAN XAVIER|0.05|122.19||MUR|09/02/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||11/05/2026|64134.94|11250|09-02-2026 to 01-05-2027|POL-MV-Feb-26-32|POL-MV-Feb-26-32|262.5|3064/26|75000.3|-64134.94850765385|","-230178.79|-230178.79|22270.08|8|QOVOLTIS LIMITEE|3983.88|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/05/2026|258054.92|18286.2|01-05-2026 to 01-05-2027|POL-HEALTH-Apr-25-44\\R1|POL-HEALTH-Apr-25-44\\R1|1949|MED/2025/00586/R1|278376|-211892.5148993019|","5709|5709|-682.69|12|ACENSI (MAURITIUS) LTD|0.31|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/06/2026|-5026.29|-683|01-05-2026 to 01-06-2026|POL-HEALTH-Jun-25-54|POL-HEALTH-Jun-25-54\\E10|-19.92|MED/2022/00742/R3/EQ/11|-5689.06|5026.307608364366|","-56714|-56714|7529.76|8|FON SING MARIE SANDRA PIT TSOU MRS|3011.6|0||MUR|01/08/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH|Mise en demeure|08/08/2025|86992.24|4518.16|01-08-2025 to 01-08-2026|POL-HEALTH-Sep-24-66\\R1|POL-HEALTH-Sep-24-66\\R1|400|MED/2024/00815/R1|94122|-52196.08027083642|","-30957|-30957|12352.4|8|GAYA SHYAMSUNDUR MR|12352.8|0||MUR|01/08/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/10/2025|142452.6|-0.400000000003274|01-08-2025 to 01-08-2026|POL-HEALTH-Aug-23-80\\R2|POL-HEALTH-Aug-23-80\\R2|400|MD08M01060/13/R4|154405|-28486.839173153323|","-19156|-19156|5061.6|12|COLLET-SERRET MARINE CELIA MRS|2784.08|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/01/2026|37518.4|2277.52|01-10-2025 to 01-10-2026|POL-HEALTH-Jul-25-88|POL-HEALTH-Jul-25-88|400|MED/2025/01440|42180|-16878.874363550964|","-15864|-15864|6314.24|8|SALEMOHAMED FAWZIA|5683.2|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||09/10/2025|73013.76|631.039999999999|01-10-2025 to 01-10-2026|POL-HEALTH-Sep-19-3130\\R6|POL-HEALTH-Sep-19-3130\\R6|400|MD06M00609/15/R4|78928|-14601.279354578459|","-23412|-23412|9316.8|12|BUCARD JOSEPHE MARIE CLAUDE MRS|7453.24|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/11/2025|68723.2|1863.56|01-09-2025 to 01-09-2026|POL-HEALTH-Sep-25-102|POL-HEALTH-Sep-25-102|400|FQ/2025/01444|77640|-20616.96|","-21473|-21473|5685.76|8|BENZOU LTD|4548.24|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/11/2025|65886.24|1137.52|01-11-2025 to 01-11-2026|POL-HEALTH-Oct-19-3194\\R6|POL-HEALTH-Oct-19-3194\\R6|500|MD18M01126/2/R5|71072|-19767.160782428884|","-58750.35|-58750.35|14063.84|8|VETOPHARMA LTD|9374.3|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/01/2026|162134.16|4689.54|01-11-2025 to 01-11-2026|POL-HEALTH-Nov-24-125\\R1|POL-HEALTH-Nov-24-125\\R1|400|MED/2024/01200/R1|175798|-54060.9918782052|","-51348|-51348|13660.8|8|RIVAUD MARIE JOSEE MRS|9562.36|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||03/12/2025|157499.2|4098.44|01-12-2025 to 01-12-2026|POL-HEALTH-Nov-23-131\\R2|POL-HEALTH-Nov-23-131\\R2|400|MED/2023/01267/R2|170760|-47249.76|","-35320|-35320|21142.08|12|CARR-BROWN ALAN|19027.52|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/12/2025|155441.92|2114.56|01-10-2025 to 01-10-2026|POL-HEALTH-Nov-25-149|POL-HEALTH-Nov-25-149|400|MED/2025/01409|176184|-31091.20086984098|","-1429694|-1429694|227140.8|8|COMPAGNIE MAURICIENNE DE TEXTILE LTEE|151420.28|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||23/12/2025|2631994.02|75720.5199999999|01-12-2025 to 01-12-2026|POL-HEALTH-May-19-2565\\R47|POL-HEALTH-May-19-2565\\R47|19874.82|MD16M00967/4/R5|2839260|-1316113.5431976167|","-51638|-51638|4099.04|8|BUSSIER ROBERT EMMANUEL MARIE ANGELO|0.04|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH|Mise en demeure|15/01/2026|47538.96|4099|01-01-2026 to 01-01-2027|POL-HEALTH-Mar-21-13\\R5|POL-HEALTH-Mar-21-13\\R5|400|MD21M00507/0/R5|51238|-47538.96|","-56545|-56545|9015.2|8|VALAYDON-JOSEPHINE RUBBY PAMELA MRS|5409.32|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/01/2026|104074.8|3605.88|01-01-2026 to 01-01-2027|POL-HEALTH-Dec-19-3277\\R6|POL-HEALTH-Dec-19-3277\\R6|400|MD18M00171/3/R5|112690|-52037.4|","-3166408|-3166408|471641.63|15|COMPAGNIE D'EXPLOITATION AGRICOLE LTEE|-0.37|11125||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||21/01/2026|2694765.92|471642|01-01-2026 to 01-01-2027|POL-MVF-Jun-19-1892\\R7|POL-MVF-Jun-19-1892\\R7|11005.05|MT200001000114/R26|3144277.5|-2694766.3029717575|","-2158923|-2158923|320037|15|REY &amp; LENFERNA LTD|0|17875||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||05/02/2026|1838885.58|320037|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1059\\R4|POL-MVF-Dec-21-1059\\R4|7467.58|25114/21/R4|2133580|-1838885.9377395276|","-151740|-151740|28900.5|15|WATERTECH LIMITED|6421.8|1750||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||20/02/2026|166193.86|22478.7|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1066\\R4|POL-MVF-Dec-21-1066\\R4|674.36|26138/21/R4|192670|-129261.84189230278|","-104108|-104108|103281.9|15|MEDITERRANEAN SHIPPING CO (MAURITIUS) LTD|95522.99|1400||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||30/01/2026|589074.02|7758.91|01-01-2026 to 01-01-2027|POL-MVF-Aug-19-6120\\R7|POL-MVF-Aug-19-6120\\R7|2409.92|56113/11/R15\n14598/21/R5\n25811/10/R15|688546|-88577.73336315229|","-67173|-67173|10715.44|8|RAJKOMAR VIMLA MRS|5358.04|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||05/02/2026|123627.56|5357.4|01-02-2026 to 01-02-2027|POL-HEALTH-Apr-24-18\\R2|POL-HEALTH-Apr-24-18\\R2|400|FD10M00005/11/R5|133943|-61815.160357294386|"]</t>
+  </si>
+  <si>
+    <t>["-30051|-30051|4776.08|8|SOOPRAMANIEN POTHEGADOO KAVINA MRS|2388.08|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||09/02/2026|55324.92|2388|01-02-2026 to 01-02-2027|POL-HEALTH-Feb-25-17\\R1|POL-HEALTH-Feb-25-17\\R1|400|MED/2025/00230/R1|59701|-27662.920266218534|","-1651|-1651|23944.66|15|SYNDICAT DES COPROPRIETAIRES LES VUES D'ANBALABA &amp;/OR ASSOCIATION FONCIÈRE EST “ANBALABA” (AFE ANBALABA)|23697.79|0||MUR|29/12/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||30/01/2026|136395.09|246.870000000003|29-12-2025 to 01-01-2027|POL-F&amp;A-Jan-26-1001|POL-F&amp;A-Jan-26-1001|708.71|712/26/N|159631.04|-1404.444584639804|","-427759|-427759|62081.28|8|PREVOIR SOLUTIONS INFORMATIQUES LTD|28216.43|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/02/2026|722082.91|33864.85|01-02-2026 to 01-02-2027|POL-HEALTH-Feb-23-11\\R3|POL-HEALTH-Feb-23-11\\R3|8148.19|MED/2023/00358/R3|776016|-393893.86487884633|","-5888|-5888|850.2|15|SKYDIVE AUSTRAL LIMITED|0.2|200||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||05/02/2026|5037.64|850|01-02-2026 to 01-02-2027|POL-MV-May-19-2761\\R7|POL-MV-May-19-2761\\R7|19.84|1249/26|5668|-5037.776896111307|","-28889|-28889|4318.2|15|CURRIMJEE GROUP|0.2|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|DIRECTORS &amp; OFFICERS LIABILITY||11/02/2026|24570.56|4318|01-01-2026 to 31-12-2026|POL-D&amp;O-Jan-22-1\\R5|POL-D&amp;O-Jan-22-1\\R5\\E2|100.76|INTERNAL PLACING SLIP|28788|-24570.764125563022|","-1033997|-1033997|257213.25|15|AIKO RESIDENCE LTD &amp;/OR MNJ PROPERTIES LTD &amp;/OR SUBSEQUENT OWNERS|102885.52|0||MUR|21/01/2028|MAURITIUS UNION ASSURANCE CO LTD|DEFECTS INSURANCE||19/02/2026|1466114.75|154327.73|21-01-2028 to 20-01-2038|POL-DEF-Jan-26-1001|POL-DEF-Jan-26-1001|8573||1714755|-879669.0201492403|Timing Difference"]</t>
+  </si>
+  <si>
+    <t>["-12738|-12738|11340.67|15|SYNDICAT DES COPROPRIETAIRES DE L’IMMEUBLE RESIDENCE ST CLEMENT COURT|9440.05|0||MUR|01/01/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|Mise en demeure|20/02/2025|64678.41|1900.62|01-01-2025 to 01-01-2026|POL-F&amp;A-Jul-19-1426\\R6|POL-F&amp;A-Jul-19-1426\\R6|414.61|13617/08/R15|75604.47|-10837.721090284176|","-36765|-36765|11907.68|15|SYNDICAT DES COPROPRIETAIRES DE L’IMMEUBLE RESIDENCE ST CLEMENT COURT|10737.15|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|Mise en demeure|25/02/2026|67904.7|1170.53|01-01-2026 to 01-01-2027|POL-F&amp;A-Jul-19-1426\\R7|POL-F&amp;A-Jul-19-1426\\R7|427.85|13617/08/R17|79384.53|-31279.812674424695|","-14657|-14657|2161.05|15|DUCHENNE LOIC DAMIEN MR|0.050000000000291|0||MUR|09/01/2025|MAURITIUS UNION ASSURANCE CO LTD|MARINE HULL &amp; TPL|Mise en demeure|30/01/2025|12496.41|2161|09-01-2025 to 01-02-2026|POL-MH+TPL-Jan-25-1002|POL-MH+TPL-Jan-25-1002|250.43|996/25/N|14407.03|-12496.01782095943|","9104|9104|-1375.72|15|DUCHENNE LOIC DAMIEN MR|0.28|0||MUR|30/05/2025|MAURITIUS UNION ASSURANCE CO LTD|MARINE HULL &amp; TPL|Mise en demeure|19/02/2026|-7727.88|-1376|30-05-2025 to 01-02-2026|POL-MH+TPL-Jan-25-1002|POL-MH+TPL-Jan-25-1002\\E1|67.89|996/25/N/E1 \nA/C No : 3601.902454|-9171.49|7728.219552704425|","-2926|-2926|33870.72|8|KASA TEXTILE &amp; CO LTD|33638.02|0||MUR|01/03/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/05/2025|392476.97|232.700000000004|01-03-2025 to 01-03-2026|POL-HEALTH-Jun-19-2719\\R48|POL-HEALTH-Jun-19-2719\\R48|2963.69|MED/2024/00392/R1\nMD08M01085/13/R4|423384|-2693.547170901759|","-68923|-68923|23068.5|15|KASA TEXTILE &amp; CO LTD|12815.38|750||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||20/02/2026|132009.77|10253.12|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1067\\R4|POL-MVF-Dec-21-1067\\R4|538.27|26063/21/R4|153790|-58670.43382486792|","-314174|-314174|37719.36|8|KASA TEXTILE &amp; CO LTD|12760.49|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/05/2026|437072.64|24958.87|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2719\\R49|POL-HEALTH-Jun-19-2719\\R49|3300|MD08M01085/13/R5|471492|-289214.7710984178|","-13131|-13131|1050.48|8|KASA TEXTILE &amp; CO LTD|0.48|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/06/2026|12080.52|1050|01-06-2026 to 01-03-2027|POL-HEALTH-Jun-19-2719\\R49|POL-HEALTH-Jun-19-2719\\R49\\E1|0|MD08M01085/13/R5/EQ/2|13131|-12080.52|","-385|-385|3565.85|15|TARTUFFE LTEE|3509.4|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|Mise en demeure|09/09/2025|20789.69|56.4499999999998|01-07-2025 to 01-07-2026|POL-F&amp;A-Jun-19-1359\\R6|POL-F&amp;A-Jun-19-1359\\R6|583.21|25773/16|23772.33|-328.6328551943418|","1131|1131|-169.04|15|TARTUFFE LTEE|-0.04|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY|Mise en demeure|15/05/2026|-961.85|-169|01-04-2026 to 01-07-2026|POL-PPL-Jun-19-1092\\R6|POL-PPL-Jun-19-1092\\R6\\E2|-3.94|25773/16/R9/E2|-1126.95|961.9435577288684|","1673|1673|-250.01|15|TARTUFFE LTEE|-0.01|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)|Mise en demeure|15/05/2026|-1422.57|-250|01-04-2026 to 01-07-2026|POL-LOP(F&amp;A)-Jun-19-1088\\R6|POL-LOP(F&amp;A)-Jun-19-1088\\R6\\E2|-5.83|25773/16/R9/E2|-1666.75|1422.92722022265|","5448|5448|-889.02|15|TARTUFFE LTEE|-0.02|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS|Mise en demeure|15/05/2026|-4558.53|-889|01-04-2026 to 01-07-2026|POL-F&amp;A-Jun-19-1359\\R6|POL-F&amp;A-Jun-19-1359\\R6\\E2|479.26|25773/16/R9/E2|-5926.81|4558.906561665336|","-4917|-4917|735|15|TARTUFFE LTEE|0|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|Mise en demeure|09/09/2025|4182.15|735|01-07-2025 to 01-07-2026|POL-PA-Jun-19-1329\\R6|POL-PA-Jun-19-1329\\R6|17.15|25773/16|4900|-4182.0224215246635|","-6709|-6709|1002.8|15|TARTUFFE LTEE|-0.2|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)|Mise en demeure|09/09/2025|5705.9|1003|01-07-2025 to 01-07-2026|POL-LOP(F&amp;A)-Jun-19-1088\\R6|POL-LOP(F&amp;A)-Jun-19-1088\\R6|23.4|25773/16|6685.3|-5706.155156736775|","1564|1564|-233.78|15|TARTUFFE LTEE|0.22|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|Mise en demeure|15/05/2026|-1330.18|-234|01-04-2026 to 01-07-2026|POL-EL-Jun-19-1268\\R6|POL-EL-Jun-19-1268\\R6\\E2|-5.45|25773/16/R9/E2|-1558.51|1330.2140208189467|","-6273|-6273|937.67|15|TARTUFFE LTEE|-0.33|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY|Mise en demeure|09/09/2025|5335.37|938|01-07-2025 to 01-07-2026|POL-EL-Jun-19-1268\\R6|POL-EL-Jun-19-1268\\R6|21.88|25773/16|6251.16|-5335.335979046842|","-4536|-4536|678.03|15|TARTUFFE LTEE|0.03|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY|Mise en demeure|09/09/2025|3857.99|678|01-07-2025 to 01-07-2026|POL-PPL-Jun-19-1092\\R6|POL-PPL-Jun-19-1092\\R6|15.82|25773/16|4520.2|-3857.972989537083|","1226|1226|-183.25|15|TARTUFFE LTEE|-0.25|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT|Mise en demeure|15/05/2026|-1042.67|-183|01-04-2026 to 01-07-2026|POL-PA-Jun-19-1329\\R6|POL-PA-Jun-19-1329\\R6\\E2|-4.28|25773/16/R9/E2|-1221.64|1042.7380416340382|","-85498|-85498|12750|15|ERC LEVAGE LTEE|0|0||MUR|30/01/2026|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||17/06/2026|72747.5|12750|30-01-2026 to 30-01-2026|POL-GIT-Jan-26-1|POL-GIT-Jan-26-1|497.5|2217/26/N|85000|-72747.92543641626|","-20270|-20270|3000|15|ERC LEVAGE LTEE|0|0||MUR|17/06/2025|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||31/07/2025|17270|3000|17-06-2025 to 17-06-2025|POL-GIT-Jun-25-5|POL-GIT-Jun-25-5|270|20990/25/N|20000|-17270|","-9881440|-9881440|2222028.75|15|ROYAL CAR RENTAL LTD|891753.83|31400||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||30/01/2026|12674744.08|1330274.92|01-01-2026 to 01-01-2027|POL-MVF-Jul-19-6113\\R7|POL-MVF-Jul-19-6113\\R7|51847.8299999998|31069/23 / 31162/23 / 31191/23|14813525|-8407507.087014845|","40842|40842|-6064.8|15|ROYAL CAR RENTAL LTD|0.2|-268||MUR|25/06/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/01/2026|-34776.72|-6065|25-06-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E43|-141.52|31162/23/R1/E35|-40432|34777.128721947665|","7452|7452|-1113.86|15|ROYAL CAR RENTAL LTD|0.140000000000146|0||MUR|26/08/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/01/2026|-6337.88|-1114|26-08-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E34|-25.99|31162/23/R1/E25|-7425.75|6338.101136110492|","-10111|-10111|1502.72|15|ROYAL CAR RENTAL LTD|-0.28|57.53||MUR|27/11/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||27/11/2025|8608.01|1503|27-11-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E47|35.06|31069/23/R1/E10|10018.14|-8608.23987090942|","-779717|-779717|116549.62|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.38|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||28/05/2026|663167.34|116550|01-05-2026 to 01-05-2027|POL-ARMISC-May-19-1048\\R7|POL-ARMISC-May-19-1048\\R7|2719.49||776997.47|-663167.3740209268|","-3485|-3485|520.93|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.0700000000000728|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||28/05/2026|2964.09|521|01-05-2026 to 01-05-2027|POL-MON-Apr-20-1058\\R6|POL-MON-Apr-20-1058\\R6|12.15||3472.87|-2964.07298953808|","-429|-429|825|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|762.01|0|Correction to be done by CBL amount not in aging|MUR|01/11/2018|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||4794|62.99|01-11-2018 to 01-11-2019|POL-CAR-TPL-May-19-1036|POL-CAR-TPL-May-19-1036|119|17636/16/N|5500|-366.01281366791244|","-95011|-95011|14202|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR PRINCIPALS &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||28/05/2026|80809.38|14202|01-05-2026 to 01-05-2027|POL-CAR-TPL(BC)-May-25-4\\R1|POL-CAR-TPL(BC)-May-25-4\\R1|331.38||94680|-80809.05680119581|","-7350|-7350|1098.64|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.359999999999854|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||28/05/2026|6251.25|1099|01-05-2026 to 01-05-2027|POL-EE-Apr-20-1086\\R6|POL-EE-Apr-20-1086\\R6|25.64||7324.25|-6251.343557522629|","-906872|-906872|135556.38|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR FASTMIX  CO LTD|0.38|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||28/05/2026|771315.81|135556|01-05-2026 to 01-05-2027|POL-ARM(P&amp;M)-Feb-20-1010\\R7|POL-ARM(P&amp;M)-Feb-20-1010\\R7|3163.01||903709.18|-771315.6484005976|","-107514|-107514|16070.81|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR FASTMIX CO LTD|-0.19|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||28/05/2026|91442.88|16071|01-05-2026 to 01-05-2027|POL-EL-Apr-20-1161\\R6|POL-EL-Apr-20-1161\\R6|374.98|9314/08/R18|107138.71|-91443.14366216991|","-92643|-92643|13848|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR FAST MIX CO LTD|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/05/2026|78795.12|13848|01-05-2026 to 01-05-2027|POL-PA-Apr-20-1154\\R6|POL-PA-Apr-20-1154\\R6|323.12||92320|-78795.01793721973|","-112057|-112057|16675.17|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR SOCIETE FOUR TWELVE &amp;/ORDISTRI-T TRADING LTD|0.169999999997672|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||28/05/2026|95381.69|16675|01-05-2026 to 01-05-2027|POL-F&amp;A-Apr-20-1182\\R6|POL-F&amp;A-Apr-20-1182\\R6|889.09|9314/08/R18|111167.77|-95381.80916661417|","-276484|-276484|41328|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/05/2026|235156.32|41328|01-05-2026 to 01-05-2027|POL-PA-Apr-20-1155\\R6|POL-PA-Apr-20-1155\\R6|964.32||275520|-235156.04783258596|","-117828|-117828|17612.55|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.45|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/05/2026|100215.41|17613|01-05-2026 to 01-05-2027|POL-PA-Apr-20-1153\\R6|POL-PA-Apr-20-1153\\R6|410.96||117417|-100215.44402092678|","-5808|-5808|868.2|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR SOCIETE FOUR TWELVE &amp;/ORDISTRI-T TRADING LTD &amp;/OR FASTMIX CO LTD|0.2|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||28/05/2026|4940.06|868|01-05-2026 to 01-05-2027|POL-PL-Apr-20-1178\\R6|POL-PL-Apr-20-1178\\R6|20.26|9314/08/R18|5788|-4939.838863962701|","1028|1028|-168.63|15|LAVASTONE LTD &amp;/OR SUBSIDIARIES &amp;/OR AFFILIATED COMPANIES|0.37|0||MUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||10/10/2025|-859.48|-169|01-10-2024 to 30-09-2025|POL-EL-Oct-19-1469\\R5|POL-EL-Oct-19-1469\\R5\\E1|96.07|33502/19/R5/E1|-1124.18|859.3880421355692|","5077|5077|-758.83|15|LAVASTONE LTD &amp;/OR SUBSIDIARIES &amp;/OR AFFILIATED COMPANIES|0.17|0||MUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||13/10/2025|-4317.73|-759|01-10-2024 to 30-09-2025|POL-PA-Oct-19-1546\\R5|POL-PA-Oct-19-1546\\R5\\E1|-17.71|33502/19/R5/E1|-5058.85|4318.104230029784|","-16533|-16533|1983.95|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.05|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|14548.96|1984|01-11-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E25|0|MED/2025/01055/EQ/55|16532.91|-14549.039199995645|","-25782|-25782|3093.89|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.11|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|22688.55|3094|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E41|0|MED/2025/01055/EQ/96|25782.44|-22688.162799952217|","7844|7844|-941.33|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.33|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|-6903.12|-941|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E40|0|MED/2025/01055/EQ/94|-7844.45|6902.723999770538|","-6277|-6277|753.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|5523.89|753|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E51|0|MED/2025/01055/EQ/112|6277.15|-5523.758000047792|","-1836|-1836|220.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||05/06/2026|1615.25|220|01-06-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E54|0|MED/2025/01055/EQ/118|1835.51|-1615.681200320347|","-6277|-6277|753.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||05/06/2026|5523.89|753|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E53|0|MED/2025/01055/EQ/114|6277.15|-5523.758000047792|","-13731|-13731|1647.68|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.32|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|12082.95|1648|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E28|0|MED/2025/01055/EQ/64|13730.63|-12083.275599881434|","3119|3119|-374.24|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.24|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/05/2026|-2744.44|-374|01-06-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E52|0|MED/2025/01055/EQ/113|-3118.68|2744.721600164172|","-11074|-11074|1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|9745.31|1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E29|0|MED/2025/01055/EQ/56|11074.22|-9745.116400071518|","-18355|-18355|2202.61|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.39|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|16152.45|2203|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E36|0|MED/2025/01055/EQ/74|18355.06|-16152.397200009153|","-7464|-7464|895.73|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.27|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|6568.66|896|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E43|0|MED/2025/01055/EQ/95|7464.39|-6568.316800167194|","-139140|-139140|16696.8|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.2|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||27/02/2026|122443.2|16697|01-07-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E19|0|MED/2025/01055/EQ/84|139140|-122443.2|","-7274|-7274|872.88|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.12|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|6401.09|873|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E35|0|MED/2025/01055/EQ/81|7273.97|-6401.116399985152|"]</t>
+  </si>
+  <si>
+    <t>["-12763.8|85840|Syndicat des Coproprietaires de L`Immeuble Residence St Clement Court|01/04/2026|31079.96||02/01/26 to 31/12/26||13617/08/R17||31079.96|22/01/2026|JRNI.260122.442|Non-Motor Corporate","-9204|1475.8|DUCHENNE Loic Damien|27/01/2026|||09/01/25 to 31/01/26||996/25/N/E1||-7828.2|27/01/2026|JRNI.260127.81|Yacht Hull/Tpl","-23068.5|155078|Kasa Textile &amp; Co Ltd|01/04/2026|73338.2|Payment done after 30.06.2026|01/01/26 to 31/12/26||26063/21/R4||73338.2|06/01/2026|JRNI.260106.450|Motor","-3143.28|39291|Kasa Textile &amp; Co Ltd|01/07/2026|20749.66||01/03/26 to 28/02/27|MD08M01085|MD08M01085/R18|MD08M01085|20749.66|31/05/2026|JRNNHZ.260531.65|Medical","-3260|40750|Kasa Textile &amp; Co Ltd|01/08/2026|||01/03/26 to 28/02/27|MD08M01085|MD08M01085/R18|MD08M01085|37490|30/06/2026|JRNNHZ.260630.468|Medical","-6919.33|46789.96|Tartuffe Ltee|01/10/2025|19409.18||01/07/25 to 30/06/26||25773/16/R9||19409.18|28/07/2025|JRNI.250728.434|Non-Motor Corporate","-11540.96|1825.13|Tartuffe Ltee|28/04/2026|100||01/07/25 to 30/06/26||25773/16/R9/E2||-9715.83|17/04/2026|JRNI.260417.279|Non-Motor Corporate","-6750|45358|ERC Levage Ltee|12/06/2026|38608|Payment done after 30.06.2026|11/05/26 to 11/05/26|POL-GIT-May-26-18|11642/26/N|POL-GIT-May-26-18|38608|12/05/2026|JRNI.260512.238|Inland Transit","-1024.8|7156|Royal Car Rental Ltd|01/02/2026|6131.2||17/10/25 to 31/10/26||32587/25/N||6131.2|20/11/2025|JRNI.251120.318|Non-Motor Corporate","-1292958.7|8666994|Royal Car Rental Ltd|15/10/2026|2938487.62||01/01/26 to 31/12/26||31162/23/R2||5167497.43|06/01/2026|JRNI.260106.423|Motor","-5260.05|35290|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/09/2026|||01/05/25 to 30/04/26||9314/08/R17/E2||30029.95|29/06/2026|JRNI.260629.452|Non-Motor Corporate","-2730.9|18570|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/08/2026|||01/05/26 to 30/04/27||22405/20/R6||15839.1|13/05/2026|JRNI.260513.103|Non-Motor Corporate","-374330.06|2504767.95|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/08/2026|||01/05/26 to 30/04/27||9314/08/R18||2130437.89|25/05/2026|JRNI.260525.474|Non-Motor Corporate","-22567.5|151477|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/06/2026|128909.5||11/07/25 to 11/09/26||7049/26/N||128909.5|26/03/2026|JRNI.260326.415|Non-Motor Corporate","-37642|5726.65|Lavastone Ltd &amp;/or Subsidiaries|09/01/2026|100||01/10/25 to 30/09/26||33502/19/R6/E1||-31915.35|08/01/2026|JRNI.260108.274|Non-Motor Corporate","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.38|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.37|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.36|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|3327.96||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|3327.96|10/03/2026|JRNNHZ.260310.35|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.252|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.251|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|57.63||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|57.63|25/06/2026|JRNNHZ.260625.250|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|10/03/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.248|Medical","-68.64|572.05|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/03/2026|75.26||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E78|MED/2025/01055|75.26|19/02/2026|JRNNHZ.260219.82|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/03/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.61|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.60|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.59|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|1624.17||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.17|19/02/2026|JRNNHZ.260219.58|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.57|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/10/2025|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.56|Medical","-367.1|3059.17|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|2692.07||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E74|MED/2025/01055|2692.07|19/02/2026|JRNNHZ.260219.37|Medical","-3396.48|28304|HARDY HENRY &amp; CIE LTEE|01/08/2026||Payment done after 30.06.2026|01/10/25 to 30/06/26|MED/2023/01269|MED/2023/01269/R2|MED/2023/01269|24907.52|30/06/2026|JRNNHZ.260630.789|Medical","-62149.68|517914|Hardy Henry Services Ltd|01/08/2026|||01/10/25 to 30/06/26|MD18M01064|MD18M01064/R7|MD18M01064|455764.32|30/06/2026|JRNNHZ.260630.599|Medical","-1014.36|8453|HARDY HENRY &amp; CIE LTEE|01/08/2026|||01/10/25 to 30/06/26|MD18M01063|MD18M01063/R7|MD18M01063|7438.64|30/06/2026|JRNNHZ.260630.598|Medical","-17714.88|147624|HARDY HENRY MANAGEMENT LTD|01/08/2026|||01/10/25 to 30/06/26|MD18M01062|MD18M01062/R7|MD18M01062|129909.12|30/06/2026|JRNNHZ.260630.597|Medical","-5604.96|46708|HARDY HENRY TEXTILES LTEE|01/08/2026|||01/10/25 to 30/06/26|MD18M01051|MD18M01051/R7|MD18M01051|41103.04|30/06/2026|JRNNHZ.260630.595|Medical","-195.99|1636|HARDY HENRY TEXTILES LTEE|01/08/2026|||01/10/25 to 30/06/26|MD04M00390|MD04M00390/R22|MD04M00390|1440.01|30/06/2026|JRNNHZ.260630.456|Medical","-3835.92|31966|Hardy Henry Services Ltd|01/08/2026|||01/10/25 to 30/06/26|MD02M00616|MD02M00616/R24|MD02M00616|28130.08|30/06/2026|JRNNHZ.260630.450|Medical","-3396.48|28304|HARDY HENRY &amp; CIE LTEE|01/07/2026|17476.02|Payment done after 30.06.2026|01/10/25 to 30/06/26|MED/2023/01269|MED/2023/01269/R2|MED/2023/01269|17476.02|31/05/2026|JRNNHZ.260531.397|Medical","-63366.36|528053|Hardy Henry Services Ltd|01/07/2026|418832.06||01/10/25 to 30/06/26|MD18M01064|MD18M01064/R7|MD18M01064|418832.06|31/05/2026|JRNNHZ.260531.197|Medical","-17714.88|147624|HARDY HENRY MANAGEMENT LTD|01/07/2026|76436.11||01/10/25 to 30/06/26|MD18M01062|MD18M01062/R7|MD18M01062|76436.11|31/05/2026|JRNNHZ.260531.195|Medical","-5604.96|46708|HARDY HENRY TEXTILES LTEE|01/07/2026|41103.04||01/10/25 to 30/06/26|MD18M01051|MD18M01051/R7|MD18M01051|41103.04|31/05/2026|JRNNHZ.260531.193|Medical","-3835.92|31966|Hardy Henry Services Ltd|01/07/2026|28130.08||01/10/25 to 30/06/26|MD02M00616|MD02M00616/R24|MD02M00616|28130.08|31/05/2026|JRNNHZ.260531.47|Medical","-86931.38|582070.94|H.VAULBERT DE CHANTILLY LTD (HVC LTD)|01/04/2026|495139.56||01/01/26 to 31/12/26||2321/20/R6||495139.56|30/01/2026|JRNI.260130.518|Non-Motor Corporate","-22324.99|1785.99|ORANGE EIGHT LTD ORANGE EIGHT LTD|31/03/2026|||01/10/25 to 30/09/26|MED/2022/01410|MED/2022/01410/R3/E7|MED/2022/01410|-20539|02/06/2026|JRNNHZ.260602.5|Medical","-45701.76|575270.9|ORANGE EIGHT LTD ORANGE EIGHT LTD|31/03/2026|217638.96||01/10/25 to 30/09/26|MED/2022/01410|MED/2022/01410/R3|MED/2022/01410|217638.96|28/11/2025|JRNNHZ.251128.28|Medical","-3865.35|26359|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/04/2026|22493.65||01/02/26 to 31/01/27||6162/25/R2||22493.65|28/01/2026|JRNI.260128.450|Non-Motor Corporate","-750|5118|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/08/2026|||16/11/25 to 15/06/26||36726/25/N/E2||4368|13/05/2026|JRNI.260513.284|Car/Ear (One Off)","-74398.8|498228|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/03/2026|278436.63||01/12/25 to 30/11/26||46037/12/R13||278436.63|30/12/2025|JRNI.251230.598|Non-Motor Corporate","-900|6121|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/09/2026|||16/11/25 to 15/08/26||36731/25/N/E3||5221|29/06/2026|JRNI.260629.604|Non-Motor Corporate","-450|3111|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/07/2026|2661||16/11/25 to 15/05/26||36731/25/N/E1||2661|23/04/2026|JRNI.260423.350|Non-Motor Corporate","-2756.85|18543|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/02/2026|9278.51||16/10/23 to 15/10/26||27489/23/N/E2||9278.51|28/11/2025|JRNI.251128.356|Car/Ear (One Off)","-18900|126630|Golden Fund Management Services Ltd &amp;/or The Mauritius Development Investment Trust Co Ltd|01/08/2026||Payment done after 30.06.2026|01/05/26 to 30/04/27|POL-C+PI-Jun-19-1003\\R7|15398/18/R8|POL-C+PI-Jun-19-1003\\R7|107730|28/05/2026|JRNI.260528.571|Financial","-7735.12|97089|Paris Onezime Marie Stephanie|02/03/2026|43569.57||01/01/26 to 31/12/26|MED/2023/00006|MED/2023/00006/R3|MED/2023/00006|43569.57|29/12/2025|JRNNHZ.251229.18|Medical","-2299.8|28747.56|Paris Onezime Marie Stephanie|02/03/2026|4969.88||01/01/26 to 31/12/26|MED/2023/00006|MED/2023/00006/R3/E1|MED/2023/00006|4969.88|22/05/2026|JRNNHZ.260522.141|Medical","-20182.35|135220|Hefty Ltd|01/06/2026|115037.65||01/04/26 to 31/03/27||6400/26/N||115037.65|20/03/2026|JRNI.260320.119|Motor","-8891.25|59582|Hefty Ltd|01/06/2026|50690.75||01/04/26 to 31/03/27||6368/26/N||50690.75|20/03/2026|JRNI.260320.18|Motor","-27536.85|184322|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/05/26||12718/24/N/E5||156785.15|30/06/2026|JRNI.260630.570|Car/Ear (One Off)","-18000|120520|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/05/26||12718/24/N/E4||102520|30/06/2026|JRNI.260630.548|Car/Ear (One Off)","-108000|722620|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/08/26||12718/24/N/E7||614620|30/06/2026|JRNI.260630.605|Car/Ear (One Off)","-20045.25|134266|Rehm Grinaker Construction Co. Ltd|01/06/2026|114220.75||01/01/26 to 31/12/26||10936/21/R4/E2||114220.75|09/03/2026|JRNI.260309.20|Motor","-44294.4|557555.76|CREDIT GUARANTEE INSURANCE CO LTD|02/03/2026|238039.16||01/01/26 to 31/12/26|MD11M00167|MD11M00167/R15|MD11M00167|238039.16|14/01/2026|JRNNHZ.260114.222|Medical","-589.95|3947|Impact Production Ltd &amp;/or Event Strategy Ltd &amp;/or Mille Feux Ltd &amp;/or Marquee Design Ltd|01/09/2026|||01/04/26 to 31/03/27||8040/21/R5/E1||3357.05|04/06/2026|JRNI.260604.342|Non-Motor Corporate","-68411.52|458172.96|Impact Production Ltd &amp;/or Event Strategy Ltd &amp;/or Mille Feux Ltd &amp;/or Marquee Design Ltd|01/07/2026|389761.44||01/04/26 to 31/03/27||8040/21/R5||389761.44|30/04/2026|JRNI.260430.631|Non-Motor Corporate","-7372.5|49772|IMPACT PRODUCTION LTD|01/04/2026|42399.5||01/01/26 to 31/12/26||54552/15/R10||42399.5|06/01/2026|JRNI.260106.400|Motor","-6255.68|78196|KASA CORPORATE SERVICES LTD|01/07/2026|71940.32||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|71940.32|31/05/2026|JRNNHZ.260531.63|Medical","-13161.28|171425.68|KASA CORPORATE SERVICES LTD|01/06/2026|158264.4||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|158264.4|30/04/2026|JRNNHZ.260430.476|Medical","-76806|514632|KASA CORPORATE SERVICES LTD|01/04/2026|243234.45|Payment done after 30.06.2026|01/01/26 to 31/12/26||32859/23/R2||243234.45|06/01/2026|JRNI.260106.408|Motor","-3986.32|49829|KASA CORPORATE SERVICES LTD|01/08/2026|||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|45842.68|30/06/2026|JRNNHZ.260630.466|Medical","-121776.21|815182.95|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|01/07/2026|462223.22||01/03/26 to 28/02/27||8187/26/N||462223.22|07/04/2026|JRNI.260407.284|Non-Motor Corporate","-57631|8614.5|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|18/05/2026|||01/12/25 to 30/11/26||29742/23/R2/E1||-49016.5|18/05/2026|JRNI.260518.268|Motor","-38187|255971|CURRIMJEE JEEWANJEE AND COMPANY LIMITED|01/04/2026|27828.27|Payment done after 30.06.2026|01/01/26 to 31/12/26||1915/26/N||27828.27|28/01/2026|JRNI.260128.526|Non-Motor Corporate","-429672.4|2875008.96|Currimjee Jeewanjee &amp; Co Ltd|01/04/2026|729243.58|Payment done after 30.06.2026|01/01/26 to 31/12/26||1918/26/N||729243.58|28/01/2026|JRNI.260128.522|Non-Motor Corporate","-150000|1005000|Currimjee Jeewanjee &amp; Co Ltd|01/04/2026|249278.65||01/01/26 to 31/12/26|POL-TER&amp;SAB-Mar-21-1002\\R5|6361/26/N|POL-TER&amp;SAB-Mar-21-1002\\R5|249278.65|18/03/2026|JRNI.260318.354|Special","-30754|4697.05|Currimjee Jeewanjee &amp; Co Ltd|03/03/2026|100||01/01/26 to 31/12/26||1918/26/N/E1||-26056.95|27/02/2026|JRNI.260227.565|Non-Motor Corporate","-29145.6|366870.24|RENTACOLOR (MAURITIUS) LTD|31/01/2026|266766.27||01/01/26 to 31/12/26|MD21M00252|MD21M00252/R5|MD21M00252|266766.27|23/02/2026|JRNNHZ.260223.99|Medical","-6290.76|52423|MAURITOURS LTD MAURITOURS LTD|01/08/2026|||01/01/26 to 31/12/26|MED/2023/00018|MED/2023/00018/R3|MED/2023/00018|46132.24|30/06/2026|JRNNHZ.260630.738|Medical","-27489.12|233886.6|MAURITOURS LTD MAURITOURS LTD|01/06/2026|206397.48||01/01/26 to 31/12/26|MED/2023/00018|MED/2023/00018/R3|MED/2023/00018|206397.48|30/04/2026|JRNNHZ.260430.757|Medical","-6872.28|57269|MAURITOURS LTD MAURITOURS LTD|01/07/2026|50396.72||01/01/26 to 31/12/26|MED/2023/00018|MED/2023/00018/R3|MED/2023/00018|50396.72|31/05/2026|JRNNHZ.260531.343|Medical","-6663.2|83290|Nassau Services Ltd|01/08/2026|||01/01/26 to 31/12/26|MD10M00493|MD10M00493/R16|MD10M00493|76626.8|30/06/2026|JRNNHZ.260630.483|Medical","-6901.04|86263|Nassau Services Ltd|01/07/2026|16093.06||01/01/26 to 31/12/26|MD10M00493|MD10M00493/R16|MD10M00493|16093.06|31/05/2026|JRNNHZ.260531.81|Medical","-31162.48|208789|Nassau Services Ltd|30/08/2026|44406.63||01/06/26 to 31/05/27||12779/21/R5||177626.52|11/06/2026|JRNI.260611.328|Financial"]</t>
+  </si>
+  <si>
+    <t>["Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure"]</t>
+  </si>
+  <si>
+    <t>["Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure","Mise en demeure"]</t>
+  </si>
+  <si>
+    <t>2026-07-28T07:16:38.348Z</t>
+  </si>
+  <si>
+    <t>["-11074|-11074|1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/02/2026|9745.31|1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E34|0|MED/2025/01055/EQ/75|11074.22|-9745.116400071518|","11074|11074|-1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/02/2026|-9745.31|-1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E33|0|MED/2025/01055/EQ/76|-11074.22|9745.116400071518|","-42083|-42083|5049.99|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.01|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|37033.25|5050|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E37|0|MED/2025/01055/EQ/80|42083.24|-37033.03880000684|","-31700|-31700|3803.97|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.03|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|27895.75|3804|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E38|0|MED/2025/01055/EQ/72|31699.72|-27895.9963999682|","-2374|-2374|284.94|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.06|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|2089.55|285|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E45|0|MED/2025/01055/EQ/107|2374.49|-2089.118800247632|","24936|24936|-2992.32|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.32|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/10/2025|-21943.68|-2992|01-07-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E14|0|MED/2025/01055|-24936|21943.68|","-2082|-2082|249.87|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.13|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|1832.41|250|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E46|0|MED/2025/01055/EQ/116|2082.28|-1832.1635995159154|","-9763|-9763|1171.52|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.48|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|8591.15|1172|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E47|0|MED/2025/01055/EQ/102|9762.67|-8591.440400013522|","-6616|-6616|793.93|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.07|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|5822.15|794|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E48|0|MED/2025/01055/EQ/101|6616.08|-5822.079600004837|","-111444|-111444|13373.34|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.34|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|98071.15|13373|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E42|0|MED/2025/01055/EQ/97|111444.49|-98070.71880000527|","38769|38769|-4636.02|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.0200000000005821|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|-34132.74|-4636|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E39|-135.22|MED/2025/01055|-38633.54|34132.951300480076|","53793|53793|-6455.21|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.21|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|-47338.2|-6455|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E22|0|MED/2025/01055/EQ/51|-53793.41|47337.8392000061|","31285|31285|-3754.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.26|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/02/2026|-27531.21|-3754|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E30|0|MED/2025/01055/EQ/73|-31285.47|27530.79640005408|","-16585|-16585|1990.24|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.24|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|14595.08|1990|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E50|0|MED/2025/01055/EQ/110|16585.32|-14594.798400030872|","6550|6550|-785.99|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.01|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||22/04/2026|-5763.91|-786|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E44|0|MED/2025/01055/EQ/99|-6549.9|5763.997999969465|","-41854|-41854|5022.48|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.479999999999418|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/01/2026|36831.55|5022|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E24|0|MED/2025/01055/EQ/48|41854.03|-36831.52359999742|","18600|18600|-2231.98|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.02|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||07/01/2026|-16367.82|-2232|01-09-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E8|0|MED/2025/01055/EQ/7|-18599.8|16367.99599995699|","-50256|-50256|6030.71|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.29|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|44225.23|6031|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E49|0|MED/2025/01055/EQ/111|50255.94|-44225.28280000334|","27159|27159|-3259.13|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.13|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/01/2026|-23900.26|-3259|01-10-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E23|0|MED/2025/01055/EQ/47|-27159.39|23899.91680004595|","33030|33030|-3963.6|12|HARDY HENRY SERVICES LTEE|0.4|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-29066.4|-3964|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E7|0|MD18M01064/3/R4/EQ/15|-33030|29066.4|","47208|47208|-5664.96|12|HARDY HENRY SERVICES LTEE|0.04|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-41543.04|-5665|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E9|0|MD18M01064/3/R4/EQ/17|-47208|41543.04|","-1884|-1884|226.08|12|HARDY HENRY SERVICES LTEE|226.16|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||01/07/2026|1657.92|-0.0800000000000125|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E21|0|MD18M01064/3/R4/EQ/43|1884|-1657.92|","-5790|-5790|694.8|12|HARDY HENRY SERVICES LTEE|-0.2|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|5095.2|695|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E10|0|MD18M01064/3/R4/EQ/18|5790|-5095.2|","-9420|-9420|1130.4|12|HARDY HENRY SERVICES LTEE|0.400000000000146|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|8289.6|1130|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E12|0|MD18M01064/3/R4/EQ/19|9420|-8289.6|","9400|9400|-1128|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/06/2026|-8272|-1128|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E22|0|MD18M01064/3/R4/EQ/42|-9400|8272|","-18840|-18840|2260.8|12|HARDY HENRY SERVICES LTEE|-0.199999999999709|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|16579.2|2261|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E8|0|MD18M01064/3/R4/EQ/16|18840|-16579.2|","-4626|-4626|555.12|12|HARDY HENRY SERVICES LTEE|0.12|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/05/2026|4070.88|555|01-05-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E18|0|MD18M01064/3/R4/EQ/30|4626|-4070.88|","-3900|-3900|468|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||01/03/2026|3432|468|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E13|0|MD18M01064/3/R4/EQ/23|3900|-3432|","27591|27591|-3310.92|12|HARDY HENRY SERVICES LTEE|0.08|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|-24280.08|-3311|01-04-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E16|0|MD18M01064/3/R4/EQ/28|-27591|24280.08|","-2111|-2111|253.32|12|HARDY HENRY SERVICES LTEE|0.32|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||14/06/2026|1857.68|253|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E20|0|MD18M01064/3/R4/EQ/37|2111|-1857.68|","17780|17780|-2133.6|12|HARDY HENRY SERVICES LTEE|0.4|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||17/12/2025|-15646.4|-2134|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E3|0|MD18M01064/3/R4/EQ/3|-17780|15646.4|","24815|24815|-2977.8|12|HARDY HENRY SERVICES LTEE|0.2|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/12/2025|-21837.2|-2978|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E6|0|MD18M01064/3/R4/EQ/12|-24815|21837.2|","6167|6167|-740.04|12|HARDY HENRY SERVICES LTEE|-0.04|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-5426.96|-740|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E5|0|MD18M01064/3/R4/EQ/14|-6167|5426.96|","-29379|-29379|3525.48|12|HARDY HENRY SERVICES LTEE|0.48|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/12/2025|25853.52|3525|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E4|0|MD18M01064/3/R4/EQ/10|29379|-25853.52|","-1762|-1762|211.44|12|HARDY HENRY SERVICES LTEE|0.44|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/05/2026|1550.56|211|01-05-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E17|0|MD18M01064/3/R4/EQ/32|1762|-1550.56|","-24687|-24687|2962.44|12|HARDY HENRY SERVICES LTEE|0.44|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/12/2025|21724.56|2962|01-10-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E1|0|MD18M01064/3/R4/EQ/9\nMD18M01064/3/R4/EQ/8\nMD02M00616/19/R5/EQ/2|24687|-21724.56|","12700|12700|-1524|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/02/2026|-11176|-1524|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E11|0|MD18M01064/3/R4/EQ/21|-12700|11176|","-14180|-14180|1701.6|12|HARDY HENRY SERVICES LTEE|-0.4|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|12478.4|1702|01-03-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E14|0|MD18M01064/3/R4/EQ/25|14180|-12478.4|","13536|13536|-1624.32|12|HARDY HENRY SERVICES LTEE|-0.32|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|-11911.68|-1624|01-04-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E15|0|MD18M01064/3/R4/EQ/26|-13536|11911.68|","1884|1884|-226.08|12|HARDY HENRY SERVICES LTEE|-0.08|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/06/2026|-1657.92|-226|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E19|0|MD18M01064/3/R4/EQ/38|-1884|1657.92|","-17559|-17559|2624.7|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.3|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||12/02/2026|14934.55|2625|01-01-2026 to 01-01-2027|POL-FID-Dec-21-9\\R4|POL-FID-Dec-21-9\\R4|61.25|2321/20/R6|17498|-14934.337369192875|","-22618|-22618|3380.83|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.17|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||12/02/2026|19236.93|3381|01-01-2026 to 01-01-2027|POL-EE-Dec-21-20\\R4|POL-EE-Dec-21-20\\R4|78.88|2321/20/R6|22538.88|-19237.134125572116|","-12042|-12042|1800|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||12/02/2026|10242|1800|01-01-2026 to 01-01-2027|POL-MON-Jan-20-1008\\R6|POL-MON-Jan-20-1008\\R6|42|2321/20/R6|12000|-10242|","-105713|-105713|15801.59|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.41|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||12/02/2026|89911.08|15802|01-01-2026 to 01-01-2027|POL-PA-Mar-20-1110\\R6|POL-PA-Mar-20-1110\\R6|368.71|2321/20/R6|105343.96|-89911.36067266109|","-34386|-34386|5139.87|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.13|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||12/02/2026|29245.89|5140|01-01-2026 to 01-01-2027|POL-EL-Jan-20-1023\\R6|POL-EL-Jan-20-1023\\R6|119.93|2321/20/R6|34265.83|-29246.094125591524|","-120816|-120816|18059.27|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.27|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||12/02/2026|102757.21|18059|01-01-2026 to 01-01-2027|POL-PPL-Jan-20-1005\\R6|POL-PPL-Jan-20-1005\\R6|421.38|2321/20/R6|120395.1|-102756.80174890049|","-136980|-136980|20475.37|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.37|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||12/02/2026|116504.87|20475|01-01-2026 to 01-01-2027|POL-LOP(F&amp;A)-Jan-20-1009\\R6|POL-LOP(F&amp;A)-Jan-20-1009\\R6|477.76|2321/20/R6|136502.48|-116504.66587443562|","-131417|-131417|19569.12|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.12|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||12/02/2026|111848.29|19569|01-01-2026 to 01-01-2027|POL-F&amp;A-Jan-20-1022\\R6|POL-F&amp;A-Jan-20-1022\\R6|956.61|2321/20/R6|130460.8|-111847.94105233089|","-2277|-2277|317.95|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.05|0||MUR|20/11/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||09/02/2026|1959.16|318|20-11-2025 to 01-01-2026|POL-F&amp;A-Jan-20-1022\\R5|POL-F&amp;A-Jan-20-1022\\R5\\E1|157.42|2321/20/R5/E2|2119.69|-1959.0653591613932|","-272603|-272603|45701.76|8|ORANGE EIGHT LTD|31739.35|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/11/2025|529569.24|13962.41|01-10-2025 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4|3999|MED/2022/01410/R3|571272|-250946.36011848328|","-30551|-30551|2444.12|8|ORANGE EIGHT LTD|2444.2|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||22/04/2026|28107.35|-0.0799999999999272|01-04-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E1|0|MED/2022/01410/R3/EQ/5|30551.47|-28106.917600036923|","25543|25543|-2043.44|8|ORANGE EIGHT LTD|-2043.88|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|-23499.6|0.440000000000055|01-05-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E3|0|MED/2022/01410/R3/EQ/6|-25543.04|23499.563199994987|","56735|56735|-4538.8|8|ORANGE EIGHT LTD|-4538.6|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||16/04/2026|-52196.22|-0.199999999999818|01-04-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E2|0|MED/2022/01410/R3/EQ/4|-56735.02|52196.20159999943|","22325|22325|-1786|8|ORANGE EIGHT LTD|-1786|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||03/06/2026|-20539|0|01-06-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E4|0|MED/2022/01410/R3/EQ/7|-22325|20539|"]</t>
+  </si>
+  <si>
+    <t>["-27050.95|2164.07|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2026|||01/01/26 to 31/12/26|MD11M00166|MD11M00166/R15/E6|MD11M00166|-24886.88|20/03/2026|JRNNHZ.260320.336|Medical","-12682.38|1014.59|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E14|MD11M00166|-8562.88|03/10/2025|JRNNHZ.251003.354|Medical","-22907.97|1832.63|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E6|MD11M00166|-7943.33|12/06/2025|JRNNHZ.250612.280|Medical","-37909.31|3032.74|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2026|||01/01/26 to 31/12/26|MD11M00166|MD11M00166/R15/E8|MD11M00166|-34876.57|05/06/2026|JRNNHZ.260605.487|Medical","-12682.38|1014.59|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E14|MD11M00166|-8562.88|03/10/2025|JRNNHZ.251003.354|Medical","-22907.97|1832.63|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E6|MD11M00166|-7943.33|12/06/2025|JRNNHZ.250612.280|Medical","-19196.43|1535.71|NEWREST (MAURITIUS) LTD NEWREST (MAURITIUS) LTD|31/03/2026|||01/10/25 to 30/09/26|MED/2024/01202|MED/2024/01202/R1/E7|MED/2024/01202|-17660.72|08/06/2026|JRNNHZ.260608.239|Medical","-895792.5|6006552|JAG SERVICES LTD|15/10/2026|2008438.85||01/01/26 to 31/12/26||31069/23/R2||3155697.21|06/01/2026|JRNI.260106.421|Motor","-52010|6861.3|JAG SERVICES LTD|13/02/2026|||01/01/26 to 31/12/26||31069/23/R2/E4||-45148.7|13/02/2026|JRNI.260213.86|Motor","-1.05|110|Panache &amp; Co.Ltd|01/09/2026|||01/07/25 to 30/06/26||17835/22/R3/E1||108.95|18/06/2026|JRNI.260618.308|Non-Motor Corporate","-48.6|325|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|26/03/26 to 26/03/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14790/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|276.4|09/06/2026|JRNI.260609.338|Marine","-37.5|251|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|08/05/26 to 08/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14789/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|213.5|09/06/2026|JRNI.260609.337|Marine","-60.9|407|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|04/05/26 to 04/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14786/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|346.1|09/06/2026|JRNI.260609.336|Marine","-37.5|251|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|01/05/26 to 01/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14778/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|213.5|09/06/2026|JRNI.260609.335|Marine","-37.5|351|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|05/05/26 to 05/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14777/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|313.5|09/06/2026|JRNI.260609.334|Marine","-180.9|1210|Panache &amp; Co.Ltd|01/09/2026|||01/07/25 to 30/06/26||9084/09/R16/E7||1029.1|03/06/2026|JRNI.260603.144|Motor","-661.05|4438|Panache &amp; Co.Ltd|01/08/2026|||01/07/25 to 30/06/26||9084/09/R16/E6||3776.95|28/05/2026|JRNI.260528.372|Motor","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|18/04/26 to 18/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12372/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.300|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|14/04/26 to 14/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12371/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.299|Marine","-304.8|2039|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|18/04/26 to 18/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12370/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|1734.2|18/05/2026|JRNI.260518.298|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|17/04/26 to 17/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12369/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.297|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|16/04/26 to 16/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12367/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.296|Marine","-57.75|386|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|09/04/26 to 09/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12366/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|328.25|18/05/2026|JRNI.260518.295|Marine","-48.6|325|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|15/04/26 to 15/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12365/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|276.4|18/05/2026|JRNI.260518.294|Marine","-104.7|700|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|02/03/26 to 02/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12364/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|595.3|18/05/2026|JRNI.260518.293|Marine","-123.15|824|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|02/02/26 to 02/02/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12363/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|700.85|18/05/2026|JRNI.260518.292|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|16/04/26 to 16/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12361/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.291|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|08/03/26 to 08/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12360/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.290|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|09/04/26 to 09/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12358/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.289|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|06/04/26 to 06/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12357/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.288|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|25/03/26 to 25/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12356/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.287|Marine","-54|461|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|28/03/26 to 28/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12355/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|407|18/05/2026|JRNI.260518.286|Marine","-5407|808.2|Panache &amp; Co.Ltd|24/04/2026|||01/07/25 to 30/06/26||9084/09/R16/E5||-4598.8|24/04/2026|JRNI.260424.167|Motor","-44.4|397|Scott &amp; Co Ltd|01/07/2026|352.6||01/10/25 to 30/09/26||33954/19/R6/E2||352.6|09/01/2026|JRNI.260109.314|Non-Motor Corporate","-457.5|3161|Scott &amp; Co Ltd|01/07/2026|2703.5||01/10/25 to 30/09/26||33954/19/R6/E1||2703.5|07/01/2026|JRNI.260107.260|Non-Motor Corporate","-195955.8|1311444|HIGHWAY PROPERTIES LTD|01/08/2026|||01/05/26 to 30/04/27||13781/26/N||1115488.2|28/05/2026|JRNI.260528.581|Non-Motor Corporate","-24269.23|162860.98|HIGHWAY PROPERTIES LTD|01/09/2026|||01/05/26 to 30/04/27||14246/26/R1||138591.75|09/06/2026|JRNI.260609.339|Non-Motor Corporate","-2059.76|14279.97|HIGHWAY PROPERTIES LTD|05/06/2026|12220.21||01/04/26 to 30/04/26||14246/26/N||12220.21|03/06/2026|JRNI.260603.381|Non-Motor Corporate","-19264.65|129381|HIGHWAY PROPERTIES LTD|06/05/2026|110116.35||01/04/26 to 30/04/26||10767/26/N||110116.35|23/04/2026|JRNI.260423.353|Non-Motor Corporate","-38641.95|258710|HIGHWAY PROPERTIES LTD|01/07/2026|176087.63|Payment done after 30.06.2026|10/04/26 to 31/03/27|POL-MV-Apr-26-95|8591/26/N|POL-MV-Apr-26-95|176087.63|10/04/2026|JRNI.260410.163|Motor","-11997.59|80763.97|ACBMS LTD|01/08/2026|||01/05/26 to 30/04/27||12079/22/R4||45845.27|07/05/2026|JRNI.260507.165|Non-Motor Corporate","-16786.56|211300.82|GAYA COLLECTIONS LIMITEE GAYA COLLECTIONS LIMITEE|30/06/2026|160619.77|Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2023/00969|MED/2023/00969/R3|MED/2023/00969|160619.77|13/05/2026|JRNNHZ.260513.423|Medical","-2119.73|26496.72|GAYA COLLECTIONS LIMITEE GAYA COLLECTIONS LIMITEE|30/06/2026|1913.1||01/05/26 to 30/04/27|MED/2023/00969|MED/2023/00969/R3/E1|MED/2023/00969|1913.1|11/06/2026|JRNNHZ.260611.54|Medical","-12676.72|158459|BELLE RIVIERE HOTEL LTD|01/08/2026|||01/05/26 to 30/04/27|MED/2025/00947|MED/2025/00947/R1|MED/2025/00947|145782.28|30/06/2026|JRNNHZ.260630.904|Medical","-11476.08|155614.12|BELLE RIVIERE HOTEL LTD|01/07/2026|131974.92||01/05/26 to 30/04/27|MED/2025/00947|MED/2025/00947/R1|MED/2025/00947|131974.92|31/05/2026|JRNNHZ.260531.511|Medical","-6485.7|43689|Osman Rezah|01/09/2026|||01/06/26 to 31/05/27||13626/10/R16||37203.3|01/06/2026|JRNI.260601.332|Non-Motor Corporate","-38910|5816.1|Partsionate Ltd|24/06/2026|||06/05/26 to 30/04/27||11100/26/N/E1||-33093.9|24/06/2026|JRNI.260624.288|Motor","-123515|18462.6|Partsionate Ltd|05/06/2026|||06/05/26 to 30/04/27||11084/26/N/E2||-105052.4|05/06/2026|JRNI.260605.166|Motor","-3078|21042|ASSOCIATION SYNDICALE DU LOTISSEMENT LES VILLAS DE CASCAVELLE|01/03/2026|17964||01/11/25 to 31/10/26||9507/20/R6||17964|03/12/2025|JRNI.251203.405|Non-Motor Corporate","-1383.3|9754|ASSOCIATION SYNDICALE MORCELLEMENT VILLAZE|01/08/2026|||01/05/26 to 30/04/27||17184/24/R2||8370.7|11/05/2026|JRNI.260511.317|Non-Motor Corporate","-263.98|1915.99|LES CAMPECHES LTEE|01/09/2026|||12/06/26 to 11/12/26||16082/26/N||1652.01|24/06/2026|JRNI.260624.397|Non-Motor Corporate","-11504.7|77466|SYNDICAT DES COPROPRIÉTAIRES DE L`ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|01/03/2026|65961.3||01/10/25 to 30/09/26||2595/17/R9||65961.3|03/12/2025|JRNI.251203.296|Non-Motor Corporate","-408.45|2783|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|01/01/2026|2374.55||01/11/25 to 31/10/26||31161/22/R3||2374.55|13/10/2025|JRNI.251013.122|Motor","-13346.85|89390|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|01/08/2026|||01/06/26 to 31/05/27||31169/22/R3||76043.15|29/05/2026|JRNI.260529.51|Motor","-457|68.25|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|08/10/2025|||01/01/25 to 31/10/25||31161/22/R2/E2||-388.75|08/10/2025|JRNI.251008.78|Motor","-408.75|2785|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|01/04/2026|2376.25||01/02/26 to 31/01/27||31164/22/R3||2376.25|12/01/2026|JRNI.260112.141|Motor","-7549.5|50606|The General Construction Company Limited|01/01/2026|43056.5||01/04/25 to 31/03/26||10359/24/R1/E1||43056.5|01/10/2025|JRNI.251001.326|Non-Motor Corporate","-242123.1|1619804|The General Construction Company Limited|17/06/2026|1377680.9||16/12/24 to 15/12/34||17764/25/N/E1||1377680.9|15/06/2026|JRNI.260615.361|Special","-768028.95|5138114|The General Construction Company Limited|01/07/2026|1456887.07||01/04/26 to 31/03/27||10359/24/R2||1456887.07|16/04/2026|JRNI.260416.322|Non-Motor Corporate","-322312.92|2156773.96|The General Construction Company Limited|01/07/2026|589013.49||01/04/26 to 31/03/27||7186/22/R4||589013.49|16/04/2026|JRNI.260416.317|Non-Motor Corporate","-12916.35|86534|The General Construction Company Limited|01/11/2025|73617.65||01/04/25 to 31/03/26||MT9900043297/R25/E15||73617.65|18/08/2025|JRNI.250818.221|Motor","-11576.25|77945|The General Construction Company Limited|01/07/2026|44248.1||01/04/26 to 31/03/27||8694/22/R4||44248.1|15/04/2026|JRNI.260415.201|Non-Motor Corporate","-9325|1393.8|The General Construction Company Limited|27/10/2025|||01/04/25 to 31/03/26||MT9900043297/R25/E27||-7931.2|27/10/2025|JRNI.251027.157|Motor","-1308|195.45|The General Construction Company Limited|05/02/2026|||01/04/25 to 31/03/26||MT9900043297/R25/E38||-1112.55|05/02/2026|JRNI.260205.45|Motor","-4762.35|32003|The General Construction Company Limited|01/10/2025|27240.65||01/04/25 to 31/03/26|POL-MVF-May-19-1121\\R6\\E14|MT9900043297/R25/E11|POL-MVF-May-19-1121\\R6\\E14|27240.65|14/07/2025|JRNI.250714.129|Motor","-3359|502.05|The General Construction Company Limited|06/11/2025|||01/04/25 to 31/03/26||MT9900043297/R25/E30||-2856.95|06/11/2025|JRNI.251106.243|Motor","-75873.75|513095|The General Construction Company Limited|01/07/2026|437221.25||01/04/26 to 31/03/27||9151/18/R8||437221.25|01/04/2026|JRNI.260401.326|Motor","-10350|69442|The General Construction Company Limited|01/07/2026|59092||01/04/26 to 31/03/27||13092/25/R1||59092|01/04/2026|JRNI.260401.324|Motor","-924635.68|6216812.99|The General Construction Company Limited|01/07/2026|3362379.92||01/04/26 to 31/03/27||MT9900043297/R26||3362379.92|01/04/2026|JRNI.260401.322|Motor","-581|86.85|The General Construction Company Limited|27/10/2025|||01/04/25 to 31/03/26||9151/18/R7/E5||-494.15|27/10/2025|JRNI.251027.149|Motor","-9693.45|64949|DESVAUX DE MARIGNY Alain Laurent|01/09/2026|||01/07/26 to 30/06/27||21359/25/R1||55255.55|16/06/2026|JRNI.260616.212|Motor","-8462.43|106180.44|Desvaux De Marigny-Montocchio Marie Pascale Anne|31/10/2026|||01/05/26 to 30/04/27|MD21M00643|MD21M00643/R5|MD21M00643|87946.25|11/05/2026|JRNNHZ.260511.367|Medical","-11246.4|94120|CHEUNG Willy|30/04/2026|66298.88|Payment done after 30.06.2026|01/03/26 to 28/02/27|MED/2026/00365|MED/2026/00365/N|MED/2026/00365|66298.88|24/04/2026|JRNNHZ.260424.75|Medical","-4703.04|39592|RAMPUTH NEELESH|30/04/2026|27911.52|Payment done after 30.06.2026|01/03/26 to 28/02/27|MED/2026/00315|MED/2026/00315/N|MED/2026/00315|27911.52|16/04/2026|JRNNHZ.260416.32|Medical","-7197.12|60376|Boodiah Maureen Vivianna|31/05/2026|53178.88|Payment done after 30.06.2026|01/04/26 to 31/03/27|MED/2026/00362|MED/2026/00362/N|MED/2026/00362|53178.88|24/04/2026|JRNNHZ.260424.21|Medical","-8138.25|54545|Comptoir Ouest OI Ltee|01/07/2026|38670.45||01/05/26 to 30/04/27|POL-MV-Apr-25-150|11301/25/R1|POL-MV-Apr-25-150|38670.45|16/04/2026|JRNI.260416.191|Motor","-5517.02|69362.87|NOMBRO MARY LYSIE IVY|30/11/2026|||01/06/26 to 31/05/27|MED/2023/00781|MED/2023/00781/R3|MED/2023/00781|56493.34|03/06/2026|JRNNHZ.260603.72|Medical","-4165.05|52563.19|Pro Wire Electrical &amp; Mechanical Ltd Pro Wire Electrical &amp; Mechanical Ltd|30/11/2026||Payment done after 30.06.2026|01/06/26 to 31/05/27|MED/2022/00714|MED/2022/00714/R4|MED/2022/00714|48398.14|15/06/2026|JRNNHZ.260615.19|Medical","-2803.5|18855|MEDLOG (MAURITIUS) LTD|01/09/2026|||01/08/25 to 31/07/26||26048/24/R1/E2||16051.5|01/06/2026|JRNI.260601.416|Non-Motor Corporate","-14031.3|93969|G. DE VILLIERS PAINT CONTRACTORS LTD|01/08/2026|||01/06/26 to 31/05/27||18210/25/R1||79937.7|27/05/2026|JRNI.260527.92|Motor","-5408.25|36381|G. DE VILLIERS PAINT CONTRACTORS LTD|01/09/2025|22655.11||01/07/25 to 30/06/26||18205/25/N||22655.11|26/06/2025|JRNI.250626.416|Motor","-8518.95|57192|G. DE VILLIERS PAINT CONTRACTORS LTD|01/09/2025|27592.64||01/07/25 to 30/06/26||18193/25/N||27592.64|26/06/2025|JRNI.250626.408|Motor","-8902.65|59759|G. DE VILLIERS PAINT CONTRACTORS LTD|01/07/2026|50856.35||01/05/26 to 30/04/27||18193/25/R1||50856.35|30/04/2026|JRNI.260430.161|Motor","-5711.1|38407|G. DE VILLIERS PAINT CONTRACTORS LTD|01/08/2026|||01/06/26 to 31/05/27||18205/25/R1||32695.9|27/05/2026|JRNI.260527.85|Motor"]</t>
+  </si>
+  <si>
+    <t>["-26357|-26357|3865.03|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND\nCLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|0.03|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||02/02/2026|22492.04|3865|01-02-2026 to 01-02-2027|POL-CAR-TPL-Jun-20-1033\\R5|POL-CAR-TPL-Jun-20-1033\\R5|590.18|6162/25|25766.89|-22491.980264877697|","-5118|-5118|750|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR CONTRACTORS &amp;/OR SUB CONTRACTORS||0||MUR|15/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||4367.5||15-05-2026 to 15-06-2026|POL-CAR-TPL-Nov-25-1054|POL-CAR-TPL-Nov-25-1054\\E2|117.5||5000|-4367.926722032243|","-6121|-6121|900|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION)||0||MUR|15/06/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY|||5221||15-06-2026 to 15-08-2026|POL-PL-Nov-25-1105|POL-PL-Nov-25-1105\\E3|121||6000|-5221|","-130114|-130114|19449|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR ECOFUEL LTEE|0|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||15/01/2026|110664.81|19449|01-12-2025 to 01-12-2026|POL-PA-Dec-19-1603\\R6|POL-PA-Dec-19-1603\\R6|453.81|46037/12/R13|129660|-110664.9715994021|","-197263|-197263|36216.93|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR ECOFUEL LTEE|6730.58|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||15/01/2026|206074.31|29486.35|01-12-2025 to 01-12-2026|POL-ARM(P&amp;M)-Dec-19-1132\\R6|POL-ARM(P&amp;M)-Dec-19-1132\\R6|845.07|46037/12/R13|241446.17|-167776.74922762375|","-15329|-15329|2216.63|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT ,SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR DIRECT CONTRACTORS &amp;/OR SUBCONTRACTORS||0||MUR|11/06/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||13112.59||11-06-2026 to 11-09-2026|POL-CAR-TPL-Jun-26-34|POL-CAR-TPL-Jun-26-34|551.72||14777.5|-13112.401812355749|","-3111|-3111|450|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION)|0|0||MUR|16/03/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||15/04/2026|2660.5|450|16-03-2026 to 15-05-2026|POL-PL-Nov-25-1105|POL-PL-Nov-25-1105\\E1|110.5||3000|-2660.9276643626426|","368|368|15750|15|GOLDEN FUND MANAGEMENT SERVICES LTD|15804.73|0|Correction to be done by CBL amount not in aging|MUR|01/05/2019|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PI-CRIME||13/05/2019|90142.5|-54.7299999999996|01-05-2019 to 01-05-2020|POL-C+PI-Jun-19-1002|POL-C+PI-Jun-19-1002|892.5|15398/18/R1|105000|313.2652454139812|","-736|-736|0|15|GOLDEN FUND MANAGEMENT SERVICES LTD|0|0|Correction to be done by CBL amount not in aging|MUR|01/05/2019|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PI-CRIME||13/05/2019|-368|0|01-05-2019 to 01-05-2020|POL-C+PI-Jun-19-1003|POL-C+PI-Jun-19-1003|-368|15398/18/R1|0|-736|","-18271|-18271|2299.8|8|PARIS-ONEZIME MARIE STEPHANIE MRS|837.96|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||09/06/2026|26447.76|1461.84|01-05-2026 to 01-01-2027|POL-HEALTH-Dec-22-157\\R3|POL-HEALTH-Dec-22-157\\R3\\E1|0|MED/2023/00006/R3|28747.56|-16809.323050721523|","-48544|-48544|7735.12|8|PARIS-ONEZIME MARIE STEPHANIE MRS|4641.24|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/12/2025|89353.88|3093.88|01-01-2026 to 01-01-2027|POL-HEALTH-Dec-22-157\\R3|POL-HEALTH-Dec-22-157\\R3|400|MED/2023/00006/R3|96689|-44676.47983520275|","-43082.59|-43082.59|14673.79|15|ROGERS CAPITAL FINANCE LTD ON LEASE TO HEFTY LTD|8240.27|99.18||MUR|04/12/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||09/12/2025|83593.07|6433.52|04-12-2025 to 01-12-2026|POL-MV-Dec-25-503|POL-MV-Dec-25-503|342.39|34294/25|97825.29|-36649.242294414405|","-135220|-135220|20182.35|15|SPICE FINANCE LTD ON FINANCE LEASE TO HEFTY LTD|0.349999999997672|200||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||06/04/2026|115037.58|20182|01-04-2026 to 01-04-2027|POL-MV-Apr-23-97\\R3|POL-MV-Apr-23-97\\R3|470.93|6400/26|134549|-115037.63955209857|","-59581|-59581|8891.1|15|INDUSTRIAL FINANCE CORPORATION OF MAURITIUS LTD (IFCM) ON FINANCE LEASE TO HEFTY LTD|0.1|100||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||06/04/2026|50690.36|8891|01-04-2026 to 01-04-2027|POL-MV-Apr-23-105\\R3|POL-MV-Apr-23-105\\R3|207.46|6368/26|59274|-50689.96864393722|","-120520|-120520|18000|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR SUB-CONTRACTORS|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|102520|18000|01-05-2026 to 31-05-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E3|520|12718/24/N|120000|-102520|","-184322|-184322|27536.85|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB-CONTRACTORS|-0.15|0||MUR|28/04/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|156784.68|27537|28-04-2026 to 31-05-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E4|742.53|12718/24/N|183579|-156785.0797840057|","-123859|-123859|92122.96|15|REHM GRINAKER CONSTRUCTION CO. LTD|92122.96|3000||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||21/01/2026|527179.71|0|01-01-2026 to 01-01-2027|POL-MVF-Jun-21-1026\\R4|POL-MVF-Jun-21-1026\\R4|2149.59|10936/21/R4|614153.08|-105434.63618668073|","-722620|-722620|108000|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB-CONTRACTORS|0|0||MUR|31/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|614620|108000|31-05-2026 to 31-08-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E5|2620|12718/24/N|720000|-614620|","-278797|-278797|44294.4|8|CREDIT GUARANTEE INSURANCE CO LTD|22146.08|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/01/2026|513261.36|22148.32|01-01-2026 to 01-01-2027|POL-HEALTH-Jan-20-22\\R6|POL-HEALTH-Jan-20-22\\R6|3875.76|MD11M00167/10/R5|553680|-256648.2810327706|","-109903|-109903|11704.53|8|CREDIT GUARANTEE INSURANCE CO LTD|2911.85|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/04/2026|134602.04|8792.68|01-03-2026 to 01-01-2027|POL-HEALTH-Jan-20-22\\R6|POL-HEALTH-Jan-20-22\\R6\\E1|0|MD11M00167/10/R5/EQ/4|146306.57|-101110.75669479504|","-4204|-4204|628.35|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|0.35|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||05/05/2026|3575.32|628|01-04-2026 to 01-04-2027|POL-MON-Apr-20-1052\\R6|POL-MON-Apr-20-1052\\R6|14.67|8040/21/R5|4189|-3575.600672745482|","-21300|-21300|3183.83|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.17|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||05/05/2026|18115.96|3184|01-04-2026 to 01-04-2027|POL-EE-Apr-20-1072\\R6|POL-EE-Apr-20-1072\\R6|74.29|8040/21/R5|21225.5|-18116.13860981728|","-3947|-3947|589.95|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.0499999999999272|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||05/05/2026|3356.82|590|01-04-2026 to 01-04-2027|POL-ARMISC-Apr-26-7|POL-ARMISC-Apr-26-7|13.77|8040/21/R5|3933|-3357.0156203680476|","-52448|-52448|7839.71|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.29|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||05/05/2026|44607.96|7840|01-04-2026 to 01-04-2027|POL-EL-Apr-20-1145\\R6|POL-EL-Apr-20-1145\\R6|182.92|8040/21/R5|52264.75|-44608.240672655236|","-197614|-197614|29538.75|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.25|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||05/05/2026|168075.49|29539|01-04-2026 to 01-04-2027|POL-PL-Apr-20-1159\\R6|POL-PL-Apr-20-1159\\R6|689.24|8040/21/R5|196925|-168075.285874439|","-115877|-115877|17320.89|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.11|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||05/05/2026|98555.9|17321|01-04-2026 to 01-04-2027|POL-PA-Apr-20-1141\\R6|POL-PA-Apr-20-1141\\R6|404.16|8040/21/R5|115472.63|-98556.0786098752|","-219576|-219576|48227.25|15|IMPACT PRODUCTION LTD|15592.78|2500||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||30/01/2026|276913.07|32634.47|01-01-2026 to 01-01-2027|POL-MVF-Sep-19-6170\\R7|POL-MVF-Sep-19-6170\\R7|1125.32|49936/17/R8\n54552/15/R10\n19969/21/R5\n30665/22/R4\n49919/17/R8|321515|-187006.84141025634|","-66231|-66231|9900|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|0|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||05/05/2026|56331|9900|01-04-2026 to 01-04-2027|POL-PA-Apr-20-1140\\R6|POL-PA-Apr-20-1140\\R6|231|8040/21/R5|66000|-56331|","-228722|-228722|76806|15|KASA CORPORATE SERVICES LTD|42670.55|800||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||20/02/2026|437826.14|34135.45|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1065\\R4|POL-MVF-Dec-21-1065\\R4|1792.14|32859/23/R2|512040|-194586.5067678828|","16632|16632|-1330.56|8|KASA CORPORATE SERVICES LTD.|0.44|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/03/2026|-15301.44|-1331|01-12-2025 to 01-03-2026|POL-HEALTH-Jun-19-2718\\R48|POL-HEALTH-Jun-19-2718\\R48\\E3|0|MD08M01076/14/R4/EQ/8|-16632|15301.44|","22341|22341|-1787.28|8|KASA CORPORATE SERVICES LTD.|-0.28|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-20553.72|-1787|01-04-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49\\E1|0|MD08M01076/14/R5/EQ/2|-22341|20553.72|","-24663|-24663|1959.36|8|KASA CORPORATE SERVICES LTD.|0.36|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|22703.64|1959|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49\\E2|171|Please refer to POL-HEALTH-Jun-19-2718\\R49 - NO Docs to follow|24492|-22703.64|","-969342|-969342|77008.32|8|KASA CORPORATE SERVICES LTD.|0.320000000009313|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|892333.68|77008|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49|6738|MD08M01076/14/R5 - please refer to POL-HEALTH-Jun-19-2718\\R49\\E2 for adjustment in  premium|962604|-892333.6799999999|","-265806|-265806|79479.3|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|39747.84|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||17/03/2026|452237.22|39731.46|01-03-2026 to 28-02-2027|POL-ARM(P&amp;M)-Mar-20-1019\\R6|POL-ARM(P&amp;M)-Mar-20-1019\\R6|1854.52|8187/26/N|529862|-226074.16165914875|","-40914|-40914|12234.05|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|6118.43|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||17/03/2026|69611.76|6115.62|01-03-2026 to 28-02-2027|POL-PA-Mar-20-1103\\R6|POL-PA-Mar-20-1103\\R6|285.46|8187/26/N|81560.35|-34798.30609092879|","-30023|-30023|8977.5|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|4489.18|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||17/03/2026|51081.97|4488.32|01-03-2026 to 28-02-2027|POL-PPL-Mar-20-1021\\R6|POL-PPL-Mar-20-1021\\R6|209.47|8187/26/N|59850|-25535.25672654121|","-30023|-30023|8977.5|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE &amp;/OR PRINCIPAL &amp;/OR CONTRACTORS &amp;/OR SUB-CONTRACTORS|4489.18|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|EAR &amp; TPL||17/03/2026|51081.98|4488.32|01-03-2026 to 28-02-2027|POL-EAR-TPL-Mar-20-1005\\R6|POL-EAR-TPL-Mar-20-1005\\R6|209.48|8187/26/N|59850|-25535.25747375768|","-8931|-8931|2596.16|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1298.65|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||17/03/2026|15272.17|1297.51|01-03-2026 to 28-02-2027|POL-F&amp;A-Mar-20-1117\\R6|POL-F&amp;A-Mar-20-1117\\R6|560.58|8187/26/N|17307.75|-7633.379855308247|","-11765|-11765|3518.25|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1759.9|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||17/03/2026|20018.87|1758.35|01-03-2026 to 28-02-2027|POL-EE-Mar-20-1049\\R6|POL-EE-Mar-20-1049\\R6|82.12|8187/26/N|23455|-10006.407136896953|","-8998|-8998|2690.78|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1345.52|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||17/03/2026|15310.51|1345.26|01-03-2026 to 28-02-2027|POL-ARMISC-Mar-20-1024\\R6|POL-ARMISC-Mar-20-1024\\R6|62.79|8187/26/N|17938.5|-7653.005366837599|","-893|-893|267.15|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|133.77|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||17/03/2026|1520.08|133.38|01-03-2026 to 28-02-2027|POL-LOP(F&amp;A)-Mar-20-1029\\R6|POL-LOP(F&amp;A)-Mar-20-1029\\R6|6.23|8187/26/N|1781|-759.5169284311477|","-10152|-10152|3035.48|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1518.42|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||08/05/2026|17271.86|1517.06|01-03-2026 to 28-02-2027|POL-EL-Mar-20-1108\\R6|POL-EL-Mar-20-1108\\R6|70.83|8187/26/N|20236.51|-8634.50962656852|","-12154.99|-12154.99|68082.09|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED  &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE  PROPERTIES LTD &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE  &amp;/OR QUALITY BEVERAGES LIMITED &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR TRAMPOLINE LIMITEE  NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|68082.14|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||06/02/2026|387387.1|-0.0500000000029104|01-01-2026 to 01-01-2027|POL-EE-Jan-26-3|POL-EE-Jan-26-3|1588.61|1918/26/N|453880.58|-10338.100644368502|"]</t>
+  </si>
+  <si>
+    <t>["-13435.2|112360|SAWMYNADEN Kisnasamy Poulay|31/05/2026|78739.85||01/04/26 to 31/03/27|MED/2026/00453|MED/2026/00453/N|MED/2026/00453|78739.85|21/05/2026|JRNNHZ.260521.163|Medical","-5286.24|44452|HUET Louise Lilette Nicole|30/06/2026|32240.48|Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2026/00429|MED/2026/00429/N|MED/2026/00429|32240.48|19/05/2026|JRNNHZ.260519.161|Medical","-10680.48|89404|SOORJUN SOTEEHALL MANISHA|30/06/2026|70314.39|Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2026/00515|MED/2026/00515/N|MED/2026/00515|70314.39|02/06/2026|JRNNHZ.260602.2|Medical","-150406.35|1006718|IKO (MAURITIUS) HOTEL LIMITED T/A CONSTANCE LE CHALAND IKO - MAURITIUS|01/04/2026|856311.65||01/01/26 to 31/12/26||1595/26/N||856311.65|23/01/2026|JRNI.260123.385|Non-Motor Corporate","-52.2|449|IKO (MAURITIUS) HOTEL LIMITED T/A CONSTANCE LE CHALAND IKO - MAURITIUS|01/09/2026|||01/01/26 to 31/12/26||1595/26/N/E3||396.8|17/06/2026|JRNI.260617.355|Non-Motor Corporate","-3529.35|23729|MERIDIS FINANCIAL SOLUTIONS LTD|01/09/2026|||04/05/26 to 30/04/27|POL-F-PI-Jun-26-23|16950/26/N|POL-F-PI-Jun-26-23|20199.65|30/06/2026|JRNI.260630.583|Financial","-8579.52|71896.01|LABELLE VICTOIRE Marie Cindy Anabelle|31/07/2026|||01/06/26 to 31/05/27|MED/2026/00624|MED/2026/00624/N|MED/2026/00624|63316.49|30/06/2026|JRNNHZ.260630.280|Medical","-3969.76|49622|VISIONWAY LTD|01/08/2026|||01/09/25 to 31/08/26|MD16M00704|MD16M00704/R9|MD16M00704|45652.24|30/06/2026|JRNNHZ.260630.553|Medical","-11250|75507|RIVALLAND CHRISTIAN ROBERT XAVIER|01/05/2026|64257||09/02/26 to 30/04/27|POL-MV-Feb-26-32|3064/26/N|POL-MV-Feb-26-32|64257|09/02/2026|JRNI.260209.147|Motor","-2808|336.96|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E7|MED/2025/00586|-2471.04|03/04/2026|JRNNHZ.260403.10|Medical","-5709.6|685.15|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E6|MED/2025/00586|-5024.45|09/03/2026|JRNNHZ.260309.114|Medical","-2808|336.96|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E7|MED/2025/00586|-2471.04|03/04/2026|JRNNHZ.260403.10|Medical","-22270.08|280324.64|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|31/10/2026||Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2025/00586|MED/2025/00586/R1|MED/2025/00586|248010.54|19/05/2026|JRNNHZ.260519.212|Medical","-5709.6|685.15|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E6|MED/2025/00586|-5024.45|09/03/2026|JRNNHZ.260309.114|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.35|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.34|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.33|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.32|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.31|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.30|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.158|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.157|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.156|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.155|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.154|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.153|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.152|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.151|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.150|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.149|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.148|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.147|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.93|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.92|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.91|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.90|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.89|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.88|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.87|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.86|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.85|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.84|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.83|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.82|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.311|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.310|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.309|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.308|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.307|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.306|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.305|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.304|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.303|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.302|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.301|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.300|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.17|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.16|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.15|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.14|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.13|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.12|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.11|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.10|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.9|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.8|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.7|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.6|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.41|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.40|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.39|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.38|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.37|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.36|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.35|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.34|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.33|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.32|Medical"]</t>
+  </si>
+  <si>
+    <t>["-27563|-27563|172922.85|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LTD &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALLI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|172922.99|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||06/02/2026|983931.06|-0.14000000001397|01-01-2026 to 01-01-2027|POL-PA-Mar-20-1106\\R6|POL-PA-Mar-20-1106\\R6|4034.9|1918/26/N|1152819.01|-23442.97025955507|","-12710|-12710|37735.58|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES &amp;/OR CURRIMJEE LIMITED &amp;/OR  CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR PRINCIPALS &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|37735.3|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||06/02/2026|214715.44|0.279999999998836|01-01-2026 to 01-01-2027|POL-CAR-TPL(BC)-Mar-20-1010\\R6|POL-CAR-TPL(BC)-Mar-20-1010\\R6|880.52|1918/26/N|251570.5|-10810.149400069764|","-19711.99|-19711.99|38186.93|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LIMITEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED  &amp;/OR LATE BAI REHMATBAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASSALI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LIMITED &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LIMITED &amp;/OR QUALITY BEVERAGES LIMITED &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR EMTEL MFS CO LTD &amp;/OR E-SKILLS LIMITED &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LIMITEE &amp;/OR ZAC (PROPERTIES) LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|38186.78|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||06/02/2026|217783.65|0.149999999994179|01-01-2026 to 01-01-2027|POL-PPL-Mar-20-1020\\R6|POL-PPL-Mar-20-1020\\R6|1391.08|1915/26/N|254579.5|-16771.259927463147|","-172|-172|34905.3|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LTD &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR SYNDICAT DES COPROPRIETAIRES DE PHOENIX CENTRAL &amp;/OR FACILICARE LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|34905.52|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||06/02/2026|198611.18|-0.219999999993888|01-01-2026 to 01-01-2027|POL-MON-Mar-20-1043\\R6|POL-MON-Mar-20-1043\\R6|814.48|1918/26/N|232702|-146.28998758460216|","-180668|-180668|29880.75|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LTD &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR SYNDICAT DES COPROPRIETAIRES DE PHOENIX CENTRAL &amp;/OR FACILICARE LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|2889.59|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||16/03/2026|170121.48|26991.16|01-01-2026 to 01-01-2027|POL-MON-Mar-20-1043\\R6|POL-MON-Mar-20-1043\\R6\\E2|797.23|1918/26/N/E1|199205|-153675.82425775955|","229698|229698|-34477.8|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LTD &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR SYNDICAT DES COPROPRIETAIRES DE PHOENIX CENTRAL &amp;/OR FACILICARE LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|-128.050000000005|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||16/03/2026|-196078.7|-34349.75|01-01-2026 to 01-01-2027|POL-MON-Mar-20-1043\\R6|POL-MON-Mar-20-1043\\R6\\E1|-704.5|1918/26/N/E1|-229852|195348.58150865405|","-14974.99|-14974.99|108863.66|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED  &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE  PROPERTIES LIMITED  &amp;/OR  LATE BAI REHMATBAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE  NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|108863.22|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||06/02/2026|619434.25|0.44000000001688|01-01-2026 to 01-01-2027|POL-EL-Mar-20-1106\\R6|POL-EL-Mar-20-1106\\R6|2540.16|1918/26/N|725757.75|-12736.576024785652|","-26952|-26952|4013.77|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED  &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE  PROPERTIES LTD &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|-0.23|0||MUR|05/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ASSETS ALL RISKS &amp; BUSINESS INTERRUPTION||26/05/2026|22938.32|4014|05-03-2026 to 01-01-2027|POL-AAR+BI-Mar-20-1003\\R6|POL-AAR+BI-Mar-20-1003\\R6\\E1|193.65||26758.44|-22938.24340301624|","34442|34442|-2755.38|8|RENTACOLOR (MAURITIUS) LIMITED|-0.38|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-31686.92|-2755|01-05-2026 to 01-01-2027|POL-HEALTH-Jan-21-3\\R5|POL-HEALTH-Jan-21-3\\R5\\E1|0|MD21M00252/0/R5/EQ/2|-34442.3|31686.64399996516|","-366870|-366870|29145.6|8|RENTACOLOR (MAURITIUS) LIMITED|2428.45|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/02/2026|337724.64|26717.15|01-01-2026 to 01-01-2027|POL-HEALTH-Jan-21-3\\R5|POL-HEALTH-Jan-21-3\\R5|2550.24|MD21M00252/0/R5|364320|-337724.41906653426|","-13076|-13076|1569.12|12|MAURITOURS LTD|0.12|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/05/2026|11506.88|1569|01-06-2026 to 01-01-2027|POL-HEALTH-Jan-26-3|POL-HEALTH-Jan-26-3\\E1|0|MED/2023/00018/R3/EQ/1|13076|-11506.880000000001|","-692039|-692039|82467.36|12|MAURITOURS LTD|27441.8|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||07/04/2026|609571.24|55025.56|01-01-2026 to 01-01-2027|POL-HEALTH-Jan-26-3|POL-HEALTH-Jan-26-3|4810.6|MED/2023/00018/R3|687228|-609571.5923336647|","-437069|-437069|69442.56|8|NASSAU SERVICES LTD|34719.69|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|804665.44|34722.87|01-01-2026 to 01-01-2027|POL-HEALTH-Feb-21-10\\R27|POL-HEALTH-Feb-21-10\\R27|6076|MD10M00493/11/R5|868032|-402346.52834130335|","-156592|-156592|31162.5|15|NASSAU SERVICES LTD &amp;/OR UHY HEERALALL &amp;/OR UHY LOSS ADJUSTERS LTD &amp;/OR UHY &amp; CO &amp;/OR UHY ADVISORY LTD &amp;/OR MR. NIRMAL HEERALALL &amp;/OR MR. DOMINIQUE SAMOUILHAN &amp;/OR MR. PRAVESH JAISHINGH PURGASS &amp;/OR MR. BENY KOWLESSUR &amp;/OR MR AVINASHSINGH MOORUTH &amp;/OR MR JEAN THOMAS SAMOUILHAN &amp;/OR CAS SERVICES LTD &amp;/OR UHY CORPORATE FINANCE LTD &amp;/OR MR ANDRE DE COMARMOND &amp;/OR MR VINCENT DESIRE NICOLAS LECORDIER &amp;/OR MR VIVEGAH THOPLAN &amp;/OR MRS SABRINA RAGAVOODOO|7790.1|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY||03/06/2026|177626.25|23372.4|01-06-2026 to 31-05-2027|POL-PI-Jun-21-15\\R5|POL-PI-Jun-21-15\\R5|1038.75|12779/21/R5 3601.902454|207750|-133220.05970149254|","-13812|-13812|1104.96|8|LA PRUDENCE LEASING FINANCE CO. LTD|-0.04|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||02/03/2026|12707.04|1105|01-01-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E2|0|MD11M00166/10/R5/EQ/2|13812|-12707.04|","27051|27051|-2164.08|8|LA PRUDENCE LEASING FINANCE CO. LTD|-0.08|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||14/04/2026|-24886.88|-2164|01-04-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E3|0|MD11M00166/10/R5/EQ/6|-27050.96|24886.91679999527|","37909|37909|-3032.75|8|LA PRUDENCE LEASING FINANCE CO. LTD|0.25|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-34876.57|-3033|01-04-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E6|0|MD11M00166/10/R5/EQ/8|-37909.32|34876.275600037145|","-21675|-21675|1734.04|8|LA PRUDENCE LEASING FINANCE CO. LTD|0.04|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/05/2026|19941.41|1734|01-05-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E5|0|MD11M00166/10/R5/EQ/7|21675.45|-19940.996000083043|","19196|19196|-1535.72|8|NEWREST (MAURITIUS) LTD|0.28|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-17660.74|-1536|01-06-2026 to 01-10-2026|POL-HEALTH-Dec-24-132\\R1|POL-HEALTH-Dec-24-132\\R1\\E3|0|MED/2024/01202/R1/EQ/7|-19196.46|17660.316800076682|","-6048|-6048|483.84|8|NEWREST (MAURITIUS) LTD|-0.16|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||10/02/2026|5564.16|484|01-02-2026 to 01-10-2026|POL-HEALTH-Dec-24-132\\R1|POL-HEALTH-Dec-24-132\\R1\\E2|0|MED/2024/01202/R1/EQ/6|6048|-5564.16|","-6447|-6447|959.67|15|MCB LEASING LIMITED ON LEASE TO JAG SERVICES LTD|-0.33|26.3||MUR|08/12/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/12/2025|5486.84|960|08-12-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E49|22.4|31069/23/R1/E12|6397.81|-5487.257055367943|","52031|52031|-7777.5|15|MCB LEASING LIMITED ON LEASE TO JAG SERVICES LTD|0.5|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||23/02/2026|-44253.98|-7778|01-01-2026 to 01-01-2027|POL-MVF-Jul-19-6113\\R7|POL-MVF-Jul-19-6113\\R7\\E2|-181.48|31069/23/R2/E4|-51850|44253.57174887203|","2|2|12938|15|PANACHE CO LTD|12937.8|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||14/09/2019|74114|0.200000000000728|01-07-2019 to 01-07-2020|POL-CAR-TPL(BC)-Jun-19-1024|POL-CAR-TPL(BC)-Jun-19-1024|802|MD07E00472/R12|86250|1.7027523778890779|","-110|-110|1.52|15|PANACHE AND COMPANY LIMITED|-0.48|0||MUR|10/06/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||30/06/2026|108.62|2|10-06-2026 to 30-06-2026|POL-CP-Jun-19-1040\\R6|POL-CP-Jun-19-1040\\R6\\E1|100.04||10.1|-108.48193208643545|","1|1|315|15|PANACHE CO LTD|315.15|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|MONEY||30/09/2019|1792|-0.149999999999977|01-07-2019 to 01-07-2020|POL-MON-Jun-19-1077|POL-MON-Jun-19-1077|7|5180/15/R5|2100|0.8504983388704319|","-1|-1|4703|15|PANACHE CO LTD|4702.35|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||30/09/2019|26756|0.649999999999636|01-07-2019 to 01-07-2020|POL-EL-Jun-19-1236|POL-EL-Jun-19-1236|109|5180/15/R5|31350|-0.8505038303824025|","-2|-2|8100|15|PANACHE CO LTD|8099.7|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||30/09/2019|46089|0.299999999999272|01-07-2019 to 01-07-2020|POL-PA-Jun-19-1304|POL-PA-Jun-19-1304|189|5180/15/R5|54000|-1.7010463378176381|","119807.99|119807.99|-102187.5|15|SCOTT &amp; CO LTD &amp;/OR RIVERSIDE HEALH LTD &amp;/OR SCOTT HEALTH LTD &amp;/OR BAGATELLE HEALTH LTD &amp;/OR GRAND BAIE FORME HEALTH LTD &amp;/OR THE BRANDHOUSE LTD &amp;/OR STANDARD PHARMACY LTD &amp;/OR BEAU VALLON HEALTH LTD &amp;/OR MOBISIL LTD &amp;/OR SCOTT TRIBECA HEALTH LTD &amp;/OR SCOTT AGROW LTD|-84278.57|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|TERRORISM &amp; SABOTAGE||09/04/2026|-584563.89|-17908.93|01-10-2025 to 01-10-2026|POL-TER&amp;SAB-Oct-19-1021\\R6|POL-TER&amp;SAB-Oct-19-1021\\R6\\E1|-5501.39||-681250|101980.75418162765|","-122866|-122866|102187.5|15|SCOTT &amp; CO LTD &amp;/OR RIVERSIDE HEALH LTD &amp;/OR SCOTT HEALTH LTD &amp;/OR BAGATELLE HEALTH LTD &amp;/OR GRAND BAIE FORME HEALTH LTD &amp;/OR THE BRANDHOUSE LTD &amp;/OR STANDARD PHARMACY LTD &amp;/OR BEAU VALLON HEALTH LTD &amp;/OR MOBISIL LTD &amp;/OR SCOTT TRIBECA HEALTH LTD &amp;/OR SCOTT AGROW LTD|83757.06|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|TERRORISM &amp; SABOTAGE||09/04/2026|582468.75|18430.44|01-10-2025 to 01-10-2026|POL-TER&amp;SAB-Oct-19-1021\\R7|POL-TER&amp;SAB-Oct-19-1021\\R7|3406.25|43624/16/R8|681250|-104527.79104477612|"]</t>
+  </si>
+  <si>
+    <t>["-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.31|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.30|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.158|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.157|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.156|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.155|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.154|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.153|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.152|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.151|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.150|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.149|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.148|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.147|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.93|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.92|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.91|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.90|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.89|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.88|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.87|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.86|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.85|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.84|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.83|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.82|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.311|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.310|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.309|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.308|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.307|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.306|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.305|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.304|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.303|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.302|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.301|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.300|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.17|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.16|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.15|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.14|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.13|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.12|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.11|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.10|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.9|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.8|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.7|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.6|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.41|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.40|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.39|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.38|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.37|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.36|Medical","-7529.76|94522|FON SING MARIE SANDRA PIT TSOU|30/09/2025|23164.95||01/08/25 to 31/07/26|MED/2024/00815|MED/2024/00815/R1|MED/2024/00815|23164.95|07/08/2025|JRNNHZ.250807.18|Medical","-12492.78|154944.97|Gaya Shyamsundur|30/09/2025|16428.91||01/08/25 to 31/07/26|MD08M01060|MD08M01060/R17|MD08M01060|16428.91|26/08/2025|JRNNHZ.250826.22|Medical","-5061.6|42580|COLLET-SERRET MARINE CELIA|30/11/2025|30014.72|Payment done after 30.06.2026|01/10/25 to 30/09/26|MED/2025/01440|MED/2025/01440/N|MED/2025/01440|30014.72|23/01/2026|JRNNHZ.260123.2|Medical","-6314.24|79328|SALEMOHAMED FAWZIA|30/11/2025|13801.66||01/10/25 to 30/09/26|MD06M00609|MD06M00609/R19|MD06M00609|13801.66|03/10/2025|JRNNHZ.251003.167|Medical","-9316.8|78040|BUCARD JOSEPHE MARIE CLAUDE|31/10/2025|14170.45||01/09/25 to 31/08/26|MED/2025/01312|MED/2025/01312/N|MED/2025/01312|14170.45|25/11/2025|JRNNHZ.251125.142|Medical","-5685.78|71572.3|BENZOU LTEE|31/12/2025|19267.44||01/11/25 to 31/10/26|MD18M01126|MD18M01126/R7|MD18M01126|19267.44|18/11/2025|JRNNHZ.251118.72|Medical","-14063.8|176197.6|VETOPHARMA LTD|31/12/2025|69323.69|Payment done after 30.06.2026|01/11/25 to 31/10/26|MED/2024/01200|MED/2024/01200/R1|MED/2024/01200|69323.69|13/01/2026|JRNNHZ.260113.134|Medical","-13858.46|171357.66|Rivaud Marie Josee|30/01/2026|62999.68|Payment done after 30.06.2026|01/12/25 to 30/11/26|MED/2023/01267|MED/2023/01267/R2|MED/2023/01267|62999.68|03/12/2025|JRNNHZ.251203.80|Medical","-21358.72|176800.64|CARR-BROWN ALAN|30/11/2025|46634.61||01/10/25 to 30/09/26|MED/2025/01409|MED/2025/01409/N|MED/2025/01409|46634.61|30/12/2025|JRNNHZ.251230.48|Medical","-20207.28|252591|COMPAGNIE MAURICIENNE DE TEXTILE LTEE|01/07/2026|232383.72||01/12/25 to 30/11/26|MD16M00967|MD16M00967/R9|MD16M00967|232383.72|31/05/2026|JRNNHZ.260531.156|Medical","-20207.28|252591|COMPAGNIE MAURICIENNE DE TEXTILE LTEE|01/08/2026|||01/12/25 to 30/11/26|MD16M00967|MD16M00967/R9|MD16M00967|232383.72|30/06/2026|JRNNHZ.260630.558|Medical","-4099.07|51638.43|BUSSIER Robert Emmanuel Marie Angelo|30/06/2026|20655.92||01/01/26 to 31/12/26|MD21M00507|MD21M00507/R5|MD21M00507|20655.92|15/01/2026|JRNNHZ.260115.177|Medical"]</t>
+  </si>
+  <si>
+    <t>["-1|-1|-28.04|15|SCOTT &amp; CO LTD &amp;/OR SCOTT HEALTH LTD &amp;/OR BAGATELLE HEALTH LTD &amp;/OR GRAND BAIE FORME HEALTH LTD &amp;/OR THE BRANDHOUSE LTD &amp;/OR STANDARD PHARMACY LTD &amp;/OR BEAU VALLON HEALTH LTD &amp;/OR MOBISIL LTD &amp;/OR TRIBECA HEALTH LTD|-28.14|0|Correction to be done by CBL amount not in aging|MUR|20/03/2024|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||13/06/2024|-159.55|0.100000000000001|20-03-2024 to 01-10-2024|POL-ARMISC-Jul-19-1112\\R5|POL-ARMISC-Jul-19-1112\\R5\\E2|-0.66|33954/19/R2/E8|-186.93|-0.850525081294312|","-17956|-17956|3578.65|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|894.27|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||18/05/2026|20362.5|2684.38|01-05-2026 to 30-04-2027|POL-EL-Mar-26-19\\R1|POL-EL-Mar-26-19\\R1|83.5|14246/26/R1|23857.65|-15271.991946919843|","-103484|-103484|38642|15|SBM BANK (MAURITIUS) LTD ON LEASE TO HIGHWAY PROPERTIES LTD|23185.21|195.07||MUR|10/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||08/05/2026|220068.02|15456.79|10-04-2026 to 01-04-2027|POL-MV-Apr-26-95|POL-MV-Apr-26-95|901.65|8591/26|257613.3|-88027.20119491313|","-118107|-118107|17579.51|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.490000000002328|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||11/05/2026|100527.45|17580|01-04-2026 to 30-04-2026|POL-F&amp;A-Mar-26-1018|POL-F&amp;A-Mar-26-1018|910.2|10767/26/N|117196.76|-100527.4840462408|","-983582|-983582|195955.58|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|48988.52|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||18/05/2026|1115487.22|146967.06|01-05-2026 to 30-04-2027|POL-CP-May-26-1008|POL-CP-May-26-1008|5072.3|13781/26/N|1306370.5|-836615.3299419845|","-11265|-11265|1683.84|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.16|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||11/05/2026|9581.04|1684|01-04-2026 to 30-04-2026|POL-LOP(F&amp;A)-Mar-26-3|POL-LOP(F&amp;A)-Mar-26-3|39.29|10767/26/N|11225.59|-9581.142062764982|","-2773|-2773|339.81|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.19|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||11/05/2026|2433.49|340|01-04-2026 to 30-04-2026|POL-PL-Mar-26-21|POL-PL-Mar-26-21|507.93|14246/26/N|2265.37|-2433.2267587350807|","-1528|-1528|228.35|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|0.35|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||11/05/2026|1299.34|228|01-04-2026 to 30-04-2026|POL-EL-Mar-26-19|POL-EL-Mar-26-19|5.33|14246/26/N|1522.36|-1299.6036630468222|","-48874|-48874|9740.63|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|2434.76|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||18/05/2026|55424.18|7305.87|01-05-2026 to 30-04-2027|POL-PA-Mar-26-17\\R1|POL-PA-Mar-26-17\\R1|227.28|14246/26/R1|64937.53|-41568.46883033957|","-1158|-1158|173.1|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|0.1|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||11/05/2026|984.92|173|01-04-2026 to 30-04-2026|POL-EE-Mar-26-8|POL-EE-Mar-26-8|4.04|14246/26/N|1153.98|-984.9029895856721|","-5001|-5001|747.58|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.42|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN||11/05/2026|4253.75|748|01-04-2026 to 30-04-2026|POL-M B-D-Mar-26-1003|POL-M B-D-Mar-26-1003|17.44|14246/26/N|4983.89|-4253.469327158976|","-55317|-55317|10950|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|2737.52|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||18/05/2026|62805.5|8212.48|01-05-2026 to 30-04-2027|POL-PL-Mar-26-21\\R1|POL-PL-Mar-26-21\\R1|755.5|14246/26/R1|73000|-47104.44432618584|","-3819|-3819|570.88|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.12|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||11/05/2026|3248.33|571|01-04-2026 to 30-04-2026|POL-PA-Mar-26-17|POL-PA-Mar-26-17|13.32|14246/26/N|3805.89|-3248.1513899471356|","-440|-440|197.03|15|ACBMS LTD|131.27|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||12/05/2026|1121.07|65.76|01-05-2026 to 01-05-2027|POL-EE-May-22-1007\\R4|POL-EE-May-22-1007\\R4|4.6|12079/22|1313.5|-374.22866246870495|","-400|-400|106.08|15|ACBMS LTD|71.1|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||12/05/2026|1103.6|34.98|01-05-2026 to 01-05-2027|POL-EL-May-22-28\\R4|POL-EL-May-22-28\\R4|502.48|12079/22|707.2|-364.9229548310297|","-6412|-6412|2874.45|15|ACBMS LTD|1916.45|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||12/05/2026|16355.62|958|01-05-2026 to 01-05-2027|POL-PA-May-22-18\\R4|POL-PA-May-22-18\\R4|67.07|12079/22|19163|-5453.554534122861|","-19672|-19672|8819.96|15|ACBMS LTD|5879.48|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||12/05/2026|50185.55|2940.48|01-05-2026 to 01-05-2027|POL-ARMISC-May-22-11\\R4|POL-ARMISC-May-22-11\\R4|205.81|12079/22|58799.7|-16731.4906624822|","-26497|-26497|2119.74|8|GAYA COLLECTIONS LIMITEE|-0.260000000000291|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/06/2026|24376.98|2120|01-06-2026 to 01-05-2027|POL-HEALTH-Aug-23-74\\R4|POL-HEALTH-Aug-23-74\\R4\\E1|0|MED/2023/00969/R3/EQ/1|26496.72|-24377.23759997464|","-140853|-140853|16786.56|8|GAYA COLLECTIONS LIMITEE|5596.22|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/05/2026|194514.44|11190.34|01-05-2026 to 01-05-2027|POL-HEALTH-Aug-23-74\\R4|POL-HEALTH-Aug-23-74\\R4|1469|MED/2023/00969/R3|209832|-129663.09869484763|","3953|3953|-474.36|12|BELLE RIVIERE HOTEL LTD|-474.72|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/05/2026|-3478.64|0.360000000000014|01-04-2026 to 01-05-2026|POL-HEALTH-Sep-21-95\\R4|POL-HEALTH-Sep-21-95\\R4\\E16|0|MED/2025/00947/EQ/40|-3953|3478.64|","-90048|-90048|7203.84|8|BELLE RIVIERE HOTEL LTD|-0.16|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/06/2026|82844.16|7204|01-05-2026 to 01-05-2027|POL-HEALTH-Sep-21-95\\R6|POL-HEALTH-Sep-21-95\\R6\\E2|0|MED/2025/00947/R1/EQ/2|90048|-82844.16|","16176|16176|-1294.08|8|BELLE RIVIERE HOTEL LTD|-0.08|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/06/2026|-14881.92|-1294|01-05-2026 to 01-05-2027|POL-HEALTH-Sep-21-95\\R6|POL-HEALTH-Sep-21-95\\R6\\E1|0|MED/2025/00947/R1/EQ/1|-16176|14881.92|","7164|7164|-859.68|12|BELLE RIVIERE HOTEL LTD|-859.36|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/05/2026|-6304.32|-0.32000000000005|01-03-2026 to 01-05-2026|POL-HEALTH-Sep-21-95\\R4|POL-HEALTH-Sep-21-95\\R4\\E15|0|MED/2025/00947/EQ/39|-7164|6304.32|","1876|1876|-225.12|12|BELLE RIVIERE HOTEL LTD|-0.12|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/04/2026|-1650.88|-225|01-03-2026 to 01-05-2026|POL-HEALTH-Sep-21-95\\R4|POL-HEALTH-Sep-21-95\\R4\\E14|0|MED/2025/00947/EQ/38|-1876|1650.88|","-1749046|-1749046|139007.04|8|BELLE RIVIERE HOTEL LTD|11584|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/07/2026|1610743.96|127423.04|01-05-2026 to 01-05-2027|POL-HEALTH-Sep-21-95\\R6|POL-HEALTH-Sep-21-95\\R6|12163|MED/2025/00947/R1|1737588|-1610094.9679481024|","-32934|-32934|4922.8|15|OSMAN DR REZAH|-0.2|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||30/06/2026|28010.71|4923|01-06-2026 to 01-06-2027|POL-ARMISC-May-20-1035\\R6|POL-ARMISC-May-20-1035\\R6|114.86|3601.902454|32818.65|-28011.12675630384|","-10906|-10906|1562.87|15|OSMAN DR REZAH|-0.13|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||30/06/2026|9342.72|1563|01-06-2026 to 01-06-2027|POL-F&amp;A-May-20-1193\\R6|POL-F&amp;A-May-20-1193\\R6|486.47|3601.902454|10419.12|-9343.071243279823|","123515|123515|-18462.61|15|PARTSIONATE LTD|0.39|0||MUR|11/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||29/06/2026|-105052.25|-18463|11-05-2026 to 01-05-2027|POL-MV-May-26-130|POL-MV-May-26-130\\E1|-430.79|11084/26|-123084.07|105052.36907324349|","38910|38910|-5816.1|15|PARTSIONATE LTD|-0.1|0||MUR|02/06/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||26/06/2026|-33093.58|-5816|02-06-2026 to 01-05-2027|POL-MV-May-26-132|POL-MV-May-26-132\\E1|-135.71|11100/26/N|-38773.97|33093.8521673784|","-590|-590|88.2|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|0.2|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||01/06/2026|501.86|88|01-05-2026 to 01-05-2027|POL-EE-May-23-1015\\R3|POL-EE-May-23-1015\\R3|2.06|3601.902454|588|-501.80896857946647|","-2768|-2768|339|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||01/06/2026|2428.91|339|01-05-2026 to 01-05-2027|POL-F&amp;A-May-20-1192\\R6|POL-F&amp;A-May-20-1192\\R6|507.91|3601.902454|2260|-2428.9889772427573|","-587|-587|87.75|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|-0.25|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN||01/06/2026|499.29|88|01-05-2026 to 01-05-2027|POL-M B-D-May-23-1003\\R3|POL-M B-D-May-23-1003\\R3|2.04|3601.902454|585|-499.255979149632|","1|1|399|15|ASSOCIATION SYNDICALE TROPICA BAIE|399.58|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||31/07/2019|2773|-0.580000000000041|01-07-2019 to 01-07-2020|POL-F&amp;A-Jun-19-1353|POL-F&amp;A-Jun-19-1353|509|19391/18/R1|2663|0.8742118537200505|","-5809|-5809|868.35|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|0.35|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||01/06/2026|4940.91|868|01-05-2026 to 01-05-2027|POL-PL-May-20-1184\\R6|POL-PL-May-20-1184\\R6|20.26|3601.902454|5789|-4940.688863986119|","-67587|-67587|14755.47|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD|4653.23|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||31/08/2020|83958.61|10102.24|01-07-2020 to 01-07-2021|POL-LOP(F&amp;A)-Jul-19-1109\\R1|POL-LOP(F&amp;A)-Jul-19-1109\\R1|344.28|29448/16|98369.8|-57484.30795353611|","-21299|-21299|3376.13|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|192.5|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||31/08/2020|19210.17|3183.63|01-07-2020 to 01-07-2021|POL-EE-Jul-19-1181\\R1|POL-EE-Jul-19-1181\\R1|78.8|29448/16|22507.5|-18115.29160730177|","-52322|-52322|11250|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|3429|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||31/08/2020|64012.5|7821|01-07-2020 to 01-07-2021|POL-PL-Jul-19-1299\\R1|POL-PL-Jul-19-1299\\R1|262.5|29448/16|75000|-44501.07324364723|","-8852|-8852|2883.87|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|1560.7|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||31/08/2020|16409.22|1323.17|01-07-2020 to 01-07-2021|POL-EL-Jul-19-1326\\R1|POL-EL-Jul-19-1326\\R1|67.29|29448/16|19225.8|-7528.831070606108|","170383|170383|25569.86|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD|50914.98|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||31/08/2020|145992.53|-25345.12|01-07-2020 to 01-07-2021|POL-F&amp;A-Jul-19-1410\\R1|POL-F&amp;A-Jul-19-1410\\R1|1096.64|29448/16|170465.75|144988.91767006743|","-20323|-20323|6724.8|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|3686.8|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||31/08/2020|38264.12|3038|01-07-2020 to 01-07-2021|POL-PA-Jul-19-1389\\R1|POL-PA-Jul-19-1389\\R1|156.92|29448/16/R4|44832|-17285.182901923406|","-1452|-1452|217.05|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|217.09|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN||19/12/2025|1235.04|-0.039999999999992|01-10-2025 to 01-10-2026|POL-M B-D-Dec-19-1066\\R6|POL-M B-D-Dec-19-1066\\R6|5.06|2595/17|1447.03|-1234.963452678553|","-58|-58|7373.44|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|7314.34|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||03/05/2021|42454.85|59.1000000000004|01-01-2021 to 01-01-2022|POL-F&amp;A-Dec-19-1623\\R1|POL-F&amp;A-Dec-19-1623\\R1|672.04|2595/17/R4 voucher not ok|49156.25|-49.41733501189786|","-987|-987|147.52|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|147.05|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||19/12/2025|839.38|0.469999999999999|01-10-2025 to 01-10-2026|POL-EL-Dec-19-1533\\R6|POL-EL-Dec-19-1533\\R6|3.44|2595/17|983.46|-839.4650521836052|","-17425|-17425|2604.6|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|2604.23|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||19/12/2025|14820.17|0.369999999999891|01-10-2025 to 01-10-2026|POL-PL-Dec-19-1523\\R6|POL-PL-Dec-19-1523\\R6|60.77|2595/17|17364|-14820.365620320958|","-57604|-57604|8535.72|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|8535.44|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||19/12/2025|49068.24|0.280000000000655|01-10-2025 to 01-10-2026|POL-F&amp;A-Dec-19-1623\\R6|POL-F&amp;A-Dec-19-1623\\R6|699.17|2595/17|56904.79|-49068.27407282416|","-2785|-2785|408.75|15|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|-0.25|50||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||27/01/2026|2375.79|409|01-02-2026 to 01-02-2027|POL-MV-Dec-24-1525\\R1|POL-MV-Dec-24-1525\\R1|9.54|31164/22|2725|-2376.18247538193|","-947|-947|786393.6|8|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|786318.01|0||MUR|01/10/2022|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/01/2023|9112335.4|75.589999999851|01-10-2022 to 01-10-2023|POL-HEALTH-Nov-21-120\\R1|POL-HEALTH-Nov-21-120\\R1|68809|MED/2021/00123/R1\nMED/2021/00123/R1/EQ/3\nMED/2021/00123/R1/EQ/4|9829920|-871.7666302209102|","-89390|-89390|13346.85|15|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|-0.15|100||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||01/06/2026|76043.58|13347|01-06-2026 to 01-06-2027|POL-MV-Dec-24-1523\\R1|POL-MV-Dec-24-1523\\R1|311.43|31169/22|88979|-76043.21420313114|","-2266447|-2266447|1031407.49|15|THE GENERAL CONSTRUCTION COMPANY LIMITED|694454.94|36900||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||28/04/2026|5905608.78|336952.55|01-04-2026 to 01-04-2027|POL-MVF-May-19-1121\\R7|POL-MVF-May-19-1121\\R7|24066.37|MT9900043297/R26/9151/18/ 13764/23/ 13092/25|6876049.9|-1929467.76851147|"]</t>
+  </si>
+  <si>
+    <t>["-84944|-84944|8462.4|8|DESVAUX DE MARIGNY-MONTOCCHIO MARIE PASCALE ANNE MRS|2539.12|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|97717.6|5923.28|01-05-2026 to 01-05-2027|POL-HEALTH-Jul-21-75\\R5|POL-HEALTH-Jul-21-75\\R5|400|MD21M00643/0/R5|105780|-78174.08|","-65884|-65884|11246.4|12|CHEUNG WILLY SOON MR|3374.32|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||27/04/2026|82873.6|7872.08|01-03-2026 to 01-03-2027|POL-HEALTH-Mar-26-26|POL-HEALTH-Mar-26-26|400|MED/2026/00365|93720|-58011.520000000004|","-27715|-27715|4703.04|12|RAMPUTH NEELESH MR|1410.88|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||16/04/2026|34888.96|3292.16|01-03-2026 to 01-03-2027|POL-HEALTH-Apr-26-28|POL-HEALTH-Apr-26-28|400|MED/2026/00315|39192|-24422.80072741968|","-54338|-54338|7197.12|12|BOODIAH MAUREEN VIVIANNA MRS|719.88|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/04/2026|53178.88|6477.24|01-04-2026 to 01-04-2027|POL-HEALTH-Apr-26-32|POL-HEALTH-Apr-26-32|400|MED/2026/00362|59976|-47860.63968199285|","-36325|-36325|8138.25|15|COMPTOIR OUEST OI LTEE|2718.72|100||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||13/05/2026|46406.64|5419.53|01-05-2026 to 01-05-2027|POL-MV-Apr-25-150\\R1|POL-MV-Apr-25-150\\R1|189.89|11301/25|54255|-30905.208498907963|","-62427|-62427|8275.56|12|NOMBRO MARY LYSIE IVY MRS|1654.6|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||04/06/2026|61087.44|6620.96|01-06-2026 to 01-06-2027|POL-HEALTH-Jul-23-49\\R3|POL-HEALTH-Jul-23-49\\R3|400|MED/2023/00781/R3|68963|-54978.96020760348|","-43008|-43008|4165.12|8|PRO WIRE ELECTRICAL &amp; MECHANICAL LTD|757.32|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/06/2026|48398.88|3407.8|01-06-2026 to 01-06-2027|POL-HEALTH-Jul-22-68\\R4|POL-HEALTH-Jul-22-68\\R4|500|MED/2022/00714/R4|52064|-39600.0881028841|","-18666|-18666|2775.13|15|MEDLOG (MAURITIUS) LTD|0.13|0||MUR|24/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||20/05/2026|15890.48|2775|24-04-2026 to 31-07-2026|POL-ARM(P&amp;M)-Jul-21-3\\R4|POL-ARM(P&amp;M)-Jul-21-3\\R4\\E2|164.75|P/10/6D99/21/3262/000/01|18500.86|-15890.812016323067|","-59758|-59758|8902.5|15|SPICE FINANCE LTD ON FINANCIAL LEASE TO G. DE VILLIERS PAINT CONTRACTORS LTD|-0.5|200||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||05/05/2026|50855.23|8903|01-05-2026 to 01-05-2027|POL-MV-Apr-26-119|POL-MV-Apr-26-119|207.73|18193/25|59350|-50855.45977633354|","-89888|-89888|13435.2|12|SAWMYNADEN KISNASAMY POULAY MR|2687.24|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|98924.8|10747.96|01-04-2026 to 01-04-2027|POL-HEALTH-Apr-26-41|POL-HEALTH-Apr-26-41|400|MED/2026/00453|111960|-79139.84|","-33338.5|-33338.5|5286.24|12|HUET LOUISE LILETTE NICOLE|1321.86|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|39165.76|3964.38|01-05-2026 to 01-05-2027|POL-HEALTH-May-26-45|POL-HEALTH-May-26-45|400|MED/2026/00429|44052|-29373.879460091783|","-71848|-71848|10680.48|12|SOORJUN SOTEEHALL MANISHA MRS|2097.77|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||04/06/2026|78723.52|8582.71|01-05-2026 to 01-05-2027|POL-HEALTH-May-26-46|POL-HEALTH-May-26-46|400|MED/2026/00515|89004|-63264.814381459444|","-449|-449|52.21|15|IKO (MAURITIUS) HOTEL LIMITED T/A ANANTARA MAURITIUS RESORTS &amp; VILLAS|0.21|0||MUR|15/05/2026|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||25/06/2026|397.09|52|15-05-2026 to 01-01-2027|POL-FID-Aug-19-1061\\R6|POL-FID-Aug-19-1061\\R6\\E2|101.22|1595/26/N|348.08|-396.82486089472513|","-23536|-23536|3500.34|15|MERIDIS FINANCIAL SOLUTIONS LTD|0.34|0||MUR|04/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY||18/06/2026|20035.27|3500|04-05-2026 to 30-04-2027|POL-F-PI-Jun-26-23|POL-F-PI-Jun-26-23|200|3601.902454 16950/26/N|23335.61|-20035.601997143902|","-71896|-71896|5719.68|8|LABELLE-VICTOIRE MARIE CINDY ANABELLE MRS|0|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/07/2026|66176.32|5719.68|01-06-2026 to 01-06-2027|POL-HEALTH-Jun-26-60|POL-HEALTH-Jun-26-60|400|MED/2026/00624|71496|-66176.32|","-93564|-93564|44603.52|8|VISIONWAY LTD|37170.16|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/09/2025|516842.13|7433.36|01-09-2025 to 01-09-2026|POL-HEALTH-Sep-19-3082\\R6|POL-HEALTH-Sep-19-3082\\R6|3901.65|MD16M00704/5/R4|557544|-86130.89628768162|","-75385|-75385|11250.05|15|MR RIVALLAND CHRISTIAN XAVIER|0.05|122.19||MUR|09/02/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||11/05/2026|64134.94|11250|09-02-2026 to 01-05-2027|POL-MV-Feb-26-32|POL-MV-Feb-26-32|262.5|3064/26|75000.3|-64134.94850765385|","-230178.79|-230178.79|22270.08|8|QOVOLTIS LIMITEE|3983.88|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/05/2026|258054.92|18286.2|01-05-2026 to 01-05-2027|POL-HEALTH-Apr-25-44\\R1|POL-HEALTH-Apr-25-44\\R1|1949|MED/2025/00586/R1|278376|-211892.5148993019|","5709|5709|-682.69|12|ACENSI (MAURITIUS) LTD|0.31|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/06/2026|-5026.29|-683|01-05-2026 to 01-06-2026|POL-HEALTH-Jun-25-54|POL-HEALTH-Jun-25-54\\E10|-19.92|MED/2022/00742/R3/EQ/11|-5689.06|5026.307608364366|","-56714|-56714|7529.76|8|FON SING MARIE SANDRA PIT TSOU MRS|3011.6|0||MUR|01/08/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH|Mise en demeure|08/08/2025|86992.24|4518.16|01-08-2025 to 01-08-2026|POL-HEALTH-Sep-24-66\\R1|POL-HEALTH-Sep-24-66\\R1|400|MED/2024/00815/R1|94122|-52196.08027083642|","-30957|-30957|12352.4|8|GAYA SHYAMSUNDUR MR|12352.8|0||MUR|01/08/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/10/2025|142452.6|-0.400000000003274|01-08-2025 to 01-08-2026|POL-HEALTH-Aug-23-80\\R2|POL-HEALTH-Aug-23-80\\R2|400|MD08M01060/13/R4|154405|-28486.839173153323|","-19156|-19156|5061.6|12|COLLET-SERRET MARINE CELIA MRS|2784.08|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/01/2026|37518.4|2277.52|01-10-2025 to 01-10-2026|POL-HEALTH-Jul-25-88|POL-HEALTH-Jul-25-88|400|MED/2025/01440|42180|-16878.874363550964|","-15864|-15864|6314.24|8|SALEMOHAMED FAWZIA|5683.2|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||09/10/2025|73013.76|631.039999999999|01-10-2025 to 01-10-2026|POL-HEALTH-Sep-19-3130\\R6|POL-HEALTH-Sep-19-3130\\R6|400|MD06M00609/15/R4|78928|-14601.279354578459|","-23412|-23412|9316.8|12|BUCARD JOSEPHE MARIE CLAUDE MRS|7453.24|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/11/2025|68723.2|1863.56|01-09-2025 to 01-09-2026|POL-HEALTH-Sep-25-102|POL-HEALTH-Sep-25-102|400|FQ/2025/01444|77640|-20616.96|","-21473|-21473|5685.76|8|BENZOU LTD|4548.24|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/11/2025|65886.24|1137.52|01-11-2025 to 01-11-2026|POL-HEALTH-Oct-19-3194\\R6|POL-HEALTH-Oct-19-3194\\R6|500|MD18M01126/2/R5|71072|-19767.160782428884|","-58750.35|-58750.35|14063.84|8|VETOPHARMA LTD|9374.3|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/01/2026|162134.16|4689.54|01-11-2025 to 01-11-2026|POL-HEALTH-Nov-24-125\\R1|POL-HEALTH-Nov-24-125\\R1|400|MED/2024/01200/R1|175798|-54060.9918782052|","-51348|-51348|13660.8|8|RIVAUD MARIE JOSEE MRS|9562.36|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||03/12/2025|157499.2|4098.44|01-12-2025 to 01-12-2026|POL-HEALTH-Nov-23-131\\R2|POL-HEALTH-Nov-23-131\\R2|400|MED/2023/01267/R2|170760|-47249.76|","-35320|-35320|21142.08|12|CARR-BROWN ALAN|19027.52|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/12/2025|155441.92|2114.56|01-10-2025 to 01-10-2026|POL-HEALTH-Nov-25-149|POL-HEALTH-Nov-25-149|400|MED/2025/01409|176184|-31091.20086984098|","-1429694|-1429694|227140.8|8|COMPAGNIE MAURICIENNE DE TEXTILE LTEE|151420.28|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||23/12/2025|2631994.02|75720.5199999999|01-12-2025 to 01-12-2026|POL-HEALTH-May-19-2565\\R47|POL-HEALTH-May-19-2565\\R47|19874.82|MD16M00967/4/R5|2839260|-1316113.5431976167|","-51638|-51638|4099.04|8|BUSSIER ROBERT EMMANUEL MARIE ANGELO|0.04|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH|Mise en demeure|15/01/2026|47538.96|4099|01-01-2026 to 01-01-2027|POL-HEALTH-Mar-21-13\\R5|POL-HEALTH-Mar-21-13\\R5|400|MD21M00507/0/R5|51238|-47538.96|"]</t>
+  </si>
+  <si>
+    <t>["-6299|-6299|-756|12|DUCRAY LENOIR LTD|-1511.76|0|Correction to be done by CBL amount not in aging|MUR|01/03/2019|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/07/2019|-5543|755.76|01-03-2019 to 01-04-2019|POL-HEALTH-Jun-19-2694|POL-HEALTH-Jun-19-2694|0|MD08M01077/MEDC/R11/E0002 MD08M01077/MEDC/R11/E0003 MD08M01077/MEDC/R11/E0004|-6299|-5543|","-5370|-5370|429.6|8|DUCRAY LENOIR LTD|-0.4|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||22/06/2026|4940.4|430|01-05-2026 to 01-03-2027|POL-HEALTH-Jun-19-2722\\R50|POL-HEALTH-Jun-19-2722\\R50\\E3|0|MD08M01077/13/R5/EQ/6|5370|-4940.4|","5208|5208|-416.64|8|DUCRAY LENOIR LTD|0.36|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/06/2026|-4791.36|-417|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2722\\R50|POL-HEALTH-Jun-19-2722\\R50\\E5|0|MD08M01077/13/R5/EQ/8|-5208|4791.36|","-15282|-15282|2269.4|15|DUCRAY LENOIR LTD &amp;/OR DUCRAY LENOIR INTERNATIONAL LTD &amp;/OR MEDLIFE SUPPLIES LTD|0.4|0||MUR|01/01/2025|MAURITIUS UNION ASSURANCE CO LTD|MARINE ANNUAL POLICY||27/05/2026|13012.89|2269|01-01-2025 to 01-01-2026|POL-AP-Dec-19-1062\\R6|POL-AP-Dec-19-1062\\R6\\E1|152.95|31535/18/R7/E1|15129.34|-13012.643064619242|","10155|10155|6596.76|12|DUCRAY LENOIR LTD|7815.36|0|Correction to be done by CBL amount not in aging|MUR|01/04/2019|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/07/2019|48376.24|-1218.6|01-04-2019 to 01-04-2020|POL-HEALTH-May-19-1518|POL-HEALTH-May-19-1518|0|NO DOCS|54973|8936.4|","1602|1602|192.24|12|DUCRAY LENOIR LTD|384.48|0|Correction to be done by CBL amount not in aging|MUR|01/03/2019|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/06/2019|1409.76|-192.24|01-03-2019 to 01-03-2020|POL-HEALTH-May-19-1003|POL-HEALTH-May-19-1003|0|MD10M00019/R10|1602|1409.76|","-5458|-5458|-655|12|DUCRAY LENOIR LTD|-1309.92|0|Correction to be done by CBL amount not in aging|MUR|01/03/2019|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/07/2019|-4803|654.92|01-03-2019 to 01-04-2019|POL-HEALTH-Jun-19-2695|POL-HEALTH-Jun-19-2695|0|MD10M00019/MCSGP/R10/E0006 MD10M00019/MCSGP/R10/E0004 MD10M00019/MCSGP/R10/E0005 MD10M00019/MCSGP/R10/E0003|-5458|-4803|","-1175990|-1175990|140137.92|8|DUCRAY LENOIR LTD|-0.0799999999813736|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||22/05/2026|1624287.08|140138|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2722\\R50|POL-HEALTH-Jun-19-2722\\R50|12701|MD08M01077/13/R5 - MD10M00019/12/R5|1751724|-1082588.0177447044|","-115753|-115753|9195.84|8|DUCRAY LENOIR INTERNATIONAL LTD|-0.16|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/05/2026|106557.16|9196|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2698\\R51|POL-HEALTH-Jun-19-2698\\R51|805|MD19M00510/2/R5|114948|-106557.16|","-213|-213|16.88|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|-0.12|0||MUR|14/08/2024|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||04/11/2024|196.07|17|14-08-2024 to 01-07-2025|POL-CP-Jul-23-8\\R1|POL-CP-Jul-23-8\\R1\\E2|100.39|19358/23|112.56|-196.1160366283165|","-48350|-48350|7212.33|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|0.33|0||MUR|06/03/2025|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||04/06/2025|41138.15|7212|06-03-2025 to 01-07-2025|POL-CP-Jul-23-8\\R1|POL-CP-Jul-23-8\\R1\\E4|268.29|19358/23|48082.19|-41137.74160049704|","-380|-380|656.95|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD|600.25|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||26/08/2024|3738.02|56.7|01-07-2024 to 01-07-2025|POL-ARMISC-Jul-23-23\\R1|POL-ARMISC-Jul-23-23\\R1|15.32|17111/23/N/E6|4379.65|-323.1984746198495|","-6643.98|-6643.98|21304.23|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|20311.45|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||26/08/2024|121221.13|992.779999999999|01-07-2024 to 01-07-2025|POL-EL-Jul-23-1039\\R1|POL-EL-Jul-23-1039\\R1|497.11|17111/23/R1|142028.25|-5650.859350907094|","-4424|-4424|1653|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|991.78|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||05/08/2025|9405.57|661.22|01-07-2025 to 01-07-2026|POL-FID-Jul-23-10\\R2|POL-FID-Jul-23-10\\R2|38.57|17111/23/R1|11020|-3762.714499252616|","-6556|-6556|1966.76|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR MR VINCENT LAGARDE &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD &amp;/OR THE HOUSE CANTEEN LTD|986.9|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|MONEY||05/08/2025|11190.87|979.86|01-07-2025 to 01-07-2026|POL-MON-Jul-23-6\\R2|POL-MON-Jul-23-6\\R2|45.93|17111/23/R1|13111.7|-5576.030312449887|","-1952|-1952|276.8|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|-0.2|0||MUR|13/08/2024|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||28/01/2025|1675|277|13-08-2024 to 01-07-2025|POL-CP-Jul-23-8\\R1|POL-CP-Jul-23-8\\R1\\E1|106.46|19358/23|1845.34|-1675.1716364381596|","-948865|-948865|251449.49|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|109616.49|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||05/08/2025|1431247.57|141833|01-07-2025 to 01-07-2026|POL-CP-Jul-23-8\\R2|POL-CP-Jul-23-8\\R2|6367.13|19358/23|1676329.93|-807073.8089410163|","-1054|-1054|1496.25|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|1338.96|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||26/08/2024|8513.67|157.29|01-07-2024 to 01-07-2025|POL-FID-Jul-23-10\\R1|POL-FID-Jul-23-10\\R1|34.92|17111/23/R1|9975|-896.4515380742304|","-39859|-39859|127825.41|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|121867.84|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||26/08/2024|727326.58|5957.56999999998|01-07-2024 to 01-07-2025|POL-PA-Jul-23-1051\\R1|POL-PA-Jul-23-1051\\R1|2982.59|17111/23/R1|852169.4|-33901.00296933181|","-813|-813|106.6|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD|-0.4|0||MUR|01/09/2023|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||20/03/2024|706.57|107|01-09-2023 to 01-07-2024|POL-CP-Jul-23-8|POL-CP-Jul-23-8\\E2|102.49|19358/23/N/E3|710.68|-706.4222856229325|","-400|-400|83.61|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD|38.33|0||MUR|01/09/2023|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||20/03/2024|575.75|45.28|01-09-2023 to 01-07-2024|POL-ARMISC-Jul-23-23|POL-ARMISC-Jul-23-23\\E1|101.95|17111/23/E4|557.41|-349.27808784275663|","-4178|-4178|2285.71|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR MR VINCENT LAGARDE &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|1661.15|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|MONEY||26/08/2024|13005.66|624.559999999999|01-07-2024 to 01-07-2025|POL-MON-Jul-23-6\\R1|POL-MON-Jul-23-6\\R1|53.29|17111/23/R1|15238.08|-3553.4845785564016|","-4272|-4272|638.47|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD|0.47|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||05/08/2025|3632.89|638|01-07-2025 to 01-07-2026|POL-ARMISC-Jul-23-23\\R2|POL-ARMISC-Jul-23-23\\R2|14.9|17111/23/N/E6|4256.46|-3633.434334731795|","-861|-861|113.81|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|-0.19|0||MUR|30/01/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||29/05/2025|747.6|114|30-01-2025 to 01-07-2025|POL-EL-Jul-23-1039\\R1|POL-EL-Jul-23-1039\\R1\\E1|102.66|17111/23/R1/E1|758.75|-747.2441694431224|","-14622|-14622|5827.5|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|3642.5|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||26/08/2024|33158.51|2185|01-07-2024 to 01-07-2025|POL-PL-Jul-23-1040\\R1|POL-PL-Jul-23-1040\\R1|136.01|17111/23/R1|38850|-12436.351737969595|","-12923|-12923|1916.71|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|-0.29|0||MUR|17/03/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||26/05/2026|11006.09|1917|17-03-2026 to 01-07-2026|POL-CP-Jul-23-8\\R2|POL-CP-Jul-23-8\\R2\\E4|144.72||12778.08|-11006.260335995295|","-25014|-25014|6118.95|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD &amp;/OR THE HOUSE CANTEEN LTD &amp;/OR AVA DCB LTD|2380.07|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||05/08/2025|34816.81|3738.88|01-07-2025 to 01-07-2026|POL-PL-Jul-23-1040\\R2|POL-PL-Jul-23-1040\\R2|142.76|19358/23|40793|-21274.98513133749|","-696|-696|89.03|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|0.03|0||MUR|31/03/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||04/06/2025|606.55|89|31-03-2025 to 01-07-2025|POL-EL-Jul-23-1039\\R1|POL-EL-Jul-23-1039\\R1\\E2|102.08|17111/23/R1|593.5|-606.9162425601656|","-4581|-4581|684.75|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|-0.25|0||MUR|30/01/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||29/05/2025|3896.23|685|30-01-2025 to 01-07-2025|POL-PA-Jul-23-1051\\R1|POL-PA-Jul-23-1051\\R1\\E1|15.98|17111/23/R1|4565|-3896.2470104650097|","-135920.99|-135920.99|103307.13|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD &amp;/OR AVA ENERGY LTD &amp;/OR THE HOUSE CANTEEN LTD|82990.12|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||05/08/2025|587817.58|20317.01|01-07-2025 to 01-07-2026|POL-PA-Jul-23-1051\\R2|POL-PA-Jul-23-1051\\R2|2410.5|17111/23/R1|688714.21|-115603.95143881369|","-11|-11|1.72|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR MR VINCENT LAGARDE &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|-0.28|0||MUR|30/01/2025|MAURITIUS UNION ASSURANCE CO LTD|MONEY||29/05/2025|9.77|2|30-01-2025 to 01-07-2025|POL-MON-Jul-23-6\\R1|POL-MON-Jul-23-6\\R1\\E1|0.04|17111/23/R1|11.45|-9.353350739773717|","-26119|-26119|17226.53|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD &amp;/OR AVA ENERGY LTD &amp;/OR THE HOUSE CANTEEN LTD|13321.94|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||05/08/2025|98018.96|3904.59|01-07-2025 to 01-07-2026|POL-EL-Jul-23-1039\\R2|POL-EL-Jul-23-1039\\R2|401.96|17111/23/R1|114843.53|-22214.814794401063|"]</t>
+  </si>
+  <si>
+    <t>["-115.96|1946|DUCRAY LENOIR LTD|01/06/2026|1830.04||01/03/26 to 28/02/27|MD10M00019|MD10M00019/R17|MD10M00019|1830.04|30/04/2026|JRNNHZ.260430.481|Medical","-23240.64|302709.34|DUCRAY LENOIR LTD|01/06/2026|279468.7||01/03/26 to 28/02/27|MD08M01077|MD08M01077/R18|MD08M01077|279468.7|30/04/2026|JRNNHZ.260430.477|Medical","-57.98|723|DUCRAY LENOIR LTD|01/04/2026|665.02||01/03/25 to 28/02/26|MD10M00019|MD10M00019/R16|MD10M00019|665.02|28/02/2026|JRNNHZ.260228.226|Medical","-10845.68|135571|DUCRAY LENOIR LTD|01/04/2026|61016.14||01/03/25 to 28/02/26|MD08M01077|MD08M01077/R17|MD08M01077|61016.14|28/02/2026|JRNNHZ.260228.222|Medical","-57.98|723|DUCRAY LENOIR LTD|01/03/2026|665.02||01/03/25 to 28/02/26|MD10M00019|MD10M00019/R16|MD10M00019|665.02|31/01/2026|JRNNHZ.260131.230|Medical","-1559|233.1|DUCRAY LENOIR LTD|26/09/2025|||01/01/25 to 31/12/25||26102/21/R3/E6||-1325.9|26/09/2025|JRNI.250926.112|Motor","-57.98|723|DUCRAY LENOIR LTD|01/02/2026|665.02||01/03/25 to 28/02/26|MD10M00019|MD10M00019/R16|MD10M00019|665.02|31/12/2025|JRNNHZ.251231.483|Medical","-1258.8|15735|DUCRAY LENOIR INTERNATIONAL LTD|01/08/2026|||01/03/26 to 28/02/27|MD19M00510|MD19M00510/R7|MD19M00510|14476.2|30/06/2026|JRNNHZ.260630.613|Medical","-766.32|9579|DUCRAY LENOIR INTERNATIONAL LTD|01/07/2026|8812.68||01/03/26 to 28/02/27|MD19M00510|MD19M00510/R7|MD19M00510|8812.68|31/05/2026|JRNNHZ.260531.211|Medical","-57.98|723|DUCRAY LENOIR LTD|01/08/2026|||01/03/26 to 28/02/27|MD10M00019|MD10M00019/R17|MD10M00019|665.02|30/06/2026|JRNNHZ.260630.470|Medical","-57.98|723|DUCRAY LENOIR LTD|01/07/2026|665.02||01/03/26 to 28/02/27|MD10M00019|MD10M00019/R17|MD10M00019|665.02|31/05/2026|JRNNHZ.260531.68|Medical","-21194.16|264927|DUCRAY LENOIR LTD|01/08/2026|||01/03/26 to 28/02/27|MD08M01077|MD08M01077/R18|MD08M01077|243732.84|30/06/2026|JRNNHZ.260630.467|Medical","-13753.2|171915|DUCRAY LENOIR LTD|01/07/2026|158161.8||01/03/26 to 28/02/27|MD08M01077|MD08M01077/R18|MD08M01077|158161.8|31/05/2026|JRNNHZ.260531.64|Medical","-251449.5|1682697|NATEC MEDICAL LTD|01/10/2025|792773.85||01/07/25 to 30/06/26||19358/23/R2||792773.85|22/07/2025|JRNI.250722.446|Non-Motor Corporate","-130910.83|876293.97|NATEC MEDICAL LTD|01/10/2025|186105.45||01/07/25 to 30/06/26||17111/23/R2||186105.45|19/07/2025|JRNI.250719.27|Non-Motor Corporate","-7684.95|51512|NATEC MEDICAL LTD|01/08/2026|||01/07/25 to 30/06/26||19358/23/R2/E5||43827.05|28/05/2026|JRNI.260528.560|Non-Motor Corporate","-1916.7|12923|NATEC MEDICAL LTD|01/07/2026|11006.3||01/07/25 to 30/06/26||19358/23/R2/E4||11006.3|15/04/2026|JRNI.260415.301|Non-Motor Corporate","-9152|1368|Bank of Mauritius|29/09/2025|||01/07/25 to 30/06/26||19120/25/N/E1||-7784|29/09/2025|JRNI.250929.287|Travel","-23068.5|155078|Kasa Textile &amp; Co Ltd|01/04/2026|73338.2|Payment done after 30.06.2026|01/01/26 to 31/12/26||26063/21/R4||73338.2|06/01/2026|JRNI.260106.450|Motor","-3143.28|39291|Kasa Textile &amp; Co Ltd|01/07/2026|20749.66||01/03/26 to 28/02/27|MD08M01085|MD08M01085/R18|MD08M01085|20749.66|31/05/2026|JRNNHZ.260531.65|Medical","-3260|40750|Kasa Textile &amp; Co Ltd|01/08/2026|||01/03/26 to 28/02/27|MD08M01085|MD08M01085/R18|MD08M01085|37490|30/06/2026|JRNNHZ.260630.468|Medical","-6750|45358|ERC Levage Ltee|12/06/2026|38608|Payment done after 30.06.2026|11/05/26 to 11/05/26|POL-GIT-May-26-18|11642/26/N|POL-GIT-May-26-18|38608|12/05/2026|JRNI.260512.238|Inland Transit","-1024.8|7156|Royal Car Rental Ltd|01/02/2026|6131.2||17/10/25 to 31/10/26||32587/25/N||6131.2|20/11/2025|JRNI.251120.318|Non-Motor Corporate","-1292958.7|8666994|Royal Car Rental Ltd|15/10/2026|2938487.62||01/01/26 to 31/12/26||31162/23/R2||5167497.43|06/01/2026|JRNI.260106.423|Motor","-5260.05|35290|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/09/2026|||01/05/25 to 30/04/26||9314/08/R17/E2||30029.95|29/06/2026|JRNI.260629.452|Non-Motor Corporate","-2730.9|18570|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/08/2026|||01/05/26 to 30/04/27||22405/20/R6||15839.1|13/05/2026|JRNI.260513.103|Non-Motor Corporate","-374330.06|2504767.95|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/08/2026|||01/05/26 to 30/04/27||9314/08/R18||2130437.89|25/05/2026|JRNI.260525.474|Non-Motor Corporate","-22567.5|151477|TAYELAMAY &amp; SONS ENTERPRISE LTD|01/06/2026|128909.5||11/07/25 to 11/09/26||7049/26/N||128909.5|26/03/2026|JRNI.260326.415|Non-Motor Corporate","-37642|5726.65|Lavastone Ltd &amp;/or Subsidiaries|09/01/2026|100||01/10/25 to 30/09/26||33502/19/R6/E1||-31915.35|08/01/2026|JRNI.260108.274|Non-Motor Corporate","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.38|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.37|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.36|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|3327.96||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|3327.96|10/03/2026|JRNNHZ.260310.35|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.252|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.251|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|57.63||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|57.63|25/06/2026|JRNNHZ.260625.250|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|10/03/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.248|Medical","-68.64|572.05|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/03/2026|75.26||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E78|MED/2025/01055|75.26|19/02/2026|JRNNHZ.260219.82|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/03/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.61|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.60|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.59|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|1624.17||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.17|19/02/2026|JRNNHZ.260219.58|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.57|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/10/2025|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.56|Medical","-367.1|3059.17|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|2692.07||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E74|MED/2025/01055|2692.07|19/02/2026|JRNNHZ.260219.37|Medical","-3396.48|28304|HARDY HENRY &amp; CIE LTEE|01/08/2026||Payment done after 30.06.2026|01/10/25 to 30/06/26|MED/2023/01269|MED/2023/01269/R2|MED/2023/01269|24907.52|30/06/2026|JRNNHZ.260630.789|Medical","-62149.68|517914|Hardy Henry Services Ltd|01/08/2026|||01/10/25 to 30/06/26|MD18M01064|MD18M01064/R7|MD18M01064|455764.32|30/06/2026|JRNNHZ.260630.599|Medical","-1014.36|8453|HARDY HENRY &amp; CIE LTEE|01/08/2026|||01/10/25 to 30/06/26|MD18M01063|MD18M01063/R7|MD18M01063|7438.64|30/06/2026|JRNNHZ.260630.598|Medical","-17714.88|147624|HARDY HENRY MANAGEMENT LTD|01/08/2026|||01/10/25 to 30/06/26|MD18M01062|MD18M01062/R7|MD18M01062|129909.12|30/06/2026|JRNNHZ.260630.597|Medical","-5604.96|46708|HARDY HENRY TEXTILES LTEE|01/08/2026|||01/10/25 to 30/06/26|MD18M01051|MD18M01051/R7|MD18M01051|41103.04|30/06/2026|JRNNHZ.260630.595|Medical","-195.99|1636|HARDY HENRY TEXTILES LTEE|01/08/2026|||01/10/25 to 30/06/26|MD04M00390|MD04M00390/R22|MD04M00390|1440.01|30/06/2026|JRNNHZ.260630.456|Medical","-3835.92|31966|Hardy Henry Services Ltd|01/08/2026|||01/10/25 to 30/06/26|MD02M00616|MD02M00616/R24|MD02M00616|28130.08|30/06/2026|JRNNHZ.260630.450|Medical","-3396.48|28304|HARDY HENRY &amp; CIE LTEE|01/07/2026|17476.02|Payment done after 30.06.2026|01/10/25 to 30/06/26|MED/2023/01269|MED/2023/01269/R2|MED/2023/01269|17476.02|31/05/2026|JRNNHZ.260531.397|Medical","-63366.36|528053|Hardy Henry Services Ltd|01/07/2026|418832.06||01/10/25 to 30/06/26|MD18M01064|MD18M01064/R7|MD18M01064|418832.06|31/05/2026|JRNNHZ.260531.197|Medical","-17714.88|147624|HARDY HENRY MANAGEMENT LTD|01/07/2026|76436.11||01/10/25 to 30/06/26|MD18M01062|MD18M01062/R7|MD18M01062|76436.11|31/05/2026|JRNNHZ.260531.195|Medical","-5604.96|46708|HARDY HENRY TEXTILES LTEE|01/07/2026|41103.04||01/10/25 to 30/06/26|MD18M01051|MD18M01051/R7|MD18M01051|41103.04|31/05/2026|JRNNHZ.260531.193|Medical","-3835.92|31966|Hardy Henry Services Ltd|01/07/2026|28130.08||01/10/25 to 30/06/26|MD02M00616|MD02M00616/R24|MD02M00616|28130.08|31/05/2026|JRNNHZ.260531.47|Medical","-86931.38|582070.94|H.VAULBERT DE CHANTILLY LTD (HVC LTD)|01/04/2026|495139.56||01/01/26 to 31/12/26||2321/20/R6||495139.56|30/01/2026|JRNI.260130.518|Non-Motor Corporate","-22324.99|1785.99|ORANGE EIGHT LTD ORANGE EIGHT LTD|31/03/2026|||01/10/25 to 30/09/26|MED/2022/01410|MED/2022/01410/R3/E7|MED/2022/01410|-20539|02/06/2026|JRNNHZ.260602.5|Medical","-45701.76|575270.9|ORANGE EIGHT LTD ORANGE EIGHT LTD|31/03/2026|217638.96||01/10/25 to 30/09/26|MED/2022/01410|MED/2022/01410/R3|MED/2022/01410|217638.96|28/11/2025|JRNNHZ.251128.28|Medical","-3865.35|26359|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/04/2026|22493.65||01/02/26 to 31/01/27||6162/25/R2||22493.65|28/01/2026|JRNI.260128.450|Non-Motor Corporate","-750|5118|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/08/2026|||16/11/25 to 15/06/26||36726/25/N/E2||4368|13/05/2026|JRNI.260513.284|Car/Ear (One Off)","-74398.8|498228|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/03/2026|278436.63||01/12/25 to 30/11/26||46037/12/R13||278436.63|30/12/2025|JRNI.251230.598|Non-Motor Corporate","-900|6121|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/09/2026|||16/11/25 to 15/08/26||36731/25/N/E3||5221|29/06/2026|JRNI.260629.604|Non-Motor Corporate","-450|3111|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/07/2026|2661||16/11/25 to 15/05/26||36731/25/N/E1||2661|23/04/2026|JRNI.260423.350|Non-Motor Corporate","-2756.85|18543|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/02/2026|9278.51||16/10/23 to 15/10/26||27489/23/N/E2||9278.51|28/11/2025|JRNI.251128.356|Car/Ear (One Off)","-18900|126630|Golden Fund Management Services Ltd &amp;/or The Mauritius Development Investment Trust Co Ltd|01/08/2026||Payment done after 30.06.2026|01/05/26 to 30/04/27|POL-C+PI-Jun-19-1003\\R7|15398/18/R8|POL-C+PI-Jun-19-1003\\R7|107730|28/05/2026|JRNI.260528.571|Financial","-7735.12|97089|Paris Onezime Marie Stephanie|02/03/2026|43569.57||01/01/26 to 31/12/26|MED/2023/00006|MED/2023/00006/R3|MED/2023/00006|43569.57|29/12/2025|JRNNHZ.251229.18|Medical","-2299.8|28747.56|Paris Onezime Marie Stephanie|02/03/2026|4969.88||01/01/26 to 31/12/26|MED/2023/00006|MED/2023/00006/R3/E1|MED/2023/00006|4969.88|22/05/2026|JRNNHZ.260522.141|Medical","-20182.35|135220|Hefty Ltd|01/06/2026|115037.65||01/04/26 to 31/03/27||6400/26/N||115037.65|20/03/2026|JRNI.260320.119|Motor","-8891.25|59582|Hefty Ltd|01/06/2026|50690.75||01/04/26 to 31/03/27||6368/26/N||50690.75|20/03/2026|JRNI.260320.18|Motor","-27536.85|184322|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/05/26||12718/24/N/E5||156785.15|30/06/2026|JRNI.260630.570|Car/Ear (One Off)","-18000|120520|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/05/26||12718/24/N/E4||102520|30/06/2026|JRNI.260630.548|Car/Ear (One Off)","-108000|722620|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/08/26||12718/24/N/E7||614620|30/06/2026|JRNI.260630.605|Car/Ear (One Off)","-20045.25|134266|Rehm Grinaker Construction Co. Ltd|01/06/2026|114220.75||01/01/26 to 31/12/26||10936/21/R4/E2||114220.75|09/03/2026|JRNI.260309.20|Motor","-44294.4|557555.76|CREDIT GUARANTEE INSURANCE CO LTD|02/03/2026|238039.16||01/01/26 to 31/12/26|MD11M00167|MD11M00167/R15|MD11M00167|238039.16|14/01/2026|JRNNHZ.260114.222|Medical","-589.95|3947|Impact Production Ltd &amp;/or Event Strategy Ltd &amp;/or Mille Feux Ltd &amp;/or Marquee Design Ltd|01/09/2026|||01/04/26 to 31/03/27||8040/21/R5/E1||3357.05|04/06/2026|JRNI.260604.342|Non-Motor Corporate","-68411.52|458172.96|Impact Production Ltd &amp;/or Event Strategy Ltd &amp;/or Mille Feux Ltd &amp;/or Marquee Design Ltd|01/07/2026|389761.44||01/04/26 to 31/03/27||8040/21/R5||389761.44|30/04/2026|JRNI.260430.631|Non-Motor Corporate","-7372.5|49772|IMPACT PRODUCTION LTD|01/04/2026|42399.5||01/01/26 to 31/12/26||54552/15/R10||42399.5|06/01/2026|JRNI.260106.400|Motor","-6255.68|78196|KASA CORPORATE SERVICES LTD|01/07/2026|71940.32||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|71940.32|31/05/2026|JRNNHZ.260531.63|Medical","-13161.28|171425.68|KASA CORPORATE SERVICES LTD|01/06/2026|158264.4||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|158264.4|30/04/2026|JRNNHZ.260430.476|Medical","-76806|514632|KASA CORPORATE SERVICES LTD|01/04/2026|243234.45|Payment done after 30.06.2026|01/01/26 to 31/12/26||32859/23/R2||243234.45|06/01/2026|JRNI.260106.408|Motor","-3986.32|49829|KASA CORPORATE SERVICES LTD|01/08/2026|||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|45842.68|30/06/2026|JRNNHZ.260630.466|Medical","-121776.21|815182.95|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|01/07/2026|462223.22||01/03/26 to 28/02/27||8187/26/N||462223.22|07/04/2026|JRNI.260407.284|Non-Motor Corporate"]</t>
+  </si>
+  <si>
+    <t>["Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging"]</t>
+  </si>
+  <si>
+    <t>["Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging","Amount not same in aging/not in aging"]</t>
+  </si>
+  <si>
+    <t>2026-07-28T07:23:03.452Z</t>
+  </si>
+  <si>
+    <t>["-656|-656|98.12|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR AVA TECHNOPARK LTD &amp;/OR AVA KNOWLEDGE LTD &amp;/OR AVA ENERGY LTD|0.12|0||MUR|30/01/2025|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||29/05/2025|558.27|98|30-01-2025 to 01-07-2025|POL-FID-Jul-23-10\\R1|POL-FID-Jul-23-10\\R1\\E1|2.29|17111/23/R1|654.1|-557.9382988771919|","-262939|-262939|208834.57|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASDCAR LTD &amp;/OR AVA TECHNOPARK LTD|169530.66|0||MUR|01/07/2024|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||26/08/2024|1188768.79|39303.91|01-07-2024 to 01-07-2025|POL-CP-Jul-23-8\\R1|POL-CP-Jul-23-8\\R1|5372.83|19358/23|1392230.53|-223649.7749073886|","-3573|-3573|534.15|15|NATEC MEDICAL LTD &amp;/OR XTRULINE CO LTD &amp;/OR ABIOLABS LTD &amp;/OR ENVASTE LTD &amp;/OR AVA MEDICAL LTD &amp;/OR TOBILI INVESTMENTS LTD &amp;/OR MAEVA CENTRE LTD &amp;/OR IPOLE PROPERTIES LTD &amp;/OR AVA REALTY LTD &amp;/OR AVA CREATION FOUNDATION &amp;/OR OSE LTD &amp;/OR AVA MADAGASCAR LTD &amp;/OR MAEVA HEALTH LTD|0.15|0||MUR|31/03/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||04/06/2025|3039.28|534|31-03-2025 to 01-07-2025|POL-PA-Jul-23-1051\\R1|POL-PA-Jul-23-1051\\R1\\E2|12.46|17111/23/R1|3560.97|-3038.9142756399315|","9048|9048|-1352.46|15|BANK OF MAURITIUS|-0.46|0||MUR|17/01/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||18/02/2025|-7695.49|-1352|17-01-2025 to 01-07-2025|POL-PA-Jun-22-34\\R2|POL-PA-Jun-22-34\\R2\\E1|-31.55|19698/24/N/E1|-9016.4|7695.532526152332|","-12744|-12744|1875|15|BANK OF MAURITIUS|0|0||MUR|07/10/2025|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||16/10/2025|10868.75|1875|07-10-2025 to 07-10-2025|POL-GIT-Oct-25-9|POL-GIT-Oct-25-9|243.75|27948/25/N|12500|-10868.963217263365|","8124|8124|-1229.36|15|BANK OF MAURITIUS|-0.359999999999854|0||MUR|29/09/2025|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL (ANNUAL COVER)||28/10/2025|-6895.08|-1229|29-09-2025 to 01-07-2026|POL-TR-ANN-Jun-25-5|POL-TR-ANN-Jun-25-5\\E3|71.31|19120/25/N/E3|-8195.75|6894.7065791611485|","-7338|-7338|1081.84|15|BANK OF MAURITIUS|-0.160000000000146|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL (ANNUAL COVER)||24/11/2025|6255.66|1082|01-11-2025 to 01-07-2026|POL-TR-ANN-Jun-25-5|POL-TR-ANN-Jun-25-5\\E4|125.24|19120/25/N|7212.26|-6256.0862800681425|","9120|9120|-1367.95|15|BANK OF MAURITIUS|0.05|0||MUR|29/08/2025|MAURITIUS UNION ASSURANCE CO LTD|TRAVEL (ANNUAL COVER)||06/10/2025|-7751.69|-1368|29-08-2025 to 01-07-2026|POL-TR-ANN-Jun-25-5|POL-TR-ANN-Jun-25-5\\E1|0||-9119.64|7751.995999842099|","-46415|-46415|6923|15|BANK OF MAURITIUS|0|0||MUR|08/11/2024|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||15/01/2025|39491.9|6923|08-11-2024 to 01-07-2025|POL-CP-Jun-22-7\\R2|POL-CP-Jun-22-7\\R2\\E2|261.54|18672/24/N|46153.36|-39491.98508453104|","-3687|-3687|506.25|15|BANK OF MAURITIUS|0.25|0||MUR|02/10/2024|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||13/11/2024|3180.56|506|02-10-2024 to 01-01-2025|POL-F&amp;A-Oct-24-1030|POL-F&amp;A-Oct-24-1030|311.81|3601.902454|3375|-3180.7239103723814|","-2926|-2926|33870.72|8|KASA TEXTILE &amp; CO LTD|33638.02|0||MUR|01/03/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/05/2025|392476.97|232.700000000004|01-03-2025 to 01-03-2026|POL-HEALTH-Jun-19-2719\\R48|POL-HEALTH-Jun-19-2719\\R48|2963.69|MED/2024/00392/R1\nMD08M01085/13/R4|423384|-2693.547170901759|","-68923|-68923|23068.5|15|KASA TEXTILE &amp; CO LTD|12815.38|750||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||20/02/2026|132009.77|10253.12|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1067\\R4|POL-MVF-Dec-21-1067\\R4|538.27|26063/21/R4|153790|-58670.43382486792|","-314174|-314174|37719.36|8|KASA TEXTILE &amp; CO LTD|12760.49|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/05/2026|437072.64|24958.87|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2719\\R49|POL-HEALTH-Jun-19-2719\\R49|3300|MD08M01085/13/R5|471492|-289214.7710984178|","-13131|-13131|1050.48|8|KASA TEXTILE &amp; CO LTD|0.48|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/06/2026|12080.52|1050|01-06-2026 to 01-03-2027|POL-HEALTH-Jun-19-2719\\R49|POL-HEALTH-Jun-19-2719\\R49\\E1|0|MD08M01085/13/R5/EQ/2|13131|-12080.52|","-85498|-85498|12750|15|ERC LEVAGE LTEE|0|0||MUR|30/01/2026|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||17/06/2026|72747.5|12750|30-01-2026 to 30-01-2026|POL-GIT-Jan-26-1|POL-GIT-Jan-26-1|497.5|2217/26/N|85000|-72747.92543641626|","-20270|-20270|3000|15|ERC LEVAGE LTEE|0|0||MUR|17/06/2025|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||31/07/2025|17270|3000|17-06-2025 to 17-06-2025|POL-GIT-Jun-25-5|POL-GIT-Jun-25-5|270|20990/25/N|20000|-17270|","-9881440|-9881440|2222028.75|15|ROYAL CAR RENTAL LTD|891753.83|31400||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||30/01/2026|12674744.08|1330274.92|01-01-2026 to 01-01-2027|POL-MVF-Jul-19-6113\\R7|POL-MVF-Jul-19-6113\\R7|51847.8299999998|31069/23 / 31162/23 / 31191/23|14813525|-8407507.087014845|","40842|40842|-6064.8|15|ROYAL CAR RENTAL LTD|0.2|-268||MUR|25/06/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/01/2026|-34776.72|-6065|25-06-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E43|-141.52|31162/23/R1/E35|-40432|34777.128721947665|","7452|7452|-1113.86|15|ROYAL CAR RENTAL LTD|0.140000000000146|0||MUR|26/08/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/01/2026|-6337.88|-1114|26-08-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E34|-25.99|31162/23/R1/E25|-7425.75|6338.101136110492|","-10111|-10111|1502.72|15|ROYAL CAR RENTAL LTD|-0.28|57.53||MUR|27/11/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||27/11/2025|8608.01|1503|27-11-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E47|35.06|31069/23/R1/E10|10018.14|-8608.23987090942|","-779717|-779717|116549.62|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.38|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||28/05/2026|663167.34|116550|01-05-2026 to 01-05-2027|POL-ARMISC-May-19-1048\\R7|POL-ARMISC-May-19-1048\\R7|2719.49||776997.47|-663167.3740209268|","-3485|-3485|520.93|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.0700000000000728|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||28/05/2026|2964.09|521|01-05-2026 to 01-05-2027|POL-MON-Apr-20-1058\\R6|POL-MON-Apr-20-1058\\R6|12.15||3472.87|-2964.07298953808|","-429|-429|825|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|762.01|0|Correction to be done by CBL amount not in aging|MUR|01/11/2018|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||4794|62.99|01-11-2018 to 01-11-2019|POL-CAR-TPL-May-19-1036|POL-CAR-TPL-May-19-1036|119|17636/16/N|5500|-366.01281366791244|","-95011|-95011|14202|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR PRINCIPALS &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||28/05/2026|80809.38|14202|01-05-2026 to 01-05-2027|POL-CAR-TPL(BC)-May-25-4\\R1|POL-CAR-TPL(BC)-May-25-4\\R1|331.38||94680|-80809.05680119581|","-7350|-7350|1098.64|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.359999999999854|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||28/05/2026|6251.25|1099|01-05-2026 to 01-05-2027|POL-EE-Apr-20-1086\\R6|POL-EE-Apr-20-1086\\R6|25.64||7324.25|-6251.343557522629|","-906872|-906872|135556.38|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR FASTMIX  CO LTD|0.38|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||28/05/2026|771315.81|135556|01-05-2026 to 01-05-2027|POL-ARM(P&amp;M)-Feb-20-1010\\R7|POL-ARM(P&amp;M)-Feb-20-1010\\R7|3163.01||903709.18|-771315.6484005976|","-107514|-107514|16070.81|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR FASTMIX CO LTD|-0.19|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||28/05/2026|91442.88|16071|01-05-2026 to 01-05-2027|POL-EL-Apr-20-1161\\R6|POL-EL-Apr-20-1161\\R6|374.98|9314/08/R18|107138.71|-91443.14366216991|","-92643|-92643|13848|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR FAST MIX CO LTD|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/05/2026|78795.12|13848|01-05-2026 to 01-05-2027|POL-PA-Apr-20-1154\\R6|POL-PA-Apr-20-1154\\R6|323.12||92320|-78795.01793721973|","-112057|-112057|16675.17|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR SOCIETE FOUR TWELVE &amp;/ORDISTRI-T TRADING LTD|0.169999999997672|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||28/05/2026|95381.69|16675|01-05-2026 to 01-05-2027|POL-F&amp;A-Apr-20-1182\\R6|POL-F&amp;A-Apr-20-1182\\R6|889.09|9314/08/R18|111167.77|-95381.80916661417|","-276484|-276484|41328|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/05/2026|235156.32|41328|01-05-2026 to 01-05-2027|POL-PA-Apr-20-1155\\R6|POL-PA-Apr-20-1155\\R6|964.32||275520|-235156.04783258596|","-117828|-117828|17612.55|15|TAYELAMAY &amp; SONS ENTERPRISE LTD|-0.45|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||28/05/2026|100215.41|17613|01-05-2026 to 01-05-2027|POL-PA-Apr-20-1153\\R6|POL-PA-Apr-20-1153\\R6|410.96||117417|-100215.44402092678|","-5808|-5808|868.2|15|TAYELAMAY &amp; SONS ENTERPRISE LTD &amp;/OR SOCIETE FOUR TWELVE &amp;/ORDISTRI-T TRADING LTD &amp;/OR FASTMIX CO LTD|0.2|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||28/05/2026|4940.06|868|01-05-2026 to 01-05-2027|POL-PL-Apr-20-1178\\R6|POL-PL-Apr-20-1178\\R6|20.26|9314/08/R18|5788|-4939.838863962701|","1028|1028|-168.63|15|LAVASTONE LTD &amp;/OR SUBSIDIARIES &amp;/OR AFFILIATED COMPANIES|0.37|0||MUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||10/10/2025|-859.48|-169|01-10-2024 to 30-09-2025|POL-EL-Oct-19-1469\\R5|POL-EL-Oct-19-1469\\R5\\E1|96.07|33502/19/R5/E1|-1124.18|859.3880421355692|","5077|5077|-758.83|15|LAVASTONE LTD &amp;/OR SUBSIDIARIES &amp;/OR AFFILIATED COMPANIES|0.17|0||MUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||13/10/2025|-4317.73|-759|01-10-2024 to 30-09-2025|POL-PA-Oct-19-1546\\R5|POL-PA-Oct-19-1546\\R5\\E1|-17.71|33502/19/R5/E1|-5058.85|4318.104230029784|","-16533|-16533|1983.95|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.05|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|14548.96|1984|01-11-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E25|0|MED/2025/01055/EQ/55|16532.91|-14549.039199995645|","-25782|-25782|3093.89|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.11|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|22688.55|3094|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E41|0|MED/2025/01055/EQ/96|25782.44|-22688.162799952217|","7844|7844|-941.33|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.33|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|-6903.12|-941|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E40|0|MED/2025/01055/EQ/94|-7844.45|6902.723999770538|","-6277|-6277|753.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|5523.89|753|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E51|0|MED/2025/01055/EQ/112|6277.15|-5523.758000047792|","-1836|-1836|220.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||05/06/2026|1615.25|220|01-06-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E54|0|MED/2025/01055/EQ/118|1835.51|-1615.681200320347|","-6277|-6277|753.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||05/06/2026|5523.89|753|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E53|0|MED/2025/01055/EQ/114|6277.15|-5523.758000047792|","-13731|-13731|1647.68|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.32|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|12082.95|1648|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E28|0|MED/2025/01055/EQ/64|13730.63|-12083.275599881434|","3119|3119|-374.24|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.24|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/05/2026|-2744.44|-374|01-06-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E52|0|MED/2025/01055/EQ/113|-3118.68|2744.721600164172|","-11074|-11074|1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|9745.31|1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E29|0|MED/2025/01055/EQ/56|11074.22|-9745.116400071518|","-18355|-18355|2202.61|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.39|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|16152.45|2203|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E36|0|MED/2025/01055/EQ/74|18355.06|-16152.397200009153|","-7464|-7464|895.73|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.27|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|6568.66|896|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E43|0|MED/2025/01055/EQ/95|7464.39|-6568.316800167194|","-139140|-139140|16696.8|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.2|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||27/02/2026|122443.2|16697|01-07-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E19|0|MED/2025/01055/EQ/84|139140|-122443.2|","-7274|-7274|872.88|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.12|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|6401.09|873|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E35|0|MED/2025/01055/EQ/81|7273.97|-6401.116399985152|","-11074|-11074|1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/02/2026|9745.31|1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E34|0|MED/2025/01055/EQ/75|11074.22|-9745.116400071518|","11074|11074|-1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/02/2026|-9745.31|-1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E33|0|MED/2025/01055/EQ/76|-11074.22|9745.116400071518|","-42083|-42083|5049.99|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.01|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|37033.25|5050|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E37|0|MED/2025/01055/EQ/80|42083.24|-37033.03880000684|"]</t>
+  </si>
+  <si>
+    <t>["-57631|8614.5|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|18/05/2026|||01/12/25 to 30/11/26||29742/23/R2/E1||-49016.5|18/05/2026|JRNI.260518.268|Motor","-38187|255971|CURRIMJEE JEEWANJEE AND COMPANY LIMITED|01/04/2026|27828.27|Payment done after 30.06.2026|01/01/26 to 31/12/26||1915/26/N||27828.27|28/01/2026|JRNI.260128.526|Non-Motor Corporate","-429672.4|2875008.96|Currimjee Jeewanjee &amp; Co Ltd|01/04/2026|729243.58|Payment done after 30.06.2026|01/01/26 to 31/12/26||1918/26/N||729243.58|28/01/2026|JRNI.260128.522|Non-Motor Corporate","-150000|1005000|Currimjee Jeewanjee &amp; Co Ltd|01/04/2026|249278.65||01/01/26 to 31/12/26|POL-TER&amp;SAB-Mar-21-1002\\R5|6361/26/N|POL-TER&amp;SAB-Mar-21-1002\\R5|249278.65|18/03/2026|JRNI.260318.354|Special","-30754|4697.05|Currimjee Jeewanjee &amp; Co Ltd|03/03/2026|100||01/01/26 to 31/12/26||1918/26/N/E1||-26056.95|27/02/2026|JRNI.260227.565|Non-Motor Corporate","-29145.6|366870.24|RENTACOLOR (MAURITIUS) LTD|31/01/2026|266766.27||01/01/26 to 31/12/26|MD21M00252|MD21M00252/R5|MD21M00252|266766.27|23/02/2026|JRNNHZ.260223.99|Medical","-6290.76|52423|MAURITOURS LTD MAURITOURS LTD|01/08/2026|||01/01/26 to 31/12/26|MED/2023/00018|MED/2023/00018/R3|MED/2023/00018|46132.24|30/06/2026|JRNNHZ.260630.738|Medical","-27489.12|233886.6|MAURITOURS LTD MAURITOURS LTD|01/06/2026|206397.48||01/01/26 to 31/12/26|MED/2023/00018|MED/2023/00018/R3|MED/2023/00018|206397.48|30/04/2026|JRNNHZ.260430.757|Medical","-6872.28|57269|MAURITOURS LTD MAURITOURS LTD|01/07/2026|50396.72||01/01/26 to 31/12/26|MED/2023/00018|MED/2023/00018/R3|MED/2023/00018|50396.72|31/05/2026|JRNNHZ.260531.343|Medical","-6663.2|83290|Nassau Services Ltd|01/08/2026|||01/01/26 to 31/12/26|MD10M00493|MD10M00493/R16|MD10M00493|76626.8|30/06/2026|JRNNHZ.260630.483|Medical","-6901.04|86263|Nassau Services Ltd|01/07/2026|16093.06||01/01/26 to 31/12/26|MD10M00493|MD10M00493/R16|MD10M00493|16093.06|31/05/2026|JRNNHZ.260531.81|Medical","-31162.48|208789|Nassau Services Ltd|30/08/2026|44406.63||01/06/26 to 31/05/27||12779/21/R5||177626.52|11/06/2026|JRNI.260611.328|Financial","-27050.95|2164.07|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2026|||01/01/26 to 31/12/26|MD11M00166|MD11M00166/R15/E6|MD11M00166|-24886.88|20/03/2026|JRNNHZ.260320.336|Medical","-12682.38|1014.59|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E14|MD11M00166|-8562.88|03/10/2025|JRNNHZ.251003.354|Medical","-22907.97|1832.63|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E6|MD11M00166|-7943.33|12/06/2025|JRNNHZ.250612.280|Medical","-37909.31|3032.74|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2026|||01/01/26 to 31/12/26|MD11M00166|MD11M00166/R15/E8|MD11M00166|-34876.57|05/06/2026|JRNNHZ.260605.487|Medical","-12682.38|1014.59|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E14|MD11M00166|-8562.88|03/10/2025|JRNNHZ.251003.354|Medical","-22907.97|1832.63|LA PRUDENCE LEASING FINANCE CO LTD|02/03/2025|||01/01/25 to 31/12/25|MD11M00166|MD11M00166/R14/E6|MD11M00166|-7943.33|12/06/2025|JRNNHZ.250612.280|Medical","-19196.43|1535.71|NEWREST (MAURITIUS) LTD NEWREST (MAURITIUS) LTD|31/03/2026|||01/10/25 to 30/09/26|MED/2024/01202|MED/2024/01202/R1/E7|MED/2024/01202|-17660.72|08/06/2026|JRNNHZ.260608.239|Medical","-895792.5|6006552|JAG SERVICES LTD|15/10/2026|2008438.85||01/01/26 to 31/12/26||31069/23/R2||3155697.21|06/01/2026|JRNI.260106.421|Motor","-52010|6861.3|JAG SERVICES LTD|13/02/2026|||01/01/26 to 31/12/26||31069/23/R2/E4||-45148.7|13/02/2026|JRNI.260213.86|Motor","-1.05|110|Panache &amp; Co.Ltd|01/09/2026|||01/07/25 to 30/06/26||17835/22/R3/E1||108.95|18/06/2026|JRNI.260618.308|Non-Motor Corporate","-48.6|325|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|26/03/26 to 26/03/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14790/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|276.4|09/06/2026|JRNI.260609.338|Marine","-37.5|251|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|08/05/26 to 08/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14789/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|213.5|09/06/2026|JRNI.260609.337|Marine","-60.9|407|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|04/05/26 to 04/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14786/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|346.1|09/06/2026|JRNI.260609.336|Marine","-37.5|251|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|01/05/26 to 01/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14778/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|213.5|09/06/2026|JRNI.260609.335|Marine","-37.5|351|Panache &amp; Co.Ltd|12/09/2026||Payment done after 30.06.2026|05/05/26 to 05/05/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|14777/26|POL-MAR-Jun-26-1273, O.Cover : 13/11/CO/HO|313.5|09/06/2026|JRNI.260609.334|Marine","-180.9|1210|Panache &amp; Co.Ltd|01/09/2026|||01/07/25 to 30/06/26||9084/09/R16/E7||1029.1|03/06/2026|JRNI.260603.144|Motor","-661.05|4438|Panache &amp; Co.Ltd|01/08/2026|||01/07/25 to 30/06/26||9084/09/R16/E6||3776.95|28/05/2026|JRNI.260528.372|Motor","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|18/04/26 to 18/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12372/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.300|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|14/04/26 to 14/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12371/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.299|Marine","-304.8|2039|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|18/04/26 to 18/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12370/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|1734.2|18/05/2026|JRNI.260518.298|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|17/04/26 to 17/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12369/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.297|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|16/04/26 to 16/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12367/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.296|Marine","-57.75|386|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|09/04/26 to 09/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12366/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|328.25|18/05/2026|JRNI.260518.295|Marine","-48.6|325|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|15/04/26 to 15/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12365/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|276.4|18/05/2026|JRNI.260518.294|Marine","-104.7|700|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|02/03/26 to 02/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12364/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|595.3|18/05/2026|JRNI.260518.293|Marine","-123.15|824|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|02/02/26 to 02/02/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12363/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|700.85|18/05/2026|JRNI.260518.292|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|16/04/26 to 16/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12361/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.291|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|08/03/26 to 08/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12360/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.290|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|09/04/26 to 09/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12358/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.289|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|06/04/26 to 06/04/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12357/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.288|Marine","-37.5|251|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|25/03/26 to 25/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12356/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|213.5|18/05/2026|JRNI.260518.287|Marine","-54|461|Panache &amp; Co.Ltd|18/08/2026||Payment done after 30.06.2026|28/03/26 to 28/03/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|12355/26|POL-MAR-May-26-1221, O.Cover : 13/11/CO/HO|407|18/05/2026|JRNI.260518.286|Marine","-5407|808.2|Panache &amp; Co.Ltd|24/04/2026|||01/07/25 to 30/06/26||9084/09/R16/E5||-4598.8|24/04/2026|JRNI.260424.167|Motor","-44.4|397|Scott &amp; Co Ltd|01/07/2026|352.6||01/10/25 to 30/09/26||33954/19/R6/E2||352.6|09/01/2026|JRNI.260109.314|Non-Motor Corporate","-457.5|3161|Scott &amp; Co Ltd|01/07/2026|2703.5||01/10/25 to 30/09/26||33954/19/R6/E1||2703.5|07/01/2026|JRNI.260107.260|Non-Motor Corporate","-195955.8|1311444|HIGHWAY PROPERTIES LTD|01/08/2026|||01/05/26 to 30/04/27||13781/26/N||1115488.2|28/05/2026|JRNI.260528.581|Non-Motor Corporate","-24269.23|162860.98|HIGHWAY PROPERTIES LTD|01/09/2026|||01/05/26 to 30/04/27||14246/26/R1||138591.75|09/06/2026|JRNI.260609.339|Non-Motor Corporate","-2059.76|14279.97|HIGHWAY PROPERTIES LTD|05/06/2026|12220.21||01/04/26 to 30/04/26||14246/26/N||12220.21|03/06/2026|JRNI.260603.381|Non-Motor Corporate","-19264.65|129381|HIGHWAY PROPERTIES LTD|06/05/2026|110116.35||01/04/26 to 30/04/26||10767/26/N||110116.35|23/04/2026|JRNI.260423.353|Non-Motor Corporate","-38641.95|258710|HIGHWAY PROPERTIES LTD|01/07/2026|176087.63|Payment done after 30.06.2026|10/04/26 to 31/03/27|POL-MV-Apr-26-95|8591/26/N|POL-MV-Apr-26-95|176087.63|10/04/2026|JRNI.260410.163|Motor","-11997.59|80763.97|ACBMS LTD|01/08/2026|||01/05/26 to 30/04/27||12079/22/R4||45845.27|07/05/2026|JRNI.260507.165|Non-Motor Corporate","-16786.56|211300.82|GAYA COLLECTIONS LIMITEE GAYA COLLECTIONS LIMITEE|30/06/2026|160619.77|Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2023/00969|MED/2023/00969/R3|MED/2023/00969|160619.77|13/05/2026|JRNNHZ.260513.423|Medical","-2119.73|26496.72|GAYA COLLECTIONS LIMITEE GAYA COLLECTIONS LIMITEE|30/06/2026|1913.1||01/05/26 to 30/04/27|MED/2023/00969|MED/2023/00969/R3/E1|MED/2023/00969|1913.1|11/06/2026|JRNNHZ.260611.54|Medical","-12676.72|158459|BELLE RIVIERE HOTEL LTD|01/08/2026|||01/05/26 to 30/04/27|MED/2025/00947|MED/2025/00947/R1|MED/2025/00947|145782.28|30/06/2026|JRNNHZ.260630.904|Medical","-11476.08|155614.12|BELLE RIVIERE HOTEL LTD|01/07/2026|131974.92||01/05/26 to 30/04/27|MED/2025/00947|MED/2025/00947/R1|MED/2025/00947|131974.92|31/05/2026|JRNNHZ.260531.511|Medical","-6485.7|43689|Osman Rezah|01/09/2026|||01/06/26 to 31/05/27||13626/10/R16||37203.3|01/06/2026|JRNI.260601.332|Non-Motor Corporate","-38910|5816.1|Partsionate Ltd|24/06/2026|||06/05/26 to 30/04/27||11100/26/N/E1||-33093.9|24/06/2026|JRNI.260624.288|Motor","-123515|18462.6|Partsionate Ltd|05/06/2026|||06/05/26 to 30/04/27||11084/26/N/E2||-105052.4|05/06/2026|JRNI.260605.166|Motor","-3078|21042|ASSOCIATION SYNDICALE DU LOTISSEMENT LES VILLAS DE CASCAVELLE|01/03/2026|17964||01/11/25 to 31/10/26||9507/20/R6||17964|03/12/2025|JRNI.251203.405|Non-Motor Corporate","-1383.3|9754|ASSOCIATION SYNDICALE MORCELLEMENT VILLAZE|01/08/2026|||01/05/26 to 30/04/27||17184/24/R2||8370.7|11/05/2026|JRNI.260511.317|Non-Motor Corporate","-263.98|1915.99|LES CAMPECHES LTEE|01/09/2026|||12/06/26 to 11/12/26||16082/26/N||1652.01|24/06/2026|JRNI.260624.397|Non-Motor Corporate","-11504.7|77466|SYNDICAT DES COPROPRIÉTAIRES DE L`ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|01/03/2026|65961.3||01/10/25 to 30/09/26||2595/17/R9||65961.3|03/12/2025|JRNI.251203.296|Non-Motor Corporate","-408.45|2783|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|01/01/2026|2374.55||01/11/25 to 31/10/26||31161/22/R3||2374.55|13/10/2025|JRNI.251013.122|Motor","-13346.85|89390|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|01/08/2026|||01/06/26 to 31/05/27||31169/22/R3||76043.15|29/05/2026|JRNI.260529.51|Motor","-457|68.25|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|08/10/2025|||01/01/25 to 31/10/25||31161/22/R2/E2||-388.75|08/10/2025|JRNI.251008.78|Motor","-408.75|2785|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|01/04/2026|2376.25||01/02/26 to 31/01/27||31164/22/R3||2376.25|12/01/2026|JRNI.260112.141|Motor","-7549.5|50606|The General Construction Company Limited|01/01/2026|43056.5||01/04/25 to 31/03/26||10359/24/R1/E1||43056.5|01/10/2025|JRNI.251001.326|Non-Motor Corporate","-242123.1|1619804|The General Construction Company Limited|17/06/2026|1377680.9||16/12/24 to 15/12/34||17764/25/N/E1||1377680.9|15/06/2026|JRNI.260615.361|Special","-768028.95|5138114|The General Construction Company Limited|01/07/2026|1456887.07||01/04/26 to 31/03/27||10359/24/R2||1456887.07|16/04/2026|JRNI.260416.322|Non-Motor Corporate","-322312.92|2156773.96|The General Construction Company Limited|01/07/2026|589013.49||01/04/26 to 31/03/27||7186/22/R4||589013.49|16/04/2026|JRNI.260416.317|Non-Motor Corporate","-12916.35|86534|The General Construction Company Limited|01/11/2025|73617.65||01/04/25 to 31/03/26||MT9900043297/R25/E15||73617.65|18/08/2025|JRNI.250818.221|Motor","-11576.25|77945|The General Construction Company Limited|01/07/2026|44248.1||01/04/26 to 31/03/27||8694/22/R4||44248.1|15/04/2026|JRNI.260415.201|Non-Motor Corporate","-9325|1393.8|The General Construction Company Limited|27/10/2025|||01/04/25 to 31/03/26||MT9900043297/R25/E27||-7931.2|27/10/2025|JRNI.251027.157|Motor","-1308|195.45|The General Construction Company Limited|05/02/2026|||01/04/25 to 31/03/26||MT9900043297/R25/E38||-1112.55|05/02/2026|JRNI.260205.45|Motor","-4762.35|32003|The General Construction Company Limited|01/10/2025|27240.65||01/04/25 to 31/03/26|POL-MVF-May-19-1121\\R6\\E14|MT9900043297/R25/E11|POL-MVF-May-19-1121\\R6\\E14|27240.65|14/07/2025|JRNI.250714.129|Motor","-3359|502.05|The General Construction Company Limited|06/11/2025|||01/04/25 to 31/03/26||MT9900043297/R25/E30||-2856.95|06/11/2025|JRNI.251106.243|Motor","-75873.75|513095|The General Construction Company Limited|01/07/2026|437221.25||01/04/26 to 31/03/27||9151/18/R8||437221.25|01/04/2026|JRNI.260401.326|Motor","-10350|69442|The General Construction Company Limited|01/07/2026|59092||01/04/26 to 31/03/27||13092/25/R1||59092|01/04/2026|JRNI.260401.324|Motor","-924635.68|6216812.99|The General Construction Company Limited|01/07/2026|3362379.92||01/04/26 to 31/03/27||MT9900043297/R26||3362379.92|01/04/2026|JRNI.260401.322|Motor","-581|86.85|The General Construction Company Limited|27/10/2025|||01/04/25 to 31/03/26||9151/18/R7/E5||-494.15|27/10/2025|JRNI.251027.149|Motor","-9693.45|64949|DESVAUX DE MARIGNY Alain Laurent|01/09/2026|||01/07/26 to 30/06/27||21359/25/R1||55255.55|16/06/2026|JRNI.260616.212|Motor","-8462.43|106180.44|Desvaux De Marigny-Montocchio Marie Pascale Anne|31/10/2026|||01/05/26 to 30/04/27|MD21M00643|MD21M00643/R5|MD21M00643|87946.25|11/05/2026|JRNNHZ.260511.367|Medical"]</t>
+  </si>
+  <si>
+    <t>["-31700|-31700|3803.97|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.03|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|27895.75|3804|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E38|0|MED/2025/01055/EQ/72|31699.72|-27895.9963999682|","-2374|-2374|284.94|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.06|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|2089.55|285|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E45|0|MED/2025/01055/EQ/107|2374.49|-2089.118800247632|","24936|24936|-2992.32|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.32|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/10/2025|-21943.68|-2992|01-07-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E14|0|MED/2025/01055|-24936|21943.68|","-2082|-2082|249.87|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.13|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|1832.41|250|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E46|0|MED/2025/01055/EQ/116|2082.28|-1832.1635995159154|","-9763|-9763|1171.52|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.48|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|8591.15|1172|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E47|0|MED/2025/01055/EQ/102|9762.67|-8591.440400013522|","-6616|-6616|793.93|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.07|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|5822.15|794|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E48|0|MED/2025/01055/EQ/101|6616.08|-5822.079600004837|","-111444|-111444|13373.34|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.34|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|98071.15|13373|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E42|0|MED/2025/01055/EQ/97|111444.49|-98070.71880000527|","38769|38769|-4636.02|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.0200000000005821|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|-34132.74|-4636|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E39|-135.22|MED/2025/01055|-38633.54|34132.951300480076|","53793|53793|-6455.21|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.21|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|-47338.2|-6455|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E22|0|MED/2025/01055/EQ/51|-53793.41|47337.8392000061|","31285|31285|-3754.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.26|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/02/2026|-27531.21|-3754|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E30|0|MED/2025/01055/EQ/73|-31285.47|27530.79640005408|","-16585|-16585|1990.24|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.24|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|14595.08|1990|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E50|0|MED/2025/01055/EQ/110|16585.32|-14594.798400030872|","6550|6550|-785.99|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.01|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||22/04/2026|-5763.91|-786|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E44|0|MED/2025/01055/EQ/99|-6549.9|5763.997999969465|","-41854|-41854|5022.48|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.479999999999418|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/01/2026|36831.55|5022|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E24|0|MED/2025/01055/EQ/48|41854.03|-36831.52359999742|","18600|18600|-2231.98|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.02|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||07/01/2026|-16367.82|-2232|01-09-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E8|0|MED/2025/01055/EQ/7|-18599.8|16367.99599995699|","-50256|-50256|6030.71|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.29|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|44225.23|6031|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E49|0|MED/2025/01055/EQ/111|50255.94|-44225.28280000334|","27159|27159|-3259.13|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.13|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/01/2026|-23900.26|-3259|01-10-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E23|0|MED/2025/01055/EQ/47|-27159.39|23899.91680004595|","33030|33030|-3963.6|12|HARDY HENRY SERVICES LTEE|0.4|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-29066.4|-3964|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E7|0|MD18M01064/3/R4/EQ/15|-33030|29066.4|","47208|47208|-5664.96|12|HARDY HENRY SERVICES LTEE|0.04|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-41543.04|-5665|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E9|0|MD18M01064/3/R4/EQ/17|-47208|41543.04|","-1884|-1884|226.08|12|HARDY HENRY SERVICES LTEE|226.16|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||01/07/2026|1657.92|-0.0800000000000125|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E21|0|MD18M01064/3/R4/EQ/43|1884|-1657.92|","-5790|-5790|694.8|12|HARDY HENRY SERVICES LTEE|-0.2|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|5095.2|695|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E10|0|MD18M01064/3/R4/EQ/18|5790|-5095.2|","-9420|-9420|1130.4|12|HARDY HENRY SERVICES LTEE|0.400000000000146|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|8289.6|1130|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E12|0|MD18M01064/3/R4/EQ/19|9420|-8289.6|","9400|9400|-1128|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/06/2026|-8272|-1128|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E22|0|MD18M01064/3/R4/EQ/42|-9400|8272|","-18840|-18840|2260.8|12|HARDY HENRY SERVICES LTEE|-0.199999999999709|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|16579.2|2261|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E8|0|MD18M01064/3/R4/EQ/16|18840|-16579.2|","-4626|-4626|555.12|12|HARDY HENRY SERVICES LTEE|0.12|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/05/2026|4070.88|555|01-05-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E18|0|MD18M01064/3/R4/EQ/30|4626|-4070.88|","-3900|-3900|468|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||01/03/2026|3432|468|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E13|0|MD18M01064/3/R4/EQ/23|3900|-3432|","27591|27591|-3310.92|12|HARDY HENRY SERVICES LTEE|0.08|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|-24280.08|-3311|01-04-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E16|0|MD18M01064/3/R4/EQ/28|-27591|24280.08|","-2111|-2111|253.32|12|HARDY HENRY SERVICES LTEE|0.32|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||14/06/2026|1857.68|253|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E20|0|MD18M01064/3/R4/EQ/37|2111|-1857.68|","17780|17780|-2133.6|12|HARDY HENRY SERVICES LTEE|0.4|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||17/12/2025|-15646.4|-2134|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E3|0|MD18M01064/3/R4/EQ/3|-17780|15646.4|","24815|24815|-2977.8|12|HARDY HENRY SERVICES LTEE|0.2|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/12/2025|-21837.2|-2978|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E6|0|MD18M01064/3/R4/EQ/12|-24815|21837.2|","6167|6167|-740.04|12|HARDY HENRY SERVICES LTEE|-0.04|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-5426.96|-740|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E5|0|MD18M01064/3/R4/EQ/14|-6167|5426.96|","-29379|-29379|3525.48|12|HARDY HENRY SERVICES LTEE|0.48|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/12/2025|25853.52|3525|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E4|0|MD18M01064/3/R4/EQ/10|29379|-25853.52|","-1762|-1762|211.44|12|HARDY HENRY SERVICES LTEE|0.44|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/05/2026|1550.56|211|01-05-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E17|0|MD18M01064/3/R4/EQ/32|1762|-1550.56|","-24687|-24687|2962.44|12|HARDY HENRY SERVICES LTEE|0.44|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/12/2025|21724.56|2962|01-10-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E1|0|MD18M01064/3/R4/EQ/9\nMD18M01064/3/R4/EQ/8\nMD02M00616/19/R5/EQ/2|24687|-21724.56|","12700|12700|-1524|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/02/2026|-11176|-1524|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E11|0|MD18M01064/3/R4/EQ/21|-12700|11176|","-14180|-14180|1701.6|12|HARDY HENRY SERVICES LTEE|-0.4|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|12478.4|1702|01-03-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E14|0|MD18M01064/3/R4/EQ/25|14180|-12478.4|","13536|13536|-1624.32|12|HARDY HENRY SERVICES LTEE|-0.32|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|-11911.68|-1624|01-04-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E15|0|MD18M01064/3/R4/EQ/26|-13536|11911.68|","1884|1884|-226.08|12|HARDY HENRY SERVICES LTEE|-0.08|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/06/2026|-1657.92|-226|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E19|0|MD18M01064/3/R4/EQ/38|-1884|1657.92|","-17559|-17559|2624.7|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.3|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||12/02/2026|14934.55|2625|01-01-2026 to 01-01-2027|POL-FID-Dec-21-9\\R4|POL-FID-Dec-21-9\\R4|61.25|2321/20/R6|17498|-14934.337369192875|","-22618|-22618|3380.83|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.17|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||12/02/2026|19236.93|3381|01-01-2026 to 01-01-2027|POL-EE-Dec-21-20\\R4|POL-EE-Dec-21-20\\R4|78.88|2321/20/R6|22538.88|-19237.134125572116|","-12042|-12042|1800|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||12/02/2026|10242|1800|01-01-2026 to 01-01-2027|POL-MON-Jan-20-1008\\R6|POL-MON-Jan-20-1008\\R6|42|2321/20/R6|12000|-10242|","-105713|-105713|15801.59|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.41|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||12/02/2026|89911.08|15802|01-01-2026 to 01-01-2027|POL-PA-Mar-20-1110\\R6|POL-PA-Mar-20-1110\\R6|368.71|2321/20/R6|105343.96|-89911.36067266109|","-34386|-34386|5139.87|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.13|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||12/02/2026|29245.89|5140|01-01-2026 to 01-01-2027|POL-EL-Jan-20-1023\\R6|POL-EL-Jan-20-1023\\R6|119.93|2321/20/R6|34265.83|-29246.094125591524|","-120816|-120816|18059.27|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.27|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||12/02/2026|102757.21|18059|01-01-2026 to 01-01-2027|POL-PPL-Jan-20-1005\\R6|POL-PPL-Jan-20-1005\\R6|421.38|2321/20/R6|120395.1|-102756.80174890049|","-136980|-136980|20475.37|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.37|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||12/02/2026|116504.87|20475|01-01-2026 to 01-01-2027|POL-LOP(F&amp;A)-Jan-20-1009\\R6|POL-LOP(F&amp;A)-Jan-20-1009\\R6|477.76|2321/20/R6|136502.48|-116504.66587443562|","-131417|-131417|19569.12|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.12|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||12/02/2026|111848.29|19569|01-01-2026 to 01-01-2027|POL-F&amp;A-Jan-20-1022\\R6|POL-F&amp;A-Jan-20-1022\\R6|956.61|2321/20/R6|130460.8|-111847.94105233089|","-2277|-2277|317.95|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.05|0||MUR|20/11/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||09/02/2026|1959.16|318|20-11-2025 to 01-01-2026|POL-F&amp;A-Jan-20-1022\\R5|POL-F&amp;A-Jan-20-1022\\R5\\E1|157.42|2321/20/R5/E2|2119.69|-1959.0653591613932|","-272603|-272603|45701.76|8|ORANGE EIGHT LTD|31739.35|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/11/2025|529569.24|13962.41|01-10-2025 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4|3999|MED/2022/01410/R3|571272|-250946.36011848328|","-30551|-30551|2444.12|8|ORANGE EIGHT LTD|2444.2|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||22/04/2026|28107.35|-0.0799999999999272|01-04-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E1|0|MED/2022/01410/R3/EQ/5|30551.47|-28106.917600036923|","25543|25543|-2043.44|8|ORANGE EIGHT LTD|-2043.88|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|-23499.6|0.440000000000055|01-05-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E3|0|MED/2022/01410/R3/EQ/6|-25543.04|23499.563199994987|","56735|56735|-4538.8|8|ORANGE EIGHT LTD|-4538.6|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||16/04/2026|-52196.22|-0.199999999999818|01-04-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E2|0|MED/2022/01410/R3/EQ/4|-56735.02|52196.20159999943|","22325|22325|-1786|8|ORANGE EIGHT LTD|-1786|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||03/06/2026|-20539|0|01-06-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E4|0|MED/2022/01410/R3/EQ/7|-22325|20539|","-26357|-26357|3865.03|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND\nCLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|0.03|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||02/02/2026|22492.04|3865|01-02-2026 to 01-02-2027|POL-CAR-TPL-Jun-20-1033\\R5|POL-CAR-TPL-Jun-20-1033\\R5|590.18|6162/25|25766.89|-22491.980264877697|","-5118|-5118|750|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR CONTRACTORS &amp;/OR SUB CONTRACTORS||0||MUR|15/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||4367.5||15-05-2026 to 15-06-2026|POL-CAR-TPL-Nov-25-1054|POL-CAR-TPL-Nov-25-1054\\E2|117.5||5000|-4367.926722032243|"]</t>
+  </si>
+  <si>
+    <t>["-11246.4|94120|CHEUNG Willy|30/04/2026|66298.88|Payment done after 30.06.2026|01/03/26 to 28/02/27|MED/2026/00365|MED/2026/00365/N|MED/2026/00365|66298.88|24/04/2026|JRNNHZ.260424.75|Medical","-4703.04|39592|RAMPUTH NEELESH|30/04/2026|27911.52|Payment done after 30.06.2026|01/03/26 to 28/02/27|MED/2026/00315|MED/2026/00315/N|MED/2026/00315|27911.52|16/04/2026|JRNNHZ.260416.32|Medical","-7197.12|60376|Boodiah Maureen Vivianna|31/05/2026|53178.88|Payment done after 30.06.2026|01/04/26 to 31/03/27|MED/2026/00362|MED/2026/00362/N|MED/2026/00362|53178.88|24/04/2026|JRNNHZ.260424.21|Medical","-8138.25|54545|Comptoir Ouest OI Ltee|01/07/2026|38670.45||01/05/26 to 30/04/27|POL-MV-Apr-25-150|11301/25/R1|POL-MV-Apr-25-150|38670.45|16/04/2026|JRNI.260416.191|Motor","-5517.02|69362.87|NOMBRO MARY LYSIE IVY|30/11/2026|||01/06/26 to 31/05/27|MED/2023/00781|MED/2023/00781/R3|MED/2023/00781|56493.34|03/06/2026|JRNNHZ.260603.72|Medical","-4165.05|52563.19|Pro Wire Electrical &amp; Mechanical Ltd Pro Wire Electrical &amp; Mechanical Ltd|30/11/2026||Payment done after 30.06.2026|01/06/26 to 31/05/27|MED/2022/00714|MED/2022/00714/R4|MED/2022/00714|48398.14|15/06/2026|JRNNHZ.260615.19|Medical","-2803.5|18855|MEDLOG (MAURITIUS) LTD|01/09/2026|||01/08/25 to 31/07/26||26048/24/R1/E2||16051.5|01/06/2026|JRNI.260601.416|Non-Motor Corporate","-14031.3|93969|G. DE VILLIERS PAINT CONTRACTORS LTD|01/08/2026|||01/06/26 to 31/05/27||18210/25/R1||79937.7|27/05/2026|JRNI.260527.92|Motor","-5408.25|36381|G. DE VILLIERS PAINT CONTRACTORS LTD|01/09/2025|22655.11||01/07/25 to 30/06/26||18205/25/N||22655.11|26/06/2025|JRNI.250626.416|Motor","-8518.95|57192|G. DE VILLIERS PAINT CONTRACTORS LTD|01/09/2025|27592.64||01/07/25 to 30/06/26||18193/25/N||27592.64|26/06/2025|JRNI.250626.408|Motor","-8902.65|59759|G. DE VILLIERS PAINT CONTRACTORS LTD|01/07/2026|50856.35||01/05/26 to 30/04/27||18193/25/R1||50856.35|30/04/2026|JRNI.260430.161|Motor","-5711.1|38407|G. DE VILLIERS PAINT CONTRACTORS LTD|01/08/2026|||01/06/26 to 31/05/27||18205/25/R1||32695.9|27/05/2026|JRNI.260527.85|Motor","-13435.2|112360|SAWMYNADEN Kisnasamy Poulay|31/05/2026|78739.85||01/04/26 to 31/03/27|MED/2026/00453|MED/2026/00453/N|MED/2026/00453|78739.85|21/05/2026|JRNNHZ.260521.163|Medical","-5286.24|44452|HUET Louise Lilette Nicole|30/06/2026|32240.48|Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2026/00429|MED/2026/00429/N|MED/2026/00429|32240.48|19/05/2026|JRNNHZ.260519.161|Medical","-10680.48|89404|SOORJUN SOTEEHALL MANISHA|30/06/2026|70314.39|Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2026/00515|MED/2026/00515/N|MED/2026/00515|70314.39|02/06/2026|JRNNHZ.260602.2|Medical","-150406.35|1006718|IKO (MAURITIUS) HOTEL LIMITED T/A CONSTANCE LE CHALAND IKO - MAURITIUS|01/04/2026|856311.65||01/01/26 to 31/12/26||1595/26/N||856311.65|23/01/2026|JRNI.260123.385|Non-Motor Corporate","-52.2|449|IKO (MAURITIUS) HOTEL LIMITED T/A CONSTANCE LE CHALAND IKO - MAURITIUS|01/09/2026|||01/01/26 to 31/12/26||1595/26/N/E3||396.8|17/06/2026|JRNI.260617.355|Non-Motor Corporate","-3529.35|23729|MERIDIS FINANCIAL SOLUTIONS LTD|01/09/2026|||04/05/26 to 30/04/27|POL-F-PI-Jun-26-23|16950/26/N|POL-F-PI-Jun-26-23|20199.65|30/06/2026|JRNI.260630.583|Financial","-8579.52|71896.01|LABELLE VICTOIRE Marie Cindy Anabelle|31/07/2026|||01/06/26 to 31/05/27|MED/2026/00624|MED/2026/00624/N|MED/2026/00624|63316.49|30/06/2026|JRNNHZ.260630.280|Medical","-3969.76|49622|VISIONWAY LTD|01/08/2026|||01/09/25 to 31/08/26|MD16M00704|MD16M00704/R9|MD16M00704|45652.24|30/06/2026|JRNNHZ.260630.553|Medical","-11250|75507|RIVALLAND CHRISTIAN ROBERT XAVIER|01/05/2026|64257||09/02/26 to 30/04/27|POL-MV-Feb-26-32|3064/26/N|POL-MV-Feb-26-32|64257|09/02/2026|JRNI.260209.147|Motor","-2808|336.96|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E7|MED/2025/00586|-2471.04|03/04/2026|JRNNHZ.260403.10|Medical","-5709.6|685.15|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E6|MED/2025/00586|-5024.45|09/03/2026|JRNNHZ.260309.114|Medical","-2808|336.96|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E7|MED/2025/00586|-2471.04|03/04/2026|JRNNHZ.260403.10|Medical","-22270.08|280324.64|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|31/10/2026||Payment done after 30.06.2026|01/05/26 to 30/04/27|MED/2025/00586|MED/2025/00586/R1|MED/2025/00586|248010.54|19/05/2026|JRNNHZ.260519.212|Medical","-5709.6|685.15|QOVOLTIS LIMITEE QOVOLTIS LIMITEE|30/06/2025|||01/05/25 to 30/04/26|MED/2025/00586|MED/2025/00586/N/E6|MED/2025/00586|-5024.45|09/03/2026|JRNNHZ.260309.114|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.35|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.34|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.33|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.32|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.31|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.30|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.158|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.157|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.156|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.155|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.154|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.153|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.152|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.151|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.150|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.149|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.148|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.147|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.93|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.92|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.91|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.90|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.89|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.88|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.87|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.86|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.85|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.84|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.83|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.82|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.311|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.310|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.309|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.308|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.307|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.306|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.305|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.304|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.303|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.302|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.301|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.300|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.17|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.16|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.15|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.14|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.13|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.12|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.11|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.10|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.9|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.8|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.7|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.6|Medical"]</t>
+  </si>
+  <si>
+    <t>["-6121|-6121|900|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION)||0||MUR|15/06/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY|||5221||15-06-2026 to 15-08-2026|POL-PL-Nov-25-1105|POL-PL-Nov-25-1105\\E3|121||6000|-5221|","-130114|-130114|19449|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR ECOFUEL LTEE|0|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||15/01/2026|110664.81|19449|01-12-2025 to 01-12-2026|POL-PA-Dec-19-1603\\R6|POL-PA-Dec-19-1603\\R6|453.81|46037/12/R13|129660|-110664.9715994021|","-197263|-197263|36216.93|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR ECOFUEL LTEE|6730.58|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||15/01/2026|206074.31|29486.35|01-12-2025 to 01-12-2026|POL-ARM(P&amp;M)-Dec-19-1132\\R6|POL-ARM(P&amp;M)-Dec-19-1132\\R6|845.07|46037/12/R13|241446.17|-167776.74922762375|","-15329|-15329|2216.63|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT ,SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR DIRECT CONTRACTORS &amp;/OR SUBCONTRACTORS||0||MUR|11/06/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||13112.59||11-06-2026 to 11-09-2026|POL-CAR-TPL-Jun-26-34|POL-CAR-TPL-Jun-26-34|551.72||14777.5|-13112.401812355749|","-3111|-3111|450|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION)|0|0||MUR|16/03/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||15/04/2026|2660.5|450|16-03-2026 to 15-05-2026|POL-PL-Nov-25-1105|POL-PL-Nov-25-1105\\E1|110.5||3000|-2660.9276643626426|","368|368|15750|15|GOLDEN FUND MANAGEMENT SERVICES LTD|15804.73|0|Correction to be done by CBL amount not in aging|MUR|01/05/2019|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PI-CRIME||13/05/2019|90142.5|-54.7299999999996|01-05-2019 to 01-05-2020|POL-C+PI-Jun-19-1002|POL-C+PI-Jun-19-1002|892.5|15398/18/R1|105000|313.2652454139812|","-736|-736|0|15|GOLDEN FUND MANAGEMENT SERVICES LTD|0|0|Correction to be done by CBL amount not in aging|MUR|01/05/2019|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PI-CRIME||13/05/2019|-368|0|01-05-2019 to 01-05-2020|POL-C+PI-Jun-19-1003|POL-C+PI-Jun-19-1003|-368|15398/18/R1|0|-736|","-18271|-18271|2299.8|8|PARIS-ONEZIME MARIE STEPHANIE MRS|837.96|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||09/06/2026|26447.76|1461.84|01-05-2026 to 01-01-2027|POL-HEALTH-Dec-22-157\\R3|POL-HEALTH-Dec-22-157\\R3\\E1|0|MED/2023/00006/R3|28747.56|-16809.323050721523|","-48544|-48544|7735.12|8|PARIS-ONEZIME MARIE STEPHANIE MRS|4641.24|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/12/2025|89353.88|3093.88|01-01-2026 to 01-01-2027|POL-HEALTH-Dec-22-157\\R3|POL-HEALTH-Dec-22-157\\R3|400|MED/2023/00006/R3|96689|-44676.47983520275|","-43082.59|-43082.59|14673.79|15|ROGERS CAPITAL FINANCE LTD ON LEASE TO HEFTY LTD|8240.27|99.18||MUR|04/12/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||09/12/2025|83593.07|6433.52|04-12-2025 to 01-12-2026|POL-MV-Dec-25-503|POL-MV-Dec-25-503|342.39|34294/25|97825.29|-36649.242294414405|","-135220|-135220|20182.35|15|SPICE FINANCE LTD ON FINANCE LEASE TO HEFTY LTD|0.349999999997672|200||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||06/04/2026|115037.58|20182|01-04-2026 to 01-04-2027|POL-MV-Apr-23-97\\R3|POL-MV-Apr-23-97\\R3|470.93|6400/26|134549|-115037.63955209857|","-59581|-59581|8891.1|15|INDUSTRIAL FINANCE CORPORATION OF MAURITIUS LTD (IFCM) ON FINANCE LEASE TO HEFTY LTD|0.1|100||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||06/04/2026|50690.36|8891|01-04-2026 to 01-04-2027|POL-MV-Apr-23-105\\R3|POL-MV-Apr-23-105\\R3|207.46|6368/26|59274|-50689.96864393722|","-120520|-120520|18000|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR SUB-CONTRACTORS|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|102520|18000|01-05-2026 to 31-05-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E3|520|12718/24/N|120000|-102520|","-184322|-184322|27536.85|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB-CONTRACTORS|-0.15|0||MUR|28/04/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|156784.68|27537|28-04-2026 to 31-05-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E4|742.53|12718/24/N|183579|-156785.0797840057|","-123859|-123859|92122.96|15|REHM GRINAKER CONSTRUCTION CO. LTD|92122.96|3000||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||21/01/2026|527179.71|0|01-01-2026 to 01-01-2027|POL-MVF-Jun-21-1026\\R4|POL-MVF-Jun-21-1026\\R4|2149.59|10936/21/R4|614153.08|-105434.63618668073|","-722620|-722620|108000|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB-CONTRACTORS|0|0||MUR|31/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|614620|108000|31-05-2026 to 31-08-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E5|2620|12718/24/N|720000|-614620|","-278797|-278797|44294.4|8|CREDIT GUARANTEE INSURANCE CO LTD|22146.08|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/01/2026|513261.36|22148.32|01-01-2026 to 01-01-2027|POL-HEALTH-Jan-20-22\\R6|POL-HEALTH-Jan-20-22\\R6|3875.76|MD11M00167/10/R5|553680|-256648.2810327706|","-109903|-109903|11704.53|8|CREDIT GUARANTEE INSURANCE CO LTD|2911.85|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/04/2026|134602.04|8792.68|01-03-2026 to 01-01-2027|POL-HEALTH-Jan-20-22\\R6|POL-HEALTH-Jan-20-22\\R6\\E1|0|MD11M00167/10/R5/EQ/4|146306.57|-101110.75669479504|","-4204|-4204|628.35|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|0.35|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||05/05/2026|3575.32|628|01-04-2026 to 01-04-2027|POL-MON-Apr-20-1052\\R6|POL-MON-Apr-20-1052\\R6|14.67|8040/21/R5|4189|-3575.600672745482|","-21300|-21300|3183.83|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.17|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||05/05/2026|18115.96|3184|01-04-2026 to 01-04-2027|POL-EE-Apr-20-1072\\R6|POL-EE-Apr-20-1072\\R6|74.29|8040/21/R5|21225.5|-18116.13860981728|","-3947|-3947|589.95|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.0499999999999272|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||05/05/2026|3356.82|590|01-04-2026 to 01-04-2027|POL-ARMISC-Apr-26-7|POL-ARMISC-Apr-26-7|13.77|8040/21/R5|3933|-3357.0156203680476|","-52448|-52448|7839.71|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.29|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||05/05/2026|44607.96|7840|01-04-2026 to 01-04-2027|POL-EL-Apr-20-1145\\R6|POL-EL-Apr-20-1145\\R6|182.92|8040/21/R5|52264.75|-44608.240672655236|","-197614|-197614|29538.75|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.25|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||05/05/2026|168075.49|29539|01-04-2026 to 01-04-2027|POL-PL-Apr-20-1159\\R6|POL-PL-Apr-20-1159\\R6|689.24|8040/21/R5|196925|-168075.285874439|","-115877|-115877|17320.89|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.11|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||05/05/2026|98555.9|17321|01-04-2026 to 01-04-2027|POL-PA-Apr-20-1141\\R6|POL-PA-Apr-20-1141\\R6|404.16|8040/21/R5|115472.63|-98556.0786098752|","-219576|-219576|48227.25|15|IMPACT PRODUCTION LTD|15592.78|2500||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||30/01/2026|276913.07|32634.47|01-01-2026 to 01-01-2027|POL-MVF-Sep-19-6170\\R7|POL-MVF-Sep-19-6170\\R7|1125.32|49936/17/R8\n54552/15/R10\n19969/21/R5\n30665/22/R4\n49919/17/R8|321515|-187006.84141025634|","-66231|-66231|9900|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|0|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||05/05/2026|56331|9900|01-04-2026 to 01-04-2027|POL-PA-Apr-20-1140\\R6|POL-PA-Apr-20-1140\\R6|231|8040/21/R5|66000|-56331|","-228722|-228722|76806|15|KASA CORPORATE SERVICES LTD|42670.55|800||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||20/02/2026|437826.14|34135.45|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1065\\R4|POL-MVF-Dec-21-1065\\R4|1792.14|32859/23/R2|512040|-194586.5067678828|","16632|16632|-1330.56|8|KASA CORPORATE SERVICES LTD.|0.44|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/03/2026|-15301.44|-1331|01-12-2025 to 01-03-2026|POL-HEALTH-Jun-19-2718\\R48|POL-HEALTH-Jun-19-2718\\R48\\E3|0|MD08M01076/14/R4/EQ/8|-16632|15301.44|","22341|22341|-1787.28|8|KASA CORPORATE SERVICES LTD.|-0.28|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-20553.72|-1787|01-04-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49\\E1|0|MD08M01076/14/R5/EQ/2|-22341|20553.72|","-24663|-24663|1959.36|8|KASA CORPORATE SERVICES LTD.|0.36|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|22703.64|1959|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49\\E2|171|Please refer to POL-HEALTH-Jun-19-2718\\R49 - NO Docs to follow|24492|-22703.64|","-969342|-969342|77008.32|8|KASA CORPORATE SERVICES LTD.|0.320000000009313|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|892333.68|77008|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49|6738|MD08M01076/14/R5 - please refer to POL-HEALTH-Jun-19-2718\\R49\\E2 for adjustment in  premium|962604|-892333.6799999999|","-265806|-265806|79479.3|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|39747.84|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||17/03/2026|452237.22|39731.46|01-03-2026 to 28-02-2027|POL-ARM(P&amp;M)-Mar-20-1019\\R6|POL-ARM(P&amp;M)-Mar-20-1019\\R6|1854.52|8187/26/N|529862|-226074.16165914875|","-40914|-40914|12234.05|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|6118.43|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||17/03/2026|69611.76|6115.62|01-03-2026 to 28-02-2027|POL-PA-Mar-20-1103\\R6|POL-PA-Mar-20-1103\\R6|285.46|8187/26/N|81560.35|-34798.30609092879|","-30023|-30023|8977.5|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|4489.18|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||17/03/2026|51081.97|4488.32|01-03-2026 to 28-02-2027|POL-PPL-Mar-20-1021\\R6|POL-PPL-Mar-20-1021\\R6|209.47|8187/26/N|59850|-25535.25672654121|","-30023|-30023|8977.5|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE &amp;/OR PRINCIPAL &amp;/OR CONTRACTORS &amp;/OR SUB-CONTRACTORS|4489.18|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|EAR &amp; TPL||17/03/2026|51081.98|4488.32|01-03-2026 to 28-02-2027|POL-EAR-TPL-Mar-20-1005\\R6|POL-EAR-TPL-Mar-20-1005\\R6|209.48|8187/26/N|59850|-25535.25747375768|","-8931|-8931|2596.16|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1298.65|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||17/03/2026|15272.17|1297.51|01-03-2026 to 28-02-2027|POL-F&amp;A-Mar-20-1117\\R6|POL-F&amp;A-Mar-20-1117\\R6|560.58|8187/26/N|17307.75|-7633.379855308247|","-11765|-11765|3518.25|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1759.9|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||17/03/2026|20018.87|1758.35|01-03-2026 to 28-02-2027|POL-EE-Mar-20-1049\\R6|POL-EE-Mar-20-1049\\R6|82.12|8187/26/N|23455|-10006.407136896953|","-8998|-8998|2690.78|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1345.52|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||17/03/2026|15310.51|1345.26|01-03-2026 to 28-02-2027|POL-ARMISC-Mar-20-1024\\R6|POL-ARMISC-Mar-20-1024\\R6|62.79|8187/26/N|17938.5|-7653.005366837599|","-893|-893|267.15|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|133.77|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||17/03/2026|1520.08|133.38|01-03-2026 to 28-02-2027|POL-LOP(F&amp;A)-Mar-20-1029\\R6|POL-LOP(F&amp;A)-Mar-20-1029\\R6|6.23|8187/26/N|1781|-759.5169284311477|","-10152|-10152|3035.48|15|GRUES LEVAGES INVESTISSEMENTS (MAURICE) LTEE|1518.42|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||08/05/2026|17271.86|1517.06|01-03-2026 to 28-02-2027|POL-EL-Mar-20-1108\\R6|POL-EL-Mar-20-1108\\R6|70.83|8187/26/N|20236.51|-8634.50962656852|","-12154.99|-12154.99|68082.09|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED  &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE  PROPERTIES LTD &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE  &amp;/OR QUALITY BEVERAGES LIMITED &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR TRAMPOLINE LIMITEE  NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|68082.14|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||06/02/2026|387387.1|-0.0500000000029104|01-01-2026 to 01-01-2027|POL-EE-Jan-26-3|POL-EE-Jan-26-3|1588.61|1918/26/N|453880.58|-10338.100644368502|","-27563|-27563|172922.85|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LTD &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALLI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|172922.99|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||06/02/2026|983931.06|-0.14000000001397|01-01-2026 to 01-01-2027|POL-PA-Mar-20-1106\\R6|POL-PA-Mar-20-1106\\R6|4034.9|1918/26/N|1152819.01|-23442.97025955507|"]</t>
+  </si>
+  <si>
+    <t>["-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.41|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.40|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.39|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.38|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.37|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.36|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.35|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.34|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.33|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.32|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.31|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.30|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.158|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.157|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.156|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.155|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.154|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.153|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.152|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.151|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.150|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.149|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.148|Medical","-1154.63|138.55|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E7|MED/2022/00742|-1016.08|05/03/2026|JRNNHZ.260305.147|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.93|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.92|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.91|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.90|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.89|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.88|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.87|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.86|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.85|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.84|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.83|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E11|MED/2022/00742|-417.2|13/05/2026|JRNNHZ.260513.82|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.311|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.310|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.309|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.308|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.307|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.306|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.305|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.304|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.303|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.302|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.301|Medical","-7.65|0.92|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E10|MED/2022/00742|-6.73|12/05/2026|JRNNHZ.260512.300|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.17|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.16|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.15|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.14|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.13|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.12|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/12/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.11|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/11/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.10|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/10/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.9|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/09/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.8|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/08/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.7|Medical","-474.09|56.89|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/07/2025|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E9|MED/2022/00742|-417.2|24/04/2026|JRNNHZ.260424.6|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/06/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.41|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|31/05/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.40|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.39|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/04/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.38|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|02/03/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.37|Medical","-932.88|111.94|ACENSI (MAURITIUS) LTD ACENSI (MAURITIUS) LTD|30/01/2026|||01/06/25 to 31/05/26|MED/2022/00742|MED/2022/00742/R3/E8|MED/2022/00742|-820.94|08/04/2026|JRNNHZ.260408.36|Medical","-12492.78|154944.97|Gaya Shyamsundur|30/09/2025|16428.91||01/08/25 to 31/07/26|MD08M01060|MD08M01060/R17|MD08M01060|16428.91|26/08/2025|JRNNHZ.250826.22|Medical","-5061.6|42580|COLLET-SERRET MARINE CELIA|30/11/2025|30014.72|Payment done after 30.06.2026|01/10/25 to 30/09/26|MED/2025/01440|MED/2025/01440/N|MED/2025/01440|30014.72|23/01/2026|JRNNHZ.260123.2|Medical","-6314.24|79328|SALEMOHAMED FAWZIA|30/11/2025|13801.66||01/10/25 to 30/09/26|MD06M00609|MD06M00609/R19|MD06M00609|13801.66|03/10/2025|JRNNHZ.251003.167|Medical","-9316.8|78040|BUCARD JOSEPHE MARIE CLAUDE|31/10/2025|14170.45||01/09/25 to 31/08/26|MED/2025/01312|MED/2025/01312/N|MED/2025/01312|14170.45|25/11/2025|JRNNHZ.251125.142|Medical","-5685.78|71572.3|BENZOU LTEE|31/12/2025|19267.44||01/11/25 to 31/10/26|MD18M01126|MD18M01126/R7|MD18M01126|19267.44|18/11/2025|JRNNHZ.251118.72|Medical","-14063.8|176197.6|VETOPHARMA LTD|31/12/2025|69323.69|Payment done after 30.06.2026|01/11/25 to 31/10/26|MED/2024/01200|MED/2024/01200/R1|MED/2024/01200|69323.69|13/01/2026|JRNNHZ.260113.134|Medical","-13858.46|171357.66|Rivaud Marie Josee|30/01/2026|62999.68|Payment done after 30.06.2026|01/12/25 to 30/11/26|MED/2023/01267|MED/2023/01267/R2|MED/2023/01267|62999.68|03/12/2025|JRNNHZ.251203.80|Medical","-21358.72|176800.64|CARR-BROWN ALAN|30/11/2025|46634.61||01/10/25 to 30/09/26|MED/2025/01409|MED/2025/01409/N|MED/2025/01409|46634.61|30/12/2025|JRNNHZ.251230.48|Medical","-20207.28|252591|COMPAGNIE MAURICIENNE DE TEXTILE LTEE|01/07/2026|232383.72||01/12/25 to 30/11/26|MD16M00967|MD16M00967/R9|MD16M00967|232383.72|31/05/2026|JRNNHZ.260531.156|Medical","-20207.28|252591|COMPAGNIE MAURICIENNE DE TEXTILE LTEE|01/08/2026|||01/12/25 to 30/11/26|MD16M00967|MD16M00967/R9|MD16M00967|232383.72|30/06/2026|JRNNHZ.260630.558|Medical","-9015.21|113090.24|VALAYDON-JOSEPHINE RUBBY PA|02/03/2026|51931.06||01/01/26 to 31/12/26|MD18M00171|MD18M00171/R8|MD18M00171|51931.06|14/01/2026|JRNNHZ.260114.35|Medical","-471641.58|3166407.94|Compagnie D`Exploitation Agricole Limitee (CEAL)|28/06/2026|2210635.51|Payment done after 30.06.2026|01/01/26 to 31/12/26||MT200001000114/R26||2662306.14|06/01/2026|JRNI.260106.373|Motor","-25914|3873.6|Compagnie D`Exploitation Agricole Limitee (CEAL)|05/06/2026|||01/01/26 to 31/12/26||MT200001000114/R26/E10||-22040.4|03/06/2026|JRNI.260603.375|Motor"]</t>
+  </si>
+  <si>
+    <t>["-12710|-12710|37735.58|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES &amp;/OR CURRIMJEE LIMITED &amp;/OR  CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR PRINCIPALS &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|37735.3|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||06/02/2026|214715.44|0.279999999998836|01-01-2026 to 01-01-2027|POL-CAR-TPL(BC)-Mar-20-1010\\R6|POL-CAR-TPL(BC)-Mar-20-1010\\R6|880.52|1918/26/N|251570.5|-10810.149400069764|","-19711.99|-19711.99|38186.93|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LIMITEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED  &amp;/OR LATE BAI REHMATBAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASSALI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LIMITED &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LIMITED &amp;/OR QUALITY BEVERAGES LIMITED &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR EMTEL MFS CO LTD &amp;/OR E-SKILLS LIMITED &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LIMITEE &amp;/OR ZAC (PROPERTIES) LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|38186.78|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||06/02/2026|217783.65|0.149999999994179|01-01-2026 to 01-01-2027|POL-PPL-Mar-20-1020\\R6|POL-PPL-Mar-20-1020\\R6|1391.08|1915/26/N|254579.5|-16771.259927463147|","-172|-172|34905.3|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LTD &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR SYNDICAT DES COPROPRIETAIRES DE PHOENIX CENTRAL &amp;/OR FACILICARE LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|34905.52|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||06/02/2026|198611.18|-0.219999999993888|01-01-2026 to 01-01-2027|POL-MON-Mar-20-1043\\R6|POL-MON-Mar-20-1043\\R6|814.48|1918/26/N|232702|-146.28998758460216|","-180668|-180668|29880.75|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LTD &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR SYNDICAT DES COPROPRIETAIRES DE PHOENIX CENTRAL &amp;/OR FACILICARE LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|2889.59|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||16/03/2026|170121.48|26991.16|01-01-2026 to 01-01-2027|POL-MON-Mar-20-1043\\R6|POL-MON-Mar-20-1043\\R6\\E2|797.23|1918/26/N/E1|199205|-153675.82425775955|","229698|229698|-34477.8|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LTD &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE PROPERTIES LIMITED &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD  &amp;/OR SYNDICAT DES COPROPRIETAIRES DE PHOENIX CENTRAL &amp;/OR FACILICARE LTD NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|-128.050000000005|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||16/03/2026|-196078.7|-34349.75|01-01-2026 to 01-01-2027|POL-MON-Mar-20-1043\\R6|POL-MON-Mar-20-1043\\R6\\E1|-704.5|1918/26/N/E1|-229852|195348.58150865405|","-14974.99|-14974.99|108863.66|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED  &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE  PROPERTIES LIMITED  &amp;/OR  LATE BAI REHMATBAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR QUALITY BEVERAGES LIMITED  &amp;/OR CREATIVE ADVERTISING BUREAU LIMITED &amp;/OR CENTRAL DISTRIBUTORS COMPANY LIMITED &amp;/OR SOAP &amp; ALLIED INDUSTRIES LIMITED &amp;/OR EMTEL LTD &amp;/OR EMTEL MFS CO LTD &amp;/OR EMTEL TECHNOPOLIS LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE  NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|108863.22|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||06/02/2026|619434.25|0.44000000001688|01-01-2026 to 01-01-2027|POL-EL-Mar-20-1106\\R6|POL-EL-Mar-20-1106\\R6|2540.16|1918/26/N|725757.75|-12736.576024785652|","-26952|-26952|4013.77|15|CURRIMJEE JEEWANJEE &amp; CO LTD &amp;/OR CURRIMJEE SECRETARIES LTD &amp;/OR CURRIMJEE LIMITED  &amp;/OR CURRIMJEE INFORMATICS LTD &amp;/OR SCREENAGE LTD &amp;/OR CURRIMJEE REAL ESTATE LTD &amp;/OR CIE IMMOBILIERE LTEE &amp;/OR CURRIMJEE JEEWANJEE  PROPERTIES LTD &amp;/OR LATE BAI REHMATABAI WAQF &amp;/OR CURRIMJEE BROTHERS WAQF &amp;/OR ABBASALI SAHEB CHARITABLE TRUST &amp;/OR  BATIMEX LTD &amp;/OR METRIC LIMITED &amp;/OR ISLAND LIFE ASSURANCE CO LTD &amp;/OR SILVER WINGS TRAVEL LTD &amp;/OR FACILICARE LTD &amp;/OR TRAMPOLINE LTEE NOW OR THEREAFTER CONSTITUTED FOR THEIR RESPECTIVE RIGHTS AND INTERESTS|-0.23|0||MUR|05/03/2026|MAURITIUS UNION ASSURANCE CO LTD|ASSETS ALL RISKS &amp; BUSINESS INTERRUPTION||26/05/2026|22938.32|4014|05-03-2026 to 01-01-2027|POL-AAR+BI-Mar-20-1003\\R6|POL-AAR+BI-Mar-20-1003\\R6\\E1|193.65||26758.44|-22938.24340301624|","34442|34442|-2755.38|8|RENTACOLOR (MAURITIUS) LIMITED|-0.38|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-31686.92|-2755|01-05-2026 to 01-01-2027|POL-HEALTH-Jan-21-3\\R5|POL-HEALTH-Jan-21-3\\R5\\E1|0|MD21M00252/0/R5/EQ/2|-34442.3|31686.64399996516|","-366870|-366870|29145.6|8|RENTACOLOR (MAURITIUS) LIMITED|2428.45|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/02/2026|337724.64|26717.15|01-01-2026 to 01-01-2027|POL-HEALTH-Jan-21-3\\R5|POL-HEALTH-Jan-21-3\\R5|2550.24|MD21M00252/0/R5|364320|-337724.41906653426|","-13076|-13076|1569.12|12|MAURITOURS LTD|0.12|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/05/2026|11506.88|1569|01-06-2026 to 01-01-2027|POL-HEALTH-Jan-26-3|POL-HEALTH-Jan-26-3\\E1|0|MED/2023/00018/R3/EQ/1|13076|-11506.880000000001|","-692039|-692039|82467.36|12|MAURITOURS LTD|27441.8|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||07/04/2026|609571.24|55025.56|01-01-2026 to 01-01-2027|POL-HEALTH-Jan-26-3|POL-HEALTH-Jan-26-3|4810.6|MED/2023/00018/R3|687228|-609571.5923336647|","-437069|-437069|69442.56|8|NASSAU SERVICES LTD|34719.69|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|804665.44|34722.87|01-01-2026 to 01-01-2027|POL-HEALTH-Feb-21-10\\R27|POL-HEALTH-Feb-21-10\\R27|6076|MD10M00493/11/R5|868032|-402346.52834130335|","-156592|-156592|31162.5|15|NASSAU SERVICES LTD &amp;/OR UHY HEERALALL &amp;/OR UHY LOSS ADJUSTERS LTD &amp;/OR UHY &amp; CO &amp;/OR UHY ADVISORY LTD &amp;/OR MR. NIRMAL HEERALALL &amp;/OR MR. DOMINIQUE SAMOUILHAN &amp;/OR MR. PRAVESH JAISHINGH PURGASS &amp;/OR MR. BENY KOWLESSUR &amp;/OR MR AVINASHSINGH MOORUTH &amp;/OR MR JEAN THOMAS SAMOUILHAN &amp;/OR CAS SERVICES LTD &amp;/OR UHY CORPORATE FINANCE LTD &amp;/OR MR ANDRE DE COMARMOND &amp;/OR MR VINCENT DESIRE NICOLAS LECORDIER &amp;/OR MR VIVEGAH THOPLAN &amp;/OR MRS SABRINA RAGAVOODOO|7790.1|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY||03/06/2026|177626.25|23372.4|01-06-2026 to 31-05-2027|POL-PI-Jun-21-15\\R5|POL-PI-Jun-21-15\\R5|1038.75|12779/21/R5 3601.902454|207750|-133220.05970149254|","-13812|-13812|1104.96|8|LA PRUDENCE LEASING FINANCE CO. LTD|-0.04|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||02/03/2026|12707.04|1105|01-01-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E2|0|MD11M00166/10/R5/EQ/2|13812|-12707.04|","27051|27051|-2164.08|8|LA PRUDENCE LEASING FINANCE CO. LTD|-0.08|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||14/04/2026|-24886.88|-2164|01-04-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E3|0|MD11M00166/10/R5/EQ/6|-27050.96|24886.91679999527|","37909|37909|-3032.75|8|LA PRUDENCE LEASING FINANCE CO. LTD|0.25|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-34876.57|-3033|01-04-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E6|0|MD11M00166/10/R5/EQ/8|-37909.32|34876.275600037145|","-21675|-21675|1734.04|8|LA PRUDENCE LEASING FINANCE CO. LTD|0.04|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/05/2026|19941.41|1734|01-05-2026 to 01-01-2027|POL-HEALTH-Feb-20-83\\R6|POL-HEALTH-Feb-20-83\\R6\\E5|0|MD11M00166/10/R5/EQ/7|21675.45|-19940.996000083043|","19196|19196|-1535.72|8|NEWREST (MAURITIUS) LTD|0.28|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-17660.74|-1536|01-06-2026 to 01-10-2026|POL-HEALTH-Dec-24-132\\R1|POL-HEALTH-Dec-24-132\\R1\\E3|0|MED/2024/01202/R1/EQ/7|-19196.46|17660.316800076682|","-6048|-6048|483.84|8|NEWREST (MAURITIUS) LTD|-0.16|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||10/02/2026|5564.16|484|01-02-2026 to 01-10-2026|POL-HEALTH-Dec-24-132\\R1|POL-HEALTH-Dec-24-132\\R1\\E2|0|MED/2024/01202/R1/EQ/6|6048|-5564.16|","-6447|-6447|959.67|15|MCB LEASING LIMITED ON LEASE TO JAG SERVICES LTD|-0.33|26.3||MUR|08/12/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/12/2025|5486.84|960|08-12-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E49|22.4|31069/23/R1/E12|6397.81|-5487.257055367943|","52031|52031|-7777.5|15|MCB LEASING LIMITED ON LEASE TO JAG SERVICES LTD|0.5|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||23/02/2026|-44253.98|-7778|01-01-2026 to 01-01-2027|POL-MVF-Jul-19-6113\\R7|POL-MVF-Jul-19-6113\\R7\\E2|-181.48|31069/23/R2/E4|-51850|44253.57174887203|","2|2|12938|15|PANACHE CO LTD|12937.8|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL (BLANKET COVER)||14/09/2019|74114|0.200000000000728|01-07-2019 to 01-07-2020|POL-CAR-TPL(BC)-Jun-19-1024|POL-CAR-TPL(BC)-Jun-19-1024|802|MD07E00472/R12|86250|1.7027523778890779|","-110|-110|1.52|15|PANACHE AND COMPANY LIMITED|-0.48|0||MUR|10/06/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||30/06/2026|108.62|2|10-06-2026 to 30-06-2026|POL-CP-Jun-19-1040\\R6|POL-CP-Jun-19-1040\\R6\\E1|100.04||10.1|-108.48193208643545|","1|1|315|15|PANACHE CO LTD|315.15|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|MONEY||30/09/2019|1792|-0.149999999999977|01-07-2019 to 01-07-2020|POL-MON-Jun-19-1077|POL-MON-Jun-19-1077|7|5180/15/R5|2100|0.8504983388704319|","-1|-1|4703|15|PANACHE CO LTD|4702.35|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||30/09/2019|26756|0.649999999999636|01-07-2019 to 01-07-2020|POL-EL-Jun-19-1236|POL-EL-Jun-19-1236|109|5180/15/R5|31350|-0.8505038303824025|","-2|-2|8100|15|PANACHE CO LTD|8099.7|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||30/09/2019|46089|0.299999999999272|01-07-2019 to 01-07-2020|POL-PA-Jun-19-1304|POL-PA-Jun-19-1304|189|5180/15/R5|54000|-1.7010463378176381|","119807.99|119807.99|-102187.5|15|SCOTT &amp; CO LTD &amp;/OR RIVERSIDE HEALH LTD &amp;/OR SCOTT HEALTH LTD &amp;/OR BAGATELLE HEALTH LTD &amp;/OR GRAND BAIE FORME HEALTH LTD &amp;/OR THE BRANDHOUSE LTD &amp;/OR STANDARD PHARMACY LTD &amp;/OR BEAU VALLON HEALTH LTD &amp;/OR MOBISIL LTD &amp;/OR SCOTT TRIBECA HEALTH LTD &amp;/OR SCOTT AGROW LTD|-84278.57|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|TERRORISM &amp; SABOTAGE||09/04/2026|-584563.89|-17908.93|01-10-2025 to 01-10-2026|POL-TER&amp;SAB-Oct-19-1021\\R6|POL-TER&amp;SAB-Oct-19-1021\\R6\\E1|-5501.39||-681250|101980.75418162765|","-122866|-122866|102187.5|15|SCOTT &amp; CO LTD &amp;/OR RIVERSIDE HEALH LTD &amp;/OR SCOTT HEALTH LTD &amp;/OR BAGATELLE HEALTH LTD &amp;/OR GRAND BAIE FORME HEALTH LTD &amp;/OR THE BRANDHOUSE LTD &amp;/OR STANDARD PHARMACY LTD &amp;/OR BEAU VALLON HEALTH LTD &amp;/OR MOBISIL LTD &amp;/OR SCOTT TRIBECA HEALTH LTD &amp;/OR SCOTT AGROW LTD|83757.06|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|TERRORISM &amp; SABOTAGE||09/04/2026|582468.75|18430.44|01-10-2025 to 01-10-2026|POL-TER&amp;SAB-Oct-19-1021\\R7|POL-TER&amp;SAB-Oct-19-1021\\R7|3406.25|43624/16/R8|681250|-104527.79104477612|","-1|-1|-28.04|15|SCOTT &amp; CO LTD &amp;/OR SCOTT HEALTH LTD &amp;/OR BAGATELLE HEALTH LTD &amp;/OR GRAND BAIE FORME HEALTH LTD &amp;/OR THE BRANDHOUSE LTD &amp;/OR STANDARD PHARMACY LTD &amp;/OR BEAU VALLON HEALTH LTD &amp;/OR MOBISIL LTD &amp;/OR TRIBECA HEALTH LTD|-28.14|0|Correction to be done by CBL amount not in aging|MUR|20/03/2024|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||13/06/2024|-159.55|0.100000000000001|20-03-2024 to 01-10-2024|POL-ARMISC-Jul-19-1112\\R5|POL-ARMISC-Jul-19-1112\\R5\\E2|-0.66|33954/19/R2/E8|-186.93|-0.850525081294312|","-17956|-17956|3578.65|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|894.27|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||18/05/2026|20362.5|2684.38|01-05-2026 to 30-04-2027|POL-EL-Mar-26-19\\R1|POL-EL-Mar-26-19\\R1|83.5|14246/26/R1|23857.65|-15271.991946919843|","-103484|-103484|38642|15|SBM BANK (MAURITIUS) LTD ON LEASE TO HIGHWAY PROPERTIES LTD|23185.21|195.07||MUR|10/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||08/05/2026|220068.02|15456.79|10-04-2026 to 01-04-2027|POL-MV-Apr-26-95|POL-MV-Apr-26-95|901.65|8591/26|257613.3|-88027.20119491313|"]</t>
+  </si>
+  <si>
+    <t>["-4140.15|27762|Compagnie D`Exploitation Agricole Limitee (CEAL)|01/08/2026|||01/01/26 to 31/12/26||MT200001000114/R26/E7||23621.85|14/05/2026|JRNI.260514.24|Motor","-4140.15|27762|Compagnie D`Exploitation Agricole Limitee (CEAL)|01/08/2026|||01/01/26 to 31/12/26||MT200001000114/R26/E6||23621.85|13/05/2026|JRNI.260513.32|Motor","-552.15|3694|Compagnie D`Exploitation Agricole Limitee (CEAL)|01/08/2026|||01/01/26 to 31/12/26|POL-MVF-Jun-19-1892\\R7\\E7|MT200001000114/R26/E8|POL-MVF-Jun-19-1892\\R7\\E7|3141.85|25/05/2026|JRNI.260525.419|Motor","-320037.58|2158926.99|Rey &amp; Lenferna Limited|07/07/2026|1783590.77||01/01/26 to 31/12/26||25114/21/R4||1783590.77|06/01/2026|JRNI.260106.427|Motor","-28900.5|195094|Watertech Limited|01/04/2026|92889.71||01/01/26 to 31/12/26||26138/21/R4||92889.71|06/01/2026|JRNI.260106.451|Motor","-17739.45|118736|Mediterranean Shipping Company (Mauritius) Ltd|01/08/2026|||01/01/26 to 31/12/26||25811/10/R15/E1||100996.55|29/05/2026|JRNI.260529.414|Motor","-43344.15|290372|Mediterranean Shipping Company (Mauritius) Ltd|01/04/2026|79196.93||01/01/26 to 31/12/26||25811/10/R15||79196.93|06/01/2026|JRNI.260106.424|Motor","-10784.22|134411.6|Rajkomar Vimla|02/04/2026|74154.66||01/02/26 to 31/01/27|FD10M00005|FD10M00005/R16|FD10M00005|74154.66|04/02/2026|JRNNHZ.260204.222|Medical","-4776.09|60101.2|SOOPRAMANIEN POTHEGADOO KAVINA|02/04/2026|30095.59|Payment done after 30.06.2026|01/02/26 to 31/01/27|MED/2025/00230|MED/2025/00230/R1|MED/2025/00230|30095.59|09/02/2026|JRNNHZ.260209.67|Medical","-31162.95|208980|LES VUES D ANBALABA|01/04/2026|1455.27||29/12/25 to 31/12/26||712/26/N||1455.27|14/01/2026|JRNI.260114.326|Non-Motor Corporate","-62081.28|781448.12|PREVOIR SOLUTIONS INFORMATIQUES LTD PREVOIR SOLUTIONS INFORMATIQUES LTD|03/03/2026|417733.72|Payment done after 30.06.2026|01/02/26 to 31/01/27|MED/2023/00358|MED/2023/00358/R3|MED/2023/00358|417733.72|19/02/2026|JRNNHZ.260219.64|Medical","-850.2|5888|SKYDIVE AUSTRAL LIMITED|01/04/2026|5037.8||01/02/26 to 31/01/27||1249/26/N||5037.8|21/01/2026|JRNI.260121.25|Motor","-850.2|5888|SKYDIVE AUSTRAL LIMITED|01/08/2026|||01/06/26 to 31/05/27||12179/26/N||5037.8|15/05/2026|JRNI.260515.213|Motor","-142500|954750|Currimjee Group of Companies|14/02/2026|34329.35||01/01/26 to 31/12/26||38813/12/R13||34329.35|21/01/2026|JRNI.260121.345|Financial","-5299.2|44560|ELLAPEN YADHAVANI|02/04/2026|23556.48|Payment done after 30.06.2026|01/02/26 to 31/01/27|MED/2026/00122|MED/2026/00122/N|MED/2026/00122|23556.48|24/02/2026|JRNNHZ.260224.28|Medical","-360712.95|2413670|OMNICANE BIO-ETHANOL OPERATIONS LIMITED|01/09/2026|||01/06/26 to 31/05/27||1772/18/R8||2052957.05|15/06/2026|JRNI.260615.424|Non-Motor Corporate"]</t>
+  </si>
+  <si>
+    <t>["-118107|-118107|17579.51|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.490000000002328|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||11/05/2026|100527.45|17580|01-04-2026 to 30-04-2026|POL-F&amp;A-Mar-26-1018|POL-F&amp;A-Mar-26-1018|910.2|10767/26/N|117196.76|-100527.4840462408|","-983582|-983582|195955.58|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|48988.52|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||18/05/2026|1115487.22|146967.06|01-05-2026 to 30-04-2027|POL-CP-May-26-1008|POL-CP-May-26-1008|5072.3|13781/26/N|1306370.5|-836615.3299419845|","-11265|-11265|1683.84|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.16|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||11/05/2026|9581.04|1684|01-04-2026 to 30-04-2026|POL-LOP(F&amp;A)-Mar-26-3|POL-LOP(F&amp;A)-Mar-26-3|39.29|10767/26/N|11225.59|-9581.142062764982|","-2773|-2773|339.81|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.19|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||11/05/2026|2433.49|340|01-04-2026 to 30-04-2026|POL-PL-Mar-26-21|POL-PL-Mar-26-21|507.93|14246/26/N|2265.37|-2433.2267587350807|","-1528|-1528|228.35|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|0.35|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||11/05/2026|1299.34|228|01-04-2026 to 30-04-2026|POL-EL-Mar-26-19|POL-EL-Mar-26-19|5.33|14246/26/N|1522.36|-1299.6036630468222|","-48874|-48874|9740.63|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|2434.76|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||18/05/2026|55424.18|7305.87|01-05-2026 to 30-04-2027|POL-PA-Mar-26-17\\R1|POL-PA-Mar-26-17\\R1|227.28|14246/26/R1|64937.53|-41568.46883033957|","-1158|-1158|173.1|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|0.1|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||11/05/2026|984.92|173|01-04-2026 to 30-04-2026|POL-EE-Mar-26-8|POL-EE-Mar-26-8|4.04|14246/26/N|1153.98|-984.9029895856721|","-5001|-5001|747.58|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.42|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN||11/05/2026|4253.75|748|01-04-2026 to 30-04-2026|POL-M B-D-Mar-26-1003|POL-M B-D-Mar-26-1003|17.44|14246/26/N|4983.89|-4253.469327158976|","-55317|-55317|10950|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|2737.52|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||18/05/2026|62805.5|8212.48|01-05-2026 to 30-04-2027|POL-PL-Mar-26-21\\R1|POL-PL-Mar-26-21\\R1|755.5|14246/26/R1|73000|-47104.44432618584|","-3819|-3819|570.88|15|HIGHWAY PROPERTIES LTD (LA CITY TRIANON)|-0.12|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||11/05/2026|3248.33|571|01-04-2026 to 30-04-2026|POL-PA-Mar-26-17|POL-PA-Mar-26-17|13.32|14246/26/N|3805.89|-3248.1513899471356|","-440|-440|197.03|15|ACBMS LTD|131.27|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||12/05/2026|1121.07|65.76|01-05-2026 to 01-05-2027|POL-EE-May-22-1007\\R4|POL-EE-May-22-1007\\R4|4.6|12079/22|1313.5|-374.22866246870495|","-400|-400|106.08|15|ACBMS LTD|71.1|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||12/05/2026|1103.6|34.98|01-05-2026 to 01-05-2027|POL-EL-May-22-28\\R4|POL-EL-May-22-28\\R4|502.48|12079/22|707.2|-364.9229548310297|","-6412|-6412|2874.45|15|ACBMS LTD|1916.45|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||12/05/2026|16355.62|958|01-05-2026 to 01-05-2027|POL-PA-May-22-18\\R4|POL-PA-May-22-18\\R4|67.07|12079/22|19163|-5453.554534122861|","-19672|-19672|8819.96|15|ACBMS LTD|5879.48|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||12/05/2026|50185.55|2940.48|01-05-2026 to 01-05-2027|POL-ARMISC-May-22-11\\R4|POL-ARMISC-May-22-11\\R4|205.81|12079/22|58799.7|-16731.4906624822|","-26497|-26497|2119.74|8|GAYA COLLECTIONS LIMITEE|-0.260000000000291|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/06/2026|24376.98|2120|01-06-2026 to 01-05-2027|POL-HEALTH-Aug-23-74\\R4|POL-HEALTH-Aug-23-74\\R4\\E1|0|MED/2023/00969/R3/EQ/1|26496.72|-24377.23759997464|","-140853|-140853|16786.56|8|GAYA COLLECTIONS LIMITEE|5596.22|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/05/2026|194514.44|11190.34|01-05-2026 to 01-05-2027|POL-HEALTH-Aug-23-74\\R4|POL-HEALTH-Aug-23-74\\R4|1469|MED/2023/00969/R3|209832|-129663.09869484763|","3953|3953|-474.36|12|BELLE RIVIERE HOTEL LTD|-474.72|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/05/2026|-3478.64|0.360000000000014|01-04-2026 to 01-05-2026|POL-HEALTH-Sep-21-95\\R4|POL-HEALTH-Sep-21-95\\R4\\E16|0|MED/2025/00947/EQ/40|-3953|3478.64|","-90048|-90048|7203.84|8|BELLE RIVIERE HOTEL LTD|-0.16|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/06/2026|82844.16|7204|01-05-2026 to 01-05-2027|POL-HEALTH-Sep-21-95\\R6|POL-HEALTH-Sep-21-95\\R6\\E2|0|MED/2025/00947/R1/EQ/2|90048|-82844.16|","16176|16176|-1294.08|8|BELLE RIVIERE HOTEL LTD|-0.08|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/06/2026|-14881.92|-1294|01-05-2026 to 01-05-2027|POL-HEALTH-Sep-21-95\\R6|POL-HEALTH-Sep-21-95\\R6\\E1|0|MED/2025/00947/R1/EQ/1|-16176|14881.92|","7164|7164|-859.68|12|BELLE RIVIERE HOTEL LTD|-859.36|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/05/2026|-6304.32|-0.32000000000005|01-03-2026 to 01-05-2026|POL-HEALTH-Sep-21-95\\R4|POL-HEALTH-Sep-21-95\\R4\\E15|0|MED/2025/00947/EQ/39|-7164|6304.32|","1876|1876|-225.12|12|BELLE RIVIERE HOTEL LTD|-0.12|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/04/2026|-1650.88|-225|01-03-2026 to 01-05-2026|POL-HEALTH-Sep-21-95\\R4|POL-HEALTH-Sep-21-95\\R4\\E14|0|MED/2025/00947/EQ/38|-1876|1650.88|","-1749046|-1749046|139007.04|8|BELLE RIVIERE HOTEL LTD|11584|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/07/2026|1610743.96|127423.04|01-05-2026 to 01-05-2027|POL-HEALTH-Sep-21-95\\R6|POL-HEALTH-Sep-21-95\\R6|12163|MED/2025/00947/R1|1737588|-1610094.9679481024|","-32934|-32934|4922.8|15|OSMAN DR REZAH|-0.2|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||30/06/2026|28010.71|4923|01-06-2026 to 01-06-2027|POL-ARMISC-May-20-1035\\R6|POL-ARMISC-May-20-1035\\R6|114.86|3601.902454|32818.65|-28011.12675630384|","-10906|-10906|1562.87|15|OSMAN DR REZAH|-0.13|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||30/06/2026|9342.72|1563|01-06-2026 to 01-06-2027|POL-F&amp;A-May-20-1193\\R6|POL-F&amp;A-May-20-1193\\R6|486.47|3601.902454|10419.12|-9343.071243279823|","123515|123515|-18462.61|15|PARTSIONATE LTD|0.39|0||MUR|11/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||29/06/2026|-105052.25|-18463|11-05-2026 to 01-05-2027|POL-MV-May-26-130|POL-MV-May-26-130\\E1|-430.79|11084/26|-123084.07|105052.36907324349|","38910|38910|-5816.1|15|PARTSIONATE LTD|-0.1|0||MUR|02/06/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||26/06/2026|-33093.58|-5816|02-06-2026 to 01-05-2027|POL-MV-May-26-132|POL-MV-May-26-132\\E1|-135.71|11100/26/N|-38773.97|33093.8521673784|","-590|-590|88.2|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|0.2|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||01/06/2026|501.86|88|01-05-2026 to 01-05-2027|POL-EE-May-23-1015\\R3|POL-EE-May-23-1015\\R3|2.06|3601.902454|588|-501.80896857946647|","-2768|-2768|339|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||01/06/2026|2428.91|339|01-05-2026 to 01-05-2027|POL-F&amp;A-May-20-1192\\R6|POL-F&amp;A-May-20-1192\\R6|507.91|3601.902454|2260|-2428.9889772427573|","-587|-587|87.75|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|-0.25|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN||01/06/2026|499.29|88|01-05-2026 to 01-05-2027|POL-M B-D-May-23-1003\\R3|POL-M B-D-May-23-1003\\R3|2.04|3601.902454|585|-499.255979149632|","1|1|399|15|ASSOCIATION SYNDICALE TROPICA BAIE|399.58|0|Correction to be done by CBL amount not in aging|MUR|01/07/2019|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||31/07/2019|2773|-0.580000000000041|01-07-2019 to 01-07-2020|POL-F&amp;A-Jun-19-1353|POL-F&amp;A-Jun-19-1353|509|19391/18/R1|2663|0.8742118537200505|","-5809|-5809|868.35|15|ASSOCIATION SYNDICALE DU MORCELLEMENT VILLAZE|0.35|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||01/06/2026|4940.91|868|01-05-2026 to 01-05-2027|POL-PL-May-20-1184\\R6|POL-PL-May-20-1184\\R6|20.26|3601.902454|5789|-4940.688863986119|","-67587|-67587|14755.47|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD|4653.23|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||31/08/2020|83958.61|10102.24|01-07-2020 to 01-07-2021|POL-LOP(F&amp;A)-Jul-19-1109\\R1|POL-LOP(F&amp;A)-Jul-19-1109\\R1|344.28|29448/16|98369.8|-57484.30795353611|","-21299|-21299|3376.13|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|192.5|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||31/08/2020|19210.17|3183.63|01-07-2020 to 01-07-2021|POL-EE-Jul-19-1181\\R1|POL-EE-Jul-19-1181\\R1|78.8|29448/16|22507.5|-18115.29160730177|","-52322|-52322|11250|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|3429|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||31/08/2020|64012.5|7821|01-07-2020 to 01-07-2021|POL-PL-Jul-19-1299\\R1|POL-PL-Jul-19-1299\\R1|262.5|29448/16|75000|-44501.07324364723|","-8852|-8852|2883.87|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|1560.7|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||31/08/2020|16409.22|1323.17|01-07-2020 to 01-07-2021|POL-EL-Jul-19-1326\\R1|POL-EL-Jul-19-1326\\R1|67.29|29448/16|19225.8|-7528.831070606108|","170383|170383|25569.86|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD|50914.98|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||31/08/2020|145992.53|-25345.12|01-07-2020 to 01-07-2021|POL-F&amp;A-Jul-19-1410\\R1|POL-F&amp;A-Jul-19-1410\\R1|1096.64|29448/16|170465.75|144988.91767006743|","-20323|-20323|6724.8|15|LES CAMPECHES LTEE &amp;/OR CYNOLOGICS LTD &amp;/OR CYNVIVO LTD|3686.8|0|Correction to be done by CBL amount not in aging|MUR|01/07/2020|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||31/08/2020|38264.12|3038|01-07-2020 to 01-07-2021|POL-PA-Jul-19-1389\\R1|POL-PA-Jul-19-1389\\R1|156.92|29448/16/R4|44832|-17285.182901923406|","-1452|-1452|217.05|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|217.09|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|MACHINERY BREAKDOWN||19/12/2025|1235.04|-0.039999999999992|01-10-2025 to 01-10-2026|POL-M B-D-Dec-19-1066\\R6|POL-M B-D-Dec-19-1066\\R6|5.06|2595/17|1447.03|-1234.963452678553|","-58|-58|7373.44|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|7314.34|0|Correction to be done by CBL amount not in aging|MUR|01/01/2021|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||03/05/2021|42454.85|59.1000000000004|01-01-2021 to 01-01-2022|POL-F&amp;A-Dec-19-1623\\R1|POL-F&amp;A-Dec-19-1623\\R1|672.04|2595/17/R4 voucher not ok|49156.25|-49.41733501189786|","-987|-987|147.52|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|147.05|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||19/12/2025|839.38|0.469999999999999|01-10-2025 to 01-10-2026|POL-EL-Dec-19-1533\\R6|POL-EL-Dec-19-1533\\R6|3.44|2595/17|983.46|-839.4650521836052|","-17425|-17425|2604.6|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|2604.23|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||19/12/2025|14820.17|0.369999999999891|01-10-2025 to 01-10-2026|POL-PL-Dec-19-1523\\R6|POL-PL-Dec-19-1523\\R6|60.77|2595/17|17364|-14820.365620320958|","-57604|-57604|8535.72|15|SYNDICAT DES COPROPRIÉTAIRES DE L’ENSEMBLE IMMOBILIER DÉNOMMÉ LES BARACHOIS DE SINFAT|8535.44|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||19/12/2025|49068.24|0.280000000000655|01-10-2025 to 01-10-2026|POL-F&amp;A-Dec-19-1623\\R6|POL-F&amp;A-Dec-19-1623\\R6|699.17|2595/17|56904.79|-49068.27407282416|","-2785|-2785|408.75|15|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|-0.25|50||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||27/01/2026|2375.79|409|01-02-2026 to 01-02-2027|POL-MV-Dec-24-1525\\R1|POL-MV-Dec-24-1525\\R1|9.54|31164/22|2725|-2376.18247538193|","-947|-947|786393.6|8|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|786318.01|0||MUR|01/10/2022|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/01/2023|9112335.4|75.589999999851|01-10-2022 to 01-10-2023|POL-HEALTH-Nov-21-120\\R1|POL-HEALTH-Nov-21-120\\R1|68809|MED/2021/00123/R1\nMED/2021/00123/R1/EQ/3\nMED/2021/00123/R1/EQ/4|9829920|-871.7666302209102|","-89390|-89390|13346.85|15|IQ EQ GLOBAL BUSINESS (MAURITIUS) LTD|-0.15|100||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||01/06/2026|76043.58|13347|01-06-2026 to 01-06-2027|POL-MV-Dec-24-1523\\R1|POL-MV-Dec-24-1523\\R1|311.43|31169/22|88979|-76043.21420313114|","-2266447|-2266447|1031407.49|15|THE GENERAL CONSTRUCTION COMPANY LIMITED|694454.94|36900||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||28/04/2026|5905608.78|336952.55|01-04-2026 to 01-04-2027|POL-MVF-May-19-1121\\R7|POL-MVF-May-19-1121\\R7|24066.37|MT9900043297/R26/9151/18/ 13764/23/ 13092/25|6876049.9|-1929467.76851147|","-84944|-84944|8462.4|8|DESVAUX DE MARIGNY-MONTOCCHIO MARIE PASCALE ANNE MRS|2539.12|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|97717.6|5923.28|01-05-2026 to 01-05-2027|POL-HEALTH-Jul-21-75\\R5|POL-HEALTH-Jul-21-75\\R5|400|MD21M00643/0/R5|105780|-78174.08|","-65884|-65884|11246.4|12|CHEUNG WILLY SOON MR|3374.32|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||27/04/2026|82873.6|7872.08|01-03-2026 to 01-03-2027|POL-HEALTH-Mar-26-26|POL-HEALTH-Mar-26-26|400|MED/2026/00365|93720|-58011.520000000004|","-27715|-27715|4703.04|12|RAMPUTH NEELESH MR|1410.88|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||16/04/2026|34888.96|3292.16|01-03-2026 to 01-03-2027|POL-HEALTH-Apr-26-28|POL-HEALTH-Apr-26-28|400|MED/2026/00315|39192|-24422.80072741968|","-54338|-54338|7197.12|12|BOODIAH MAUREEN VIVIANNA MRS|719.88|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/04/2026|53178.88|6477.24|01-04-2026 to 01-04-2027|POL-HEALTH-Apr-26-32|POL-HEALTH-Apr-26-32|400|MED/2026/00362|59976|-47860.63968199285|","-36325|-36325|8138.25|15|COMPTOIR OUEST OI LTEE|2718.72|100||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||13/05/2026|46406.64|5419.53|01-05-2026 to 01-05-2027|POL-MV-Apr-25-150\\R1|POL-MV-Apr-25-150\\R1|189.89|11301/25|54255|-30905.208498907963|"]</t>
+  </si>
+  <si>
+    <t>["-62427|-62427|8275.56|12|NOMBRO MARY LYSIE IVY MRS|1654.6|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||04/06/2026|61087.44|6620.96|01-06-2026 to 01-06-2027|POL-HEALTH-Jul-23-49\\R3|POL-HEALTH-Jul-23-49\\R3|400|MED/2023/00781/R3|68963|-54978.96020760348|","-43008|-43008|4165.12|8|PRO WIRE ELECTRICAL &amp; MECHANICAL LTD|757.32|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/06/2026|48398.88|3407.8|01-06-2026 to 01-06-2027|POL-HEALTH-Jul-22-68\\R4|POL-HEALTH-Jul-22-68\\R4|500|MED/2022/00714/R4|52064|-39600.0881028841|","-18666|-18666|2775.13|15|MEDLOG (MAURITIUS) LTD|0.13|0||MUR|24/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||20/05/2026|15890.48|2775|24-04-2026 to 31-07-2026|POL-ARM(P&amp;M)-Jul-21-3\\R4|POL-ARM(P&amp;M)-Jul-21-3\\R4\\E2|164.75|P/10/6D99/21/3262/000/01|18500.86|-15890.812016323067|","-59758|-59758|8902.5|15|SPICE FINANCE LTD ON FINANCIAL LEASE TO G. DE VILLIERS PAINT CONTRACTORS LTD|-0.5|200||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||05/05/2026|50855.23|8903|01-05-2026 to 01-05-2027|POL-MV-Apr-26-119|POL-MV-Apr-26-119|207.73|18193/25|59350|-50855.45977633354|","-89888|-89888|13435.2|12|SAWMYNADEN KISNASAMY POULAY MR|2687.24|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|98924.8|10747.96|01-04-2026 to 01-04-2027|POL-HEALTH-Apr-26-41|POL-HEALTH-Apr-26-41|400|MED/2026/00453|111960|-79139.84|","-33338.5|-33338.5|5286.24|12|HUET LOUISE LILETTE NICOLE|1321.86|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|39165.76|3964.38|01-05-2026 to 01-05-2027|POL-HEALTH-May-26-45|POL-HEALTH-May-26-45|400|MED/2026/00429|44052|-29373.879460091783|","-71848|-71848|10680.48|12|SOORJUN SOTEEHALL MANISHA MRS|2097.77|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||04/06/2026|78723.52|8582.71|01-05-2026 to 01-05-2027|POL-HEALTH-May-26-46|POL-HEALTH-May-26-46|400|MED/2026/00515|89004|-63264.814381459444|","-449|-449|52.21|15|IKO (MAURITIUS) HOTEL LIMITED T/A ANANTARA MAURITIUS RESORTS &amp; VILLAS|0.21|0||MUR|15/05/2026|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||25/06/2026|397.09|52|15-05-2026 to 01-01-2027|POL-FID-Aug-19-1061\\R6|POL-FID-Aug-19-1061\\R6\\E2|101.22|1595/26/N|348.08|-396.82486089472513|","-23536|-23536|3500.34|15|MERIDIS FINANCIAL SOLUTIONS LTD|0.34|0||MUR|04/05/2026|MAURITIUS UNION ASSURANCE CO LTD|PROFESSIONAL INDEMNITY||18/06/2026|20035.27|3500|04-05-2026 to 30-04-2027|POL-F-PI-Jun-26-23|POL-F-PI-Jun-26-23|200|3601.902454 16950/26/N|23335.61|-20035.601997143902|","-71896|-71896|5719.68|8|LABELLE-VICTOIRE MARIE CINDY ANABELLE MRS|0|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/07/2026|66176.32|5719.68|01-06-2026 to 01-06-2027|POL-HEALTH-Jun-26-60|POL-HEALTH-Jun-26-60|400|MED/2026/00624|71496|-66176.32|","-93564|-93564|44603.52|8|VISIONWAY LTD|37170.16|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/09/2025|516842.13|7433.36|01-09-2025 to 01-09-2026|POL-HEALTH-Sep-19-3082\\R6|POL-HEALTH-Sep-19-3082\\R6|3901.65|MD16M00704/5/R4|557544|-86130.89628768162|","-75385|-75385|11250.05|15|MR RIVALLAND CHRISTIAN XAVIER|0.05|122.19||MUR|09/02/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||11/05/2026|64134.94|11250|09-02-2026 to 01-05-2027|POL-MV-Feb-26-32|POL-MV-Feb-26-32|262.5|3064/26|75000.3|-64134.94850765385|","-230178.79|-230178.79|22270.08|8|QOVOLTIS LIMITEE|3983.88|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/05/2026|258054.92|18286.2|01-05-2026 to 01-05-2027|POL-HEALTH-Apr-25-44\\R1|POL-HEALTH-Apr-25-44\\R1|1949|MED/2025/00586/R1|278376|-211892.5148993019|","5709|5709|-682.69|12|ACENSI (MAURITIUS) LTD|0.31|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/06/2026|-5026.29|-683|01-05-2026 to 01-06-2026|POL-HEALTH-Jun-25-54|POL-HEALTH-Jun-25-54\\E10|-19.92|MED/2022/00742/R3/EQ/11|-5689.06|5026.307608364366|","-30957|-30957|12352.4|8|GAYA SHYAMSUNDUR MR|12352.8|0||MUR|01/08/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/10/2025|142452.6|-0.400000000003274|01-08-2025 to 01-08-2026|POL-HEALTH-Aug-23-80\\R2|POL-HEALTH-Aug-23-80\\R2|400|MD08M01060/13/R4|154405|-28486.839173153323|","-19156|-19156|5061.6|12|COLLET-SERRET MARINE CELIA MRS|2784.08|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/01/2026|37518.4|2277.52|01-10-2025 to 01-10-2026|POL-HEALTH-Jul-25-88|POL-HEALTH-Jul-25-88|400|MED/2025/01440|42180|-16878.874363550964|","-15864|-15864|6314.24|8|SALEMOHAMED FAWZIA|5683.2|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||09/10/2025|73013.76|631.039999999999|01-10-2025 to 01-10-2026|POL-HEALTH-Sep-19-3130\\R6|POL-HEALTH-Sep-19-3130\\R6|400|MD06M00609/15/R4|78928|-14601.279354578459|","-23412|-23412|9316.8|12|BUCARD JOSEPHE MARIE CLAUDE MRS|7453.24|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/11/2025|68723.2|1863.56|01-09-2025 to 01-09-2026|POL-HEALTH-Sep-25-102|POL-HEALTH-Sep-25-102|400|FQ/2025/01444|77640|-20616.96|","-21473|-21473|5685.76|8|BENZOU LTD|4548.24|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/11/2025|65886.24|1137.52|01-11-2025 to 01-11-2026|POL-HEALTH-Oct-19-3194\\R6|POL-HEALTH-Oct-19-3194\\R6|500|MD18M01126/2/R5|71072|-19767.160782428884|","-58750.35|-58750.35|14063.84|8|VETOPHARMA LTD|9374.3|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/01/2026|162134.16|4689.54|01-11-2025 to 01-11-2026|POL-HEALTH-Nov-24-125\\R1|POL-HEALTH-Nov-24-125\\R1|400|MED/2024/01200/R1|175798|-54060.9918782052|","-51348|-51348|13660.8|8|RIVAUD MARIE JOSEE MRS|9562.36|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||03/12/2025|157499.2|4098.44|01-12-2025 to 01-12-2026|POL-HEALTH-Nov-23-131\\R2|POL-HEALTH-Nov-23-131\\R2|400|MED/2023/01267/R2|170760|-47249.76|","-35320|-35320|21142.08|12|CARR-BROWN ALAN|19027.52|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/12/2025|155441.92|2114.56|01-10-2025 to 01-10-2026|POL-HEALTH-Nov-25-149|POL-HEALTH-Nov-25-149|400|MED/2025/01409|176184|-31091.20086984098|","-1429694|-1429694|227140.8|8|COMPAGNIE MAURICIENNE DE TEXTILE LTEE|151420.28|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||23/12/2025|2631994.02|75720.5199999999|01-12-2025 to 01-12-2026|POL-HEALTH-May-19-2565\\R47|POL-HEALTH-May-19-2565\\R47|19874.82|MD16M00967/4/R5|2839260|-1316113.5431976167|","-56545|-56545|9015.2|8|VALAYDON-JOSEPHINE RUBBY PAMELA MRS|5409.32|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/01/2026|104074.8|3605.88|01-01-2026 to 01-01-2027|POL-HEALTH-Dec-19-3277\\R6|POL-HEALTH-Dec-19-3277\\R6|400|MD18M00171/3/R5|112690|-52037.4|","-3166408|-3166408|471641.63|15|COMPAGNIE D'EXPLOITATION AGRICOLE LTEE|-0.37|11125||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||21/01/2026|2694765.92|471642|01-01-2026 to 01-01-2027|POL-MVF-Jun-19-1892\\R7|POL-MVF-Jun-19-1892\\R7|11005.05|MT200001000114/R26|3144277.5|-2694766.3029717575|","-2158923|-2158923|320037|15|REY &amp; LENFERNA LTD|0|17875||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||05/02/2026|1838885.58|320037|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1059\\R4|POL-MVF-Dec-21-1059\\R4|7467.58|25114/21/R4|2133580|-1838885.9377395276|","-151740|-151740|28900.5|15|WATERTECH LIMITED|6421.8|1750||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||20/02/2026|166193.86|22478.7|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1066\\R4|POL-MVF-Dec-21-1066\\R4|674.36|26138/21/R4|192670|-129261.84189230278|","-104108|-104108|103281.9|15|MEDITERRANEAN SHIPPING CO (MAURITIUS) LTD|95522.99|1400||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||30/01/2026|589074.02|7758.91|01-01-2026 to 01-01-2027|POL-MVF-Aug-19-6120\\R7|POL-MVF-Aug-19-6120\\R7|2409.92|56113/11/R15\n14598/21/R5\n25811/10/R15|688546|-88577.73336315229|","-67173|-67173|10715.44|8|RAJKOMAR VIMLA MRS|5358.04|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||05/02/2026|123627.56|5357.4|01-02-2026 to 01-02-2027|POL-HEALTH-Apr-24-18\\R2|POL-HEALTH-Apr-24-18\\R2|400|FD10M00005/11/R5|133943|-61815.160357294386|","-30051|-30051|4776.08|8|SOOPRAMANIEN POTHEGADOO KAVINA MRS|2388.08|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||09/02/2026|55324.92|2388|01-02-2026 to 01-02-2027|POL-HEALTH-Feb-25-17\\R1|POL-HEALTH-Feb-25-17\\R1|400|MED/2025/00230/R1|59701|-27662.920266218534|","-1651|-1651|23944.66|15|SYNDICAT DES COPROPRIETAIRES LES VUES D'ANBALABA &amp;/OR ASSOCIATION FONCIÈRE EST “ANBALABA” (AFE ANBALABA)|23697.79|0||MUR|29/12/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||30/01/2026|136395.09|246.870000000003|29-12-2025 to 01-01-2027|POL-F&amp;A-Jan-26-1001|POL-F&amp;A-Jan-26-1001|708.71|712/26/N|159631.04|-1404.444584639804|","-427759|-427759|62081.28|8|PREVOIR SOLUTIONS INFORMATIQUES LTD|28216.43|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/02/2026|722082.91|33864.85|01-02-2026 to 01-02-2027|POL-HEALTH-Feb-23-11\\R3|POL-HEALTH-Feb-23-11\\R3|8148.19|MED/2023/00358/R3|776016|-393893.86487884633|","-5888|-5888|850.2|15|SKYDIVE AUSTRAL LIMITED|0.2|200||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||05/02/2026|5037.64|850|01-02-2026 to 01-02-2027|POL-MV-May-19-2761\\R7|POL-MV-May-19-2761\\R7|19.84|1249/26|5668|-5037.776896111307|","-28889|-28889|4318.2|15|CURRIMJEE GROUP|0.2|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|DIRECTORS &amp; OFFICERS LIABILITY||11/02/2026|24570.56|4318|01-01-2026 to 31-12-2026|POL-D&amp;O-Jan-22-1\\R5|POL-D&amp;O-Jan-22-1\\R5\\E2|100.76|INTERNAL PLACING SLIP|28788|-24570.764125563022|","-22280|-22280|5299.2|12|ELLAPEN YADHAVANI MS|2649.8|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/02/2026|39260.8|2649.4|01-02-2026 to 01-02-2027|POL-HEALTH-Feb-26-11|POL-HEALTH-Feb-26-11|400|MED/2026/00122|44160|-19630.4|","-51355|-2383385.55|7674.53|15|OMNICANE BIO-ETHANOL OPERATIONS LTD &amp;/OR OMNICANE ETHANOL PRODUCTION LTD|-0.47|0|Correction to be done by CBL amount not same as in aging|USD|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||11/06/2026|43680.04|7675|01-06-2026 to 31-05-2027|POL-CP-Jan-20-1001\\R6|POL-CP-Jan-20-1001\\R6|191.07||51163.5|-2027207.6303904792|"]</t>
+  </si>
+  <si>
+    <t>["-2926|-2926|33870.72|8|KASA TEXTILE &amp; CO LTD|33638.02|0||MUR|01/03/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/05/2025|392476.97|232.700000000004|01-03-2025 to 01-03-2026|POL-HEALTH-Jun-19-2719\\R48|POL-HEALTH-Jun-19-2719\\R48|2963.69|MED/2024/00392/R1\nMD08M01085/13/R4|423384|-2693.547170901759|","-68923|-68923|23068.5|15|KASA TEXTILE &amp; CO LTD|12815.38|750||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||20/02/2026|132009.77|10253.12|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1067\\R4|POL-MVF-Dec-21-1067\\R4|538.27|26063/21/R4|153790|-58670.43382486792|","-314174|-314174|37719.36|8|KASA TEXTILE &amp; CO LTD|12760.49|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/05/2026|437072.64|24958.87|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2719\\R49|POL-HEALTH-Jun-19-2719\\R49|3300|MD08M01085/13/R5|471492|-289214.7710984178|","-13131|-13131|1050.48|8|KASA TEXTILE &amp; CO LTD|0.48|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/06/2026|12080.52|1050|01-06-2026 to 01-03-2027|POL-HEALTH-Jun-19-2719\\R49|POL-HEALTH-Jun-19-2719\\R49\\E1|0|MD08M01085/13/R5/EQ/2|13131|-12080.52|","-85498|-85498|12750|15|ERC LEVAGE LTEE|0|0||MUR|30/01/2026|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||17/06/2026|72747.5|12750|30-01-2026 to 30-01-2026|POL-GIT-Jan-26-1|POL-GIT-Jan-26-1|497.5|2217/26/N|85000|-72747.92543641626|","-20270|-20270|3000|15|ERC LEVAGE LTEE|0|0||MUR|17/06/2025|MAURITIUS UNION ASSURANCE CO LTD|INLAND TRANSIT||31/07/2025|17270|3000|17-06-2025 to 17-06-2025|POL-GIT-Jun-25-5|POL-GIT-Jun-25-5|270|20990/25/N|20000|-17270|","-9881440|-9881440|2222028.75|15|ROYAL CAR RENTAL LTD|891753.83|31400||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||30/01/2026|12674744.08|1330274.92|01-01-2026 to 01-01-2027|POL-MVF-Jul-19-6113\\R7|POL-MVF-Jul-19-6113\\R7|51847.8299999998|31069/23 / 31162/23 / 31191/23|14813525|-8407507.087014845|","40842|40842|-6064.8|15|ROYAL CAR RENTAL LTD|0.2|-268||MUR|25/06/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/01/2026|-34776.72|-6065|25-06-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E43|-141.52|31162/23/R1/E35|-40432|34777.128721947665|","7452|7452|-1113.86|15|ROYAL CAR RENTAL LTD|0.140000000000146|0||MUR|26/08/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||09/01/2026|-6337.88|-1114|26-08-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E34|-25.99|31162/23/R1/E25|-7425.75|6338.101136110492|","-10111|-10111|1502.72|15|ROYAL CAR RENTAL LTD|-0.28|57.53||MUR|27/11/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||27/11/2025|8608.01|1503|27-11-2025 to 01-01-2026|POL-MVF-Jul-19-6113\\R6|POL-MVF-Jul-19-6113\\R6\\E47|35.06|31069/23/R1/E10|10018.14|-8608.23987090942|","1028|1028|-168.63|15|LAVASTONE LTD &amp;/OR SUBSIDIARIES &amp;/OR AFFILIATED COMPANIES|0.37|0||MUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||10/10/2025|-859.48|-169|01-10-2024 to 30-09-2025|POL-EL-Oct-19-1469\\R5|POL-EL-Oct-19-1469\\R5\\E1|96.07|33502/19/R5/E1|-1124.18|859.3880421355692|","5077|5077|-758.83|15|LAVASTONE LTD &amp;/OR SUBSIDIARIES &amp;/OR AFFILIATED COMPANIES|0.17|0||MUR|01/10/2024|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||13/10/2025|-4317.73|-759|01-10-2024 to 30-09-2025|POL-PA-Oct-19-1546\\R5|POL-PA-Oct-19-1546\\R5\\E1|-17.71|33502/19/R5/E1|-5058.85|4318.104230029784|","-16533|-16533|1983.95|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.05|0||MUR|01/11/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|14548.96|1984|01-11-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E25|0|MED/2025/01055/EQ/55|16532.91|-14549.039199995645|","-25782|-25782|3093.89|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.11|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|22688.55|3094|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E41|0|MED/2025/01055/EQ/96|25782.44|-22688.162799952217|","7844|7844|-941.33|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.33|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|-6903.12|-941|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E40|0|MED/2025/01055/EQ/94|-7844.45|6902.723999770538|","-6277|-6277|753.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|5523.89|753|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E51|0|MED/2025/01055/EQ/112|6277.15|-5523.758000047792|","-1836|-1836|220.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||05/06/2026|1615.25|220|01-06-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E54|0|MED/2025/01055/EQ/118|1835.51|-1615.681200320347|","-6277|-6277|753.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.26|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||05/06/2026|5523.89|753|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E53|0|MED/2025/01055/EQ/114|6277.15|-5523.758000047792|","-13731|-13731|1647.68|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.32|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|12082.95|1648|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E28|0|MED/2025/01055/EQ/64|13730.63|-12083.275599881434|","3119|3119|-374.24|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.24|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||28/05/2026|-2744.44|-374|01-06-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E52|0|MED/2025/01055/EQ/113|-3118.68|2744.721600164172|","-11074|-11074|1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|9745.31|1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E29|0|MED/2025/01055/EQ/56|11074.22|-9745.116400071518|","-18355|-18355|2202.61|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.39|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|16152.45|2203|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E36|0|MED/2025/01055/EQ/74|18355.06|-16152.397200009153|","-7464|-7464|895.73|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.27|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|6568.66|896|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E43|0|MED/2025/01055/EQ/95|7464.39|-6568.316800167194|","-139140|-139140|16696.8|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.2|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||27/02/2026|122443.2|16697|01-07-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E19|0|MED/2025/01055/EQ/84|139140|-122443.2|","-7274|-7274|872.88|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.12|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|6401.09|873|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E35|0|MED/2025/01055/EQ/81|7273.97|-6401.116399985152|","-11074|-11074|1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/02/2026|9745.31|1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E34|0|MED/2025/01055/EQ/75|11074.22|-9745.116400071518|","11074|11074|-1328.91|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.09|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/02/2026|-9745.31|-1329|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E33|0|MED/2025/01055/EQ/76|-11074.22|9745.116400071518|","-42083|-42083|5049.99|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.01|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|37033.25|5050|01-01-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E37|0|MED/2025/01055/EQ/80|42083.24|-37033.03880000684|","-31700|-31700|3803.97|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.03|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||13/05/2026|27895.75|3804|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E38|0|MED/2025/01055/EQ/72|31699.72|-27895.9963999682|","-2374|-2374|284.94|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.06|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|2089.55|285|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E45|0|MED/2025/01055/EQ/107|2374.49|-2089.118800247632|","24936|24936|-2992.32|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.32|0||MUR|01/07/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/10/2025|-21943.68|-2992|01-07-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E14|0|MED/2025/01055|-24936|21943.68|","-2082|-2082|249.87|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.13|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|1832.41|250|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E46|0|MED/2025/01055/EQ/116|2082.28|-1832.1635995159154|","-9763|-9763|1171.52|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.48|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|8591.15|1172|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E47|0|MED/2025/01055/EQ/102|9762.67|-8591.440400013522|","-6616|-6616|793.93|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.07|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|5822.15|794|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E48|0|MED/2025/01055/EQ/101|6616.08|-5822.079600004837|","-111444|-111444|13373.34|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.34|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/05/2026|98071.15|13373|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E42|0|MED/2025/01055/EQ/97|111444.49|-98070.71880000527|","38769|38769|-4636.02|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.0200000000005821|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|-34132.74|-4636|01-03-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E39|-135.22|MED/2025/01055|-38633.54|34132.951300480076|","53793|53793|-6455.21|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.21|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/02/2026|-47338.2|-6455|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E22|0|MED/2025/01055/EQ/51|-53793.41|47337.8392000061|","31285|31285|-3754.26|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.26|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/02/2026|-27531.21|-3754|01-02-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E30|0|MED/2025/01055/EQ/73|-31285.47|27530.79640005408|","-16585|-16585|1990.24|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.24|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|14595.08|1990|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E50|0|MED/2025/01055/EQ/110|16585.32|-14594.798400030872|","6550|6550|-785.99|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.01|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||22/04/2026|-5763.91|-786|01-05-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E44|0|MED/2025/01055/EQ/99|-6549.9|5763.997999969465|","-41854|-41854|5022.48|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.479999999999418|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/01/2026|36831.55|5022|01-12-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E24|0|MED/2025/01055/EQ/48|41854.03|-36831.52359999742|","18600|18600|-2231.98|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|0.02|0||MUR|01/09/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||07/01/2026|-16367.82|-2232|01-09-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E8|0|MED/2025/01055/EQ/7|-18599.8|16367.99599995699|","-50256|-50256|6030.71|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.29|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||08/06/2026|44225.23|6031|01-04-2026 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E49|0|MED/2025/01055/EQ/111|50255.94|-44225.28280000334|","27159|27159|-3259.13|12|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|-0.13|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/01/2026|-23900.26|-3259|01-10-2025 to 01-07-2026|POL-HEALTH-Sep-24-94\\R1|POL-HEALTH-Sep-24-94\\R1\\E23|0|MED/2025/01055/EQ/47|-27159.39|23899.91680004595|","33030|33030|-3963.6|12|HARDY HENRY SERVICES LTEE|0.4|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-29066.4|-3964|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E7|0|MD18M01064/3/R4/EQ/15|-33030|29066.4|","47208|47208|-5664.96|12|HARDY HENRY SERVICES LTEE|0.04|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-41543.04|-5665|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E9|0|MD18M01064/3/R4/EQ/17|-47208|41543.04|","-1884|-1884|226.08|12|HARDY HENRY SERVICES LTEE|226.16|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||01/07/2026|1657.92|-0.0800000000000125|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E21|0|MD18M01064/3/R4/EQ/43|1884|-1657.92|","-5790|-5790|694.8|12|HARDY HENRY SERVICES LTEE|-0.2|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|5095.2|695|01-01-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E10|0|MD18M01064/3/R4/EQ/18|5790|-5095.2|","-9420|-9420|1130.4|12|HARDY HENRY SERVICES LTEE|0.400000000000146|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|8289.6|1130|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E12|0|MD18M01064/3/R4/EQ/19|9420|-8289.6|","9400|9400|-1128|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/06/2026|-8272|-1128|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E22|0|MD18M01064/3/R4/EQ/42|-9400|8272|","-18840|-18840|2260.8|12|HARDY HENRY SERVICES LTEE|-0.199999999999709|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|16579.2|2261|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E8|0|MD18M01064/3/R4/EQ/16|18840|-16579.2|","-4626|-4626|555.12|12|HARDY HENRY SERVICES LTEE|0.12|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/05/2026|4070.88|555|01-05-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E18|0|MD18M01064/3/R4/EQ/30|4626|-4070.88|","-3900|-3900|468|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||01/03/2026|3432|468|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E13|0|MD18M01064/3/R4/EQ/23|3900|-3432|"]</t>
+  </si>
+  <si>
+    <t>["-23068.5|155078|Kasa Textile &amp; Co Ltd|01/04/2026|73338.2|Payment done after 30.06.2026|01/01/26 to 31/12/26||26063/21/R4||73338.2|06/01/2026|JRNI.260106.450|Motor","-3143.28|39291|Kasa Textile &amp; Co Ltd|01/07/2026|20749.66||01/03/26 to 28/02/27|MD08M01085|MD08M01085/R18|MD08M01085|20749.66|31/05/2026|JRNNHZ.260531.65|Medical","-3260|40750|Kasa Textile &amp; Co Ltd|01/08/2026|||01/03/26 to 28/02/27|MD08M01085|MD08M01085/R18|MD08M01085|37490|30/06/2026|JRNNHZ.260630.468|Medical","-6750|45358|ERC Levage Ltee|12/06/2026|38608|Payment done after 30.06.2026|11/05/26 to 11/05/26|POL-GIT-May-26-18|11642/26/N|POL-GIT-May-26-18|38608|12/05/2026|JRNI.260512.238|Inland Transit","-1024.8|7156|Royal Car Rental Ltd|01/02/2026|6131.2||17/10/25 to 31/10/26||32587/25/N||6131.2|20/11/2025|JRNI.251120.318|Non-Motor Corporate","-1292958.7|8666994|Royal Car Rental Ltd|15/10/2026|2938487.62||01/01/26 to 31/12/26||31162/23/R2||5167497.43|06/01/2026|JRNI.260106.423|Motor","-37642|5726.65|Lavastone Ltd &amp;/or Subsidiaries|09/01/2026|100||01/10/25 to 30/09/26||33502/19/R6/E1||-31915.35|08/01/2026|JRNI.260108.274|Non-Motor Corporate","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.38|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.37|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|5666.25||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|5666.25|10/03/2026|JRNNHZ.260310.36|Medical","-772.66|6438.91|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|3327.96||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E89|MED/2025/01055|3327.96|10/03/2026|JRNNHZ.260310.35|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.252|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.251|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|57.63||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|57.63|25/06/2026|JRNNHZ.260625.250|Medical","-96.2|801.72|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|10/03/2026|705.52||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E121|MED/2025/01055|705.52|25/06/2026|JRNNHZ.260625.248|Medical","-68.64|572.05|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/03/2026|75.26||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E78|MED/2025/01055|75.26|19/02/2026|JRNNHZ.260219.82|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/03/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.61|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/02/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.60|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/01/2026|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.59|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/12/2025|1624.17||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.17|19/02/2026|JRNNHZ.260219.58|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.57|Medical","-221.48|1845.7|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/10/2025|1624.22||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E75|MED/2025/01055|1624.22|19/02/2026|JRNNHZ.260219.56|Medical","-367.1|3059.17|PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD PUBLICIS PRODIGIOUS BRAND LOGISTICS LTD|15/11/2025|2692.07||01/07/25 to 30/06/26|MED/2025/01055|MED/2025/01055/N/E74|MED/2025/01055|2692.07|19/02/2026|JRNNHZ.260219.37|Medical","-3396.48|28304|HARDY HENRY &amp; CIE LTEE|01/08/2026||Payment done after 30.06.2026|01/10/25 to 30/06/26|MED/2023/01269|MED/2023/01269/R2|MED/2023/01269|24907.52|30/06/2026|JRNNHZ.260630.789|Medical","-62149.68|517914|Hardy Henry Services Ltd|01/08/2026|||01/10/25 to 30/06/26|MD18M01064|MD18M01064/R7|MD18M01064|455764.32|30/06/2026|JRNNHZ.260630.599|Medical","-1014.36|8453|HARDY HENRY &amp; CIE LTEE|01/08/2026|||01/10/25 to 30/06/26|MD18M01063|MD18M01063/R7|MD18M01063|7438.64|30/06/2026|JRNNHZ.260630.598|Medical","-17714.88|147624|HARDY HENRY MANAGEMENT LTD|01/08/2026|||01/10/25 to 30/06/26|MD18M01062|MD18M01062/R7|MD18M01062|129909.12|30/06/2026|JRNNHZ.260630.597|Medical","-5604.96|46708|HARDY HENRY TEXTILES LTEE|01/08/2026|||01/10/25 to 30/06/26|MD18M01051|MD18M01051/R7|MD18M01051|41103.04|30/06/2026|JRNNHZ.260630.595|Medical","-195.99|1636|HARDY HENRY TEXTILES LTEE|01/08/2026|||01/10/25 to 30/06/26|MD04M00390|MD04M00390/R22|MD04M00390|1440.01|30/06/2026|JRNNHZ.260630.456|Medical","-3835.92|31966|Hardy Henry Services Ltd|01/08/2026|||01/10/25 to 30/06/26|MD02M00616|MD02M00616/R24|MD02M00616|28130.08|30/06/2026|JRNNHZ.260630.450|Medical","-3396.48|28304|HARDY HENRY &amp; CIE LTEE|01/07/2026|17476.02|Payment done after 30.06.2026|01/10/25 to 30/06/26|MED/2023/01269|MED/2023/01269/R2|MED/2023/01269|17476.02|31/05/2026|JRNNHZ.260531.397|Medical","-63366.36|528053|Hardy Henry Services Ltd|01/07/2026|418832.06||01/10/25 to 30/06/26|MD18M01064|MD18M01064/R7|MD18M01064|418832.06|31/05/2026|JRNNHZ.260531.197|Medical","-17714.88|147624|HARDY HENRY MANAGEMENT LTD|01/07/2026|76436.11||01/10/25 to 30/06/26|MD18M01062|MD18M01062/R7|MD18M01062|76436.11|31/05/2026|JRNNHZ.260531.195|Medical","-5604.96|46708|HARDY HENRY TEXTILES LTEE|01/07/2026|41103.04||01/10/25 to 30/06/26|MD18M01051|MD18M01051/R7|MD18M01051|41103.04|31/05/2026|JRNNHZ.260531.193|Medical","-3835.92|31966|Hardy Henry Services Ltd|01/07/2026|28130.08||01/10/25 to 30/06/26|MD02M00616|MD02M00616/R24|MD02M00616|28130.08|31/05/2026|JRNNHZ.260531.47|Medical","-86931.38|582070.94|H.VAULBERT DE CHANTILLY LTD (HVC LTD)|01/04/2026|495139.56||01/01/26 to 31/12/26||2321/20/R6||495139.56|30/01/2026|JRNI.260130.518|Non-Motor Corporate","-22324.99|1785.99|ORANGE EIGHT LTD ORANGE EIGHT LTD|31/03/2026|||01/10/25 to 30/09/26|MED/2022/01410|MED/2022/01410/R3/E7|MED/2022/01410|-20539|02/06/2026|JRNNHZ.260602.5|Medical","-45701.76|575270.9|ORANGE EIGHT LTD ORANGE EIGHT LTD|31/03/2026|217638.96||01/10/25 to 30/09/26|MED/2022/01410|MED/2022/01410/R3|MED/2022/01410|217638.96|28/11/2025|JRNNHZ.251128.28|Medical","-3865.35|26359|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/04/2026|22493.65||01/02/26 to 31/01/27||6162/25/R2||22493.65|28/01/2026|JRNI.260128.450|Non-Motor Corporate","-750|5118|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/08/2026|||16/11/25 to 15/06/26||36726/25/N/E2||4368|13/05/2026|JRNI.260513.284|Car/Ear (One Off)","-74398.8|498228|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/03/2026|278436.63||01/12/25 to 30/11/26||46037/12/R13||278436.63|30/12/2025|JRNI.251230.598|Non-Motor Corporate","-900|6121|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/09/2026|||16/11/25 to 15/08/26||36731/25/N/E3||5221|29/06/2026|JRNI.260629.604|Non-Motor Corporate","-450|3111|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/07/2026|2661||16/11/25 to 15/05/26||36731/25/N/E1||2661|23/04/2026|JRNI.260423.350|Non-Motor Corporate","-2756.85|18543|COMPAGNIE REGIONALE DE SERVICES ET DE L`ENVIRONNEMENT LTEE|01/02/2026|9278.51||16/10/23 to 15/10/26||27489/23/N/E2||9278.51|28/11/2025|JRNI.251128.356|Car/Ear (One Off)","-7735.12|97089|Paris Onezime Marie Stephanie|02/03/2026|43569.57||01/01/26 to 31/12/26|MED/2023/00006|MED/2023/00006/R3|MED/2023/00006|43569.57|29/12/2025|JRNNHZ.251229.18|Medical","-2299.8|28747.56|Paris Onezime Marie Stephanie|02/03/2026|4969.88||01/01/26 to 31/12/26|MED/2023/00006|MED/2023/00006/R3/E1|MED/2023/00006|4969.88|22/05/2026|JRNNHZ.260522.141|Medical","-20182.35|135220|Hefty Ltd|01/06/2026|115037.65||01/04/26 to 31/03/27||6400/26/N||115037.65|20/03/2026|JRNI.260320.119|Motor","-8891.25|59582|Hefty Ltd|01/06/2026|50690.75||01/04/26 to 31/03/27||6368/26/N||50690.75|20/03/2026|JRNI.260320.18|Motor","-27536.85|184322|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/05/26||12718/24/N/E5||156785.15|30/06/2026|JRNI.260630.570|Car/Ear (One Off)","-18000|120520|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/05/26||12718/24/N/E4||102520|30/06/2026|JRNI.260630.548|Car/Ear (One Off)","-108000|722620|Rehm Grinaker Construction Co Ltd|01/09/2026|||15/04/24 to 31/08/26||12718/24/N/E7||614620|30/06/2026|JRNI.260630.605|Car/Ear (One Off)","-20045.25|134266|Rehm Grinaker Construction Co. Ltd|01/06/2026|114220.75||01/01/26 to 31/12/26||10936/21/R4/E2||114220.75|09/03/2026|JRNI.260309.20|Motor","-44294.4|557555.76|CREDIT GUARANTEE INSURANCE CO LTD|02/03/2026|238039.16||01/01/26 to 31/12/26|MD11M00167|MD11M00167/R15|MD11M00167|238039.16|14/01/2026|JRNNHZ.260114.222|Medical","-589.95|3947|Impact Production Ltd &amp;/or Event Strategy Ltd &amp;/or Mille Feux Ltd &amp;/or Marquee Design Ltd|01/09/2026|||01/04/26 to 31/03/27||8040/21/R5/E1||3357.05|04/06/2026|JRNI.260604.342|Non-Motor Corporate","-68411.52|458172.96|Impact Production Ltd &amp;/or Event Strategy Ltd &amp;/or Mille Feux Ltd &amp;/or Marquee Design Ltd|01/07/2026|389761.44||01/04/26 to 31/03/27||8040/21/R5||389761.44|30/04/2026|JRNI.260430.631|Non-Motor Corporate","-7372.5|49772|IMPACT PRODUCTION LTD|01/04/2026|42399.5||01/01/26 to 31/12/26||54552/15/R10||42399.5|06/01/2026|JRNI.260106.400|Motor","-6255.68|78196|KASA CORPORATE SERVICES LTD|01/07/2026|71940.32||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|71940.32|31/05/2026|JRNNHZ.260531.63|Medical","-13161.28|171425.68|KASA CORPORATE SERVICES LTD|01/06/2026|158264.4||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|158264.4|30/04/2026|JRNNHZ.260430.476|Medical","-76806|514632|KASA CORPORATE SERVICES LTD|01/04/2026|243234.45|Payment done after 30.06.2026|01/01/26 to 31/12/26||32859/23/R2||243234.45|06/01/2026|JRNI.260106.408|Motor","-3986.32|49829|KASA CORPORATE SERVICES LTD|01/08/2026|||01/03/26 to 28/02/27|MD08M01076|MD08M01076/R19|MD08M01076|45842.68|30/06/2026|JRNNHZ.260630.466|Medical"]</t>
+  </si>
+  <si>
+    <t>["Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026"]</t>
+  </si>
+  <si>
+    <t>["Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026","Timing Payment After 30.06.2026"]</t>
+  </si>
+  <si>
+    <t>2026-07-28T09:30:07.256Z</t>
+  </si>
+  <si>
+    <t>["27591|27591|-3310.92|12|HARDY HENRY SERVICES LTEE|0.08|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|-24280.08|-3311|01-04-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E16|0|MD18M01064/3/R4/EQ/28|-27591|24280.08|","-2111|-2111|253.32|12|HARDY HENRY SERVICES LTEE|0.32|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||14/06/2026|1857.68|253|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E20|0|MD18M01064/3/R4/EQ/37|2111|-1857.68|","17780|17780|-2133.6|12|HARDY HENRY SERVICES LTEE|0.4|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||17/12/2025|-15646.4|-2134|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E3|0|MD18M01064/3/R4/EQ/3|-17780|15646.4|","24815|24815|-2977.8|12|HARDY HENRY SERVICES LTEE|0.2|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||31/12/2025|-21837.2|-2978|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E6|0|MD18M01064/3/R4/EQ/12|-24815|21837.2|","6167|6167|-740.04|12|HARDY HENRY SERVICES LTEE|-0.04|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||06/02/2026|-5426.96|-740|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E5|0|MD18M01064/3/R4/EQ/14|-6167|5426.96|","-29379|-29379|3525.48|12|HARDY HENRY SERVICES LTEE|0.48|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||18/12/2025|25853.52|3525|01-12-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E4|0|MD18M01064/3/R4/EQ/10|29379|-25853.52|","-1762|-1762|211.44|12|HARDY HENRY SERVICES LTEE|0.44|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/05/2026|1550.56|211|01-05-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E17|0|MD18M01064/3/R4/EQ/32|1762|-1550.56|","-24687|-24687|2962.44|12|HARDY HENRY SERVICES LTEE|0.44|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||21/12/2025|21724.56|2962|01-10-2025 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E1|0|MD18M01064/3/R4/EQ/9\nMD18M01064/3/R4/EQ/8\nMD02M00616/19/R5/EQ/2|24687|-21724.56|","12700|12700|-1524|12|HARDY HENRY SERVICES LTEE|0|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/02/2026|-11176|-1524|01-02-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E11|0|MD18M01064/3/R4/EQ/21|-12700|11176|","-14180|-14180|1701.6|12|HARDY HENRY SERVICES LTEE|-0.4|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|12478.4|1702|01-03-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E14|0|MD18M01064/3/R4/EQ/25|14180|-12478.4|","13536|13536|-1624.32|12|HARDY HENRY SERVICES LTEE|-0.32|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||15/04/2026|-11911.68|-1624|01-04-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E15|0|MD18M01064/3/R4/EQ/26|-13536|11911.68|","1884|1884|-226.08|12|HARDY HENRY SERVICES LTEE|-0.08|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/06/2026|-1657.92|-226|01-06-2026 to 01-07-2026|POL-HEALTH-Oct-25-129|POL-HEALTH-Oct-25-129\\E19|0|MD18M01064/3/R4/EQ/38|-1884|1657.92|","-17559|-17559|2624.7|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.3|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||12/02/2026|14934.55|2625|01-01-2026 to 01-01-2027|POL-FID-Dec-21-9\\R4|POL-FID-Dec-21-9\\R4|61.25|2321/20/R6|17498|-14934.337369192875|","-22618|-22618|3380.83|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.17|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||12/02/2026|19236.93|3381|01-01-2026 to 01-01-2027|POL-EE-Dec-21-20\\R4|POL-EE-Dec-21-20\\R4|78.88|2321/20/R6|22538.88|-19237.134125572116|","-12042|-12042|1800|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||12/02/2026|10242|1800|01-01-2026 to 01-01-2027|POL-MON-Jan-20-1008\\R6|POL-MON-Jan-20-1008\\R6|42|2321/20/R6|12000|-10242|","-105713|-105713|15801.59|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.41|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||12/02/2026|89911.08|15802|01-01-2026 to 01-01-2027|POL-PA-Mar-20-1110\\R6|POL-PA-Mar-20-1110\\R6|368.71|2321/20/R6|105343.96|-89911.36067266109|","-34386|-34386|5139.87|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.13|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||12/02/2026|29245.89|5140|01-01-2026 to 01-01-2027|POL-EL-Jan-20-1023\\R6|POL-EL-Jan-20-1023\\R6|119.93|2321/20/R6|34265.83|-29246.094125591524|","-120816|-120816|18059.27|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.27|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC &amp; PRODUCTS LIABILITY||12/02/2026|102757.21|18059|01-01-2026 to 01-01-2027|POL-PPL-Jan-20-1005\\R6|POL-PPL-Jan-20-1005\\R6|421.38|2321/20/R6|120395.1|-102756.80174890049|","-136980|-136980|20475.37|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.37|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|LOSS OF PROFITS-REVENUE (FIRE &amp; ALLIED PERILS)||12/02/2026|116504.87|20475|01-01-2026 to 01-01-2027|POL-LOP(F&amp;A)-Jan-20-1009\\R6|POL-LOP(F&amp;A)-Jan-20-1009\\R6|477.76|2321/20/R6|136502.48|-116504.66587443562|","-131417|-131417|19569.12|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|0.12|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||12/02/2026|111848.29|19569|01-01-2026 to 01-01-2027|POL-F&amp;A-Jan-20-1022\\R6|POL-F&amp;A-Jan-20-1022\\R6|956.61|2321/20/R6|130460.8|-111847.94105233089|","-2277|-2277|317.95|15|H. VAULBERT DE CHANTILLY LTD (HVC LTD)|-0.05|0||MUR|20/11/2025|MAURITIUS UNION ASSURANCE CO LTD|FIRE &amp; ALLIED PERILS||09/02/2026|1959.16|318|20-11-2025 to 01-01-2026|POL-F&amp;A-Jan-20-1022\\R5|POL-F&amp;A-Jan-20-1022\\R5\\E1|157.42|2321/20/R5/E2|2119.69|-1959.0653591613932|","-272603|-272603|45701.76|8|ORANGE EIGHT LTD|31739.35|0||MUR|01/10/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||30/11/2025|529569.24|13962.41|01-10-2025 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4|3999|MED/2022/01410/R3|571272|-250946.36011848328|","-30551|-30551|2444.12|8|ORANGE EIGHT LTD|2444.2|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||22/04/2026|28107.35|-0.0799999999999272|01-04-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E1|0|MED/2022/01410/R3/EQ/5|30551.47|-28106.917600036923|","25543|25543|-2043.44|8|ORANGE EIGHT LTD|-2043.88|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||12/05/2026|-23499.6|0.440000000000055|01-05-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E3|0|MED/2022/01410/R3/EQ/6|-25543.04|23499.563199994987|","56735|56735|-4538.8|8|ORANGE EIGHT LTD|-4538.6|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||16/04/2026|-52196.22|-0.199999999999818|01-04-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E2|0|MED/2022/01410/R3/EQ/4|-56735.02|52196.20159999943|","22325|22325|-1786|8|ORANGE EIGHT LTD|-1786|0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||03/06/2026|-20539|0|01-06-2026 to 01-10-2026|POL-HEALTH-Oct-22-131\\R4|POL-HEALTH-Oct-22-131\\R4\\E4|0|MED/2022/01410/R3/EQ/7|-22325|20539|","-26357|-26357|3865.03|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND\nCLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB CONTRACTORS|0.03|0||MUR|01/02/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||02/02/2026|22492.04|3865|01-02-2026 to 01-02-2027|POL-CAR-TPL-Jun-20-1033\\R5|POL-CAR-TPL-Jun-20-1033\\R5|590.18|6162/25|25766.89|-22491.980264877697|","-5118|-5118|750|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR CONTRACTORS &amp;/OR SUB CONTRACTORS||0||MUR|15/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||4367.5||15-05-2026 to 15-06-2026|POL-CAR-TPL-Nov-25-1054|POL-CAR-TPL-Nov-25-1054\\E2|117.5||5000|-4367.926722032243|","-6121|-6121|900|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION)||0||MUR|15/06/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY|||5221||15-06-2026 to 15-08-2026|POL-PL-Nov-25-1105|POL-PL-Nov-25-1105\\E3|121||6000|-5221|","-130114|-130114|19449|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR ECOFUEL LTEE|0|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||15/01/2026|110664.81|19449|01-12-2025 to 01-12-2026|POL-PA-Dec-19-1603\\R6|POL-PA-Dec-19-1603\\R6|453.81|46037/12/R13|129660|-110664.9715994021|","-197263|-197263|36216.93|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR ECOFUEL LTEE|6730.58|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (PLANT &amp; MACHINERY)||15/01/2026|206074.31|29486.35|01-12-2025 to 01-12-2026|POL-ARM(P&amp;M)-Dec-19-1132\\R6|POL-ARM(P&amp;M)-Dec-19-1132\\R6|845.07|46037/12/R13|241446.17|-167776.74922762375|","-15329|-15329|2216.63|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT ,SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION) &amp;/OR DIRECT CONTRACTORS &amp;/OR SUBCONTRACTORS||0||MUR|11/06/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL|||13112.59||11-06-2026 to 11-09-2026|POL-CAR-TPL-Jun-26-34|POL-CAR-TPL-Jun-26-34|551.72||14777.5|-13112.401812355749|","-3111|-3111|450|15|COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE COMPAGNIE REGIONALE DE SERVICES ET DE L'ENVIRONNEMENT LTEE &amp;/OR MINISTRY OF ENVIRONMENT, SOLID WASTE MANAGEMENT AND CLIMATE CHANGE (SOLID WASTE MANAGEMENT DIVISION)|0|0||MUR|16/03/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||15/04/2026|2660.5|450|16-03-2026 to 15-05-2026|POL-PL-Nov-25-1105|POL-PL-Nov-25-1105\\E1|110.5||3000|-2660.9276643626426|","-18271|-18271|2299.8|8|PARIS-ONEZIME MARIE STEPHANIE MRS|837.96|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||09/06/2026|26447.76|1461.84|01-05-2026 to 01-01-2027|POL-HEALTH-Dec-22-157\\R3|POL-HEALTH-Dec-22-157\\R3\\E1|0|MED/2023/00006/R3|28747.56|-16809.323050721523|","-48544|-48544|7735.12|8|PARIS-ONEZIME MARIE STEPHANIE MRS|4641.24|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||29/12/2025|89353.88|3093.88|01-01-2026 to 01-01-2027|POL-HEALTH-Dec-22-157\\R3|POL-HEALTH-Dec-22-157\\R3|400|MED/2023/00006/R3|96689|-44676.47983520275|","-43082.59|-43082.59|14673.79|15|ROGERS CAPITAL FINANCE LTD ON LEASE TO HEFTY LTD|8240.27|99.18||MUR|04/12/2025|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||09/12/2025|83593.07|6433.52|04-12-2025 to 01-12-2026|POL-MV-Dec-25-503|POL-MV-Dec-25-503|342.39|34294/25|97825.29|-36649.242294414405|","-135220|-135220|20182.35|15|SPICE FINANCE LTD ON FINANCE LEASE TO HEFTY LTD|0.349999999997672|200||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||06/04/2026|115037.58|20182|01-04-2026 to 01-04-2027|POL-MV-Apr-23-97\\R3|POL-MV-Apr-23-97\\R3|470.93|6400/26|134549|-115037.63955209857|","-59581|-59581|8891.1|15|INDUSTRIAL FINANCE CORPORATION OF MAURITIUS LTD (IFCM) ON FINANCE LEASE TO HEFTY LTD|0.1|100||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE||06/04/2026|50690.36|8891|01-04-2026 to 01-04-2027|POL-MV-Apr-23-105\\R3|POL-MV-Apr-23-105\\R3|207.46|6368/26|59274|-50689.96864393722|","-120520|-120520|18000|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR SUB-CONTRACTORS|0|0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|102520|18000|01-05-2026 to 31-05-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E3|520|12718/24/N|120000|-102520|","-184322|-184322|27536.85|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB-CONTRACTORS|-0.15|0||MUR|28/04/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|156784.68|27537|28-04-2026 to 31-05-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E4|742.53|12718/24/N|183579|-156785.0797840057|","-123859|-123859|92122.96|15|REHM GRINAKER CONSTRUCTION CO. LTD|92122.96|3000||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||21/01/2026|527179.71|0|01-01-2026 to 01-01-2027|POL-MVF-Jun-21-1026\\R4|POL-MVF-Jun-21-1026\\R4|2149.59|10936/21/R4|614153.08|-105434.63618668073|","-722620|-722620|108000|15|REHM GRINAKER CONSTRUCTION CO. LTD &amp;/OR MILESTONES LTD &amp;/OR DIRECT CONTRACTORS &amp;/OR SUB-CONTRACTORS|0|0||MUR|31/05/2026|MAURITIUS UNION ASSURANCE CO LTD|CAR &amp; TPL||09/06/2026|614620|108000|31-05-2026 to 31-08-2026|POL-CAR-TPL-Apr-24-13|POL-CAR-TPL-Apr-24-13\\E5|2620|12718/24/N|720000|-614620|","-278797|-278797|44294.4|8|CREDIT GUARANTEE INSURANCE CO LTD|22146.08|0||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||20/01/2026|513261.36|22148.32|01-01-2026 to 01-01-2027|POL-HEALTH-Jan-20-22\\R6|POL-HEALTH-Jan-20-22\\R6|3875.76|MD11M00167/10/R5|553680|-256648.2810327706|","-109903|-109903|11704.53|8|CREDIT GUARANTEE INSURANCE CO LTD|2911.85|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||24/04/2026|134602.04|8792.68|01-03-2026 to 01-01-2027|POL-HEALTH-Jan-20-22\\R6|POL-HEALTH-Jan-20-22\\R6\\E1|0|MD11M00167/10/R5/EQ/4|146306.57|-101110.75669479504|","-4204|-4204|628.35|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|0.35|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|MONEY||05/05/2026|3575.32|628|01-04-2026 to 01-04-2027|POL-MON-Apr-20-1052\\R6|POL-MON-Apr-20-1052\\R6|14.67|8040/21/R5|4189|-3575.600672745482|","-21300|-21300|3183.83|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.17|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ELECTRONIC EQUIPMENT||05/05/2026|18115.96|3184|01-04-2026 to 01-04-2027|POL-EE-Apr-20-1072\\R6|POL-EE-Apr-20-1072\\R6|74.29|8040/21/R5|21225.5|-18116.13860981728|","-3947|-3947|589.95|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.0499999999999272|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|ALL RISKS (MISCELLANEOUS)||05/05/2026|3356.82|590|01-04-2026 to 01-04-2027|POL-ARMISC-Apr-26-7|POL-ARMISC-Apr-26-7|13.77|8040/21/R5|3933|-3357.0156203680476|","-52448|-52448|7839.71|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.29|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|EMPLOYERS LIABILITY||05/05/2026|44607.96|7840|01-04-2026 to 01-04-2027|POL-EL-Apr-20-1145\\R6|POL-EL-Apr-20-1145\\R6|182.92|8040/21/R5|52264.75|-44608.240672655236|","-197614|-197614|29538.75|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.25|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||05/05/2026|168075.49|29539|01-04-2026 to 01-04-2027|POL-PL-Apr-20-1159\\R6|POL-PL-Apr-20-1159\\R6|689.24|8040/21/R5|196925|-168075.285874439|"]</t>
+  </si>
+  <si>
+    <t>["-115877|-115877|17320.89|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|-0.11|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||05/05/2026|98555.9|17321|01-04-2026 to 01-04-2027|POL-PA-Apr-20-1141\\R6|POL-PA-Apr-20-1141\\R6|404.16|8040/21/R5|115472.63|-98556.0786098752|","-219576|-219576|48227.25|15|IMPACT PRODUCTION LTD|15592.78|2500||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||30/01/2026|276913.07|32634.47|01-01-2026 to 01-01-2027|POL-MVF-Sep-19-6170\\R7|POL-MVF-Sep-19-6170\\R7|1125.32|49936/17/R8\n54552/15/R10\n19969/21/R5\n30665/22/R4\n49919/17/R8|321515|-187006.84141025634|","-66231|-66231|9900|15|IMPACT PRODUCTION LTD &amp;/OR MILLE FEUX LTÉE &amp;/OR EVENT STRATEGY LTD|0|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PERSONAL ACCIDENT||05/05/2026|56331|9900|01-04-2026 to 01-04-2027|POL-PA-Apr-20-1140\\R6|POL-PA-Apr-20-1140\\R6|231|8040/21/R5|66000|-56331|","-228722|-228722|76806|15|KASA CORPORATE SERVICES LTD|42670.55|800||MUR|01/01/2026|MAURITIUS UNION ASSURANCE CO LTD|MOTOR VEHICLE FLEET||20/02/2026|437826.14|34135.45|01-01-2026 to 01-01-2027|POL-MVF-Dec-21-1065\\R4|POL-MVF-Dec-21-1065\\R4|1792.14|32859/23/R2|512040|-194586.5067678828|","16632|16632|-1330.56|8|KASA CORPORATE SERVICES LTD.|0.44|0||MUR|01/12/2025|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||26/03/2026|-15301.44|-1331|01-12-2025 to 01-03-2026|POL-HEALTH-Jun-19-2718\\R48|POL-HEALTH-Jun-19-2718\\R48\\E3|0|MD08M01076/14/R4/EQ/8|-16632|15301.44|","22341|22341|-1787.28|8|KASA CORPORATE SERVICES LTD.|-0.28|0||MUR|01/04/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||19/06/2026|-20553.72|-1787|01-04-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49\\E1|0|MD08M01076/14/R5/EQ/2|-22341|20553.72|","-24663|-24663|1959.36|8|KASA CORPORATE SERVICES LTD.|0.36|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|22703.64|1959|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49\\E2|171|Please refer to POL-HEALTH-Jun-19-2718\\R49 - NO Docs to follow|24492|-22703.64|","-969342|-969342|77008.32|8|KASA CORPORATE SERVICES LTD.|0.320000000009313|0||MUR|01/03/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||25/05/2026|892333.68|77008|01-03-2026 to 01-03-2027|POL-HEALTH-Jun-19-2718\\R49|POL-HEALTH-Jun-19-2718\\R49|6738|MD08M01076/14/R5 - please refer to POL-HEALTH-Jun-19-2718\\R49\\E2 for adjustment in  premium|962604|-892333.6799999999|"]</t>
+  </si>
+  <si>
+    <t>["-449|-449|52.21|15|IKO (MAURITIUS) HOTEL LIMITED T/A ANANTARA MAURITIUS RESORTS &amp; VILLAS|0.21|0||MUR|15/05/2026|MAURITIUS UNION ASSURANCE CO LTD|FIDELITY GUARANTEE||25/06/2026|397.09|52|15-05-2026 to 01-01-2027|POL-FID-Aug-19-1061\\R6|POL-FID-Aug-19-1061\\R6\\E2|101.22|1595/26/N|348.08|-396.82486089472513|"]</t>
+  </si>
+  <si>
+    <t>["-52.2|449|IKO (MAURITIUS) HOTEL LIMITED T/A CONSTANCE LE CHALAND IKO - MAURITIUS|01/09/2026|||01/01/26 to 31/12/26||1595/26/N/E3||396.8|17/06/2026|JRNI.260617.355|Non-Motor Corporate","-3529.35|23729|MERIDIS FINANCIAL SOLUTIONS LTD|01/09/2026|||04/05/26 to 30/04/27|POL-F-PI-Jun-26-23|16950/26/N|POL-F-PI-Jun-26-23|20199.65|30/06/2026|JRNI.260630.583|Financial"]</t>
+  </si>
+  <si>
+    <t>["Exact match"]</t>
+  </si>
+  <si>
+    <t>["Exact match","Exact match"]</t>
+  </si>
+  <si>
+    <t>exact</t>
+  </si>
+  <si>
+    <t>2026-07-28T09:31:18.630Z</t>
+  </si>
+  <si>
+    <t>["-242123.1|1619804|The General Construction Company Limited|17/06/2026|1377680.9||16/12/24 to 15/12/34||17764/25/N/E1||1377680.9|15/06/2026|JRNI.260615.361|Special"]</t>
+  </si>
+  <si>
+    <t>["Paid in Aug&amp;Sept 25"]</t>
+  </si>
+  <si>
+    <t>allocation_issues</t>
+  </si>
+  <si>
+    <t>2026-07-28T09:33:47.812Z</t>
+  </si>
+  <si>
+    <t>["-4318040|-4318040|0|0|AMAZON SUPPORT SERVICES MUS LIMITED||0||MUR|01/05/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||03/06/2026|4318040||01-05-2026 to 01-01-2027|POL-HEALTH-Jun-26-54|POL-HEALTH-Jun-26-54|30016|MED/2022/00586/R4|4288024|-4318040|","149527|149527|0|0|AMAZON SUPPORT SERVICES MUS LIMITED||0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/06/2026|-149527||01-06-2026 to 01-01-2027|POL-HEALTH-Jun-26-54|POL-HEALTH-Jun-26-54\\E1|0|MED/2022/00586/R4/EQ/3|-149527|149527|"]</t>
+  </si>
+  <si>
+    <t>["MUA account to another client ","MUA account to another client "]</t>
+  </si>
+  <si>
+    <t>2026-07-28T10:31:40.965Z</t>
+  </si>
+  <si>
+    <t>["-150406.35|1006718|IKO (MAURITIUS) HOTEL LIMITED T/A CONSTANCE LE CHALAND IKO - MAURITIUS|01/04/2026|856311.65||01/01/26 to 31/12/26||1595/26/N||856311.65|23/01/2026|JRNI.260123.385|Non-Motor Corporate"]</t>
   </si>
   <si>
     <t>["Error system double"]</t>
   </si>
   <si>
-    <t>2026-07-29T12:11:52.492Z</t>
-  </si>
-  <si>
-    <t>["-89605|-89605|39732.9|15|WESTBYMJ LTD &amp;/OR CHINA JIANGSU CONSTRUCTION GROUP CORPORATION &amp;/OR CONTRACTORS &amp;/OR SUB CONTRACTORS|26438.95|0|MUR|30/06/2025|SANLAM GENERAL INSURANCE LTD|CAR &amp; TPL|09/07/2025|228080.2|13293.95|30-06-2025 to 31-12-2025|POL-CAR-TPL-Jun-23-1039|POL-CAR-TPL-Jun-23-1039\\E4|2927.1|DN5270601225000025|264886|-76311.15252017172|"]</t>
-  </si>
-  <si>
-    <t>["151768.05||WEST BY MJ LTD (SITE A)||07/07/2025||267813|01/05/2023 - 31/12/2025|DN52706012025000025|116044.95|24/11/2025|RC5272025000019|151768.05","417548.44||WEST BY MJ LTD (SITE A)||11/10/2023||497961|11/10/2023 - 31/05/2024|DN52706092023000025|80412.56|11/03/2024|RC0012024000999|417548.44"]</t>
-  </si>
-  <si>
-    <t>[""]</t>
-  </si>
-  <si>
-    <t>["",""]</t>
-  </si>
-  <si>
-    <t>allocation_issues</t>
-  </si>
-  <si>
-    <t>2026-08-03T09:37:13.510Z</t>
+    <t>correction_to_be_done_by_insurer</t>
+  </si>
+  <si>
+    <t>2026-07-28T10:52:18.764Z</t>
+  </si>
+  <si>
+    <t>["-71057.95|1426588|Liquid Telecommunications Holdings Limited &amp;/or its Subsidiaries|30/08/2026|||01/11/25 to 31/10/26||14100/26/N||1355530.05|31/05/2026|JRNI.260531.16|Special","-14781|297110|Liquid Telecommunications Holdings Limited &amp;/or its Subsidiaries|01/09/2026|||01/11/25 to 31/10/26||13982/26/N||282329|01/06/2026|JRNI.260601.426|Non-Motor Corporate"]</t>
+  </si>
+  <si>
+    <t>["Close In July 2026 in Oasis","Close In July 2026 in Oasis"]</t>
+  </si>
+  <si>
+    <t>2026-07-28T11:41:06.755Z</t>
+  </si>
+  <si>
+    <t>["-7549.5|50606|The General Construction Company Limited|01/01/2026|43056.5||01/04/25 to 31/03/26||10359/24/R1/E1||43056.5|01/10/2025|JRNI.251001.326|Non-Motor Corporate","-768028.95|5138114|The General Construction Company Limited|01/07/2026|1456887.07||01/04/26 to 31/03/27||10359/24/R2||1456887.07|16/04/2026|JRNI.260416.322|Non-Motor Corporate","-322312.92|2156773.96|The General Construction Company Limited|01/07/2026|589013.49||01/04/26 to 31/03/27||7186/22/R4||589013.49|16/04/2026|JRNI.260416.317|Non-Motor Corporate","-11576.25|77945|The General Construction Company Limited|01/07/2026|44248.1||01/04/26 to 31/03/27||8694/22/R4||44248.1|15/04/2026|JRNI.260415.201|Non-Motor Corporate"]</t>
+  </si>
+  <si>
+    <t>["Payment done in July 2026","Payment done in July 2026","Payment done in July 2026","Payment done in July 2026"]</t>
+  </si>
+  <si>
+    <t>2026-07-28T11:42:16.529Z</t>
+  </si>
+  <si>
+    <t>["-251449.5|1682697|NATEC MEDICAL LTD|01/10/2025|792773.85||01/07/25 to 30/06/26||19358/23/R2||792773.85|22/07/2025|JRNI.250722.446|Non-Motor Corporate"]</t>
+  </si>
+  <si>
+    <t>["Paid in Aug 2025"]</t>
+  </si>
+  <si>
+    <t>2026-07-28T11:54:31.678Z</t>
+  </si>
+  <si>
+    <t>["under query with insurer"]</t>
+  </si>
+  <si>
+    <t>2026-07-28T12:07:54.190Z</t>
+  </si>
+  <si>
+    <t>["-36417|-36417|5443.56|15|DYOSPOWER LTD &amp;/OR ECOASIS ENERGY SOLUTIONS LTD|5443.06|0||MUR|09/04/2026|MAURITIUS UNION ASSURANCE CO LTD|PUBLIC LIABILITY||18/06/2026|30973.87|0.5|09-04-2026 to 01-04-2027|POL-PL-Apr-26-31|POL-PL-Apr-26-31|127.02||36290.41|-30973.504275013365|","-685061|-685061|102326.01|15|DYOSPOWER LTD &amp;/OR THE MAURITIUS COMMERCIAL BANK LTD &amp;/OR MCB REAL ASSETS LTD &amp;/OR OMNICANE-CALYCÉ JV LTD|102326.02|0||MUR|09/04/2026|MAURITIUS UNION ASSURANCE CO LTD|COMBINED PACKAGE||18/06/2026|582735.01|-0.00999999999476131|09-04-2026 to 01-04-2027|POL-CP-Apr-26-1007|POL-CP-Apr-26-1007|2887.6||682173.42|-582734.9929873546|"]</t>
+  </si>
+  <si>
+    <t>["-107769.3|721477|OMNI PV 1 LTD|01/09/2026|||09/04/26 to 01/04/27||16287/26/N||613707.7|25/06/2026|JRNI.260625.418|Non-Motor Corporate"]</t>
+  </si>
+  <si>
+    <t>2026-07-28T12:23:06.416Z</t>
+  </si>
+  <si>
+    <t>["Insurer Confirm they wrongly allocate"]</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:52:53.127Z</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:53:23.606Z</t>
+  </si>
+  <si>
+    <t>["149527|149527|0|0|AMAZON SUPPORT SERVICES MUS LIMITED||0||MUR|01/06/2026|MAURITIUS UNION ASSURANCE CO LTD|HEALTH||11/06/2026|-149527||01-06-2026 to 01-01-2027|POL-HEALTH-Jun-26-54|POL-HEALTH-Jun-26-54\\E1|0|MED/2022/00586/R4/EQ/3|-149527|149527|"]</t>
+  </si>
+  <si>
+    <t>["MUA account to another client "]</t>
+  </si>
+  <si>
+    <t>2026-07-30T11:55:49.329Z</t>
   </si>
 </sst>
 </file>
@@ -560,7 +788,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:12">
@@ -612,22 +840,22 @@
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J2" t="s">
         <v>16</v>
@@ -644,34 +872,34 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H3" t="s">
+        <v>14</v>
+      </c>
+      <c r="I3" t="s">
         <v>20</v>
       </c>
-      <c r="I3" t="s">
-        <v>13</v>
-      </c>
       <c r="J3" t="s">
+        <v>16</v>
+      </c>
+      <c r="K3" t="s">
         <v>21</v>
-      </c>
-      <c r="K3" t="s">
-        <v>17</v>
       </c>
       <c r="L3" t="s">
         <v>22</v>
@@ -685,31 +913,31 @@
         <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H4" t="s">
         <v>24</v>
       </c>
       <c r="I4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="J4" t="s">
         <v>16</v>
       </c>
       <c r="K4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="L4" t="s">
         <v>25</v>
@@ -720,28 +948,28 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H5" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="I5" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="J5" t="s">
         <v>16</v>
@@ -755,78 +983,78 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="C6" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I6" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="J6" t="s">
         <v>16</v>
       </c>
       <c r="K6" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="L6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I7" t="s">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="J7" t="s">
         <v>16</v>
       </c>
       <c r="K7" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="L7" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -834,37 +1062,37 @@
         <v>12</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>14</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>34</v>
+      </c>
+      <c r="I8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" t="s">
+        <v>16</v>
+      </c>
+      <c r="K8" t="s">
+        <v>35</v>
+      </c>
+      <c r="L8" t="s">
         <v>36</v>
-      </c>
-      <c r="D8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" t="s">
-        <v>37</v>
-      </c>
-      <c r="J8" t="s">
-        <v>21</v>
-      </c>
-      <c r="K8" t="s">
-        <v>17</v>
-      </c>
-      <c r="L8" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -872,80 +1100,80 @@
         <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
         <v>39</v>
-      </c>
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" t="s">
-        <v>13</v>
-      </c>
-      <c r="H9" t="s">
-        <v>13</v>
       </c>
       <c r="I9" t="s">
         <v>40</v>
       </c>
       <c r="J9" t="s">
+        <v>41</v>
+      </c>
+      <c r="K9" t="s">
         <v>21</v>
       </c>
-      <c r="K9" t="s">
-        <v>17</v>
-      </c>
       <c r="L9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
+        <v>44</v>
+      </c>
+      <c r="D10" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" t="s">
+        <v>14</v>
+      </c>
+      <c r="J10" t="s">
+        <v>41</v>
+      </c>
+      <c r="K10" t="s">
+        <v>21</v>
+      </c>
+      <c r="L10" t="s">
         <v>42</v>
-      </c>
-      <c r="D10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" t="s">
-        <v>13</v>
-      </c>
-      <c r="H10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I10" t="s">
-        <v>43</v>
-      </c>
-      <c r="J10" t="s">
-        <v>21</v>
-      </c>
-      <c r="K10" t="s">
-        <v>28</v>
-      </c>
-      <c r="L10" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>30</v>
       </c>
       <c r="B11" t="s">
         <v>45</v>
@@ -954,37 +1182,1329 @@
         <v>46</v>
       </c>
       <c r="D11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H11" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" t="s">
+        <v>41</v>
+      </c>
+      <c r="K11" t="s">
+        <v>21</v>
+      </c>
+      <c r="L11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
         <v>47</v>
       </c>
-      <c r="I11" t="s">
+      <c r="C12" t="s">
         <v>48</v>
       </c>
-      <c r="J11" t="s">
+      <c r="D12" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>14</v>
+      </c>
+      <c r="H12" t="s">
+        <v>14</v>
+      </c>
+      <c r="I12" t="s">
+        <v>14</v>
+      </c>
+      <c r="J12" t="s">
+        <v>41</v>
+      </c>
+      <c r="K12" t="s">
+        <v>21</v>
+      </c>
+      <c r="L12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" t="s">
+        <v>14</v>
+      </c>
+      <c r="G13" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J13" t="s">
+        <v>41</v>
+      </c>
+      <c r="K13" t="s">
+        <v>21</v>
+      </c>
+      <c r="L13" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" t="s">
+        <v>14</v>
+      </c>
+      <c r="F14" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" t="s">
+        <v>14</v>
+      </c>
+      <c r="I14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J14" t="s">
+        <v>41</v>
+      </c>
+      <c r="K14" t="s">
+        <v>21</v>
+      </c>
+      <c r="L14" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" t="s">
+        <v>14</v>
+      </c>
+      <c r="F15" t="s">
+        <v>14</v>
+      </c>
+      <c r="G15" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" t="s">
+        <v>14</v>
+      </c>
+      <c r="J15" t="s">
+        <v>41</v>
+      </c>
+      <c r="K15" t="s">
+        <v>21</v>
+      </c>
+      <c r="L15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" t="s">
+        <v>14</v>
+      </c>
+      <c r="E16" t="s">
+        <v>14</v>
+      </c>
+      <c r="F16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G16" t="s">
+        <v>14</v>
+      </c>
+      <c r="H16" t="s">
+        <v>14</v>
+      </c>
+      <c r="I16" t="s">
+        <v>14</v>
+      </c>
+      <c r="J16" t="s">
+        <v>41</v>
+      </c>
+      <c r="K16" t="s">
+        <v>21</v>
+      </c>
+      <c r="L16" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C17" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" t="s">
+        <v>14</v>
+      </c>
+      <c r="G17" t="s">
+        <v>14</v>
+      </c>
+      <c r="H17" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J17" t="s">
+        <v>41</v>
+      </c>
+      <c r="K17" t="s">
+        <v>21</v>
+      </c>
+      <c r="L17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" t="s">
+        <v>55</v>
+      </c>
+      <c r="C18" t="s">
+        <v>56</v>
+      </c>
+      <c r="D18" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" t="s">
+        <v>14</v>
+      </c>
+      <c r="F18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G18" t="s">
+        <v>14</v>
+      </c>
+      <c r="H18" t="s">
+        <v>57</v>
+      </c>
+      <c r="I18" t="s">
+        <v>58</v>
+      </c>
+      <c r="J18" t="s">
+        <v>41</v>
+      </c>
+      <c r="K18" t="s">
+        <v>17</v>
+      </c>
+      <c r="L18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" t="s">
+        <v>60</v>
+      </c>
+      <c r="C19" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+      <c r="F19" t="s">
+        <v>14</v>
+      </c>
+      <c r="G19" t="s">
+        <v>14</v>
+      </c>
+      <c r="H19" t="s">
+        <v>14</v>
+      </c>
+      <c r="I19" t="s">
+        <v>14</v>
+      </c>
+      <c r="J19" t="s">
+        <v>41</v>
+      </c>
+      <c r="K19" t="s">
+        <v>17</v>
+      </c>
+      <c r="L19" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C20" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" t="s">
+        <v>14</v>
+      </c>
+      <c r="F20" t="s">
+        <v>14</v>
+      </c>
+      <c r="G20" t="s">
+        <v>14</v>
+      </c>
+      <c r="H20" t="s">
+        <v>14</v>
+      </c>
+      <c r="I20" t="s">
+        <v>14</v>
+      </c>
+      <c r="J20" t="s">
+        <v>41</v>
+      </c>
+      <c r="K20" t="s">
+        <v>17</v>
+      </c>
+      <c r="L20" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C21" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>14</v>
+      </c>
+      <c r="G21" t="s">
+        <v>14</v>
+      </c>
+      <c r="H21" t="s">
+        <v>14</v>
+      </c>
+      <c r="I21" t="s">
+        <v>14</v>
+      </c>
+      <c r="J21" t="s">
+        <v>41</v>
+      </c>
+      <c r="K21" t="s">
+        <v>17</v>
+      </c>
+      <c r="L21" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" t="s">
+        <v>66</v>
+      </c>
+      <c r="C22" t="s">
+        <v>14</v>
+      </c>
+      <c r="D22" t="s">
+        <v>14</v>
+      </c>
+      <c r="E22" t="s">
+        <v>14</v>
+      </c>
+      <c r="F22" t="s">
+        <v>14</v>
+      </c>
+      <c r="G22" t="s">
+        <v>14</v>
+      </c>
+      <c r="H22" t="s">
+        <v>14</v>
+      </c>
+      <c r="I22" t="s">
+        <v>14</v>
+      </c>
+      <c r="J22" t="s">
+        <v>41</v>
+      </c>
+      <c r="K22" t="s">
+        <v>17</v>
+      </c>
+      <c r="L22" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" t="s">
+        <v>14</v>
+      </c>
+      <c r="D23" t="s">
+        <v>14</v>
+      </c>
+      <c r="E23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F23" t="s">
+        <v>14</v>
+      </c>
+      <c r="G23" t="s">
+        <v>14</v>
+      </c>
+      <c r="H23" t="s">
+        <v>14</v>
+      </c>
+      <c r="I23" t="s">
+        <v>14</v>
+      </c>
+      <c r="J23" t="s">
+        <v>41</v>
+      </c>
+      <c r="K23" t="s">
+        <v>17</v>
+      </c>
+      <c r="L23" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" t="s">
+        <v>69</v>
+      </c>
+      <c r="D24" t="s">
+        <v>14</v>
+      </c>
+      <c r="E24" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" t="s">
+        <v>14</v>
+      </c>
+      <c r="G24" t="s">
+        <v>14</v>
+      </c>
+      <c r="H24" t="s">
+        <v>70</v>
+      </c>
+      <c r="I24" t="s">
+        <v>71</v>
+      </c>
+      <c r="J24" t="s">
+        <v>41</v>
+      </c>
+      <c r="K24" t="s">
+        <v>28</v>
+      </c>
+      <c r="L24" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D25" t="s">
+        <v>14</v>
+      </c>
+      <c r="E25" t="s">
+        <v>14</v>
+      </c>
+      <c r="F25" t="s">
+        <v>14</v>
+      </c>
+      <c r="G25" t="s">
+        <v>14</v>
+      </c>
+      <c r="H25" t="s">
+        <v>14</v>
+      </c>
+      <c r="I25" t="s">
+        <v>14</v>
+      </c>
+      <c r="J25" t="s">
+        <v>41</v>
+      </c>
+      <c r="K25" t="s">
+        <v>28</v>
+      </c>
+      <c r="L25" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12">
+      <c r="A26" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" t="s">
+        <v>76</v>
+      </c>
+      <c r="D26" t="s">
+        <v>14</v>
+      </c>
+      <c r="E26" t="s">
+        <v>14</v>
+      </c>
+      <c r="F26" t="s">
+        <v>14</v>
+      </c>
+      <c r="G26" t="s">
+        <v>14</v>
+      </c>
+      <c r="H26" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" t="s">
+        <v>14</v>
+      </c>
+      <c r="J26" t="s">
+        <v>41</v>
+      </c>
+      <c r="K26" t="s">
+        <v>28</v>
+      </c>
+      <c r="L26" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12">
+      <c r="A27" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" t="s">
+        <v>77</v>
+      </c>
+      <c r="C27" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" t="s">
+        <v>14</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
+      </c>
+      <c r="F27" t="s">
+        <v>14</v>
+      </c>
+      <c r="G27" t="s">
+        <v>14</v>
+      </c>
+      <c r="H27" t="s">
+        <v>14</v>
+      </c>
+      <c r="I27" t="s">
+        <v>14</v>
+      </c>
+      <c r="J27" t="s">
+        <v>41</v>
+      </c>
+      <c r="K27" t="s">
+        <v>28</v>
+      </c>
+      <c r="L27" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12">
+      <c r="A28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C28" t="s">
+        <v>80</v>
+      </c>
+      <c r="D28" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" t="s">
+        <v>14</v>
+      </c>
+      <c r="F28" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>14</v>
+      </c>
+      <c r="H28" t="s">
+        <v>14</v>
+      </c>
+      <c r="I28" t="s">
+        <v>14</v>
+      </c>
+      <c r="J28" t="s">
+        <v>41</v>
+      </c>
+      <c r="K28" t="s">
+        <v>28</v>
+      </c>
+      <c r="L28" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" t="s">
+        <v>14</v>
+      </c>
+      <c r="E29" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>14</v>
+      </c>
+      <c r="H29" t="s">
+        <v>14</v>
+      </c>
+      <c r="I29" t="s">
+        <v>14</v>
+      </c>
+      <c r="J29" t="s">
+        <v>41</v>
+      </c>
+      <c r="K29" t="s">
+        <v>28</v>
+      </c>
+      <c r="L29" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" t="s">
+        <v>14</v>
+      </c>
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" t="s">
+        <v>14</v>
+      </c>
+      <c r="H30" t="s">
+        <v>14</v>
+      </c>
+      <c r="I30" t="s">
+        <v>14</v>
+      </c>
+      <c r="J30" t="s">
+        <v>41</v>
+      </c>
+      <c r="K30" t="s">
+        <v>28</v>
+      </c>
+      <c r="L30" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
+      <c r="A31" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" t="s">
+        <v>83</v>
+      </c>
+      <c r="C31" t="s">
+        <v>84</v>
+      </c>
+      <c r="D31" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" t="s">
+        <v>14</v>
+      </c>
+      <c r="F31" t="s">
+        <v>14</v>
+      </c>
+      <c r="G31" t="s">
+        <v>14</v>
+      </c>
+      <c r="H31" t="s">
+        <v>85</v>
+      </c>
+      <c r="I31" t="s">
+        <v>86</v>
+      </c>
+      <c r="J31" t="s">
+        <v>41</v>
+      </c>
+      <c r="K31" t="s">
+        <v>21</v>
+      </c>
+      <c r="L31" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12">
+      <c r="A32" t="s">
+        <v>30</v>
+      </c>
+      <c r="B32" t="s">
+        <v>88</v>
+      </c>
+      <c r="C32" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32" t="s">
+        <v>14</v>
+      </c>
+      <c r="F32" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>14</v>
+      </c>
+      <c r="H32" t="s">
+        <v>14</v>
+      </c>
+      <c r="I32" t="s">
+        <v>14</v>
+      </c>
+      <c r="J32" t="s">
+        <v>41</v>
+      </c>
+      <c r="K32" t="s">
+        <v>21</v>
+      </c>
+      <c r="L32" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12">
+      <c r="A33" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" t="s">
+        <v>89</v>
+      </c>
+      <c r="C33" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" t="s">
+        <v>14</v>
+      </c>
+      <c r="E33" t="s">
+        <v>14</v>
+      </c>
+      <c r="F33" t="s">
+        <v>14</v>
+      </c>
+      <c r="G33" t="s">
+        <v>14</v>
+      </c>
+      <c r="H33" t="s">
+        <v>14</v>
+      </c>
+      <c r="I33" t="s">
+        <v>14</v>
+      </c>
+      <c r="J33" t="s">
+        <v>41</v>
+      </c>
+      <c r="K33" t="s">
+        <v>21</v>
+      </c>
+      <c r="L33" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12">
+      <c r="A34" t="s">
+        <v>12</v>
+      </c>
+      <c r="B34" t="s">
+        <v>90</v>
+      </c>
+      <c r="C34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D34" t="s">
+        <v>14</v>
+      </c>
+      <c r="E34" t="s">
+        <v>14</v>
+      </c>
+      <c r="F34" t="s">
+        <v>14</v>
+      </c>
+      <c r="G34" t="s">
+        <v>14</v>
+      </c>
+      <c r="H34" t="s">
+        <v>92</v>
+      </c>
+      <c r="I34" t="s">
+        <v>93</v>
+      </c>
+      <c r="J34" t="s">
+        <v>41</v>
+      </c>
+      <c r="K34" t="s">
+        <v>94</v>
+      </c>
+      <c r="L34" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12">
+      <c r="A35" t="s">
+        <v>12</v>
+      </c>
+      <c r="B35" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" t="s">
+        <v>96</v>
+      </c>
+      <c r="D35" t="s">
+        <v>14</v>
+      </c>
+      <c r="E35" t="s">
+        <v>14</v>
+      </c>
+      <c r="F35" t="s">
+        <v>14</v>
+      </c>
+      <c r="G35" t="s">
+        <v>14</v>
+      </c>
+      <c r="H35" t="s">
+        <v>14</v>
+      </c>
+      <c r="I35" t="s">
+        <v>97</v>
+      </c>
+      <c r="J35" t="s">
+        <v>41</v>
+      </c>
+      <c r="K35" t="s">
+        <v>98</v>
+      </c>
+      <c r="L35" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12">
+      <c r="A36" t="s">
+        <v>12</v>
+      </c>
+      <c r="B36" t="s">
+        <v>100</v>
+      </c>
+      <c r="C36" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" t="s">
+        <v>14</v>
+      </c>
+      <c r="E36" t="s">
+        <v>14</v>
+      </c>
+      <c r="F36" t="s">
+        <v>14</v>
+      </c>
+      <c r="G36" t="s">
+        <v>14</v>
+      </c>
+      <c r="H36" t="s">
+        <v>101</v>
+      </c>
+      <c r="I36" t="s">
+        <v>14</v>
+      </c>
+      <c r="J36" t="s">
         <v>16</v>
       </c>
-      <c r="K11" t="s">
-        <v>49</v>
-      </c>
-      <c r="L11" t="s">
-        <v>50</v>
+      <c r="K36" t="s">
+        <v>35</v>
+      </c>
+      <c r="L36" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12">
+      <c r="A37" t="s">
+        <v>12</v>
+      </c>
+      <c r="B37" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" t="s">
+        <v>103</v>
+      </c>
+      <c r="D37" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" t="s">
+        <v>14</v>
+      </c>
+      <c r="I37" t="s">
+        <v>104</v>
+      </c>
+      <c r="J37" t="s">
+        <v>16</v>
+      </c>
+      <c r="K37" t="s">
+        <v>105</v>
+      </c>
+      <c r="L37" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12">
+      <c r="A38" t="s">
+        <v>12</v>
+      </c>
+      <c r="B38" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" t="s">
+        <v>107</v>
+      </c>
+      <c r="D38" t="s">
+        <v>14</v>
+      </c>
+      <c r="E38" t="s">
+        <v>14</v>
+      </c>
+      <c r="F38" t="s">
+        <v>14</v>
+      </c>
+      <c r="G38" t="s">
+        <v>14</v>
+      </c>
+      <c r="H38" t="s">
+        <v>14</v>
+      </c>
+      <c r="I38" t="s">
+        <v>108</v>
+      </c>
+      <c r="J38" t="s">
+        <v>16</v>
+      </c>
+      <c r="K38" t="s">
+        <v>21</v>
+      </c>
+      <c r="L38" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12">
+      <c r="A39" t="s">
+        <v>12</v>
+      </c>
+      <c r="B39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" t="s">
+        <v>110</v>
+      </c>
+      <c r="D39" t="s">
+        <v>14</v>
+      </c>
+      <c r="E39" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" t="s">
+        <v>14</v>
+      </c>
+      <c r="G39" t="s">
+        <v>14</v>
+      </c>
+      <c r="H39" t="s">
+        <v>14</v>
+      </c>
+      <c r="I39" t="s">
+        <v>111</v>
+      </c>
+      <c r="J39" t="s">
+        <v>16</v>
+      </c>
+      <c r="K39" t="s">
+        <v>21</v>
+      </c>
+      <c r="L39" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12">
+      <c r="A40" t="s">
+        <v>12</v>
+      </c>
+      <c r="B40" t="s">
+        <v>14</v>
+      </c>
+      <c r="C40" t="s">
+        <v>113</v>
+      </c>
+      <c r="D40" t="s">
+        <v>14</v>
+      </c>
+      <c r="E40" t="s">
+        <v>14</v>
+      </c>
+      <c r="F40" t="s">
+        <v>14</v>
+      </c>
+      <c r="G40" t="s">
+        <v>14</v>
+      </c>
+      <c r="H40" t="s">
+        <v>14</v>
+      </c>
+      <c r="I40" t="s">
+        <v>114</v>
+      </c>
+      <c r="J40" t="s">
+        <v>16</v>
+      </c>
+      <c r="K40" t="s">
+        <v>98</v>
+      </c>
+      <c r="L40" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12">
+      <c r="A41" t="s">
+        <v>12</v>
+      </c>
+      <c r="B41" t="s">
+        <v>14</v>
+      </c>
+      <c r="C41" t="s">
+        <v>103</v>
+      </c>
+      <c r="D41" t="s">
+        <v>14</v>
+      </c>
+      <c r="E41" t="s">
+        <v>14</v>
+      </c>
+      <c r="F41" t="s">
+        <v>14</v>
+      </c>
+      <c r="G41" t="s">
+        <v>14</v>
+      </c>
+      <c r="H41" t="s">
+        <v>14</v>
+      </c>
+      <c r="I41" t="s">
+        <v>116</v>
+      </c>
+      <c r="J41" t="s">
+        <v>16</v>
+      </c>
+      <c r="K41" t="s">
+        <v>35</v>
+      </c>
+      <c r="L41" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12">
+      <c r="A42" t="s">
+        <v>12</v>
+      </c>
+      <c r="B42" t="s">
+        <v>118</v>
+      </c>
+      <c r="C42" t="s">
+        <v>119</v>
+      </c>
+      <c r="D42" t="s">
+        <v>14</v>
+      </c>
+      <c r="E42" t="s">
+        <v>14</v>
+      </c>
+      <c r="F42" t="s">
+        <v>14</v>
+      </c>
+      <c r="G42" t="s">
+        <v>14</v>
+      </c>
+      <c r="H42" t="s">
+        <v>93</v>
+      </c>
+      <c r="I42" t="s">
+        <v>92</v>
+      </c>
+      <c r="J42" t="s">
+        <v>16</v>
+      </c>
+      <c r="K42" t="s">
+        <v>94</v>
+      </c>
+      <c r="L42" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12">
+      <c r="A43" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" t="s">
+        <v>14</v>
+      </c>
+      <c r="C43" t="s">
+        <v>103</v>
+      </c>
+      <c r="D43" t="s">
+        <v>14</v>
+      </c>
+      <c r="E43" t="s">
+        <v>14</v>
+      </c>
+      <c r="F43" t="s">
+        <v>14</v>
+      </c>
+      <c r="G43" t="s">
+        <v>14</v>
+      </c>
+      <c r="H43" t="s">
+        <v>14</v>
+      </c>
+      <c r="I43" t="s">
+        <v>121</v>
+      </c>
+      <c r="J43" t="s">
+        <v>35</v>
+      </c>
+      <c r="K43" t="s">
+        <v>98</v>
+      </c>
+      <c r="L43" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12">
+      <c r="A44" t="s">
+        <v>12</v>
+      </c>
+      <c r="B44" t="s">
+        <v>14</v>
+      </c>
+      <c r="C44" t="s">
+        <v>103</v>
+      </c>
+      <c r="D44" t="s">
+        <v>14</v>
+      </c>
+      <c r="E44" t="s">
+        <v>14</v>
+      </c>
+      <c r="F44" t="s">
+        <v>14</v>
+      </c>
+      <c r="G44" t="s">
+        <v>14</v>
+      </c>
+      <c r="H44" t="s">
+        <v>14</v>
+      </c>
+      <c r="I44" t="s">
+        <v>104</v>
+      </c>
+      <c r="J44" t="s">
+        <v>105</v>
+      </c>
+      <c r="K44" t="s">
+        <v>35</v>
+      </c>
+      <c r="L44" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12">
+      <c r="A45" t="s">
+        <v>12</v>
+      </c>
+      <c r="B45" t="s">
+        <v>124</v>
+      </c>
+      <c r="C45" t="s">
+        <v>14</v>
+      </c>
+      <c r="D45" t="s">
+        <v>14</v>
+      </c>
+      <c r="E45" t="s">
+        <v>14</v>
+      </c>
+      <c r="F45" t="s">
+        <v>14</v>
+      </c>
+      <c r="G45" t="s">
+        <v>14</v>
+      </c>
+      <c r="H45" t="s">
+        <v>125</v>
+      </c>
+      <c r="I45" t="s">
+        <v>14</v>
+      </c>
+      <c r="J45" t="s">
+        <v>16</v>
+      </c>
+      <c r="K45" t="s">
+        <v>35</v>
+      </c>
+      <c r="L45" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L11" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L45" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1143,13 +2663,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{83311AB4-90CC-4A04-9265-FD3C26947DC6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0A92803E-9F96-4C31-8492-E7EA1A888A3F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D630CF28-A847-4464-9934-3B22E7B89F3C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FF43559C-BF50-47EF-A62A-63920082D190}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D61E1145-834D-4F65-8504-4F457A2B41BA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{821E4950-752C-4CBC-BCD0-0EE703FCA48F}"/>
 </file>
</xml_diff>